<commit_message>
Update amplitude website 2026-09-07
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4421542aaa514ac5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2d6aea3a74d44825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R28c02c52488f4aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R09092d9c6f384d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rec27dde1fce54c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R340ea6c5a8f3478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc7638fd1891d49c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R2c4dc9f40d194fde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9d9b6b01523a4197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R8a680614cb334464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R6f1c0072f0634882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re507ab25437e49c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ree375e15868f4865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4adb059d8e144c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2353385c41494e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R84b1f49ec91e4023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5b5093134f704f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R8fe77a816e6e46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R47c3c595e6b24fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R8ee50f001cb143c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7717.93</x:v>
+        <x:v>7669.84</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7464.98</x:v>
+        <x:v>7541.14</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>253</x:v>
+        <x:v>128.7</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>570.4</x:v>
+        <x:v>699.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>142.6</x:v>
+        <x:v>139.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7850.4</x:v>
+        <x:v>7791.79</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7610.58</x:v>
+        <x:v>7672.99</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>239.8</x:v>
+        <x:v>118.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>546.6</x:v>
+        <x:v>665.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>136.7</x:v>
+        <x:v>133.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3980.2</x:v>
+        <x:v>3948.42</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3915.22</x:v>
+        <x:v>3916.49</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>65</x:v>
+        <x:v>31.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>155</x:v>
+        <x:v>186.9</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>38.8</x:v>
+        <x:v>37.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7824.2</x:v>
+        <x:v>7784.2</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7568</x:v>
+        <x:v>7651.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>256.2</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>672.4</x:v>
+        <x:v>805.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>168.1</x:v>
+        <x:v>161.1</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4594</x:v>
+        <x:v>4576.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4519</x:v>
+        <x:v>4537.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>75</x:v>
+        <x:v>39.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>237</x:v>
+        <x:v>276.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>59.3</x:v>
+        <x:v>55.3</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2949.4</x:v>
+        <x:v>2931.4</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2904.8</x:v>
+        <x:v>2892.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>44.6</x:v>
+        <x:v>39.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>132.6</x:v>
+        <x:v>171.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>33.2</x:v>
+        <x:v>34.4</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1198,843 +1198,951 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B6" s="28" t="n">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="n">
+        <x:v>7551.02</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7669.84</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7541.14</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7639.36</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:f>ROUND(F6-F5,1)</x:f>
+        <x:v>131.3</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="n">
+        <x:f>IFERROR(F6/F5-1,"")</x:f>
+        <x:v>0.017483807466346146</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="n">
+        <x:f>ROUND(D6-E6,1)</x:f>
+        <x:v>128.7</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="28"/>
-      <x:c r="D6" s="28"/>
-      <x:c r="E6" s="28"/>
-      <x:c r="F6" s="28"/>
-      <x:c r="G6" s="28"/>
-      <x:c r="H6" s="28"/>
-      <x:c r="I6" s="30" t="n">
-        <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>308.1</x:v>
-      </x:c>
-      <x:c r="J6" s="28"/>
-      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B7" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C7" s="28"/>
       <x:c r="D7" s="28"/>
       <x:c r="E7" s="28"/>
       <x:c r="F7" s="28"/>
       <x:c r="G7" s="28"/>
       <x:c r="H7" s="28"/>
-      <x:c r="I7" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>308.1</x:v>
+      <x:c r="I7" s="30" t="n">
+        <x:f>ROUND(SUM(I5:I6),1)</x:f>
+        <x:v>436.8</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="17" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
+        <x:v>218.4</x:v>
+      </x:c>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B9" s="17"/>
-      <x:c r="C9" s="17"/>
-      <x:c r="D9" s="17"/>
-      <x:c r="E9" s="17"/>
-      <x:c r="F9" s="17"/>
-      <x:c r="G9" s="17"/>
-      <x:c r="H9" s="17"/>
-      <x:c r="I9" s="17"/>
-      <x:c r="J9" s="17"/>
-      <x:c r="K9" s="17"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="20" t="str">
+      <x:c r="B10" s="17"/>
+      <x:c r="C10" s="17"/>
+      <x:c r="D10" s="17"/>
+      <x:c r="E10" s="17"/>
+      <x:c r="F10" s="17"/>
+      <x:c r="G10" s="17"/>
+      <x:c r="H10" s="17"/>
+      <x:c r="I10" s="17"/>
+      <x:c r="J10" s="17"/>
+      <x:c r="K10" s="17"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B10" s="20" t="str">
+      <x:c r="B11" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C10" s="20" t="str">
+      <x:c r="C11" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D10" s="20" t="str">
+      <x:c r="D11" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E10" s="20" t="str">
+      <x:c r="E11" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F10" s="20" t="str">
+      <x:c r="F11" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G10" s="20" t="str">
+      <x:c r="G11" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H10" s="20" t="str">
+      <x:c r="H11" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I10" s="20" t="str">
+      <x:c r="I11" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J10" s="20" t="str">
+      <x:c r="J11" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K10" s="20" t="str">
+      <x:c r="K11" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="22" t="n">
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B11" s="22" t="str">
+      <x:c r="B12" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C11" s="23" t="n">
+      <x:c r="C12" s="23" t="n">
         <x:v>7944.29</x:v>
       </x:c>
-      <x:c r="D11" s="23" t="n">
+      <x:c r="D12" s="23" t="n">
         <x:v>7955.57</x:v>
       </x:c>
-      <x:c r="E11" s="23" t="n">
+      <x:c r="E12" s="23" t="n">
         <x:v>7610.58</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="n">
+      <x:c r="F12" s="23" t="n">
         <x:v>7652.69</x:v>
       </x:c>
-      <x:c r="G11" s="23"/>
-      <x:c r="H11" s="24"/>
-      <x:c r="I11" s="26" t="n">
-        <x:f>ROUND(D11-E11,1)</x:f>
+      <x:c r="G12" s="23"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="26" t="n">
+        <x:f>ROUND(D12-E12,1)</x:f>
         <x:v>345</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="str">
+      <x:c r="J12" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="K11" s="22" t="n">
+      <x:c r="K12" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="n">
+        <x:v>7687.47</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7791.79</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7672.99</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7759.37</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:f>ROUND(F13-F12,1)</x:f>
+        <x:v>106.7</x:v>
+      </x:c>
+      <x:c r="H13" s="24" t="n">
+        <x:f>IFERROR(F13/F12-1,"")</x:f>
+        <x:v>0.013940196192449905</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:f>ROUND(D13-E13,1)</x:f>
+        <x:v>118.8</x:v>
+      </x:c>
+      <x:c r="J13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="n">
+      <x:c r="B14" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="30" t="n">
+        <x:f>ROUND(SUM(I12:I13),1)</x:f>
+        <x:v>463.8</x:v>
+      </x:c>
+      <x:c r="J14" s="28"/>
+      <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
+        <x:v>231.9</x:v>
+      </x:c>
+      <x:c r="J15" s="28"/>
+      <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B17" s="17"/>
+      <x:c r="C17" s="17"/>
+      <x:c r="D17" s="17"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="17"/>
+      <x:c r="G17" s="17"/>
+      <x:c r="H17" s="17"/>
+      <x:c r="I17" s="17"/>
+      <x:c r="J17" s="17"/>
+      <x:c r="K17" s="17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J18" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K18" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="30" t="n">
-        <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="J12" s="28"/>
-      <x:c r="K12" s="28"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
+      <x:c r="B19" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>3979.88</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3995.18</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3915.22</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3930.12</x:v>
+      </x:c>
+      <x:c r="G19" s="23"/>
+      <x:c r="H19" s="24"/>
+      <x:c r="I19" s="26" t="n">
+        <x:f>ROUND(D19-E19,1)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="n">
+        <x:v>3942.51</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3948.42</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3916.49</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3932.7</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:f>ROUND(F20-F19,1)</x:f>
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="H20" s="24" t="n">
+        <x:f>IFERROR(F20/F19-1,"")</x:f>
+        <x:v>0.0006564685047785179</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:f>ROUND(D20-E20,1)</x:f>
+        <x:v>31.9</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
+      <x:c r="E21" s="28"/>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28"/>
+      <x:c r="H21" s="28"/>
+      <x:c r="I21" s="30" t="n">
+        <x:f>ROUND(SUM(I19:I20),1)</x:f>
+        <x:v>111.9</x:v>
+      </x:c>
+      <x:c r="J21" s="28"/>
+      <x:c r="K21" s="28"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="28"/>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="J13" s="28"/>
-      <x:c r="K13" s="28"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B15" s="17"/>
-      <x:c r="C15" s="17"/>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="17"/>
-      <x:c r="F15" s="17"/>
-      <x:c r="G15" s="17"/>
-      <x:c r="H15" s="17"/>
-      <x:c r="I15" s="17"/>
-      <x:c r="J15" s="17"/>
-      <x:c r="K15" s="17"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="20" t="str">
+      <x:c r="B22" s="28"/>
+      <x:c r="C22" s="28"/>
+      <x:c r="D22" s="28"/>
+      <x:c r="E22" s="28"/>
+      <x:c r="F22" s="28"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="J22" s="28"/>
+      <x:c r="K22" s="28"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B24" s="17"/>
+      <x:c r="C24" s="17"/>
+      <x:c r="D24" s="17"/>
+      <x:c r="E24" s="17"/>
+      <x:c r="F24" s="17"/>
+      <x:c r="G24" s="17"/>
+      <x:c r="H24" s="17"/>
+      <x:c r="I24" s="17"/>
+      <x:c r="J24" s="17"/>
+      <x:c r="K24" s="17"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B16" s="20" t="str">
+      <x:c r="B25" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C16" s="20" t="str">
+      <x:c r="C25" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D16" s="20" t="str">
+      <x:c r="D25" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E16" s="20" t="str">
+      <x:c r="E25" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F16" s="20" t="str">
+      <x:c r="F25" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G16" s="20" t="str">
+      <x:c r="G25" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H16" s="20" t="str">
+      <x:c r="H25" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I16" s="20" t="str">
+      <x:c r="I25" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J16" s="20" t="str">
+      <x:c r="J25" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K16" s="20" t="str">
+      <x:c r="K25" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="22" t="n">
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B17" s="22" t="str">
+      <x:c r="B26" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C17" s="23" t="n">
-        <x:v>3979.88</x:v>
-      </x:c>
-      <x:c r="D17" s="23" t="n">
-        <x:v>3995.18</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="n">
-        <x:v>3915.22</x:v>
-      </x:c>
-      <x:c r="F17" s="23" t="n">
-        <x:v>3930.12</x:v>
-      </x:c>
-      <x:c r="G17" s="23"/>
-      <x:c r="H17" s="24"/>
-      <x:c r="I17" s="26" t="n">
-        <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J17" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K17" s="22" t="n">
+      <x:c r="C26" s="23" t="n">
+        <x:v>7713.4</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>7721</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>7432</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>7468.2</x:v>
+      </x:c>
+      <x:c r="G26" s="23"/>
+      <x:c r="H26" s="24"/>
+      <x:c r="I26" s="26" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+    <x:row r="27">
+      <x:c r="A27" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="28" t="n">
+      <x:c r="B27" s="28" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="30" t="n">
-        <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J18" s="28"/>
-      <x:c r="K18" s="28"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="C27" s="28"/>
+      <x:c r="D27" s="28"/>
+      <x:c r="E27" s="28"/>
+      <x:c r="F27" s="28"/>
+      <x:c r="G27" s="28"/>
+      <x:c r="H27" s="28"/>
+      <x:c r="I27" s="30" t="n">
+        <x:f>ROUND(SUM(I26:I26),1)</x:f>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="J27" s="28"/>
+      <x:c r="K27" s="28"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="28"/>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J19" s="28"/>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B21" s="17"/>
-      <x:c r="C21" s="17"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="17"/>
-      <x:c r="G21" s="17"/>
-      <x:c r="H21" s="17"/>
-      <x:c r="I21" s="17"/>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
+      <x:c r="B28" s="28"/>
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="28"/>
+      <x:c r="E28" s="28"/>
+      <x:c r="F28" s="28"/>
+      <x:c r="G28" s="28"/>
+      <x:c r="H28" s="28"/>
+      <x:c r="I28" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I26:I26),0),1)</x:f>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="J28" s="28"/>
+      <x:c r="K28" s="28"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B30" s="17"/>
+      <x:c r="C30" s="17"/>
+      <x:c r="D30" s="17"/>
+      <x:c r="E30" s="17"/>
+      <x:c r="F30" s="17"/>
+      <x:c r="G30" s="17"/>
+      <x:c r="H30" s="17"/>
+      <x:c r="I30" s="17"/>
+      <x:c r="J30" s="17"/>
+      <x:c r="K30" s="17"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B22" s="20" t="str">
+      <x:c r="B31" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="str">
+      <x:c r="C31" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="str">
+      <x:c r="D31" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="str">
+      <x:c r="E31" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
+      <x:c r="F31" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="str">
+      <x:c r="G31" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H22" s="20" t="str">
+      <x:c r="H31" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I22" s="20" t="str">
+      <x:c r="I31" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J22" s="20" t="str">
+      <x:c r="J31" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K22" s="20" t="str">
+      <x:c r="K31" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="22" t="n">
+    <x:row r="32">
+      <x:c r="A32" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B23" s="22" t="str">
+      <x:c r="B32" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C23" s="23" t="n">
-        <x:v>7713.4</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="n">
-        <x:v>7721</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="n">
-        <x:v>7432</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="n">
-        <x:v>7468.2</x:v>
-      </x:c>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
-      <x:c r="I23" s="26" t="n">
-        <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J23" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K23" s="22" t="n">
+      <x:c r="C32" s="23" t="n">
+        <x:v>7880.8</x:v>
+      </x:c>
+      <x:c r="D32" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="E32" s="23" t="n">
+        <x:v>7568</x:v>
+      </x:c>
+      <x:c r="F32" s="23" t="n">
+        <x:v>7608</x:v>
+      </x:c>
+      <x:c r="G32" s="23"/>
+      <x:c r="H32" s="24"/>
+      <x:c r="I32" s="26" t="n">
+        <x:f>ROUND(D32-E32,1)</x:f>
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="J32" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K32" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7665.6</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7784.2</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>7651.2</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>7716.2</x:v>
+      </x:c>
+      <x:c r="G33" s="23" t="n">
+        <x:f>ROUND(F33-F32,1)</x:f>
+        <x:v>108.2</x:v>
+      </x:c>
+      <x:c r="H33" s="24" t="n">
+        <x:f>IFERROR(F33/F32-1,"")</x:f>
+        <x:v>0.014221871713985257</x:v>
+      </x:c>
+      <x:c r="I33" s="23" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B34" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C34" s="28"/>
+      <x:c r="D34" s="28"/>
+      <x:c r="E34" s="28"/>
+      <x:c r="F34" s="28"/>
+      <x:c r="G34" s="28"/>
+      <x:c r="H34" s="28"/>
+      <x:c r="I34" s="30" t="n">
+        <x:f>ROUND(SUM(I32:I33),1)</x:f>
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="J34" s="28"/>
+      <x:c r="K34" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B35" s="28"/>
+      <x:c r="C35" s="28"/>
+      <x:c r="D35" s="28"/>
+      <x:c r="E35" s="28"/>
+      <x:c r="F35" s="28"/>
+      <x:c r="G35" s="28"/>
+      <x:c r="H35" s="28"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I32:I33),0),1)</x:f>
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="J35" s="28"/>
+      <x:c r="K35" s="28"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B37" s="17"/>
+      <x:c r="C37" s="17"/>
+      <x:c r="D37" s="17"/>
+      <x:c r="E37" s="17"/>
+      <x:c r="F37" s="17"/>
+      <x:c r="G37" s="17"/>
+      <x:c r="H37" s="17"/>
+      <x:c r="I37" s="17"/>
+      <x:c r="J37" s="17"/>
+      <x:c r="K37" s="17"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C38" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D38" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E38" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F38" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G38" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H38" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I38" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J38" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K38" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="28"/>
-      <x:c r="E24" s="28"/>
-      <x:c r="F24" s="28"/>
-      <x:c r="G24" s="28"/>
-      <x:c r="H24" s="28"/>
-      <x:c r="I24" s="30" t="n">
-        <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J24" s="28"/>
-      <x:c r="K24" s="28"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="28"/>
-      <x:c r="E25" s="28"/>
-      <x:c r="F25" s="28"/>
-      <x:c r="G25" s="28"/>
-      <x:c r="H25" s="28"/>
-      <x:c r="I25" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J25" s="28"/>
-      <x:c r="K25" s="28"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B28" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C28" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D28" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E28" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F28" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G28" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H28" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I28" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J28" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K28" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
+      <x:c r="B39" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C39" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="D39" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="E39" s="23" t="n">
+        <x:v>4497.6</x:v>
+      </x:c>
+      <x:c r="F39" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="G39" s="23"/>
+      <x:c r="H39" s="24"/>
+      <x:c r="I39" s="26" t="n">
+        <x:f>ROUND(D39-E39,1)</x:f>
+        <x:v>120.2</x:v>
+      </x:c>
+      <x:c r="J39" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K39" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B40" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C40" s="23" t="n">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="D40" s="23" t="n">
+        <x:v>4576.8</x:v>
+      </x:c>
+      <x:c r="E40" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="F40" s="23" t="n">
+        <x:v>4555.6</x:v>
+      </x:c>
+      <x:c r="G40" s="23" t="n">
+        <x:f>ROUND(F40-F39,1)</x:f>
+        <x:v>18.2</x:v>
+      </x:c>
+      <x:c r="H40" s="24" t="n">
+        <x:f>IFERROR(F40/F39-1,"")</x:f>
+        <x:v>0.004011107682814208</x:v>
+      </x:c>
+      <x:c r="I40" s="23" t="n">
+        <x:f>ROUND(D40-E40,1)</x:f>
+        <x:v>39.4</x:v>
+      </x:c>
+      <x:c r="J40" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K40" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7880.8</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7903</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>7568</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7608</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="29" t="str">
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B30" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="28"/>
-      <x:c r="D30" s="28"/>
-      <x:c r="E30" s="28"/>
-      <x:c r="F30" s="28"/>
-      <x:c r="G30" s="28"/>
-      <x:c r="H30" s="28"/>
-      <x:c r="I30" s="30" t="n">
-        <x:f>ROUND(SUM(I29:I29),1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J30" s="28"/>
-      <x:c r="K30" s="28"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B31" s="28"/>
-      <x:c r="C31" s="28"/>
-      <x:c r="D31" s="28"/>
-      <x:c r="E31" s="28"/>
-      <x:c r="F31" s="28"/>
-      <x:c r="G31" s="28"/>
-      <x:c r="H31" s="28"/>
-      <x:c r="I31" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J31" s="28"/>
-      <x:c r="K31" s="28"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B33" s="17"/>
-      <x:c r="C33" s="17"/>
-      <x:c r="D33" s="17"/>
-      <x:c r="E33" s="17"/>
-      <x:c r="F33" s="17"/>
-      <x:c r="G33" s="17"/>
-      <x:c r="H33" s="17"/>
-      <x:c r="I33" s="17"/>
-      <x:c r="J33" s="17"/>
-      <x:c r="K33" s="17"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B34" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C34" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D34" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E34" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F34" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G34" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H34" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I34" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J34" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K34" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B35" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C35" s="23" t="n">
-        <x:v>4602</x:v>
-      </x:c>
-      <x:c r="D35" s="23" t="n">
-        <x:v>4617.8</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="n">
-        <x:v>4497.6</x:v>
-      </x:c>
-      <x:c r="F35" s="23" t="n">
-        <x:v>4537.4</x:v>
-      </x:c>
-      <x:c r="G35" s="23"/>
-      <x:c r="H35" s="24"/>
-      <x:c r="I35" s="26" t="n">
-        <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J35" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K35" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B36" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="30" t="n">
-        <x:f>ROUND(SUM(I35:I35),1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B37" s="28"/>
-      <x:c r="C37" s="28"/>
-      <x:c r="D37" s="28"/>
-      <x:c r="E37" s="28"/>
-      <x:c r="F37" s="28"/>
-      <x:c r="G37" s="28"/>
-      <x:c r="H37" s="28"/>
-      <x:c r="I37" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J37" s="28"/>
-      <x:c r="K37" s="28"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B39" s="17"/>
-      <x:c r="C39" s="17"/>
-      <x:c r="D39" s="17"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="17"/>
-      <x:c r="G39" s="17"/>
-      <x:c r="H39" s="17"/>
-      <x:c r="I39" s="17"/>
-      <x:c r="J39" s="17"/>
-      <x:c r="K39" s="17"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B40" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C40" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D40" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E40" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F40" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G40" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H40" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I40" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J40" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K40" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>2913</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>2949.4</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>2881.4</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>2915.8</x:v>
-      </x:c>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
+      <x:c r="B41" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C41" s="28"/>
+      <x:c r="D41" s="28"/>
+      <x:c r="E41" s="28"/>
+      <x:c r="F41" s="28"/>
+      <x:c r="G41" s="28"/>
+      <x:c r="H41" s="28"/>
+      <x:c r="I41" s="30" t="n">
+        <x:f>ROUND(SUM(I39:I40),1)</x:f>
+        <x:v>159.6</x:v>
+      </x:c>
+      <x:c r="J41" s="28"/>
+      <x:c r="K41" s="28"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B42" s="28"/>
       <x:c r="C42" s="28"/>
       <x:c r="D42" s="28"/>
       <x:c r="E42" s="28"/>
       <x:c r="F42" s="28"/>
       <x:c r="G42" s="28"/>
       <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
-        <x:f>ROUND(SUM(I41:I41),1)</x:f>
-        <x:v>68</x:v>
+      <x:c r="I42" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I39:I40),0),1)</x:f>
+        <x:v>79.8</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
     </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
+    <x:row r="44">
+      <x:c r="A44" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B44" s="17"/>
+      <x:c r="C44" s="17"/>
+      <x:c r="D44" s="17"/>
+      <x:c r="E44" s="17"/>
+      <x:c r="F44" s="17"/>
+      <x:c r="G44" s="17"/>
+      <x:c r="H44" s="17"/>
+      <x:c r="I44" s="17"/>
+      <x:c r="J44" s="17"/>
+      <x:c r="K44" s="17"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E45" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F45" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G45" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I45" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J45" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K45" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="n">
+        <x:v>2913</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="n">
+        <x:v>2949.4</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="n">
+        <x:v>2881.4</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="n">
+        <x:v>2915.8</x:v>
+      </x:c>
+      <x:c r="G46" s="23"/>
+      <x:c r="H46" s="24"/>
+      <x:c r="I46" s="26" t="n">
+        <x:f>ROUND(D46-E46,1)</x:f>
         <x:v>68</x:v>
       </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C46" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E46" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F46" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I46" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J46" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str">
-        <x:v>交易日</x:v>
+      <x:c r="J46" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K46" s="22" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="n">
+        <x:v>2923.2</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="n">
+        <x:v>2931.4</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="n">
+        <x:v>2892.2</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="n">
+        <x:v>2898.8</x:v>
+      </x:c>
+      <x:c r="G47" s="23" t="n">
+        <x:f>ROUND(F47-F46,1)</x:f>
+        <x:v>-17</x:v>
+      </x:c>
+      <x:c r="H47" s="24" t="n">
+        <x:f>IFERROR(F47/F46-1,"")</x:f>
+        <x:v>-0.0058303038617189</x:v>
+      </x:c>
+      <x:c r="I47" s="23" t="n">
+        <x:f>ROUND(D47-E47,1)</x:f>
+        <x:v>39.2</x:v>
+      </x:c>
+      <x:c r="J47" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K47" s="22" t="n">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>159000</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>160480</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>140940</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>140980</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>19540</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2042,7 +2150,7 @@
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B48" s="28" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="28"/>
       <x:c r="D48" s="28"/>
@@ -2051,8 +2159,8 @@
       <x:c r="G48" s="28"/>
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
-        <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>19540</x:v>
+        <x:f>ROUND(SUM(I46:I47),1)</x:f>
+        <x:v>107.2</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -2069,23 +2177,143 @@
       <x:c r="G49" s="28"/>
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>19540</x:v>
+        <x:f>ROUND(IFERROR(AVERAGE(I46:I47),0),1)</x:f>
+        <x:v>53.6</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B51" s="17"/>
+      <x:c r="C51" s="17"/>
+      <x:c r="D51" s="17"/>
+      <x:c r="E51" s="17"/>
+      <x:c r="F51" s="17"/>
+      <x:c r="G51" s="17"/>
+      <x:c r="H51" s="17"/>
+      <x:c r="I51" s="17"/>
+      <x:c r="J51" s="17"/>
+      <x:c r="K51" s="17"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B52" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C52" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D52" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E52" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F52" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G52" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H52" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I52" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J52" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K52" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B53" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C53" s="23" t="n">
+        <x:v>159000</x:v>
+      </x:c>
+      <x:c r="D53" s="23" t="n">
+        <x:v>160480</x:v>
+      </x:c>
+      <x:c r="E53" s="23" t="n">
+        <x:v>140940</x:v>
+      </x:c>
+      <x:c r="F53" s="23" t="n">
+        <x:v>140980</x:v>
+      </x:c>
+      <x:c r="G53" s="23"/>
+      <x:c r="H53" s="24"/>
+      <x:c r="I53" s="26" t="n">
+        <x:f>ROUND(D53-E53,1)</x:f>
+        <x:v>19540</x:v>
+      </x:c>
+      <x:c r="J53" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K53" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B54" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C54" s="28"/>
+      <x:c r="D54" s="28"/>
+      <x:c r="E54" s="28"/>
+      <x:c r="F54" s="28"/>
+      <x:c r="G54" s="28"/>
+      <x:c r="H54" s="28"/>
+      <x:c r="I54" s="30" t="n">
+        <x:f>ROUND(SUM(I53:I53),1)</x:f>
+        <x:v>19540</x:v>
+      </x:c>
+      <x:c r="J54" s="28"/>
+      <x:c r="K54" s="28"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B55" s="28"/>
+      <x:c r="C55" s="28"/>
+      <x:c r="D55" s="28"/>
+      <x:c r="E55" s="28"/>
+      <x:c r="F55" s="28"/>
+      <x:c r="G55" s="28"/>
+      <x:c r="H55" s="28"/>
+      <x:c r="I55" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I53:I53),0),1)</x:f>
+        <x:v>19540</x:v>
+      </x:c>
+      <x:c r="J55" s="28"/>
+      <x:c r="K55" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A9:K9"/>
-    <x:mergeCell ref="A15:K15"/>
-    <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A33:K33"/>
-    <x:mergeCell ref="A39:K39"/>
-    <x:mergeCell ref="A45:K45"/>
+    <x:mergeCell ref="A10:K10"/>
+    <x:mergeCell ref="A17:K17"/>
+    <x:mergeCell ref="A24:K24"/>
+    <x:mergeCell ref="A30:K30"/>
+    <x:mergeCell ref="A37:K37"/>
+    <x:mergeCell ref="A44:K44"/>
+    <x:mergeCell ref="A51:K51"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2292,31 +2520,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>570.4</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7551.02</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7669.84</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7541.14</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7639.36</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>131.3</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.017483807466346146</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>128.7</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2324,11 +2570,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>142.6</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>699.0999999999999</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>139.8</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2539,31 +2803,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>546.6</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7687.47</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7791.79</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7672.99</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7759.37</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>106.7</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.013940196192449905</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>118.8</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2571,11 +2853,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>136.7</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>665.4</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>133.1</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2786,31 +3086,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>3942.51</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>3948.42</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>3916.49</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>3932.7</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.0006564685047785179</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>31.9</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -2818,11 +3136,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>38.8</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>186.9</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>37.4</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3280,31 +3616,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>672.4</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7665.6</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7784.2</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7651.2</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>7716.2</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>108.2</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.014221871713985257</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3312,11 +3666,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>168.1</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>805.4</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>161.1</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3527,31 +3899,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>4576.8</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>4555.6</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>18.2</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>0.004011107682814208</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>39.4</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3559,11 +3949,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>59.3</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>276.4</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>55.3</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3774,31 +4182,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>132.6</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>9月7日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>2923.2</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>2931.4</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>2892.2</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>2898.8</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-17</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.0058303038617189</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>39.2</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B11" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="28"/>
       <x:c r="E11" s="28"/>
@@ -3806,11 +4232,29 @@
       <x:c r="G11" s="28"/>
       <x:c r="H11" s="28"/>
       <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>33.2</x:v>
+      <x:c r="J11" s="30" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>171.8</x:v>
       </x:c>
       <x:c r="K11" s="28"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B12" s="28"/>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>34.4</x:v>
+      </x:c>
+      <x:c r="K12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-08
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4d68833dcead400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R4be66a6724924229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6cc88e75e51d4d0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R1bfc0802906e4fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc3f0a913fcdb4e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5d582af0203f42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re99dc128ec384947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rc76cadcb6fb34e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R340f0cb8d58f4d46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R5994bd1c9a1545c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rbd014a4a968e42c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R531599f4319d4c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R308cf15ec1444832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R2a7dc7f3a84e449c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rb4df23ca764840af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R25f4aaba29024945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R8321b531cb804df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R639f78fb25504a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf100675b78494f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R0283b112a5f04ab1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,6 +201,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -216,12 +222,6 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7669.84</x:v>
+        <x:v>7724.94</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7541.14</x:v>
+        <x:v>7622.9</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>128.7</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>699.1</x:v>
+        <x:v>801.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>139.8</x:v>
+        <x:v>133.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7791.79</x:v>
+        <x:v>7830.16</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7672.99</x:v>
+        <x:v>7736.44</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>118.8</x:v>
+        <x:v>93.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>665.4</x:v>
+        <x:v>759.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>133.1</x:v>
+        <x:v>126.5</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3948.42</x:v>
+        <x:v>3951.32</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3916.49</x:v>
+        <x:v>3925.72</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>31.9</x:v>
+        <x:v>25.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>186.9</x:v>
+        <x:v>212.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>37.4</x:v>
+        <x:v>35.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7784.2</x:v>
+        <x:v>7817.2</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7651.2</x:v>
+        <x:v>7703.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>133</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>805.4</x:v>
+        <x:v>919.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>161.1</x:v>
+        <x:v>153.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2931.4</x:v>
+        <x:v>2917.4</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2892.2</x:v>
+        <x:v>2891</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>39.2</x:v>
+        <x:v>26.4</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>171.8</x:v>
+        <x:v>198.2</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>34.4</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>142800</x:v>
+        <x:v>143200</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>139880</x:v>
+        <x:v>141320</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>2920</x:v>
+        <x:v>1880</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>29140</x:v>
+        <x:v>31020</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5828</x:v>
+        <x:v>5170</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-08</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>155820</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-3180</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>155000</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>-820</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>148900</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>-6100</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>140980</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="n">
+      <x:c r="H7" s="28" t="n">
         <x:v>-7920</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1069,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
+      <x:c r="H8" s="28" t="n">
         <x:v>-480</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1083,43 +1083,79 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>143200</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>143200</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>141320</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>141320</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="n">
+        <x:v>820</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.005836298932384354</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>1880</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>29140</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>31020</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>5828</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>5170</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1238,76 +1274,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7551.02</x:v>
       </x:c>
       <x:c r="D6" s="23" t="n">
-        <x:v>7669.84</x:v>
+        <x:v>7724.94</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:v>7541.14</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7639.36</x:v>
-      </x:c>
-      <x:c r="G6" s="23" t="n">
+        <x:v>7659.61</x:v>
+      </x:c>
+      <x:c r="G6" s="28" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>131.3</x:v>
+        <x:v>151.5</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.017483807466346146</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="n">
+        <x:v>0.02018089820447</x:v>
+      </x:c>
+      <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>128.7</x:v>
+        <x:v>183.8</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="str">
+      <x:c r="A7" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="28" t="n">
+      <x:c r="B7" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="30" t="n">
+      <x:c r="C7" s="30"/>
+      <x:c r="D7" s="30"/>
+      <x:c r="E7" s="30"/>
+      <x:c r="F7" s="30"/>
+      <x:c r="G7" s="30"/>
+      <x:c r="H7" s="30"/>
+      <x:c r="I7" s="32" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>436.8</x:v>
-      </x:c>
-      <x:c r="J7" s="28"/>
-      <x:c r="K7" s="28"/>
+        <x:v>491.9</x:v>
+      </x:c>
+      <x:c r="J7" s="30"/>
+      <x:c r="K7" s="30"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="A8" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="28"/>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="32" t="n">
+      <x:c r="B8" s="30"/>
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="30"/>
+      <x:c r="E8" s="30"/>
+      <x:c r="F8" s="30"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>218.4</x:v>
-      </x:c>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="28"/>
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
@@ -1396,76 +1432,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7687.47</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>7791.79</x:v>
+        <x:v>7830.16</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
         <x:v>7672.99</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7759.37</x:v>
+        <x:v>7770.73</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>106.7</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.013940196192449905</x:v>
+        <x:v>0.015424641531278649</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>118.8</x:v>
+        <x:v>157.2</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="29" t="str">
+      <x:c r="A14" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B14" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="30" t="n">
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="32" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>463.8</x:v>
-      </x:c>
-      <x:c r="J14" s="28"/>
-      <x:c r="K14" s="28"/>
+        <x:v>502.2</x:v>
+      </x:c>
+      <x:c r="J14" s="30"/>
+      <x:c r="K14" s="30"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="A15" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="28"/>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="32" t="n">
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>231.9</x:v>
-      </x:c>
-      <x:c r="J15" s="28"/>
-      <x:c r="K15" s="28"/>
+        <x:v>251.1</x:v>
+      </x:c>
+      <x:c r="J15" s="30"/>
+      <x:c r="K15" s="30"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="17" t="str">
@@ -1554,76 +1590,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3942.51</x:v>
       </x:c>
       <x:c r="D20" s="23" t="n">
-        <x:v>3948.42</x:v>
+        <x:v>3951.32</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
         <x:v>3916.49</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3932.7</x:v>
+        <x:v>3940.55</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>2.6</x:v>
+        <x:v>10.4</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.0006564685047785179</x:v>
+        <x:v>0.0026538629863719354</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>31.9</x:v>
+        <x:v>34.8</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="29" t="str">
+      <x:c r="A21" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B21" s="28" t="n">
+      <x:c r="B21" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C21" s="28"/>
-      <x:c r="D21" s="28"/>
-      <x:c r="E21" s="28"/>
-      <x:c r="F21" s="28"/>
-      <x:c r="G21" s="28"/>
-      <x:c r="H21" s="28"/>
-      <x:c r="I21" s="30" t="n">
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="32" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>111.9</x:v>
-      </x:c>
-      <x:c r="J21" s="28"/>
-      <x:c r="K21" s="28"/>
+        <x:v>114.8</x:v>
+      </x:c>
+      <x:c r="J21" s="30"/>
+      <x:c r="K21" s="30"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29" t="str">
+      <x:c r="A22" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="28"/>
-      <x:c r="C22" s="28"/>
-      <x:c r="D22" s="28"/>
-      <x:c r="E22" s="28"/>
-      <x:c r="F22" s="28"/>
-      <x:c r="G22" s="28"/>
-      <x:c r="H22" s="28"/>
-      <x:c r="I22" s="32" t="n">
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="J22" s="28"/>
-      <x:c r="K22" s="28"/>
+        <x:v>57.4</x:v>
+      </x:c>
+      <x:c r="J22" s="30"/>
+      <x:c r="K22" s="30"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="17" t="str">
@@ -1746,42 +1782,42 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="29" t="str">
+      <x:c r="A28" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="n">
+      <x:c r="B28" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C28" s="28"/>
-      <x:c r="D28" s="28"/>
-      <x:c r="E28" s="28"/>
-      <x:c r="F28" s="28"/>
-      <x:c r="G28" s="28"/>
-      <x:c r="H28" s="28"/>
-      <x:c r="I28" s="30" t="n">
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="32" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
         <x:v>438.6</x:v>
       </x:c>
-      <x:c r="J28" s="28"/>
-      <x:c r="K28" s="28"/>
+      <x:c r="J28" s="30"/>
+      <x:c r="K28" s="30"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="29" t="str">
+      <x:c r="A29" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="28"/>
-      <x:c r="C29" s="28"/>
-      <x:c r="D29" s="28"/>
-      <x:c r="E29" s="28"/>
-      <x:c r="F29" s="28"/>
-      <x:c r="G29" s="28"/>
-      <x:c r="H29" s="28"/>
-      <x:c r="I29" s="32" t="n">
+      <x:c r="B29" s="30"/>
+      <x:c r="C29" s="30"/>
+      <x:c r="D29" s="30"/>
+      <x:c r="E29" s="30"/>
+      <x:c r="F29" s="30"/>
+      <x:c r="G29" s="30"/>
+      <x:c r="H29" s="30"/>
+      <x:c r="I29" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
         <x:v>219.3</x:v>
       </x:c>
-      <x:c r="J29" s="28"/>
-      <x:c r="K29" s="28"/>
+      <x:c r="J29" s="30"/>
+      <x:c r="K29" s="30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="17" t="str">
@@ -1870,76 +1906,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C34" s="23" t="n">
         <x:v>7665.6</x:v>
       </x:c>
       <x:c r="D34" s="23" t="n">
-        <x:v>7784.2</x:v>
+        <x:v>7817.2</x:v>
       </x:c>
       <x:c r="E34" s="23" t="n">
         <x:v>7651.2</x:v>
       </x:c>
       <x:c r="F34" s="23" t="n">
-        <x:v>7716.2</x:v>
+        <x:v>7743.4</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
         <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>108.2</x:v>
+        <x:v>135.4</x:v>
       </x:c>
       <x:c r="H34" s="24" t="n">
         <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>0.014221871713985257</x:v>
-      </x:c>
-      <x:c r="I34" s="23" t="n">
+        <x:v>0.017797055730809586</x:v>
+      </x:c>
+      <x:c r="I34" s="26" t="n">
         <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>133</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="J34" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K34" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="29" t="str">
+      <x:c r="A35" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B35" s="28" t="n">
+      <x:c r="B35" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C35" s="28"/>
-      <x:c r="D35" s="28"/>
-      <x:c r="E35" s="28"/>
-      <x:c r="F35" s="28"/>
-      <x:c r="G35" s="28"/>
-      <x:c r="H35" s="28"/>
-      <x:c r="I35" s="30" t="n">
+      <x:c r="C35" s="30"/>
+      <x:c r="D35" s="30"/>
+      <x:c r="E35" s="30"/>
+      <x:c r="F35" s="30"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="32" t="n">
         <x:f>ROUND(SUM(I33:I34),1)</x:f>
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="J35" s="28"/>
-      <x:c r="K35" s="28"/>
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="J35" s="30"/>
+      <x:c r="K35" s="30"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="29" t="str">
+      <x:c r="A36" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B36" s="28"/>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="32" t="n">
+      <x:c r="B36" s="30"/>
+      <x:c r="C36" s="30"/>
+      <x:c r="D36" s="30"/>
+      <x:c r="E36" s="30"/>
+      <x:c r="F36" s="30"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
+        <x:v>250.5</x:v>
+      </x:c>
+      <x:c r="J36" s="30"/>
+      <x:c r="K36" s="30"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="17" t="str">
@@ -2062,42 +2098,42 @@
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="29" t="str">
+      <x:c r="A42" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B42" s="28" t="n">
+      <x:c r="B42" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C42" s="28"/>
-      <x:c r="D42" s="28"/>
-      <x:c r="E42" s="28"/>
-      <x:c r="F42" s="28"/>
-      <x:c r="G42" s="28"/>
-      <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
+      <x:c r="C42" s="30"/>
+      <x:c r="D42" s="30"/>
+      <x:c r="E42" s="30"/>
+      <x:c r="F42" s="30"/>
+      <x:c r="G42" s="30"/>
+      <x:c r="H42" s="30"/>
+      <x:c r="I42" s="32" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
         <x:v>159.6</x:v>
       </x:c>
-      <x:c r="J42" s="28"/>
-      <x:c r="K42" s="28"/>
+      <x:c r="J42" s="30"/>
+      <x:c r="K42" s="30"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="29" t="str">
+      <x:c r="A43" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
+      <x:c r="B43" s="30"/>
+      <x:c r="C43" s="30"/>
+      <x:c r="D43" s="30"/>
+      <x:c r="E43" s="30"/>
+      <x:c r="F43" s="30"/>
+      <x:c r="G43" s="30"/>
+      <x:c r="H43" s="30"/>
+      <x:c r="I43" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
         <x:v>79.8</x:v>
       </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
+      <x:c r="J43" s="30"/>
+      <x:c r="K43" s="30"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="17" t="str">
@@ -2186,7 +2222,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2923.2</x:v>
@@ -2195,67 +2231,67 @@
         <x:v>2931.4</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2892.2</x:v>
+        <x:v>2891</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2898.8</x:v>
+        <x:v>2897</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-17</x:v>
+        <x:v>-18.8</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.0058303038617189</x:v>
+        <x:v>-0.0064476301529597935</x:v>
       </x:c>
       <x:c r="I48" s="23" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>39.2</x:v>
+        <x:v>40.4</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29" t="str">
+      <x:c r="A49" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B49" s="28" t="n">
+      <x:c r="B49" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="30" t="n">
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="32" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>107.2</x:v>
-      </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
+        <x:v>108.4</x:v>
+      </x:c>
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="29" t="str">
+      <x:c r="A50" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B50" s="28"/>
-      <x:c r="C50" s="28"/>
-      <x:c r="D50" s="28"/>
-      <x:c r="E50" s="28"/>
-      <x:c r="F50" s="28"/>
-      <x:c r="G50" s="28"/>
-      <x:c r="H50" s="28"/>
-      <x:c r="I50" s="32" t="n">
+      <x:c r="B50" s="30"/>
+      <x:c r="C50" s="30"/>
+      <x:c r="D50" s="30"/>
+      <x:c r="E50" s="30"/>
+      <x:c r="F50" s="30"/>
+      <x:c r="G50" s="30"/>
+      <x:c r="H50" s="30"/>
+      <x:c r="I50" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>53.6</x:v>
-      </x:c>
-      <x:c r="J50" s="28"/>
-      <x:c r="K50" s="28"/>
+        <x:v>54.2</x:v>
+      </x:c>
+      <x:c r="J50" s="30"/>
+      <x:c r="K50" s="30"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="17" t="str">
@@ -2344,76 +2380,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>9月7日</x:v>
+        <x:v>9月7日-9月8日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>142120</x:v>
       </x:c>
       <x:c r="D55" s="23" t="n">
-        <x:v>142800</x:v>
+        <x:v>143200</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
         <x:v>139880</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>140500</x:v>
-      </x:c>
-      <x:c r="G55" s="34" t="n">
+        <x:v>141320</x:v>
+      </x:c>
+      <x:c r="G55" s="28" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-480</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.003404738260746165</x:v>
+        <x:v>0.002411689601361955</x:v>
       </x:c>
       <x:c r="I55" s="23" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>2920</x:v>
+        <x:v>3320</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="29" t="str">
+      <x:c r="A56" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B56" s="28" t="n">
+      <x:c r="B56" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C56" s="28"/>
-      <x:c r="D56" s="28"/>
-      <x:c r="E56" s="28"/>
-      <x:c r="F56" s="28"/>
-      <x:c r="G56" s="28"/>
-      <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
+      <x:c r="C56" s="30"/>
+      <x:c r="D56" s="30"/>
+      <x:c r="E56" s="30"/>
+      <x:c r="F56" s="30"/>
+      <x:c r="G56" s="30"/>
+      <x:c r="H56" s="30"/>
+      <x:c r="I56" s="32" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>22460</x:v>
-      </x:c>
-      <x:c r="J56" s="28"/>
-      <x:c r="K56" s="28"/>
+        <x:v>22860</x:v>
+      </x:c>
+      <x:c r="J56" s="30"/>
+      <x:c r="K56" s="30"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29" t="str">
+      <x:c r="A57" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
+      <x:c r="B57" s="30"/>
+      <x:c r="C57" s="30"/>
+      <x:c r="D57" s="30"/>
+      <x:c r="E57" s="30"/>
+      <x:c r="F57" s="30"/>
+      <x:c r="G57" s="30"/>
+      <x:c r="H57" s="30"/>
+      <x:c r="I57" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
-        <x:v>11230</x:v>
-      </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+        <x:v>11430</x:v>
+      </x:c>
+      <x:c r="J57" s="30"/>
+      <x:c r="K57" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2668,43 +2704,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7650.06</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7724.94</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7622.9</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>7659.61</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>20.3</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.0026507456121978024</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>699.0999999999999</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>801.0999999999999</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>139.8</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>133.5</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2951,43 +3023,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7773.28</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7830.16</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7736.44</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>7770.73</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>11.4</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.0014640363843971826</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>93.7</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>665.4</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>759.1</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>133.1</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>126.5</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3234,43 +3342,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>3935.55</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>3951.32</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>3925.72</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>3940.55</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.001996084115238883</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>25.6</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>186.9</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>212.5</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>37.4</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>35.4</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3518,42 +3662,42 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="30" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
         <x:f>SUM(J4:J8)</x:f>
         <x:v>781</x:v>
       </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="K11" s="30"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
         <x:v>156.2</x:v>
       </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3800,43 +3944,79 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7734</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7817.2</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7703.2</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>7743.4</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>27.2</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>0.003525051191000772</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>805.4</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>919.4</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>161.1</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>153.2</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4084,42 +4264,42 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
+      <x:c r="B11" s="30" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
         <x:f>SUM(J4:J8)</x:f>
         <x:v>276.4</x:v>
       </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="K11" s="30"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
         <x:v>55.3</x:v>
       </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4366,43 +4546,79 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>9月8日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>2904.8</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>2917.4</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>2891</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>2897</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-1.8</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.0006209465985925755</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>26.4</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="30" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>171.8</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>198.20000000000002</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="28"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>34.4</x:v>
-      </x:c>
-      <x:c r="K12" s="28"/>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-09
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2a763a7270c34097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rcc18b4eb980c4833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rc8e5077aa9e74535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R2fa15d7683454ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R56e8428ef2cd4b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Read726e503344ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R237e4b8d1b4e4983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R5156a54f8b574de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R4a5a8ae9662b4479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Re65efeeccb13418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4155bcf6305e4be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R0265ddd84034425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rbc4bc2058aff478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R507f851da1424f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R59291e888561422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R35a21b3cceff42a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd6f21753894e4294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd6c81c1d78b148ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb5f206676dc840e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R95e6ec74dd994b01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,12 +201,6 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -222,6 +216,12 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7724.94</x:v>
+        <x:v>7715.08</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7622.9</x:v>
+        <x:v>7602.5</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>102</x:v>
+        <x:v>112.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>801.1</x:v>
+        <x:v>913.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>133.5</x:v>
+        <x:v>130.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7830.16</x:v>
+        <x:v>7816.66</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7736.44</x:v>
+        <x:v>7723.82</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>93.7</x:v>
+        <x:v>92.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>759.1</x:v>
+        <x:v>851.9</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>126.5</x:v>
+        <x:v>121.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3951.32</x:v>
+        <x:v>3958.12</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3925.72</x:v>
+        <x:v>3933.47</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>25.6</x:v>
+        <x:v>24.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>212.5</x:v>
+        <x:v>237.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.4</x:v>
+        <x:v>33.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7714.6</x:v>
+        <x:v>7705</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7592.4</x:v>
+        <x:v>7575</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>122.2</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>903.2</x:v>
+        <x:v>1033.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>150.5</x:v>
+        <x:v>147.6</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4584</x:v>
+        <x:v>4574.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4532.8</x:v>
+        <x:v>4535.6</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>51.2</x:v>
+        <x:v>38.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>327.6</x:v>
+        <x:v>366.2</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>54.6</x:v>
+        <x:v>52.3</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2917.4</x:v>
+        <x:v>2909.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2891</x:v>
+        <x:v>2887.6</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>26.4</x:v>
+        <x:v>22.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>198.2</x:v>
+        <x:v>220.4</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>33</x:v>
+        <x:v>31.5</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-08</x:v>
+        <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>155820</x:v>
       </x:c>
-      <x:c r="H4" s="28" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>-3180</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>155000</x:v>
       </x:c>
-      <x:c r="H5" s="28" t="n">
+      <x:c r="H5" s="34" t="n">
         <x:v>-820</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>148900</x:v>
       </x:c>
-      <x:c r="H6" s="28" t="n">
+      <x:c r="H6" s="34" t="n">
         <x:v>-6100</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>140980</x:v>
       </x:c>
-      <x:c r="H7" s="28" t="n">
+      <x:c r="H7" s="34" t="n">
         <x:v>-7920</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1069,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="n">
+      <x:c r="H8" s="34" t="n">
         <x:v>-480</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1105,7 +1105,7 @@
       <x:c r="G9" s="23" t="n">
         <x:v>141320</x:v>
       </x:c>
-      <x:c r="H9" s="28" t="n">
+      <x:c r="H9" s="34" t="n">
         <x:v>820</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
@@ -1120,42 +1120,42 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+      <x:c r="A12" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
+      <x:c r="B12" s="28" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="30" t="n">
         <x:f>SUM(J4:J9)</x:f>
         <x:v>31020</x:v>
       </x:c>
-      <x:c r="K12" s="30"/>
+      <x:c r="K12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="A13" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
         <x:v>5170</x:v>
       </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1274,7 +1274,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7551.02</x:v>
@@ -1286,15 +1286,15 @@
         <x:v>7541.14</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7659.61</x:v>
-      </x:c>
-      <x:c r="G6" s="28" t="n">
+        <x:v>7648.8</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>151.5</x:v>
+        <x:v>140.7</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.02018089820447</x:v>
+        <x:v>0.018741117914143235</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
@@ -1304,46 +1304,46 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="30"/>
-      <x:c r="D7" s="30"/>
-      <x:c r="E7" s="30"/>
-      <x:c r="F7" s="30"/>
-      <x:c r="G7" s="30"/>
-      <x:c r="H7" s="30"/>
-      <x:c r="I7" s="32" t="n">
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
         <x:v>491.9</x:v>
       </x:c>
-      <x:c r="J7" s="30"/>
-      <x:c r="K7" s="30"/>
+      <x:c r="J7" s="28"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="31" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="30"/>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="30"/>
-      <x:c r="E8" s="30"/>
-      <x:c r="F8" s="30"/>
-      <x:c r="G8" s="30"/>
-      <x:c r="H8" s="30"/>
-      <x:c r="I8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
         <x:v>246</x:v>
       </x:c>
-      <x:c r="J8" s="30"/>
-      <x:c r="K8" s="30"/>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
@@ -1432,7 +1432,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7687.47</x:v>
@@ -1444,15 +1444,15 @@
         <x:v>7672.99</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7770.73</x:v>
+        <x:v>7768.11</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>118</x:v>
+        <x:v>115.4</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.015424641531278649</x:v>
+        <x:v>0.01508227825771069</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
@@ -1462,46 +1462,46 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="32" t="n">
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
         <x:v>502.2</x:v>
       </x:c>
-      <x:c r="J14" s="30"/>
-      <x:c r="K14" s="30"/>
+      <x:c r="J14" s="28"/>
+      <x:c r="K14" s="28"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="31" t="str">
+      <x:c r="A15" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="30"/>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="34" t="n">
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
         <x:v>251.1</x:v>
       </x:c>
-      <x:c r="J15" s="30"/>
-      <x:c r="K15" s="30"/>
+      <x:c r="J15" s="28"/>
+      <x:c r="K15" s="28"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="17" t="str">
@@ -1590,76 +1590,76 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3942.51</x:v>
       </x:c>
       <x:c r="D20" s="23" t="n">
-        <x:v>3951.32</x:v>
+        <x:v>3958.12</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
         <x:v>3916.49</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3940.55</x:v>
+        <x:v>3951.51</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>10.4</x:v>
+        <x:v>21.4</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.0026538629863719354</x:v>
+        <x:v>0.005442581905896082</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>34.8</x:v>
+        <x:v>41.6</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="32" t="n">
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
+      <x:c r="E21" s="28"/>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28"/>
+      <x:c r="H21" s="28"/>
+      <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>114.8</x:v>
-      </x:c>
-      <x:c r="J21" s="30"/>
-      <x:c r="K21" s="30"/>
+        <x:v>121.6</x:v>
+      </x:c>
+      <x:c r="J21" s="28"/>
+      <x:c r="K21" s="28"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="31" t="str">
+      <x:c r="A22" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="30"/>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="34" t="n">
+      <x:c r="B22" s="28"/>
+      <x:c r="C22" s="28"/>
+      <x:c r="D22" s="28"/>
+      <x:c r="E22" s="28"/>
+      <x:c r="F22" s="28"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>57.4</x:v>
-      </x:c>
-      <x:c r="J22" s="30"/>
-      <x:c r="K22" s="30"/>
+        <x:v>60.8</x:v>
+      </x:c>
+      <x:c r="J22" s="28"/>
+      <x:c r="K22" s="28"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="17" t="str">
@@ -1748,7 +1748,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7527.2</x:v>
@@ -1760,15 +1760,15 @@
         <x:v>7512.6</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>7633.4</x:v>
-      </x:c>
-      <x:c r="G27" s="28" t="n">
+        <x:v>7618.6</x:v>
+      </x:c>
+      <x:c r="G27" s="34" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>165.2</x:v>
+        <x:v>150.4</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>0.022120457406068272</x:v>
+        <x:v>0.020138721512546587</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
@@ -1778,46 +1778,46 @@
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B28" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B28" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C28" s="30"/>
-      <x:c r="D28" s="30"/>
-      <x:c r="E28" s="30"/>
-      <x:c r="F28" s="30"/>
-      <x:c r="G28" s="30"/>
-      <x:c r="H28" s="30"/>
-      <x:c r="I28" s="32" t="n">
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="28"/>
+      <x:c r="E28" s="28"/>
+      <x:c r="F28" s="28"/>
+      <x:c r="G28" s="28"/>
+      <x:c r="H28" s="28"/>
+      <x:c r="I28" s="30" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
         <x:v>491</x:v>
       </x:c>
-      <x:c r="J28" s="30"/>
-      <x:c r="K28" s="30"/>
+      <x:c r="J28" s="28"/>
+      <x:c r="K28" s="28"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="31" t="str">
+      <x:c r="A29" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="30"/>
-      <x:c r="C29" s="30"/>
-      <x:c r="D29" s="30"/>
-      <x:c r="E29" s="30"/>
-      <x:c r="F29" s="30"/>
-      <x:c r="G29" s="30"/>
-      <x:c r="H29" s="30"/>
-      <x:c r="I29" s="34" t="n">
+      <x:c r="B29" s="28"/>
+      <x:c r="C29" s="28"/>
+      <x:c r="D29" s="28"/>
+      <x:c r="E29" s="28"/>
+      <x:c r="F29" s="28"/>
+      <x:c r="G29" s="28"/>
+      <x:c r="H29" s="28"/>
+      <x:c r="I29" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
         <x:v>245.5</x:v>
       </x:c>
-      <x:c r="J29" s="30"/>
-      <x:c r="K29" s="30"/>
+      <x:c r="J29" s="28"/>
+      <x:c r="K29" s="28"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="17" t="str">
@@ -1940,42 +1940,42 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="31" t="str">
+      <x:c r="A35" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B35" s="30" t="n">
+      <x:c r="B35" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C35" s="30"/>
-      <x:c r="D35" s="30"/>
-      <x:c r="E35" s="30"/>
-      <x:c r="F35" s="30"/>
-      <x:c r="G35" s="30"/>
-      <x:c r="H35" s="30"/>
-      <x:c r="I35" s="32" t="n">
+      <x:c r="C35" s="28"/>
+      <x:c r="D35" s="28"/>
+      <x:c r="E35" s="28"/>
+      <x:c r="F35" s="28"/>
+      <x:c r="G35" s="28"/>
+      <x:c r="H35" s="28"/>
+      <x:c r="I35" s="30" t="n">
         <x:f>ROUND(SUM(I33:I34),1)</x:f>
         <x:v>501</x:v>
       </x:c>
-      <x:c r="J35" s="30"/>
-      <x:c r="K35" s="30"/>
+      <x:c r="J35" s="28"/>
+      <x:c r="K35" s="28"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="31" t="str">
+      <x:c r="A36" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B36" s="30"/>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="30"/>
-      <x:c r="E36" s="30"/>
-      <x:c r="F36" s="30"/>
-      <x:c r="G36" s="30"/>
-      <x:c r="H36" s="30"/>
-      <x:c r="I36" s="34" t="n">
+      <x:c r="B36" s="28"/>
+      <x:c r="C36" s="28"/>
+      <x:c r="D36" s="28"/>
+      <x:c r="E36" s="28"/>
+      <x:c r="F36" s="28"/>
+      <x:c r="G36" s="28"/>
+      <x:c r="H36" s="28"/>
+      <x:c r="I36" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
         <x:v>250.5</x:v>
       </x:c>
-      <x:c r="J36" s="30"/>
-      <x:c r="K36" s="30"/>
+      <x:c r="J36" s="28"/>
+      <x:c r="K36" s="28"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="17" t="str">
@@ -2064,7 +2064,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>4562</x:v>
@@ -2076,15 +2076,15 @@
         <x:v>4532.8</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>4547</x:v>
+        <x:v>4560</x:v>
       </x:c>
       <x:c r="G41" s="23" t="n">
         <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>9.6</x:v>
+        <x:v>22.6</x:v>
       </x:c>
       <x:c r="H41" s="24" t="n">
         <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>0.0021157491074184076</x:v>
+        <x:v>0.00498082602371408</x:v>
       </x:c>
       <x:c r="I41" s="23" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
@@ -2094,46 +2094,46 @@
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B42" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C42" s="30"/>
-      <x:c r="D42" s="30"/>
-      <x:c r="E42" s="30"/>
-      <x:c r="F42" s="30"/>
-      <x:c r="G42" s="30"/>
-      <x:c r="H42" s="30"/>
-      <x:c r="I42" s="32" t="n">
+      <x:c r="C42" s="28"/>
+      <x:c r="D42" s="28"/>
+      <x:c r="E42" s="28"/>
+      <x:c r="F42" s="28"/>
+      <x:c r="G42" s="28"/>
+      <x:c r="H42" s="28"/>
+      <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
         <x:v>171.4</x:v>
       </x:c>
-      <x:c r="J42" s="30"/>
-      <x:c r="K42" s="30"/>
+      <x:c r="J42" s="28"/>
+      <x:c r="K42" s="28"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="31" t="str">
+      <x:c r="A43" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="30"/>
-      <x:c r="C43" s="30"/>
-      <x:c r="D43" s="30"/>
-      <x:c r="E43" s="30"/>
-      <x:c r="F43" s="30"/>
-      <x:c r="G43" s="30"/>
-      <x:c r="H43" s="30"/>
-      <x:c r="I43" s="34" t="n">
+      <x:c r="B43" s="28"/>
+      <x:c r="C43" s="28"/>
+      <x:c r="D43" s="28"/>
+      <x:c r="E43" s="28"/>
+      <x:c r="F43" s="28"/>
+      <x:c r="G43" s="28"/>
+      <x:c r="H43" s="28"/>
+      <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
         <x:v>85.7</x:v>
       </x:c>
-      <x:c r="J43" s="30"/>
-      <x:c r="K43" s="30"/>
+      <x:c r="J43" s="28"/>
+      <x:c r="K43" s="28"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="17" t="str">
@@ -2222,7 +2222,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>9月7日-9月8日</x:v>
+        <x:v>9月7日-9月9日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2923.2</x:v>
@@ -2231,67 +2231,67 @@
         <x:v>2931.4</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2891</x:v>
+        <x:v>2887.6</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2897</x:v>
+        <x:v>2901.2</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-18.8</x:v>
+        <x:v>-14.6</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.0064476301529597935</x:v>
+        <x:v>-0.0050072021400645594</x:v>
       </x:c>
       <x:c r="I48" s="23" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>40.4</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B49" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B49" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="32" t="n">
+      <x:c r="C49" s="28"/>
+      <x:c r="D49" s="28"/>
+      <x:c r="E49" s="28"/>
+      <x:c r="F49" s="28"/>
+      <x:c r="G49" s="28"/>
+      <x:c r="H49" s="28"/>
+      <x:c r="I49" s="30" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>108.4</x:v>
-      </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
+        <x:v>111.8</x:v>
+      </x:c>
+      <x:c r="J49" s="28"/>
+      <x:c r="K49" s="28"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="31" t="str">
+      <x:c r="A50" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B50" s="30"/>
-      <x:c r="C50" s="30"/>
-      <x:c r="D50" s="30"/>
-      <x:c r="E50" s="30"/>
-      <x:c r="F50" s="30"/>
-      <x:c r="G50" s="30"/>
-      <x:c r="H50" s="30"/>
-      <x:c r="I50" s="34" t="n">
+      <x:c r="B50" s="28"/>
+      <x:c r="C50" s="28"/>
+      <x:c r="D50" s="28"/>
+      <x:c r="E50" s="28"/>
+      <x:c r="F50" s="28"/>
+      <x:c r="G50" s="28"/>
+      <x:c r="H50" s="28"/>
+      <x:c r="I50" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>54.2</x:v>
-      </x:c>
-      <x:c r="J50" s="30"/>
-      <x:c r="K50" s="30"/>
+        <x:v>55.9</x:v>
+      </x:c>
+      <x:c r="J50" s="28"/>
+      <x:c r="K50" s="28"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="17" t="str">
@@ -2394,7 +2394,7 @@
       <x:c r="F55" s="23" t="n">
         <x:v>141320</x:v>
       </x:c>
-      <x:c r="G55" s="28" t="n">
+      <x:c r="G55" s="34" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
         <x:v>340</x:v>
       </x:c>
@@ -2414,42 +2414,42 @@
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="31" t="str">
+      <x:c r="A56" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B56" s="30" t="n">
+      <x:c r="B56" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
+      <x:c r="C56" s="28"/>
+      <x:c r="D56" s="28"/>
+      <x:c r="E56" s="28"/>
+      <x:c r="F56" s="28"/>
+      <x:c r="G56" s="28"/>
+      <x:c r="H56" s="28"/>
+      <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
         <x:v>22860</x:v>
       </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
+      <x:c r="J56" s="28"/>
+      <x:c r="K56" s="28"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="31" t="str">
+      <x:c r="A57" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
+      <x:c r="B57" s="28"/>
+      <x:c r="C57" s="28"/>
+      <x:c r="D57" s="28"/>
+      <x:c r="E57" s="28"/>
+      <x:c r="F57" s="28"/>
+      <x:c r="G57" s="28"/>
+      <x:c r="H57" s="28"/>
+      <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
         <x:v>11430</x:v>
       </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
+      <x:c r="J57" s="28"/>
+      <x:c r="K57" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2740,43 +2740,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>7676.86</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>7715.08</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>7602.5</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>7648.8</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-10.8</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.0014112990086961874</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>112.6</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>801.0999999999999</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>913.6999999999999</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>133.5</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>130.5</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3059,43 +3095,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>7793.04</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>7816.66</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>7723.82</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>7768.11</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-2.6</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.0003371626603935196</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>92.8</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>759.1</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>851.9</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>126.5</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>121.7</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3378,43 +3450,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>3943.92</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>3958.12</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>3933.47</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>3951.51</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>0.0027813376305338977</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>24.7</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>212.5</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>237.2</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>35.4</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3697,43 +3805,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>7671.8</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>7705</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>7575</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>7618.6</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>-14.8</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>-0.001938847695653223</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>903.2</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1033.2</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>150.5</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>147.6</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4017,42 +4161,42 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+      <x:c r="A12" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
+      <x:c r="B12" s="28" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="30" t="n">
         <x:f>SUM(J4:J9)</x:f>
         <x:v>919.4</x:v>
       </x:c>
-      <x:c r="K12" s="30"/>
+      <x:c r="K12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="A13" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
         <x:v>153.2</x:v>
       </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="K13" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4335,43 +4479,79 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>4564.2</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>4574.2</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>4535.6</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>4560</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>0.0028590279305036326</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>38.6</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>327.59999999999997</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>366.2</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>54.6</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>52.3</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4654,43 +4834,79 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="22" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>9月9日</x:v>
+      </x:c>
+      <x:c r="D10" s="23" t="n">
+        <x:v>2903.2</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="n">
+        <x:v>2909.8</x:v>
+      </x:c>
+      <x:c r="F10" s="23" t="n">
+        <x:v>2887.6</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="n">
+        <x:v>2901.2</x:v>
+      </x:c>
+      <x:c r="H10" s="23" t="n">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="I10" s="24" t="n">
+        <x:v>0.001449775629962069</x:v>
+      </x:c>
+      <x:c r="J10" s="23" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>22.2</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>198.20000000000002</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
+      <x:c r="B13" s="28" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="30" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>220.4</x:v>
+      </x:c>
+      <x:c r="K13" s="28"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="30"/>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="B14" s="28"/>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>31.5</x:v>
+      </x:c>
+      <x:c r="K14" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-10
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra43035a8c579445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2df3182e019a4b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R4ff0ac52df1d4731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R34cb832d7ee34852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3145353c23934a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rbf834805b71e4830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R3428758aaefd4cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R3bfe4397d0454d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R60c2c5c6d9c34b18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rdad28e337e0b43bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc46102d30f4a4c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rd07c33c1355c410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R59c1cabeff78444e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re53a24802835483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2fc132173f574c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R74df81fd4b5d4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R38bed62df0a740dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R387ac6b6d91c4095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rdfa9c3f390ed4cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R4b824e8871244371"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7715.08</x:v>
+        <x:v>7641.86</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7602.5</x:v>
+        <x:v>7564.67</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>112.6</x:v>
+        <x:v>77.2</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>913.7</x:v>
+        <x:v>990.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>130.5</x:v>
+        <x:v>123.9</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7816.66</x:v>
+        <x:v>7766.35</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7723.82</x:v>
+        <x:v>7696.55</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>92.8</x:v>
+        <x:v>69.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>851.9</x:v>
+        <x:v>921.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>121.7</x:v>
+        <x:v>115.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3958.12</x:v>
+        <x:v>3949.25</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3933.47</x:v>
+        <x:v>3927.35</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>24.7</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>237.2</x:v>
+        <x:v>259.1</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>33.9</x:v>
+        <x:v>32.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7804.8</x:v>
+        <x:v>7754.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7695.4</x:v>
+        <x:v>7664</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>109.4</x:v>
+        <x:v>90.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1028.8</x:v>
+        <x:v>1119.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>147</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4574.2</x:v>
+        <x:v>4565.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4535.6</x:v>
+        <x:v>4517.6</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>38.6</x:v>
+        <x:v>48.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>366.2</x:v>
+        <x:v>414.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>52.3</x:v>
+        <x:v>51.8</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2909.8</x:v>
+        <x:v>2908.4</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2887.6</x:v>
+        <x:v>2879.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>22.2</x:v>
+        <x:v>29.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>220.4</x:v>
+        <x:v>249.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>31.5</x:v>
+        <x:v>31.2</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-09</x:v>
+        <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1310,7 +1310,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7551.02</x:v>
@@ -1322,15 +1322,15 @@
         <x:v>7541.14</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7648.8</x:v>
+        <x:v>7587.75</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>140.7</x:v>
+        <x:v>79.7</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.018741117914143235</x:v>
+        <x:v>0.010609888799947731</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
@@ -1340,7 +1340,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1468,7 +1468,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7687.47</x:v>
@@ -1480,15 +1480,15 @@
         <x:v>7672.99</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7768.11</x:v>
+        <x:v>7717.8</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>115.4</x:v>
+        <x:v>65.1</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.01508227825771069</x:v>
+        <x:v>0.00850811936717677</x:v>
       </x:c>
       <x:c r="I13" s="23" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
@@ -1498,7 +1498,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1626,7 +1626,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3942.51</x:v>
@@ -1638,15 +1638,15 @@
         <x:v>3916.49</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3951.51</x:v>
+        <x:v>3934.4</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>21.4</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.005442581905896082</x:v>
+        <x:v>0.001089025271493016</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
@@ -1656,7 +1656,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1942,7 +1942,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C34" s="23" t="n">
         <x:v>7665.6</x:v>
@@ -1954,15 +1954,15 @@
         <x:v>7651.2</x:v>
       </x:c>
       <x:c r="F34" s="23" t="n">
-        <x:v>7738.6</x:v>
+        <x:v>7705.8</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
         <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>130.6</x:v>
+        <x:v>97.8</x:v>
       </x:c>
       <x:c r="H34" s="24" t="n">
         <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>0.017166140904311344</x:v>
+        <x:v>0.012854889589905438</x:v>
       </x:c>
       <x:c r="I34" s="26" t="n">
         <x:f>ROUND(D34-E34,1)</x:f>
@@ -1972,7 +1972,7 @@
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K34" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2100,7 +2100,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>4562</x:v>
@@ -2109,28 +2109,28 @@
         <x:v>4584</x:v>
       </x:c>
       <x:c r="E41" s="23" t="n">
-        <x:v>4532.8</x:v>
+        <x:v>4517.6</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>4560</x:v>
+        <x:v>4542.2</x:v>
       </x:c>
       <x:c r="G41" s="23" t="n">
         <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>22.6</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="H41" s="24" t="n">
         <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>0.00498082602371408</x:v>
+        <x:v>0.0010578745537093148</x:v>
       </x:c>
       <x:c r="I41" s="23" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>51.2</x:v>
+        <x:v>66.4</x:v>
       </x:c>
       <x:c r="J41" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2148,7 +2148,7 @@
       <x:c r="H42" s="28"/>
       <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>171.4</x:v>
+        <x:v>186.6</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
@@ -2166,7 +2166,7 @@
       <x:c r="H43" s="28"/>
       <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>85.7</x:v>
+        <x:v>93.3</x:v>
       </x:c>
       <x:c r="J43" s="28"/>
       <x:c r="K43" s="28"/>
@@ -2258,7 +2258,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>9月7日-9月9日</x:v>
+        <x:v>9月7日-9月10日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2923.2</x:v>
@@ -2267,28 +2267,28 @@
         <x:v>2931.4</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2887.6</x:v>
+        <x:v>2879.2</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2901.2</x:v>
+        <x:v>2897</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-14.6</x:v>
+        <x:v>-18.8</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.0050072021400645594</x:v>
+        <x:v>-0.0064476301529597935</x:v>
       </x:c>
       <x:c r="I48" s="23" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>43.8</x:v>
+        <x:v>52.2</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2306,7 +2306,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="30" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>111.8</x:v>
+        <x:v>120.2</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2324,7 +2324,7 @@
       <x:c r="H50" s="28"/>
       <x:c r="I50" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>55.9</x:v>
+        <x:v>60.1</x:v>
       </x:c>
       <x:c r="J50" s="28"/>
       <x:c r="K50" s="28"/>
@@ -2812,31 +2812,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>913.6999999999999</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7611.52</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7641.86</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7564.67</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>7587.75</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-61.1</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.007981644179479108</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>77.2</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -2844,11 +2862,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>130.5</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>990.9</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>123.9</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3167,31 +3203,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>851.9</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7731.63</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7766.35</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7696.55</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>7717.8</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-50.3</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.006476478834619992</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>69.8</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -3199,11 +3253,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>121.7</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>921.6999999999999</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>115.2</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3522,31 +3594,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>237.2</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>3939.09</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>3949.25</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>3927.35</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>3934.4</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-17.1</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.004329990307502696</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -3554,11 +3644,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>33.9</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>259.09999999999997</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>32.4</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4232,31 +4340,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1028.8</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7696.8</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7754.8</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7664</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>7705.8</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-32.8</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.00423849275062671</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>90.8</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -4264,11 +4390,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>147</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1119.6</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4587,31 +4731,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>366.2</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>4535.6</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>4565.8</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>4517.6</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>4542.2</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-17.8</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.003903508771929909</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>48.2</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -4619,11 +4781,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>52.3</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>414.4</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>51.8</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4942,31 +5122,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="28"/>
-      <x:c r="J13" s="30" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>220.4</x:v>
-      </x:c>
-      <x:c r="K13" s="28"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>9月10日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>2892</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>2908.4</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>2879.2</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>2897</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>-4.2</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>-0.0014476768233833148</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>29.2</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="28"/>
       <x:c r="D14" s="28"/>
       <x:c r="E14" s="28"/>
@@ -4974,11 +5172,29 @@
       <x:c r="G14" s="28"/>
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="28"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>31.5</x:v>
+      <x:c r="J14" s="30" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>249.6</x:v>
       </x:c>
       <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>31.2</x:v>
+      </x:c>
+      <x:c r="K15" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-11
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5df3ddae7e59455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re0d6d0bf6213454c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rea8705f8702843d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R56e439b0dbd44c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9eae1e2a4bdd4655"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re0e0255b73504064"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4462c2b789c74059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rcc9b75189e6e4fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R8442c124207a425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R09cc1293569645f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R79635d2925904f25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfb83d253b0834d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R2ae3c79ca5ec49b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R196fbcc2f3134630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rccd843930b584fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re82673bb0c804cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Redb925ade6494f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R88ecdf527d9040f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc495cd896d894730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rf06841941ea44f44"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7641.86</x:v>
+        <x:v>7506.24</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7564.67</x:v>
+        <x:v>7284.53</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>77.2</x:v>
+        <x:v>221.7</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>990.9</x:v>
+        <x:v>1212.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>123.9</x:v>
+        <x:v>134.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7766.35</x:v>
+        <x:v>7638.63</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7696.55</x:v>
+        <x:v>7451.12</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>69.8</x:v>
+        <x:v>187.5</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>921.7</x:v>
+        <x:v>1109.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>115.2</x:v>
+        <x:v>123.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3949.25</x:v>
+        <x:v>3912.32</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3927.35</x:v>
+        <x:v>3852.03</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>21.9</x:v>
+        <x:v>60.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>259.1</x:v>
+        <x:v>319.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>32.4</x:v>
+        <x:v>35.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7627.8</x:v>
+        <x:v>7488.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7534</x:v>
+        <x:v>7259.4</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>93.8</x:v>
+        <x:v>229.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1127</x:v>
+        <x:v>1356.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>140.9</x:v>
+        <x:v>150.7</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7754.8</x:v>
+        <x:v>7626</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7664</x:v>
+        <x:v>7418.8</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>90.8</x:v>
+        <x:v>207.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1119.6</x:v>
+        <x:v>1326.8</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>140</x:v>
+        <x:v>147.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4565.8</x:v>
+        <x:v>4514</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4517.6</x:v>
+        <x:v>4451.6</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>48.2</x:v>
+        <x:v>62.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>414.4</x:v>
+        <x:v>476.8</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>51.8</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2908.4</x:v>
+        <x:v>2876.6</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2879.2</x:v>
+        <x:v>2836.8</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>29.2</x:v>
+        <x:v>39.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>249.6</x:v>
+        <x:v>289.4</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>31.2</x:v>
+        <x:v>32.2</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2609</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>142500</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>139000</x:v>
+        <x:v>131900</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>3500</x:v>
+        <x:v>3600</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>37600</x:v>
+        <x:v>41200</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>4700</x:v>
+        <x:v>4577.8</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-10</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1191,31 +1191,49 @@
         <x:v>LC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>37600</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>134480</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>135500</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>131900</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>135500</x:v>
+      </x:c>
+      <x:c r="H12" s="34" t="n">
+        <x:v>-5020</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.035724452035297505</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -1223,11 +1241,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>4700</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>41200</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>4577.8</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1346,7 +1382,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7551.02</x:v>
@@ -1355,28 +1391,28 @@
         <x:v>7724.94</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
-        <x:v>7541.14</x:v>
+        <x:v>7284.53</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7587.75</x:v>
+        <x:v>7427.24</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>79.7</x:v>
+        <x:v>-80.9</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>0.010609888799947731</x:v>
+        <x:v>-0.010768384502583217</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>183.8</x:v>
+        <x:v>440.4</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1394,7 +1430,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>491.9</x:v>
+        <x:v>748.5</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1412,7 +1448,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>246</x:v>
+        <x:v>374.3</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1504,7 +1540,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7687.47</x:v>
@@ -1513,28 +1549,28 @@
         <x:v>7830.16</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>7672.99</x:v>
+        <x:v>7451.12</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7717.8</x:v>
+        <x:v>7580.54</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>65.1</x:v>
+        <x:v>-72.1</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>0.00850811936717677</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="n">
+        <x:v>-0.009428057323633832</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>157.2</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1552,7 +1588,7 @@
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>502.2</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="J14" s="28"/>
       <x:c r="K14" s="28"/>
@@ -1570,7 +1606,7 @@
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>251.1</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="J15" s="28"/>
       <x:c r="K15" s="28"/>
@@ -1662,7 +1698,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3942.51</x:v>
@@ -1671,28 +1707,28 @@
         <x:v>3958.12</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3916.49</x:v>
+        <x:v>3852.03</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3934.4</x:v>
+        <x:v>3888.11</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>4.3</x:v>
+        <x:v>-42</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>0.001089025271493016</x:v>
-      </x:c>
-      <x:c r="I20" s="23" t="n">
+        <x:v>-0.010689241040986008</x:v>
+      </x:c>
+      <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>41.6</x:v>
+        <x:v>106.1</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1710,7 +1746,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>121.6</x:v>
+        <x:v>186.1</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1728,7 +1764,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>60.8</x:v>
+        <x:v>93.1</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -1820,7 +1856,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7527.2</x:v>
@@ -1829,28 +1865,28 @@
         <x:v>7714.6</x:v>
       </x:c>
       <x:c r="E27" s="23" t="n">
-        <x:v>7512.6</x:v>
+        <x:v>7259.4</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>7574</x:v>
+        <x:v>7415.2</x:v>
       </x:c>
       <x:c r="G27" s="23" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>105.8</x:v>
+        <x:v>-53</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>0.014166733617203553</x:v>
+        <x:v>-0.007096756915990432</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>202</x:v>
+        <x:v>455.2</x:v>
       </x:c>
       <x:c r="J27" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1868,7 +1904,7 @@
       <x:c r="H28" s="28"/>
       <x:c r="I28" s="30" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>491</x:v>
+        <x:v>744.2</x:v>
       </x:c>
       <x:c r="J28" s="28"/>
       <x:c r="K28" s="28"/>
@@ -1886,7 +1922,7 @@
       <x:c r="H29" s="28"/>
       <x:c r="I29" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>245.5</x:v>
+        <x:v>372.1</x:v>
       </x:c>
       <x:c r="J29" s="28"/>
       <x:c r="K29" s="28"/>
@@ -1978,7 +2014,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C34" s="23" t="n">
         <x:v>7665.6</x:v>
@@ -1987,28 +2023,28 @@
         <x:v>7817.2</x:v>
       </x:c>
       <x:c r="E34" s="23" t="n">
-        <x:v>7651.2</x:v>
+        <x:v>7418.8</x:v>
       </x:c>
       <x:c r="F34" s="23" t="n">
-        <x:v>7705.8</x:v>
+        <x:v>7569</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
         <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>97.8</x:v>
+        <x:v>-39</x:v>
       </x:c>
       <x:c r="H34" s="24" t="n">
         <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>0.012854889589905438</x:v>
+        <x:v>-0.005126182965299653</x:v>
       </x:c>
       <x:c r="I34" s="26" t="n">
         <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>166</x:v>
+        <x:v>398.4</x:v>
       </x:c>
       <x:c r="J34" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K34" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2026,7 +2062,7 @@
       <x:c r="H35" s="28"/>
       <x:c r="I35" s="30" t="n">
         <x:f>ROUND(SUM(I33:I34),1)</x:f>
-        <x:v>501</x:v>
+        <x:v>733.4</x:v>
       </x:c>
       <x:c r="J35" s="28"/>
       <x:c r="K35" s="28"/>
@@ -2044,7 +2080,7 @@
       <x:c r="H36" s="28"/>
       <x:c r="I36" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
-        <x:v>250.5</x:v>
+        <x:v>366.7</x:v>
       </x:c>
       <x:c r="J36" s="28"/>
       <x:c r="K36" s="28"/>
@@ -2136,7 +2172,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>4562</x:v>
@@ -2145,28 +2181,28 @@
         <x:v>4584</x:v>
       </x:c>
       <x:c r="E41" s="23" t="n">
-        <x:v>4517.6</x:v>
+        <x:v>4451.6</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>4542.2</x:v>
+        <x:v>4503.4</x:v>
       </x:c>
       <x:c r="G41" s="23" t="n">
         <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>4.8</x:v>
+        <x:v>-34</x:v>
       </x:c>
       <x:c r="H41" s="24" t="n">
         <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>0.0010578745537093148</x:v>
-      </x:c>
-      <x:c r="I41" s="23" t="n">
+        <x:v>-0.007493278088773314</x:v>
+      </x:c>
+      <x:c r="I41" s="26" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>66.4</x:v>
+        <x:v>132.4</x:v>
       </x:c>
       <x:c r="J41" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2184,7 +2220,7 @@
       <x:c r="H42" s="28"/>
       <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>186.6</x:v>
+        <x:v>252.6</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
@@ -2202,7 +2238,7 @@
       <x:c r="H43" s="28"/>
       <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>93.3</x:v>
+        <x:v>126.3</x:v>
       </x:c>
       <x:c r="J43" s="28"/>
       <x:c r="K43" s="28"/>
@@ -2294,7 +2330,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2923.2</x:v>
@@ -2303,28 +2339,28 @@
         <x:v>2931.4</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2879.2</x:v>
+        <x:v>2836.8</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2897</x:v>
+        <x:v>2867</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-18.8</x:v>
+        <x:v>-48.8</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.0064476301529597935</x:v>
-      </x:c>
-      <x:c r="I48" s="23" t="n">
+        <x:v>-0.01673640167364021</x:v>
+      </x:c>
+      <x:c r="I48" s="26" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>52.2</x:v>
+        <x:v>94.6</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2342,7 +2378,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="30" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>120.2</x:v>
+        <x:v>162.6</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2360,7 +2396,7 @@
       <x:c r="H50" s="28"/>
       <x:c r="I50" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>60.1</x:v>
+        <x:v>81.3</x:v>
       </x:c>
       <x:c r="J50" s="28"/>
       <x:c r="K50" s="28"/>
@@ -2452,7 +2488,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>9月7日-9月10日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>142120</x:v>
@@ -2461,28 +2497,28 @@
         <x:v>143200</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
-        <x:v>139000</x:v>
+        <x:v>131900</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>140520</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="G55" s="34" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-460</x:v>
+        <x:v>-5480</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.0032628741665484684</x:v>
-      </x:c>
-      <x:c r="I55" s="23" t="n">
+        <x:v>-0.038870761810185894</x:v>
+      </x:c>
+      <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>4200</x:v>
+        <x:v>11300</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>LC2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2500,7 +2536,7 @@
       <x:c r="H56" s="28"/>
       <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>23740</x:v>
+        <x:v>30840</x:v>
       </x:c>
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
@@ -2518,7 +2554,7 @@
       <x:c r="H57" s="28"/>
       <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
-        <x:v>11870</x:v>
+        <x:v>15420</x:v>
       </x:c>
       <x:c r="J57" s="28"/>
       <x:c r="K57" s="28"/>
@@ -2884,31 +2920,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>990.9</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>7504.66</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>7506.24</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7284.53</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7427.24</x:v>
+      </x:c>
+      <x:c r="H12" s="34" t="n">
+        <x:v>-160.5</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.021153833481598605</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>221.7</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -2916,11 +2970,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>123.9</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1212.6</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>134.7</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3275,31 +3347,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>921.6999999999999</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>7638.63</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>7638.63</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7451.12</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7580.54</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-137.3</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.017784860970742944</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>187.5</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -3307,11 +3397,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>115.2</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1109.1999999999998</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>123.2</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3666,31 +3774,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>259.09999999999997</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>3910.92</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>3912.32</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>3852.03</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>3888.11</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-46.3</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.011765453436356266</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>60.3</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -3698,11 +3824,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>32.4</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>319.4</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>35.5</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4057,31 +4201,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1127</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>7480</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>7488.8</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7259.4</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7415.2</x:v>
+      </x:c>
+      <x:c r="H12" s="34" t="n">
+        <x:v>-158.8</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.020966464219698944</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>229.4</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -4089,11 +4251,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>140.9</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1356.4</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>150.7</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4448,31 +4628,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1119.6</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>7626</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>7626</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>7418.8</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>7569</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-136.8</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.017752861480962445</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>207.2</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -4480,11 +4678,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>140</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1326.8</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>147.4</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4839,31 +5055,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>414.4</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>4508.2</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>4514</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>4451.6</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>4503.4</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-38.8</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.00854211615516709</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>62.4</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -4871,11 +5105,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>51.8</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>476.79999999999995</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5230,31 +5482,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="28"/>
-      <x:c r="J14" s="30" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>249.6</x:v>
-      </x:c>
-      <x:c r="K14" s="28"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>9月11日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>2872.4</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>2876.6</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>2836.8</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>2867</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-30</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.010355540214014525</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>39.8</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="28"/>
       <x:c r="D15" s="28"/>
       <x:c r="E15" s="28"/>
@@ -5262,11 +5532,29 @@
       <x:c r="G15" s="28"/>
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="28"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>31.2</x:v>
+      <x:c r="J15" s="30" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>289.4</x:v>
       </x:c>
       <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="28"/>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>32.2</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-14
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R79635d2925904f25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfb83d253b0834d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R2ae3c79ca5ec49b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R196fbcc2f3134630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rccd843930b584fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re82673bb0c804cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Redb925ade6494f62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R88ecdf527d9040f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc495cd896d894730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rf06841941ea44f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra7552cfc5e30495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R04568498b09d40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ra753228ef1ae454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rfdf532450bc14cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rbcddd9b08c9a4c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R850c298251934675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re6bc2b2754c54f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Ra7f1b2b6d72d4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R512cdf205b3f4fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="Rf1fdb065f5bc4b5f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7506.24</x:v>
+        <x:v>7501.14</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7284.53</x:v>
+        <x:v>7329.6</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>221.7</x:v>
+        <x:v>171.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1212.6</x:v>
+        <x:v>1384.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>134.7</x:v>
+        <x:v>138.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,22 +514,22 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7638.63</x:v>
+        <x:v>7610.03</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7451.12</x:v>
+        <x:v>7487.46</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>187.5</x:v>
+        <x:v>122.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1109.2</x:v>
+        <x:v>1231.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
         <x:v>123.2</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3912.32</x:v>
+        <x:v>3895.51</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3852.03</x:v>
+        <x:v>3867.02</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>60.3</x:v>
+        <x:v>28.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>319.4</x:v>
+        <x:v>347.9</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.5</x:v>
+        <x:v>34.8</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7488.8</x:v>
+        <x:v>7483</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7259.4</x:v>
+        <x:v>7283.4</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>229.4</x:v>
+        <x:v>199.6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1356.4</x:v>
+        <x:v>1556</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>150.7</x:v>
+        <x:v>155.6</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4514</x:v>
+        <x:v>4500.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4451.6</x:v>
+        <x:v>4458</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>62.4</x:v>
+        <x:v>42.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>476.8</x:v>
+        <x:v>519.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>53</x:v>
+        <x:v>51.9</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2876.6</x:v>
+        <x:v>2864.6</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2836.8</x:v>
+        <x:v>2843.8</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>39.8</x:v>
+        <x:v>20.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>289.4</x:v>
+        <x:v>310.2</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>32.2</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1416,1160 +1416,1388 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="30" t="n">
-        <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>748.5</x:v>
-      </x:c>
-      <x:c r="J7" s="28"/>
-      <x:c r="K7" s="28"/>
+      <x:c r="A7" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="n">
+        <x:v>7363.42</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>7501.14</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7329.6</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>7468.3</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:f>ROUND(F7-F6,1)</x:f>
+        <x:v>41.1</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="n">
+        <x:f>IFERROR(F7/F6-1,"")</x:f>
+        <x:v>0.005528298533506337</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>171.5</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
       <x:c r="F8" s="28"/>
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
-      <x:c r="I8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>374.3</x:v>
+      <x:c r="I8" s="30" t="n">
+        <x:f>ROUND(SUM(I5:I7),1)</x:f>
+        <x:v>920</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="17" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
+        <x:v>306.7</x:v>
+      </x:c>
+      <x:c r="J9" s="28"/>
+      <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B10" s="17"/>
-      <x:c r="C10" s="17"/>
-      <x:c r="D10" s="17"/>
-      <x:c r="E10" s="17"/>
-      <x:c r="F10" s="17"/>
-      <x:c r="G10" s="17"/>
-      <x:c r="H10" s="17"/>
-      <x:c r="I10" s="17"/>
-      <x:c r="J10" s="17"/>
-      <x:c r="K10" s="17"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="20" t="str">
+      <x:c r="B11" s="17"/>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="17"/>
+      <x:c r="E11" s="17"/>
+      <x:c r="F11" s="17"/>
+      <x:c r="G11" s="17"/>
+      <x:c r="H11" s="17"/>
+      <x:c r="I11" s="17"/>
+      <x:c r="J11" s="17"/>
+      <x:c r="K11" s="17"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
+      <x:c r="B12" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="str">
+      <x:c r="C12" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D11" s="20" t="str">
+      <x:c r="D12" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E11" s="20" t="str">
+      <x:c r="E12" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F11" s="20" t="str">
+      <x:c r="F12" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G11" s="20" t="str">
+      <x:c r="G12" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H11" s="20" t="str">
+      <x:c r="H12" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I11" s="20" t="str">
+      <x:c r="I12" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J11" s="20" t="str">
+      <x:c r="J12" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K11" s="20" t="str">
+      <x:c r="K12" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B12" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C12" s="23" t="n">
-        <x:v>7944.29</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="n">
-        <x:v>7955.57</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="n">
-        <x:v>7610.58</x:v>
-      </x:c>
-      <x:c r="F12" s="23" t="n">
-        <x:v>7652.69</x:v>
-      </x:c>
-      <x:c r="G12" s="23"/>
-      <x:c r="H12" s="24"/>
-      <x:c r="I12" s="26" t="n">
-        <x:f>ROUND(D12-E12,1)</x:f>
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="J12" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K12" s="22" t="n">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
-        <x:v>7687.47</x:v>
+        <x:v>7944.29</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>7830.16</x:v>
+        <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>7451.12</x:v>
+        <x:v>7610.58</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7580.54</x:v>
-      </x:c>
-      <x:c r="G13" s="23" t="n">
-        <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-72.1</x:v>
-      </x:c>
-      <x:c r="H13" s="24" t="n">
-        <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.009428057323633832</x:v>
-      </x:c>
+        <x:v>7652.69</x:v>
+      </x:c>
+      <x:c r="G13" s="23"/>
+      <x:c r="H13" s="24"/>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>379</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="n">
+        <x:v>7687.47</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7830.16</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7451.12</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7580.54</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:f>ROUND(F14-F13,1)</x:f>
+        <x:v>-72.1</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="n">
+        <x:f>IFERROR(F14/F13-1,"")</x:f>
+        <x:v>-0.009428057323633832</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="n">
+        <x:f>ROUND(D14-E14,1)</x:f>
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="n">
+        <x:v>7511.04</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7610.03</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7487.46</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7571.2</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:f>ROUND(F15-F14,1)</x:f>
+        <x:v>-9.3</x:v>
+      </x:c>
+      <x:c r="H15" s="24" t="n">
+        <x:f>IFERROR(F15/F14-1,"")</x:f>
+        <x:v>-0.0012321021985240987</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="n">
+        <x:f>ROUND(D15-E15,1)</x:f>
+        <x:v>122.6</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B16" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="30" t="n">
+        <x:f>ROUND(SUM(I13:I15),1)</x:f>
+        <x:v>846.6</x:v>
+      </x:c>
+      <x:c r="J16" s="28"/>
+      <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
+        <x:v>282.2</x:v>
+      </x:c>
+      <x:c r="J17" s="28"/>
+      <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B19" s="17"/>
+      <x:c r="C19" s="17"/>
+      <x:c r="D19" s="17"/>
+      <x:c r="E19" s="17"/>
+      <x:c r="F19" s="17"/>
+      <x:c r="G19" s="17"/>
+      <x:c r="H19" s="17"/>
+      <x:c r="I19" s="17"/>
+      <x:c r="J19" s="17"/>
+      <x:c r="K19" s="17"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E20" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G20" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J20" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K20" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="n">
+        <x:v>3979.88</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>3995.18</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>3915.22</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>3930.12</x:v>
+      </x:c>
+      <x:c r="G21" s="23"/>
+      <x:c r="H21" s="24"/>
+      <x:c r="I21" s="26" t="n">
+        <x:f>ROUND(D21-E21,1)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="30" t="n">
-        <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>724</x:v>
-      </x:c>
-      <x:c r="J14" s="28"/>
-      <x:c r="K14" s="28"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="B22" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="n">
+        <x:v>3942.51</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>3958.12</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>3852.03</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>3888.11</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:f>ROUND(F22-F21,1)</x:f>
+        <x:v>-42</x:v>
+      </x:c>
+      <x:c r="H22" s="24" t="n">
+        <x:f>IFERROR(F22/F21-1,"")</x:f>
+        <x:v>-0.010689241040986008</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="n">
+        <x:f>ROUND(D22-E22,1)</x:f>
+        <x:v>106.1</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>3895.51</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>3885.33</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:f>ROUND(F23-F22,1)</x:f>
+        <x:v>-2.8</x:v>
+      </x:c>
+      <x:c r="H23" s="24" t="n">
+        <x:f>IFERROR(F23/F22-1,"")</x:f>
+        <x:v>-0.0007150003472125022</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="n">
+        <x:f>ROUND(D23-E23,1)</x:f>
+        <x:v>28.5</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="28"/>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="30" t="n">
+        <x:f>ROUND(SUM(I21:I23),1)</x:f>
+        <x:v>214.6</x:v>
+      </x:c>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="28"/>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>362</x:v>
-      </x:c>
-      <x:c r="J15" s="28"/>
-      <x:c r="K15" s="28"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B17" s="17"/>
-      <x:c r="C17" s="17"/>
-      <x:c r="D17" s="17"/>
-      <x:c r="E17" s="17"/>
-      <x:c r="F17" s="17"/>
-      <x:c r="G17" s="17"/>
-      <x:c r="H17" s="17"/>
-      <x:c r="I17" s="17"/>
-      <x:c r="J17" s="17"/>
-      <x:c r="K17" s="17"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="20" t="str">
+      <x:c r="B25" s="28"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
+        <x:v>71.5</x:v>
+      </x:c>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
+      <x:c r="E27" s="17"/>
+      <x:c r="F27" s="17"/>
+      <x:c r="G27" s="17"/>
+      <x:c r="H27" s="17"/>
+      <x:c r="I27" s="17"/>
+      <x:c r="J27" s="17"/>
+      <x:c r="K27" s="17"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B18" s="20" t="str">
+      <x:c r="B28" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C18" s="20" t="str">
+      <x:c r="C28" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D18" s="20" t="str">
+      <x:c r="D28" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E18" s="20" t="str">
+      <x:c r="E28" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F18" s="20" t="str">
+      <x:c r="F28" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G18" s="20" t="str">
+      <x:c r="G28" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H18" s="20" t="str">
+      <x:c r="H28" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I18" s="20" t="str">
+      <x:c r="I28" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J18" s="20" t="str">
+      <x:c r="J28" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K18" s="20" t="str">
+      <x:c r="K28" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="22" t="n">
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B19" s="22" t="str">
+      <x:c r="B29" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C19" s="23" t="n">
-        <x:v>3979.88</x:v>
-      </x:c>
-      <x:c r="D19" s="23" t="n">
-        <x:v>3995.18</x:v>
-      </x:c>
-      <x:c r="E19" s="23" t="n">
-        <x:v>3915.22</x:v>
-      </x:c>
-      <x:c r="F19" s="23" t="n">
-        <x:v>3930.12</x:v>
-      </x:c>
-      <x:c r="G19" s="23"/>
-      <x:c r="H19" s="24"/>
-      <x:c r="I19" s="26" t="n">
-        <x:f>ROUND(D19-E19,1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J19" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K19" s="22" t="n">
+      <x:c r="C29" s="23" t="n">
+        <x:v>7713.4</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>7721</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>7432</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>7468.2</x:v>
+      </x:c>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="22" t="n">
+    <x:row r="30">
+      <x:c r="A30" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B20" s="22" t="str">
+      <x:c r="B30" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C20" s="23" t="n">
-        <x:v>3942.51</x:v>
-      </x:c>
-      <x:c r="D20" s="23" t="n">
-        <x:v>3958.12</x:v>
-      </x:c>
-      <x:c r="E20" s="23" t="n">
-        <x:v>3852.03</x:v>
-      </x:c>
-      <x:c r="F20" s="23" t="n">
-        <x:v>3888.11</x:v>
-      </x:c>
-      <x:c r="G20" s="23" t="n">
-        <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-42</x:v>
-      </x:c>
-      <x:c r="H20" s="24" t="n">
-        <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.010689241040986008</x:v>
-      </x:c>
-      <x:c r="I20" s="26" t="n">
-        <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>106.1</x:v>
-      </x:c>
-      <x:c r="J20" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K20" s="22" t="n">
+      <x:c r="C30" s="23" t="n">
+        <x:v>7527.2</x:v>
+      </x:c>
+      <x:c r="D30" s="23" t="n">
+        <x:v>7714.6</x:v>
+      </x:c>
+      <x:c r="E30" s="23" t="n">
+        <x:v>7259.4</x:v>
+      </x:c>
+      <x:c r="F30" s="23" t="n">
+        <x:v>7415.2</x:v>
+      </x:c>
+      <x:c r="G30" s="23" t="n">
+        <x:f>ROUND(F30-F29,1)</x:f>
+        <x:v>-53</x:v>
+      </x:c>
+      <x:c r="H30" s="24" t="n">
+        <x:f>IFERROR(F30/F29-1,"")</x:f>
+        <x:v>-0.007096756915990432</x:v>
+      </x:c>
+      <x:c r="I30" s="26" t="n">
+        <x:f>ROUND(D30-E30,1)</x:f>
+        <x:v>455.2</x:v>
+      </x:c>
+      <x:c r="J30" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K30" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="29" t="str">
+    <x:row r="31">
+      <x:c r="A31" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B31" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C31" s="23" t="n">
+        <x:v>7312</x:v>
+      </x:c>
+      <x:c r="D31" s="23" t="n">
+        <x:v>7483</x:v>
+      </x:c>
+      <x:c r="E31" s="23" t="n">
+        <x:v>7283.4</x:v>
+      </x:c>
+      <x:c r="F31" s="23" t="n">
+        <x:v>7470</x:v>
+      </x:c>
+      <x:c r="G31" s="23" t="n">
+        <x:f>ROUND(F31-F30,1)</x:f>
+        <x:v>54.8</x:v>
+      </x:c>
+      <x:c r="H31" s="24" t="n">
+        <x:f>IFERROR(F31/F30-1,"")</x:f>
+        <x:v>0.007390225482792223</x:v>
+      </x:c>
+      <x:c r="I31" s="26" t="n">
+        <x:f>ROUND(D31-E31,1)</x:f>
+        <x:v>199.6</x:v>
+      </x:c>
+      <x:c r="J31" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K31" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B21" s="28" t="n">
+      <x:c r="B32" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C32" s="28"/>
+      <x:c r="D32" s="28"/>
+      <x:c r="E32" s="28"/>
+      <x:c r="F32" s="28"/>
+      <x:c r="G32" s="28"/>
+      <x:c r="H32" s="28"/>
+      <x:c r="I32" s="30" t="n">
+        <x:f>ROUND(SUM(I29:I31),1)</x:f>
+        <x:v>943.8</x:v>
+      </x:c>
+      <x:c r="J32" s="28"/>
+      <x:c r="K32" s="28"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B33" s="28"/>
+      <x:c r="C33" s="28"/>
+      <x:c r="D33" s="28"/>
+      <x:c r="E33" s="28"/>
+      <x:c r="F33" s="28"/>
+      <x:c r="G33" s="28"/>
+      <x:c r="H33" s="28"/>
+      <x:c r="I33" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
+        <x:v>314.6</x:v>
+      </x:c>
+      <x:c r="J33" s="28"/>
+      <x:c r="K33" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B35" s="17"/>
+      <x:c r="C35" s="17"/>
+      <x:c r="D35" s="17"/>
+      <x:c r="E35" s="17"/>
+      <x:c r="F35" s="17"/>
+      <x:c r="G35" s="17"/>
+      <x:c r="H35" s="17"/>
+      <x:c r="I35" s="17"/>
+      <x:c r="J35" s="17"/>
+      <x:c r="K35" s="17"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C36" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D36" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E36" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F36" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G36" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H36" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I36" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J36" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K36" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C37" s="23" t="n">
+        <x:v>7880.8</x:v>
+      </x:c>
+      <x:c r="D37" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="E37" s="23" t="n">
+        <x:v>7568</x:v>
+      </x:c>
+      <x:c r="F37" s="23" t="n">
+        <x:v>7608</x:v>
+      </x:c>
+      <x:c r="G37" s="23"/>
+      <x:c r="H37" s="24"/>
+      <x:c r="I37" s="26" t="n">
+        <x:f>ROUND(D37-E37,1)</x:f>
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="J37" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K37" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C21" s="28"/>
-      <x:c r="D21" s="28"/>
-      <x:c r="E21" s="28"/>
-      <x:c r="F21" s="28"/>
-      <x:c r="G21" s="28"/>
-      <x:c r="H21" s="28"/>
-      <x:c r="I21" s="30" t="n">
-        <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>186.1</x:v>
-      </x:c>
-      <x:c r="J21" s="28"/>
-      <x:c r="K21" s="28"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="29" t="str">
+      <x:c r="B38" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C38" s="23" t="n">
+        <x:v>7665.6</x:v>
+      </x:c>
+      <x:c r="D38" s="23" t="n">
+        <x:v>7817.2</x:v>
+      </x:c>
+      <x:c r="E38" s="23" t="n">
+        <x:v>7418.8</x:v>
+      </x:c>
+      <x:c r="F38" s="23" t="n">
+        <x:v>7569</x:v>
+      </x:c>
+      <x:c r="G38" s="23" t="n">
+        <x:f>ROUND(F38-F37,1)</x:f>
+        <x:v>-39</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="n">
+        <x:f>IFERROR(F38/F37-1,"")</x:f>
+        <x:v>-0.005126182965299653</x:v>
+      </x:c>
+      <x:c r="I38" s="26" t="n">
+        <x:f>ROUND(D38-E38,1)</x:f>
+        <x:v>398.4</x:v>
+      </x:c>
+      <x:c r="J38" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K38" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B39" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C39" s="28"/>
+      <x:c r="D39" s="28"/>
+      <x:c r="E39" s="28"/>
+      <x:c r="F39" s="28"/>
+      <x:c r="G39" s="28"/>
+      <x:c r="H39" s="28"/>
+      <x:c r="I39" s="30" t="n">
+        <x:f>ROUND(SUM(I37:I38),1)</x:f>
+        <x:v>733.4</x:v>
+      </x:c>
+      <x:c r="J39" s="28"/>
+      <x:c r="K39" s="28"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="28"/>
-      <x:c r="C22" s="28"/>
-      <x:c r="D22" s="28"/>
-      <x:c r="E22" s="28"/>
-      <x:c r="F22" s="28"/>
-      <x:c r="G22" s="28"/>
-      <x:c r="H22" s="28"/>
-      <x:c r="I22" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>93.1</x:v>
-      </x:c>
-      <x:c r="J22" s="28"/>
-      <x:c r="K22" s="28"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B24" s="17"/>
-      <x:c r="C24" s="17"/>
-      <x:c r="D24" s="17"/>
-      <x:c r="E24" s="17"/>
-      <x:c r="F24" s="17"/>
-      <x:c r="G24" s="17"/>
-      <x:c r="H24" s="17"/>
-      <x:c r="I24" s="17"/>
-      <x:c r="J24" s="17"/>
-      <x:c r="K24" s="17"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="20" t="str">
+      <x:c r="B40" s="28"/>
+      <x:c r="C40" s="28"/>
+      <x:c r="D40" s="28"/>
+      <x:c r="E40" s="28"/>
+      <x:c r="F40" s="28"/>
+      <x:c r="G40" s="28"/>
+      <x:c r="H40" s="28"/>
+      <x:c r="I40" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I37:I38),0),1)</x:f>
+        <x:v>366.7</x:v>
+      </x:c>
+      <x:c r="J40" s="28"/>
+      <x:c r="K40" s="28"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B42" s="17"/>
+      <x:c r="C42" s="17"/>
+      <x:c r="D42" s="17"/>
+      <x:c r="E42" s="17"/>
+      <x:c r="F42" s="17"/>
+      <x:c r="G42" s="17"/>
+      <x:c r="H42" s="17"/>
+      <x:c r="I42" s="17"/>
+      <x:c r="J42" s="17"/>
+      <x:c r="K42" s="17"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B25" s="20" t="str">
+      <x:c r="B43" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C25" s="20" t="str">
+      <x:c r="C43" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D25" s="20" t="str">
+      <x:c r="D43" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E25" s="20" t="str">
+      <x:c r="E43" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F25" s="20" t="str">
+      <x:c r="F43" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G25" s="20" t="str">
+      <x:c r="G43" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H25" s="20" t="str">
+      <x:c r="H43" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I25" s="20" t="str">
+      <x:c r="I43" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J25" s="20" t="str">
+      <x:c r="J43" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K25" s="20" t="str">
+      <x:c r="K43" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="22" t="n">
+    <x:row r="44">
+      <x:c r="A44" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B26" s="22" t="str">
+      <x:c r="B44" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C26" s="23" t="n">
-        <x:v>7713.4</x:v>
-      </x:c>
-      <x:c r="D26" s="23" t="n">
-        <x:v>7721</x:v>
-      </x:c>
-      <x:c r="E26" s="23" t="n">
-        <x:v>7432</x:v>
-      </x:c>
-      <x:c r="F26" s="23" t="n">
-        <x:v>7468.2</x:v>
-      </x:c>
-      <x:c r="G26" s="23"/>
-      <x:c r="H26" s="24"/>
-      <x:c r="I26" s="26" t="n">
-        <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J26" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K26" s="22" t="n">
+      <x:c r="C44" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="D44" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="E44" s="23" t="n">
+        <x:v>4497.6</x:v>
+      </x:c>
+      <x:c r="F44" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="G44" s="23"/>
+      <x:c r="H44" s="24"/>
+      <x:c r="I44" s="26" t="n">
+        <x:f>ROUND(D44-E44,1)</x:f>
+        <x:v>120.2</x:v>
+      </x:c>
+      <x:c r="J44" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K44" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="22" t="n">
+    <x:row r="45">
+      <x:c r="A45" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B27" s="22" t="str">
+      <x:c r="B45" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C27" s="23" t="n">
-        <x:v>7527.2</x:v>
-      </x:c>
-      <x:c r="D27" s="23" t="n">
-        <x:v>7714.6</x:v>
-      </x:c>
-      <x:c r="E27" s="23" t="n">
-        <x:v>7259.4</x:v>
-      </x:c>
-      <x:c r="F27" s="23" t="n">
-        <x:v>7415.2</x:v>
-      </x:c>
-      <x:c r="G27" s="23" t="n">
-        <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>-53</x:v>
-      </x:c>
-      <x:c r="H27" s="24" t="n">
-        <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>-0.007096756915990432</x:v>
-      </x:c>
-      <x:c r="I27" s="26" t="n">
-        <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>455.2</x:v>
-      </x:c>
-      <x:c r="J27" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K27" s="22" t="n">
+      <x:c r="C45" s="23" t="n">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="n">
+        <x:v>4584</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="n">
+        <x:v>4451.6</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="n">
+        <x:v>4503.4</x:v>
+      </x:c>
+      <x:c r="G45" s="23" t="n">
+        <x:f>ROUND(F45-F44,1)</x:f>
+        <x:v>-34</x:v>
+      </x:c>
+      <x:c r="H45" s="24" t="n">
+        <x:f>IFERROR(F45/F44-1,"")</x:f>
+        <x:v>-0.007493278088773314</x:v>
+      </x:c>
+      <x:c r="I45" s="26" t="n">
+        <x:f>ROUND(D45-E45,1)</x:f>
+        <x:v>132.4</x:v>
+      </x:c>
+      <x:c r="J45" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K45" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="29" t="str">
+    <x:row r="46">
+      <x:c r="A46" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="n">
+        <x:v>4468</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="n">
+        <x:v>4500.6</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="n">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="n">
+        <x:v>4480.2</x:v>
+      </x:c>
+      <x:c r="G46" s="23" t="n">
+        <x:f>ROUND(F46-F45,1)</x:f>
+        <x:v>-23.2</x:v>
+      </x:c>
+      <x:c r="H46" s="24" t="n">
+        <x:f>IFERROR(F46/F45-1,"")</x:f>
+        <x:v>-0.005151663187813571</x:v>
+      </x:c>
+      <x:c r="I46" s="23" t="n">
+        <x:f>ROUND(D46-E46,1)</x:f>
+        <x:v>42.6</x:v>
+      </x:c>
+      <x:c r="J46" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K46" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B28" s="28" t="n">
+      <x:c r="B47" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C47" s="28"/>
+      <x:c r="D47" s="28"/>
+      <x:c r="E47" s="28"/>
+      <x:c r="F47" s="28"/>
+      <x:c r="G47" s="28"/>
+      <x:c r="H47" s="28"/>
+      <x:c r="I47" s="30" t="n">
+        <x:f>ROUND(SUM(I44:I46),1)</x:f>
+        <x:v>295.2</x:v>
+      </x:c>
+      <x:c r="J47" s="28"/>
+      <x:c r="K47" s="28"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B48" s="28"/>
+      <x:c r="C48" s="28"/>
+      <x:c r="D48" s="28"/>
+      <x:c r="E48" s="28"/>
+      <x:c r="F48" s="28"/>
+      <x:c r="G48" s="28"/>
+      <x:c r="H48" s="28"/>
+      <x:c r="I48" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I44:I46),0),1)</x:f>
+        <x:v>98.4</x:v>
+      </x:c>
+      <x:c r="J48" s="28"/>
+      <x:c r="K48" s="28"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B50" s="17"/>
+      <x:c r="C50" s="17"/>
+      <x:c r="D50" s="17"/>
+      <x:c r="E50" s="17"/>
+      <x:c r="F50" s="17"/>
+      <x:c r="G50" s="17"/>
+      <x:c r="H50" s="17"/>
+      <x:c r="I50" s="17"/>
+      <x:c r="J50" s="17"/>
+      <x:c r="K50" s="17"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B51" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C51" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D51" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E51" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F51" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G51" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H51" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I51" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J51" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K51" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B52" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C52" s="23" t="n">
+        <x:v>2913</x:v>
+      </x:c>
+      <x:c r="D52" s="23" t="n">
+        <x:v>2949.4</x:v>
+      </x:c>
+      <x:c r="E52" s="23" t="n">
+        <x:v>2881.4</x:v>
+      </x:c>
+      <x:c r="F52" s="23" t="n">
+        <x:v>2915.8</x:v>
+      </x:c>
+      <x:c r="G52" s="23"/>
+      <x:c r="H52" s="24"/>
+      <x:c r="I52" s="26" t="n">
+        <x:f>ROUND(D52-E52,1)</x:f>
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="J52" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K52" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C28" s="28"/>
-      <x:c r="D28" s="28"/>
-      <x:c r="E28" s="28"/>
-      <x:c r="F28" s="28"/>
-      <x:c r="G28" s="28"/>
-      <x:c r="H28" s="28"/>
-      <x:c r="I28" s="30" t="n">
-        <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>744.2</x:v>
-      </x:c>
-      <x:c r="J28" s="28"/>
-      <x:c r="K28" s="28"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B29" s="28"/>
-      <x:c r="C29" s="28"/>
-      <x:c r="D29" s="28"/>
-      <x:c r="E29" s="28"/>
-      <x:c r="F29" s="28"/>
-      <x:c r="G29" s="28"/>
-      <x:c r="H29" s="28"/>
-      <x:c r="I29" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>372.1</x:v>
-      </x:c>
-      <x:c r="J29" s="28"/>
-      <x:c r="K29" s="28"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B32" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C32" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D32" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E32" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F32" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G32" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H32" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I32" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J32" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K32" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B33" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C33" s="23" t="n">
-        <x:v>7880.8</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="n">
-        <x:v>7903</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="n">
-        <x:v>7568</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="n">
-        <x:v>7608</x:v>
-      </x:c>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="24"/>
-      <x:c r="I33" s="26" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J33" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K33" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B34" s="22" t="str">
+      <x:c r="B53" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C34" s="23" t="n">
-        <x:v>7665.6</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="n">
-        <x:v>7817.2</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="n">
-        <x:v>7418.8</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="n">
-        <x:v>7569</x:v>
-      </x:c>
-      <x:c r="G34" s="23" t="n">
-        <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>-39</x:v>
-      </x:c>
-      <x:c r="H34" s="24" t="n">
-        <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>-0.005126182965299653</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>398.4</x:v>
-      </x:c>
-      <x:c r="J34" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K34" s="22" t="n">
+      <x:c r="C53" s="23" t="n">
+        <x:v>2923.2</x:v>
+      </x:c>
+      <x:c r="D53" s="23" t="n">
+        <x:v>2931.4</x:v>
+      </x:c>
+      <x:c r="E53" s="23" t="n">
+        <x:v>2836.8</x:v>
+      </x:c>
+      <x:c r="F53" s="23" t="n">
+        <x:v>2867</x:v>
+      </x:c>
+      <x:c r="G53" s="23" t="n">
+        <x:f>ROUND(F53-F52,1)</x:f>
+        <x:v>-48.8</x:v>
+      </x:c>
+      <x:c r="H53" s="24" t="n">
+        <x:f>IFERROR(F53/F52-1,"")</x:f>
+        <x:v>-0.01673640167364021</x:v>
+      </x:c>
+      <x:c r="I53" s="26" t="n">
+        <x:f>ROUND(D53-E53,1)</x:f>
+        <x:v>94.6</x:v>
+      </x:c>
+      <x:c r="J53" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K53" s="22" t="n">
         <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B35" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C35" s="28"/>
-      <x:c r="D35" s="28"/>
-      <x:c r="E35" s="28"/>
-      <x:c r="F35" s="28"/>
-      <x:c r="G35" s="28"/>
-      <x:c r="H35" s="28"/>
-      <x:c r="I35" s="30" t="n">
-        <x:f>ROUND(SUM(I33:I34),1)</x:f>
-        <x:v>733.4</x:v>
-      </x:c>
-      <x:c r="J35" s="28"/>
-      <x:c r="K35" s="28"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B36" s="28"/>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
-        <x:v>366.7</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B38" s="17"/>
-      <x:c r="C38" s="17"/>
-      <x:c r="D38" s="17"/>
-      <x:c r="E38" s="17"/>
-      <x:c r="F38" s="17"/>
-      <x:c r="G38" s="17"/>
-      <x:c r="H38" s="17"/>
-      <x:c r="I38" s="17"/>
-      <x:c r="J38" s="17"/>
-      <x:c r="K38" s="17"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B39" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C39" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D39" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E39" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F39" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G39" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H39" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I39" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J39" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K39" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B40" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C40" s="23" t="n">
-        <x:v>4602</x:v>
-      </x:c>
-      <x:c r="D40" s="23" t="n">
-        <x:v>4617.8</x:v>
-      </x:c>
-      <x:c r="E40" s="23" t="n">
-        <x:v>4497.6</x:v>
-      </x:c>
-      <x:c r="F40" s="23" t="n">
-        <x:v>4537.4</x:v>
-      </x:c>
-      <x:c r="G40" s="23"/>
-      <x:c r="H40" s="24"/>
-      <x:c r="I40" s="26" t="n">
-        <x:f>ROUND(D40-E40,1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J40" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K40" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>4562</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>4584</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>4451.6</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>4503.4</x:v>
-      </x:c>
-      <x:c r="G41" s="23" t="n">
-        <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>-34</x:v>
-      </x:c>
-      <x:c r="H41" s="24" t="n">
-        <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>-0.007493278088773314</x:v>
-      </x:c>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>132.4</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C42" s="28"/>
-      <x:c r="D42" s="28"/>
-      <x:c r="E42" s="28"/>
-      <x:c r="F42" s="28"/>
-      <x:c r="G42" s="28"/>
-      <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
-        <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>252.6</x:v>
-      </x:c>
-      <x:c r="J42" s="28"/>
-      <x:c r="K42" s="28"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>126.3</x:v>
-      </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C46" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E46" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F46" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I46" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J46" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>2913</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>2949.4</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>2881.4</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>2915.8</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B48" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C48" s="23" t="n">
-        <x:v>2923.2</x:v>
-      </x:c>
-      <x:c r="D48" s="23" t="n">
-        <x:v>2931.4</x:v>
-      </x:c>
-      <x:c r="E48" s="23" t="n">
-        <x:v>2836.8</x:v>
-      </x:c>
-      <x:c r="F48" s="23" t="n">
-        <x:v>2867</x:v>
-      </x:c>
-      <x:c r="G48" s="23" t="n">
-        <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-48.8</x:v>
-      </x:c>
-      <x:c r="H48" s="24" t="n">
-        <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.01673640167364021</x:v>
-      </x:c>
-      <x:c r="I48" s="26" t="n">
-        <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>94.6</x:v>
-      </x:c>
-      <x:c r="J48" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K48" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B49" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="30" t="n">
-        <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>162.6</x:v>
-      </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B50" s="28"/>
-      <x:c r="C50" s="28"/>
-      <x:c r="D50" s="28"/>
-      <x:c r="E50" s="28"/>
-      <x:c r="F50" s="28"/>
-      <x:c r="G50" s="28"/>
-      <x:c r="H50" s="28"/>
-      <x:c r="I50" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>81.3</x:v>
-      </x:c>
-      <x:c r="J50" s="28"/>
-      <x:c r="K50" s="28"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="17" t="str">
-        <x:v>碳酸锂2609</x:v>
-      </x:c>
-      <x:c r="B52" s="17"/>
-      <x:c r="C52" s="17"/>
-      <x:c r="D52" s="17"/>
-      <x:c r="E52" s="17"/>
-      <x:c r="F52" s="17"/>
-      <x:c r="G52" s="17"/>
-      <x:c r="H52" s="17"/>
-      <x:c r="I52" s="17"/>
-      <x:c r="J52" s="17"/>
-      <x:c r="K52" s="17"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B53" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C53" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D53" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E53" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F53" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G53" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H53" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I53" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J53" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K53" s="20" t="str">
-        <x:v>交易日</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B54" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="C54" s="23" t="n">
+        <x:v>2849.2</x:v>
+      </x:c>
+      <x:c r="D54" s="23" t="n">
+        <x:v>2864.6</x:v>
+      </x:c>
+      <x:c r="E54" s="23" t="n">
+        <x:v>2843.8</x:v>
+      </x:c>
+      <x:c r="F54" s="23" t="n">
+        <x:v>2860.4</x:v>
+      </x:c>
+      <x:c r="G54" s="23" t="n">
+        <x:f>ROUND(F54-F53,1)</x:f>
+        <x:v>-6.6</x:v>
+      </x:c>
+      <x:c r="H54" s="24" t="n">
+        <x:f>IFERROR(F54/F53-1,"")</x:f>
+        <x:v>-0.002302057900244181</x:v>
+      </x:c>
+      <x:c r="I54" s="23" t="n">
+        <x:f>ROUND(D54-E54,1)</x:f>
+        <x:v>20.8</x:v>
+      </x:c>
+      <x:c r="J54" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K54" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>159000</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>160480</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>140940</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>140980</x:v>
-      </x:c>
-      <x:c r="G54" s="23"/>
-      <x:c r="H54" s="24"/>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>19540</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>142120</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>143200</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>131900</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>135500</x:v>
-      </x:c>
-      <x:c r="G55" s="34" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-5480</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.038870761810185894</x:v>
-      </x:c>
-      <x:c r="I55" s="26" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>11300</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>LC2609</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
+      <x:c r="A55" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B55" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C55" s="28"/>
+      <x:c r="D55" s="28"/>
+      <x:c r="E55" s="28"/>
+      <x:c r="F55" s="28"/>
+      <x:c r="G55" s="28"/>
+      <x:c r="H55" s="28"/>
+      <x:c r="I55" s="30" t="n">
+        <x:f>ROUND(SUM(I52:I54),1)</x:f>
+        <x:v>183.4</x:v>
+      </x:c>
+      <x:c r="J55" s="28"/>
+      <x:c r="K55" s="28"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B56" s="28"/>
       <x:c r="C56" s="28"/>
       <x:c r="D56" s="28"/>
       <x:c r="E56" s="28"/>
       <x:c r="F56" s="28"/>
       <x:c r="G56" s="28"/>
       <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
-        <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>30840</x:v>
+      <x:c r="I56" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I52:I54),0),1)</x:f>
+        <x:v>61.1</x:v>
       </x:c>
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
     </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="29" t="str">
+    <x:row r="58">
+      <x:c r="A58" s="17" t="str">
+        <x:v>碳酸锂2609</x:v>
+      </x:c>
+      <x:c r="B58" s="17"/>
+      <x:c r="C58" s="17"/>
+      <x:c r="D58" s="17"/>
+      <x:c r="E58" s="17"/>
+      <x:c r="F58" s="17"/>
+      <x:c r="G58" s="17"/>
+      <x:c r="H58" s="17"/>
+      <x:c r="I58" s="17"/>
+      <x:c r="J58" s="17"/>
+      <x:c r="K58" s="17"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B59" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C59" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D59" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E59" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F59" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G59" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H59" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I59" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J59" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K59" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B60" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C60" s="23" t="n">
+        <x:v>159000</x:v>
+      </x:c>
+      <x:c r="D60" s="23" t="n">
+        <x:v>160480</x:v>
+      </x:c>
+      <x:c r="E60" s="23" t="n">
+        <x:v>140940</x:v>
+      </x:c>
+      <x:c r="F60" s="23" t="n">
+        <x:v>140980</x:v>
+      </x:c>
+      <x:c r="G60" s="23"/>
+      <x:c r="H60" s="24"/>
+      <x:c r="I60" s="26" t="n">
+        <x:f>ROUND(D60-E60,1)</x:f>
+        <x:v>19540</x:v>
+      </x:c>
+      <x:c r="J60" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K60" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B61" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C61" s="23" t="n">
+        <x:v>142120</x:v>
+      </x:c>
+      <x:c r="D61" s="23" t="n">
+        <x:v>143200</x:v>
+      </x:c>
+      <x:c r="E61" s="23" t="n">
+        <x:v>131900</x:v>
+      </x:c>
+      <x:c r="F61" s="23" t="n">
+        <x:v>135500</x:v>
+      </x:c>
+      <x:c r="G61" s="34" t="n">
+        <x:f>ROUND(F61-F60,1)</x:f>
+        <x:v>-5480</x:v>
+      </x:c>
+      <x:c r="H61" s="24" t="n">
+        <x:f>IFERROR(F61/F60-1,"")</x:f>
+        <x:v>-0.038870761810185894</x:v>
+      </x:c>
+      <x:c r="I61" s="26" t="n">
+        <x:f>ROUND(D61-E61,1)</x:f>
+        <x:v>11300</x:v>
+      </x:c>
+      <x:c r="J61" s="22" t="str">
+        <x:v>LC2609</x:v>
+      </x:c>
+      <x:c r="K61" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B62" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C62" s="28"/>
+      <x:c r="D62" s="28"/>
+      <x:c r="E62" s="28"/>
+      <x:c r="F62" s="28"/>
+      <x:c r="G62" s="28"/>
+      <x:c r="H62" s="28"/>
+      <x:c r="I62" s="30" t="n">
+        <x:f>ROUND(SUM(I60:I61),1)</x:f>
+        <x:v>30840</x:v>
+      </x:c>
+      <x:c r="J62" s="28"/>
+      <x:c r="K62" s="28"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
+      <x:c r="B63" s="28"/>
+      <x:c r="C63" s="28"/>
+      <x:c r="D63" s="28"/>
+      <x:c r="E63" s="28"/>
+      <x:c r="F63" s="28"/>
+      <x:c r="G63" s="28"/>
+      <x:c r="H63" s="28"/>
+      <x:c r="I63" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I60:I61),0),1)</x:f>
         <x:v>15420</x:v>
       </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+      <x:c r="J63" s="28"/>
+      <x:c r="K63" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A10:K10"/>
-    <x:mergeCell ref="A17:K17"/>
-    <x:mergeCell ref="A24:K24"/>
-    <x:mergeCell ref="A31:K31"/>
-    <x:mergeCell ref="A38:K38"/>
-    <x:mergeCell ref="A45:K45"/>
-    <x:mergeCell ref="A52:K52"/>
+    <x:mergeCell ref="A11:K11"/>
+    <x:mergeCell ref="A19:K19"/>
+    <x:mergeCell ref="A27:K27"/>
+    <x:mergeCell ref="A35:K35"/>
+    <x:mergeCell ref="A42:K42"/>
+    <x:mergeCell ref="A50:K50"/>
+    <x:mergeCell ref="A58:K58"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2956,31 +3184,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1212.6</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7363.42</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7501.14</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7329.6</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7468.3</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>41.1</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.005528298533506337</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>171.5</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -2988,11 +3234,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>134.7</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1384.1</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>138.4</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3383,31 +3647,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1109.1999999999998</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7511.04</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7610.03</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7487.46</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7571.2</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-9.3</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.0012321021985240987</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>122.6</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -3415,11 +3697,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1231.7999999999997</x:v>
+      </x:c>
+      <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>123.2</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3810,31 +4110,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>319.4</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>3895.51</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>3885.33</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-2.8</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.0007150003472125022</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>28.5</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -3842,11 +4160,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>35.5</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>347.9</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>34.8</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4237,31 +4573,49 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1356.4</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7312</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7483</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7283.4</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>7470</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>54.8</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.007390225482792223</x:v>
+      </x:c>
+      <x:c r="J13" s="26" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>199.6</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -4269,11 +4623,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>150.7</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1556</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>155.6</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5091,31 +5463,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>476.79999999999995</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>4468</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>4500.6</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>4480.2</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-23.2</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.005151663187813571</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>42.6</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -5123,11 +5513,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>53</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>519.4</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5518,31 +5926,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="28"/>
-      <x:c r="J15" s="30" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>289.4</x:v>
-      </x:c>
-      <x:c r="K15" s="28"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>9月14日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>2849.2</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>2864.6</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>2843.8</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>2860.4</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-6.6</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.002302057900244181</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>20.8</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="28"/>
       <x:c r="E16" s="28"/>
@@ -5550,11 +5976,29 @@
       <x:c r="G16" s="28"/>
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="28"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>32.2</x:v>
+      <x:c r="J16" s="30" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>310.2</x:v>
       </x:c>
       <x:c r="K16" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="K17" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-15
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1d3066adabb247b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rca5843f633da4f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R661f1733ac84486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R01f7538c7f754ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R569add9bfc084ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R54f25e71ee444a76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra8e4b1680b6a4fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R38111ff722624871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R8eea5beee54044cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R3876f2a11f144911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R47e67d63a8944264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R166e35c752094ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Reca4b5427f0e414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R32abd6ed66e04ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R4627cb948eba4fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2de4e66695bc4add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9d04326ca2604a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd91d34a1f5b34aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Re8edafd11f5a457d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R6c5813f33e424753"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7501.14</x:v>
+        <x:v>7524.61</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7329.6</x:v>
+        <x:v>7426.9</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>171.5</x:v>
+        <x:v>97.7</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1384.1</x:v>
+        <x:v>1481.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>138.4</x:v>
+        <x:v>134.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7610.03</x:v>
+        <x:v>7641.54</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7487.46</x:v>
+        <x:v>7543.95</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>122.6</x:v>
+        <x:v>97.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1231.8</x:v>
+        <x:v>1329.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>123.2</x:v>
+        <x:v>120.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3895.51</x:v>
+        <x:v>3891.62</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3867.02</x:v>
+        <x:v>3858.15</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>28.5</x:v>
+        <x:v>33.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>347.9</x:v>
+        <x:v>381.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>34.8</x:v>
+        <x:v>34.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7595.2</x:v>
+        <x:v>7418.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7452.2</x:v>
+        <x:v>7311</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>143</x:v>
+        <x:v>107.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1469.8</x:v>
+        <x:v>1577.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>147</x:v>
+        <x:v>143.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4500.6</x:v>
+        <x:v>4405</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4458</x:v>
+        <x:v>4347.8</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>42.6</x:v>
+        <x:v>57.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>519.4</x:v>
+        <x:v>576.6</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>51.9</x:v>
+        <x:v>52.4</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2864.6</x:v>
+        <x:v>2867</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2843.8</x:v>
+        <x:v>2840</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>20.8</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>310.2</x:v>
+        <x:v>337.2</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>31</x:v>
+        <x:v>30.7</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -691,12 +691,14 @@
         <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
+        <x:v>135500</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="n">
+        <x:v>135500</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D11" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="12" t="str"/>
       <x:c r="F11" s="9" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -718,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-14</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1236,13 +1238,13 @@
         <x:v>9月14日</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="G13" s="23" t="n">
         <x:v>135500</x:v>
@@ -1454,37 +1456,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7363.42</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>7501.14</x:v>
+        <x:v>7524.61</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>7329.6</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7468.3</x:v>
+        <x:v>7437.7</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>41.1</x:v>
+        <x:v>10.5</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.005528298533506337</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="n">
+        <x:v>0.0014083293390276808</x:v>
+      </x:c>
+      <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>171.5</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1502,7 +1504,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="30" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>920</x:v>
+        <x:v>943.5</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1520,7 +1522,7 @@
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>306.7</x:v>
+        <x:v>314.5</x:v>
       </x:c>
       <x:c r="J9" s="28"/>
       <x:c r="K9" s="28"/>
@@ -1650,37 +1652,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>7511.04</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7610.03</x:v>
+        <x:v>7641.54</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>7487.46</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7571.2</x:v>
+        <x:v>7561.59</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-9.3</x:v>
+        <x:v>-18.9</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.0012321021985240987</x:v>
+        <x:v>-0.00249982191242315</x:v>
       </x:c>
       <x:c r="I15" s="23" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>122.6</x:v>
+        <x:v>154.1</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1698,7 +1700,7 @@
       <x:c r="H16" s="28"/>
       <x:c r="I16" s="30" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>846.6</x:v>
+        <x:v>878.1</x:v>
       </x:c>
       <x:c r="J16" s="28"/>
       <x:c r="K16" s="28"/>
@@ -1716,7 +1718,7 @@
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>282.2</x:v>
+        <x:v>292.7</x:v>
       </x:c>
       <x:c r="J17" s="28"/>
       <x:c r="K17" s="28"/>
@@ -1846,7 +1848,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3867.02</x:v>
@@ -1855,28 +1857,28 @@
         <x:v>3895.51</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3867.02</x:v>
+        <x:v>3858.15</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3885.33</x:v>
+        <x:v>3864.28</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-2.8</x:v>
+        <x:v>-23.8</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.0007150003472125022</x:v>
+        <x:v>-0.006128941825205514</x:v>
       </x:c>
       <x:c r="I23" s="23" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>28.5</x:v>
+        <x:v>37.4</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1894,7 +1896,7 @@
       <x:c r="H24" s="28"/>
       <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>214.6</x:v>
+        <x:v>223.5</x:v>
       </x:c>
       <x:c r="J24" s="28"/>
       <x:c r="K24" s="28"/>
@@ -1912,7 +1914,7 @@
       <x:c r="H25" s="28"/>
       <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>71.5</x:v>
+        <x:v>74.5</x:v>
       </x:c>
       <x:c r="J25" s="28"/>
       <x:c r="K25" s="28"/>
@@ -2238,7 +2240,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7482.2</x:v>
@@ -2247,28 +2249,28 @@
         <x:v>7595.2</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
-        <x:v>7452.2</x:v>
+        <x:v>7311</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>7573.6</x:v>
-      </x:c>
-      <x:c r="G39" s="23" t="n">
+        <x:v>7350.8</x:v>
+      </x:c>
+      <x:c r="G39" s="34" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>4.6</x:v>
+        <x:v>-218.2</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.0006077421059584864</x:v>
-      </x:c>
-      <x:c r="I39" s="23" t="n">
+        <x:v>-0.02882811467829305</x:v>
+      </x:c>
+      <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>143</x:v>
+        <x:v>284.2</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2286,7 +2288,7 @@
       <x:c r="H40" s="28"/>
       <x:c r="I40" s="30" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>876.4</x:v>
+        <x:v>1017.6</x:v>
       </x:c>
       <x:c r="J40" s="28"/>
       <x:c r="K40" s="28"/>
@@ -2304,7 +2306,7 @@
       <x:c r="H41" s="28"/>
       <x:c r="I41" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>292.1</x:v>
+        <x:v>339.2</x:v>
       </x:c>
       <x:c r="J41" s="28"/>
       <x:c r="K41" s="28"/>
@@ -2434,7 +2436,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>4468</x:v>
@@ -2443,28 +2445,28 @@
         <x:v>4500.6</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>4458</x:v>
+        <x:v>4347.8</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>4480.2</x:v>
+        <x:v>4355.8</x:v>
       </x:c>
       <x:c r="G47" s="23" t="n">
         <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>-23.2</x:v>
+        <x:v>-147.6</x:v>
       </x:c>
       <x:c r="H47" s="24" t="n">
         <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>-0.005151663187813571</x:v>
-      </x:c>
-      <x:c r="I47" s="23" t="n">
+        <x:v>-0.03277523648798675</x:v>
+      </x:c>
+      <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>42.6</x:v>
+        <x:v>152.8</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>IF2609</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2482,7 +2484,7 @@
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>295.2</x:v>
+        <x:v>405.4</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -2500,7 +2502,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>98.4</x:v>
+        <x:v>135.1</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2630,37 +2632,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>9月14日</x:v>
+        <x:v>9月14日-9月15日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>2849.2</x:v>
       </x:c>
       <x:c r="D55" s="23" t="n">
-        <x:v>2864.6</x:v>
+        <x:v>2867</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
-        <x:v>2843.8</x:v>
+        <x:v>2840</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>2860.4</x:v>
+        <x:v>2845</x:v>
       </x:c>
       <x:c r="G55" s="23" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-6.6</x:v>
+        <x:v>-22</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.002302057900244181</x:v>
+        <x:v>-0.007673526334147196</x:v>
       </x:c>
       <x:c r="I55" s="23" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>20.8</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2678,7 +2680,7 @@
       <x:c r="H56" s="28"/>
       <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>183.4</x:v>
+        <x:v>189.6</x:v>
       </x:c>
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
@@ -2696,7 +2698,7 @@
       <x:c r="H57" s="28"/>
       <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>61.1</x:v>
+        <x:v>63.2</x:v>
       </x:c>
       <x:c r="J57" s="28"/>
       <x:c r="K57" s="28"/>
@@ -2829,13 +2831,13 @@
         <x:v>9月14日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="D63" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="E63" s="23" t="n">
-        <x:v>0</x:v>
+        <x:v>135500</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
         <x:v>135500</x:v>
@@ -3330,31 +3332,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1384.1</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7453.47</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7524.61</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7426.9</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>7437.7</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-30.6</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.004097317997402428</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>97.7</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -3362,11 +3382,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>138.4</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1481.8</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>134.7</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3793,31 +3831,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1231.7999999999997</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7550.68</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7641.54</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7543.95</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>7561.59</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-9.6</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.0012692836010143038</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>97.6</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -3825,11 +3881,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>123.2</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1329.3999999999996</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>120.9</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4256,31 +4330,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>347.9</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>3879.73</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>3891.62</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>3858.15</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>3864.28</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-21</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.005417815217754973</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>33.5</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -4288,11 +4380,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>34.8</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>381.4</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>34.7</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5182,31 +5292,49 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1469.8</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7351.6</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>7418.8</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>7311</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>7350.8</x:v>
+      </x:c>
+      <x:c r="H14" s="34" t="n">
+        <x:v>-222.8</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.02941797824020287</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>107.8</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -5214,11 +5342,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>147</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1577.6</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>143.4</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5645,31 +5791,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>519.4</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>4383</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>4405</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>4347.8</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>4355.8</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-124.4</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.027766617561715945</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>57.2</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -5677,11 +5841,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>51.9</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>576.6</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>52.4</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6108,31 +6290,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>310.2</x:v>
-      </x:c>
-      <x:c r="K16" s="28"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>9月15日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>2858</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>2867</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>2840</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>2845</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-15.4</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.005383862396867611</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="28"/>
       <x:c r="D17" s="28"/>
       <x:c r="E17" s="28"/>
@@ -6140,11 +6340,29 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
       <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>31</x:v>
+      <x:c r="J17" s="30" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>337.2</x:v>
       </x:c>
       <x:c r="K17" s="28"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="28"/>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>30.7</x:v>
+      </x:c>
+      <x:c r="K18" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-16
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R0e360bb7dab3445a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1c9301830e764666"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R2272e6f495674665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R122f8dc30a9e4942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R25bcf701ddab489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R92b477e516424ea0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re457d634019d4617"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rc43af6a8ae424f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R424ed98dc85546a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R418d9a53a6224f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R61de7af2bfd84a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rc849680e72f74481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R4b4769e2c9c2403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re753a7cecb9f4eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3141eea88f854ddc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R72db82ef80394279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4b1b1856a5684b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R660fd9828a2e49f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R00dbdf8d4e454391"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2609" sheetId="10" r:id="R712b7508a96a4a33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,6 +201,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -216,12 +222,6 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7524.61</x:v>
+        <x:v>7607.89</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7426.9</x:v>
+        <x:v>7402.37</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>97.7</x:v>
+        <x:v>205.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1481.8</x:v>
+        <x:v>1687.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>134.7</x:v>
+        <x:v>140.6</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7641.54</x:v>
+        <x:v>7696.47</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7543.95</x:v>
+        <x:v>7523.82</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>97.6</x:v>
+        <x:v>172.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1329.4</x:v>
+        <x:v>1502.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>120.9</x:v>
+        <x:v>125.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3891.62</x:v>
+        <x:v>3894.66</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3858.15</x:v>
+        <x:v>3842.72</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>33.5</x:v>
+        <x:v>51.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>381.4</x:v>
+        <x:v>433.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>34.7</x:v>
+        <x:v>36.1</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7523.8</x:v>
+        <x:v>7623.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7413.2</x:v>
+        <x:v>7401.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>110.6</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1666.6</x:v>
+        <x:v>1888.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>151.5</x:v>
+        <x:v>157.4</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -601,25 +601,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7641.8</x:v>
+        <x:v>7710</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7531</x:v>
+        <x:v>7516.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>110.8</x:v>
+        <x:v>193.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1580.6</x:v>
+        <x:v>1774.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>143.7</x:v>
+        <x:v>147.9</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2867</x:v>
+        <x:v>2873.2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2840</x:v>
+        <x:v>2829.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>27</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>337.2</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>30.7</x:v>
+        <x:v>31.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-09-16</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>155820</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-3180</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>155000</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>-820</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>148900</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>-6100</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>140980</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="n">
+      <x:c r="H7" s="28" t="n">
         <x:v>-7920</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1069,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>140500</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
+      <x:c r="H8" s="28" t="n">
         <x:v>-480</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1105,7 +1105,7 @@
       <x:c r="G9" s="23" t="n">
         <x:v>141320</x:v>
       </x:c>
-      <x:c r="H9" s="34" t="n">
+      <x:c r="H9" s="28" t="n">
         <x:v>820</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
@@ -1177,7 +1177,7 @@
       <x:c r="G11" s="23" t="n">
         <x:v>140520</x:v>
       </x:c>
-      <x:c r="H11" s="34" t="n">
+      <x:c r="H11" s="28" t="n">
         <x:v>-740</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
@@ -1213,7 +1213,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>135500</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-5020</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -1264,42 +1264,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="28"/>
-      <x:c r="J16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="32" t="n">
         <x:f>SUM(J4:J13)</x:f>
         <x:v>41200</x:v>
       </x:c>
-      <x:c r="K16" s="28"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
         <x:v>4120</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1456,76 +1456,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7363.42</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>7524.61</x:v>
+        <x:v>7607.89</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>7329.6</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7437.7</x:v>
-      </x:c>
-      <x:c r="G7" s="23" t="n">
+        <x:v>7587.43</x:v>
+      </x:c>
+      <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>10.5</x:v>
+        <x:v>160.2</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.0014083293390276808</x:v>
+        <x:v>0.021567904093579893</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>195</x:v>
+        <x:v>278.3</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="A8" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B8" s="28" t="n">
+      <x:c r="B8" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="30" t="n">
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="30"/>
+      <x:c r="E8" s="30"/>
+      <x:c r="F8" s="30"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>943.5</x:v>
-      </x:c>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="28"/>
+        <x:v>1026.8</x:v>
+      </x:c>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="str">
+      <x:c r="A9" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B9" s="28"/>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="32" t="n">
+      <x:c r="B9" s="30"/>
+      <x:c r="C9" s="30"/>
+      <x:c r="D9" s="30"/>
+      <x:c r="E9" s="30"/>
+      <x:c r="F9" s="30"/>
+      <x:c r="G9" s="30"/>
+      <x:c r="H9" s="30"/>
+      <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>314.5</x:v>
-      </x:c>
-      <x:c r="J9" s="28"/>
-      <x:c r="K9" s="28"/>
+        <x:v>342.3</x:v>
+      </x:c>
+      <x:c r="J9" s="30"/>
+      <x:c r="K9" s="30"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="17" t="str">
@@ -1652,76 +1652,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>7511.04</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7641.54</x:v>
+        <x:v>7696.47</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>7487.46</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7561.59</x:v>
+        <x:v>7683.47</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-18.9</x:v>
+        <x:v>102.9</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.00249982191242315</x:v>
-      </x:c>
-      <x:c r="I15" s="23" t="n">
+        <x:v>0.013578188361251353</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>154.1</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>878.1</x:v>
-      </x:c>
-      <x:c r="J16" s="28"/>
-      <x:c r="K16" s="28"/>
+        <x:v>933</x:v>
+      </x:c>
+      <x:c r="J16" s="30"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>292.7</x:v>
-      </x:c>
-      <x:c r="J17" s="28"/>
-      <x:c r="K17" s="28"/>
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="J17" s="30"/>
+      <x:c r="K17" s="30"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="17" t="str">
@@ -1848,7 +1848,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3867.02</x:v>
@@ -1857,67 +1857,67 @@
         <x:v>3895.51</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3858.15</x:v>
+        <x:v>3842.72</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3864.28</x:v>
+        <x:v>3891.6</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-23.8</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.006128941825205514</x:v>
-      </x:c>
-      <x:c r="I23" s="23" t="n">
+        <x:v>0.0008976083495579879</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>37.4</x:v>
+        <x:v>52.8</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+      <x:c r="A24" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B24" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="28"/>
-      <x:c r="E24" s="28"/>
-      <x:c r="F24" s="28"/>
-      <x:c r="G24" s="28"/>
-      <x:c r="H24" s="28"/>
-      <x:c r="I24" s="30" t="n">
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>223.5</x:v>
-      </x:c>
-      <x:c r="J24" s="28"/>
-      <x:c r="K24" s="28"/>
+        <x:v>238.9</x:v>
+      </x:c>
+      <x:c r="J24" s="30"/>
+      <x:c r="K24" s="30"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29" t="str">
+      <x:c r="A25" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="28"/>
-      <x:c r="E25" s="28"/>
-      <x:c r="F25" s="28"/>
-      <x:c r="G25" s="28"/>
-      <x:c r="H25" s="28"/>
-      <x:c r="I25" s="32" t="n">
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>74.5</x:v>
-      </x:c>
-      <x:c r="J25" s="28"/>
-      <x:c r="K25" s="28"/>
+        <x:v>79.6</x:v>
+      </x:c>
+      <x:c r="J25" s="30"/>
+      <x:c r="K25" s="30"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
@@ -2044,76 +2044,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>7312</x:v>
       </x:c>
       <x:c r="D31" s="23" t="n">
-        <x:v>7523.8</x:v>
+        <x:v>7623.6</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
         <x:v>7283.4</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>7443.2</x:v>
-      </x:c>
-      <x:c r="G31" s="23" t="n">
+        <x:v>7593</x:v>
+      </x:c>
+      <x:c r="G31" s="28" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>28</x:v>
+        <x:v>177.8</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.0037760276189449105</x:v>
+        <x:v>0.02397777538029988</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>240.4</x:v>
+        <x:v>340.2</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="29" t="str">
+      <x:c r="A32" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="28" t="n">
+      <x:c r="B32" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="28"/>
-      <x:c r="D32" s="28"/>
-      <x:c r="E32" s="28"/>
-      <x:c r="F32" s="28"/>
-      <x:c r="G32" s="28"/>
-      <x:c r="H32" s="28"/>
-      <x:c r="I32" s="30" t="n">
+      <x:c r="C32" s="30"/>
+      <x:c r="D32" s="30"/>
+      <x:c r="E32" s="30"/>
+      <x:c r="F32" s="30"/>
+      <x:c r="G32" s="30"/>
+      <x:c r="H32" s="30"/>
+      <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>984.6</x:v>
-      </x:c>
-      <x:c r="J32" s="28"/>
-      <x:c r="K32" s="28"/>
+        <x:v>1084.4</x:v>
+      </x:c>
+      <x:c r="J32" s="30"/>
+      <x:c r="K32" s="30"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29" t="str">
+      <x:c r="A33" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="28"/>
-      <x:c r="C33" s="28"/>
-      <x:c r="D33" s="28"/>
-      <x:c r="E33" s="28"/>
-      <x:c r="F33" s="28"/>
-      <x:c r="G33" s="28"/>
-      <x:c r="H33" s="28"/>
-      <x:c r="I33" s="32" t="n">
+      <x:c r="B33" s="30"/>
+      <x:c r="C33" s="30"/>
+      <x:c r="D33" s="30"/>
+      <x:c r="E33" s="30"/>
+      <x:c r="F33" s="30"/>
+      <x:c r="G33" s="30"/>
+      <x:c r="H33" s="30"/>
+      <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>328.2</x:v>
-      </x:c>
-      <x:c r="J33" s="28"/>
-      <x:c r="K33" s="28"/>
+        <x:v>361.5</x:v>
+      </x:c>
+      <x:c r="J33" s="30"/>
+      <x:c r="K33" s="30"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="17" t="str">
@@ -2240,76 +2240,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7482.2</x:v>
       </x:c>
       <x:c r="D39" s="23" t="n">
-        <x:v>7641.8</x:v>
+        <x:v>7710</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
         <x:v>7452.2</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>7567.8</x:v>
+        <x:v>7689.6</x:v>
       </x:c>
       <x:c r="G39" s="23" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>-1.2</x:v>
+        <x:v>120.6</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>-0.00015854141894566798</x:v>
+        <x:v>0.015933412604042907</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>189.6</x:v>
+        <x:v>257.8</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="29" t="str">
+      <x:c r="A40" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="28" t="n">
+      <x:c r="B40" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C40" s="28"/>
-      <x:c r="D40" s="28"/>
-      <x:c r="E40" s="28"/>
-      <x:c r="F40" s="28"/>
-      <x:c r="G40" s="28"/>
-      <x:c r="H40" s="28"/>
-      <x:c r="I40" s="30" t="n">
+      <x:c r="C40" s="30"/>
+      <x:c r="D40" s="30"/>
+      <x:c r="E40" s="30"/>
+      <x:c r="F40" s="30"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>923</x:v>
-      </x:c>
-      <x:c r="J40" s="28"/>
-      <x:c r="K40" s="28"/>
+        <x:v>991.2</x:v>
+      </x:c>
+      <x:c r="J40" s="30"/>
+      <x:c r="K40" s="30"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="29" t="str">
+      <x:c r="A41" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="28"/>
-      <x:c r="C41" s="28"/>
-      <x:c r="D41" s="28"/>
-      <x:c r="E41" s="28"/>
-      <x:c r="F41" s="28"/>
-      <x:c r="G41" s="28"/>
-      <x:c r="H41" s="28"/>
-      <x:c r="I41" s="32" t="n">
+      <x:c r="B41" s="30"/>
+      <x:c r="C41" s="30"/>
+      <x:c r="D41" s="30"/>
+      <x:c r="E41" s="30"/>
+      <x:c r="F41" s="30"/>
+      <x:c r="G41" s="30"/>
+      <x:c r="H41" s="30"/>
+      <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>307.7</x:v>
-      </x:c>
-      <x:c r="J41" s="28"/>
-      <x:c r="K41" s="28"/>
+        <x:v>330.4</x:v>
+      </x:c>
+      <x:c r="J41" s="30"/>
+      <x:c r="K41" s="30"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="17" t="str">
@@ -2470,42 +2470,42 @@
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="29" t="str">
+      <x:c r="A48" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="28" t="n">
+      <x:c r="B48" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C48" s="28"/>
-      <x:c r="D48" s="28"/>
-      <x:c r="E48" s="28"/>
-      <x:c r="F48" s="28"/>
-      <x:c r="G48" s="28"/>
-      <x:c r="H48" s="28"/>
-      <x:c r="I48" s="30" t="n">
+      <x:c r="C48" s="30"/>
+      <x:c r="D48" s="30"/>
+      <x:c r="E48" s="30"/>
+      <x:c r="F48" s="30"/>
+      <x:c r="G48" s="30"/>
+      <x:c r="H48" s="30"/>
+      <x:c r="I48" s="32" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
         <x:v>312.2</x:v>
       </x:c>
-      <x:c r="J48" s="28"/>
-      <x:c r="K48" s="28"/>
+      <x:c r="J48" s="30"/>
+      <x:c r="K48" s="30"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29" t="str">
+      <x:c r="A49" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="28"/>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="32" t="n">
+      <x:c r="B49" s="30"/>
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
         <x:v>104.1</x:v>
       </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="17" t="str">
@@ -2632,76 +2632,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>9月14日-9月15日</x:v>
+        <x:v>9月14日-9月16日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>2849.2</x:v>
       </x:c>
       <x:c r="D55" s="23" t="n">
-        <x:v>2867</x:v>
+        <x:v>2873.2</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
-        <x:v>2840</x:v>
+        <x:v>2829.4</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>2845</x:v>
+        <x:v>2865</x:v>
       </x:c>
       <x:c r="G55" s="23" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-22</x:v>
+        <x:v>-2</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.007673526334147196</x:v>
+        <x:v>-0.0006975933031042603</x:v>
       </x:c>
       <x:c r="I55" s="23" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>27</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>IH2609</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="29" t="str">
+      <x:c r="A56" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B56" s="28" t="n">
+      <x:c r="B56" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C56" s="28"/>
-      <x:c r="D56" s="28"/>
-      <x:c r="E56" s="28"/>
-      <x:c r="F56" s="28"/>
-      <x:c r="G56" s="28"/>
-      <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
+      <x:c r="C56" s="30"/>
+      <x:c r="D56" s="30"/>
+      <x:c r="E56" s="30"/>
+      <x:c r="F56" s="30"/>
+      <x:c r="G56" s="30"/>
+      <x:c r="H56" s="30"/>
+      <x:c r="I56" s="32" t="n">
         <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>189.6</x:v>
-      </x:c>
-      <x:c r="J56" s="28"/>
-      <x:c r="K56" s="28"/>
+        <x:v>206.4</x:v>
+      </x:c>
+      <x:c r="J56" s="30"/>
+      <x:c r="K56" s="30"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29" t="str">
+      <x:c r="A57" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
+      <x:c r="B57" s="30"/>
+      <x:c r="C57" s="30"/>
+      <x:c r="D57" s="30"/>
+      <x:c r="E57" s="30"/>
+      <x:c r="F57" s="30"/>
+      <x:c r="G57" s="30"/>
+      <x:c r="H57" s="30"/>
+      <x:c r="I57" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>63.2</x:v>
-      </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="J57" s="30"/>
+      <x:c r="K57" s="30"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="17" t="str">
@@ -2804,7 +2804,7 @@
       <x:c r="F62" s="23" t="n">
         <x:v>135500</x:v>
       </x:c>
-      <x:c r="G62" s="34" t="n">
+      <x:c r="G62" s="28" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
         <x:v>-5480</x:v>
       </x:c>
@@ -2862,42 +2862,42 @@
       </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="29" t="str">
+      <x:c r="A64" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B64" s="28" t="n">
+      <x:c r="B64" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C64" s="28"/>
-      <x:c r="D64" s="28"/>
-      <x:c r="E64" s="28"/>
-      <x:c r="F64" s="28"/>
-      <x:c r="G64" s="28"/>
-      <x:c r="H64" s="28"/>
-      <x:c r="I64" s="30" t="n">
+      <x:c r="C64" s="30"/>
+      <x:c r="D64" s="30"/>
+      <x:c r="E64" s="30"/>
+      <x:c r="F64" s="30"/>
+      <x:c r="G64" s="30"/>
+      <x:c r="H64" s="30"/>
+      <x:c r="I64" s="32" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
         <x:v>30840</x:v>
       </x:c>
-      <x:c r="J64" s="28"/>
-      <x:c r="K64" s="28"/>
+      <x:c r="J64" s="30"/>
+      <x:c r="K64" s="30"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="29" t="str">
+      <x:c r="A65" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B65" s="28"/>
-      <x:c r="C65" s="28"/>
-      <x:c r="D65" s="28"/>
-      <x:c r="E65" s="28"/>
-      <x:c r="F65" s="28"/>
-      <x:c r="G65" s="28"/>
-      <x:c r="H65" s="28"/>
-      <x:c r="I65" s="32" t="n">
+      <x:c r="B65" s="30"/>
+      <x:c r="C65" s="30"/>
+      <x:c r="D65" s="30"/>
+      <x:c r="E65" s="30"/>
+      <x:c r="F65" s="30"/>
+      <x:c r="G65" s="30"/>
+      <x:c r="H65" s="30"/>
+      <x:c r="I65" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
         <x:v>10280</x:v>
       </x:c>
-      <x:c r="J65" s="28"/>
-      <x:c r="K65" s="28"/>
+      <x:c r="J65" s="30"/>
+      <x:c r="K65" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3282,7 +3282,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7427.24</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-160.5</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -3368,43 +3368,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7437.82</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7607.89</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7402.37</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>7587.43</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>149.7</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.020131223362060968</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>205.5</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1481.8</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1687.3</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>134.7</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>140.6</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3867,43 +3903,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7556.9</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7696.47</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7523.82</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>7683.47</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>121.9</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.016118303161107628</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>172.7</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1329.3999999999996</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1502.0999999999997</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>120.9</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>125.2</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4366,43 +4438,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>3861.75</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>3894.66</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>3842.72</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>3891.6</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>27.3</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.007069881064519112</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>381.4</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>433.29999999999995</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>34.7</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>36.1</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4779,7 +4887,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7415.2</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-158.8</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -4865,43 +4973,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7456.2</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7623.6</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7401.6</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>7593</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>149.8</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.020125752364574367</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1666.6</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1888.6</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>151.5</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>157.4</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5364,43 +5508,79 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>7571.8</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>7710</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>7516.2</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>7689.6</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>121.8</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.016094505668754477</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>193.8</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1580.6</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>1774.3999999999999</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>143.7</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>147.9</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5864,42 +6044,42 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
+      <x:c r="B17" s="30" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="32" t="n">
         <x:f>SUM(J4:J14)</x:f>
         <x:v>574.1999999999999</x:v>
       </x:c>
-      <x:c r="K17" s="28"/>
+      <x:c r="K17" s="30"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="A18" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
         <x:v>52.2</x:v>
       </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6362,43 +6542,79 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>9月16日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>2848.2</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>2873.2</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>2829.4</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>2865</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.007029876977152849</x:v>
+      </x:c>
+      <x:c r="J15" s="23" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>43.8</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B17" s="28" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="28"/>
-      <x:c r="J17" s="30" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>337.2</x:v>
-      </x:c>
-      <x:c r="K17" s="28"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="28"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>30.7</x:v>
-      </x:c>
-      <x:c r="K18" s="28"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>31.8</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-17
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R315739b2fec741ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R6d8620e9ce8a46ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R957e9d613ed947b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re96c78c61ac44551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9040bd18b34c4dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd548f891c00f4665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra878f45ac8f9431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R5b5b9ea2fac940d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R05c4132095ec4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rbede1135f15b4125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R230cbf2ee6c44424"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R114335d81dba4ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rfeea35fde6b54db5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R962a8ac736824935"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R16707cb2688f4a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Ref8a6d09a9c94601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd2eae34dfc81426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rade25e1aaa6e4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R30ceb238dcb14508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Ra80cff5d90e3401b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,12 +201,6 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -222,6 +216,12 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-16</x:v>
+        <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7607.89</x:v>
+        <x:v>7632.53</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7402.37</x:v>
+        <x:v>7522.77</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>205.5</x:v>
+        <x:v>109.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1687.3</x:v>
+        <x:v>1797.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>140.6</x:v>
+        <x:v>138.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-16</x:v>
+        <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7696.47</x:v>
+        <x:v>7738.03</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7523.82</x:v>
+        <x:v>7622.55</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>172.7</x:v>
+        <x:v>115.5</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1502.1</x:v>
+        <x:v>1617.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>125.2</x:v>
+        <x:v>124.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-16</x:v>
+        <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3894.66</x:v>
+        <x:v>3898.84</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3842.72</x:v>
+        <x:v>3866.89</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>51.9</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>433.3</x:v>
+        <x:v>465.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>36.1</x:v>
+        <x:v>35.8</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-16</x:v>
+        <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>130660</x:v>
+        <x:v>133760</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>126200</x:v>
+        <x:v>127900</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>4460</x:v>
+        <x:v>5860</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>67360</x:v>
+        <x:v>73220</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5613.3</x:v>
+        <x:v>5632.3</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-16</x:v>
+        <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>156920</x:v>
       </x:c>
-      <x:c r="H4" s="28" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>-2360</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>153680</x:v>
       </x:c>
-      <x:c r="H5" s="28" t="n">
+      <x:c r="H5" s="34" t="n">
         <x:v>-3240</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>149080</x:v>
       </x:c>
-      <x:c r="H6" s="28" t="n">
+      <x:c r="H6" s="34" t="n">
         <x:v>-4600</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>142000</x:v>
       </x:c>
-      <x:c r="H7" s="28" t="n">
+      <x:c r="H7" s="34" t="n">
         <x:v>-7080</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1069,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>141140</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="n">
+      <x:c r="H8" s="34" t="n">
         <x:v>-860</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1105,7 +1105,7 @@
       <x:c r="G9" s="23" t="n">
         <x:v>142640</x:v>
       </x:c>
-      <x:c r="H9" s="28" t="n">
+      <x:c r="H9" s="34" t="n">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
@@ -1141,7 +1141,7 @@
       <x:c r="G10" s="23" t="n">
         <x:v>141140</x:v>
       </x:c>
-      <x:c r="H10" s="28" t="n">
+      <x:c r="H10" s="34" t="n">
         <x:v>-1500</x:v>
       </x:c>
       <x:c r="I10" s="24" t="n">
@@ -1177,7 +1177,7 @@
       <x:c r="G11" s="23" t="n">
         <x:v>140960</x:v>
       </x:c>
-      <x:c r="H11" s="28" t="n">
+      <x:c r="H11" s="34" t="n">
         <x:v>-180</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
@@ -1213,7 +1213,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>134340</x:v>
       </x:c>
-      <x:c r="H12" s="28" t="n">
+      <x:c r="H12" s="34" t="n">
         <x:v>-6620</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -1249,7 +1249,7 @@
       <x:c r="G13" s="23" t="n">
         <x:v>132580</x:v>
       </x:c>
-      <x:c r="H13" s="28" t="n">
+      <x:c r="H13" s="34" t="n">
         <x:v>-1760</x:v>
       </x:c>
       <x:c r="I13" s="24" t="n">
@@ -1285,7 +1285,7 @@
       <x:c r="G14" s="23" t="n">
         <x:v>130000</x:v>
       </x:c>
-      <x:c r="H14" s="28" t="n">
+      <x:c r="H14" s="34" t="n">
         <x:v>-2580</x:v>
       </x:c>
       <x:c r="I14" s="24" t="n">
@@ -1321,7 +1321,7 @@
       <x:c r="G15" s="23" t="n">
         <x:v>127460</x:v>
       </x:c>
-      <x:c r="H15" s="28" t="n">
+      <x:c r="H15" s="34" t="n">
         <x:v>-2540</x:v>
       </x:c>
       <x:c r="I15" s="24" t="n">
@@ -1335,43 +1335,79 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>9月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>129900</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>133760</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>127900</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>132280</x:v>
+      </x:c>
+      <x:c r="H16" s="34" t="n">
+        <x:v>4820</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>0.03781578534442187</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>5860</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>67360</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B19" s="28" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="30" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>73220</x:v>
+      </x:c>
+      <x:c r="K19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>5613.3</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="B20" s="28"/>
+      <x:c r="C20" s="28"/>
+      <x:c r="D20" s="28"/>
+      <x:c r="E20" s="28"/>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28"/>
+      <x:c r="H20" s="28"/>
+      <x:c r="I20" s="28"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>5632.3</x:v>
+      </x:c>
+      <x:c r="K20" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1528,76 +1564,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>9月14日-9月16日</x:v>
+        <x:v>9月14日-9月17日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7363.42</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>7607.89</x:v>
+        <x:v>7632.53</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>7329.6</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7587.43</x:v>
-      </x:c>
-      <x:c r="G7" s="28" t="n">
+        <x:v>7548.82</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>160.2</x:v>
+        <x:v>121.6</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.021567904093579893</x:v>
+        <x:v>0.01636947237466413</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>278.3</x:v>
+        <x:v>302.9</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="30"/>
-      <x:c r="E8" s="30"/>
-      <x:c r="F8" s="30"/>
-      <x:c r="G8" s="30"/>
-      <x:c r="H8" s="30"/>
-      <x:c r="I8" s="32" t="n">
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="30" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1026.8</x:v>
-      </x:c>
-      <x:c r="J8" s="30"/>
-      <x:c r="K8" s="30"/>
+        <x:v>1051.4</x:v>
+      </x:c>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="31" t="str">
+      <x:c r="A9" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B9" s="30"/>
-      <x:c r="C9" s="30"/>
-      <x:c r="D9" s="30"/>
-      <x:c r="E9" s="30"/>
-      <x:c r="F9" s="30"/>
-      <x:c r="G9" s="30"/>
-      <x:c r="H9" s="30"/>
-      <x:c r="I9" s="34" t="n">
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>342.3</x:v>
-      </x:c>
-      <x:c r="J9" s="30"/>
-      <x:c r="K9" s="30"/>
+        <x:v>350.5</x:v>
+      </x:c>
+      <x:c r="J9" s="28"/>
+      <x:c r="K9" s="28"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="17" t="str">
@@ -1724,76 +1760,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月14日-9月16日</x:v>
+        <x:v>9月14日-9月17日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>7511.04</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7696.47</x:v>
+        <x:v>7738.03</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>7487.46</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7683.47</x:v>
+        <x:v>7654.98</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>102.9</x:v>
+        <x:v>74.4</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.013578188361251353</x:v>
+        <x:v>0.009819880905581835</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>209</x:v>
+        <x:v>250.6</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="32" t="n">
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="30" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>933</x:v>
-      </x:c>
-      <x:c r="J16" s="30"/>
-      <x:c r="K16" s="30"/>
+        <x:v>974.6</x:v>
+      </x:c>
+      <x:c r="J16" s="28"/>
+      <x:c r="K16" s="28"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="31" t="str">
+      <x:c r="A17" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="34" t="n">
+      <x:c r="B17" s="28"/>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>311</x:v>
-      </x:c>
-      <x:c r="J17" s="30"/>
-      <x:c r="K17" s="30"/>
+        <x:v>324.9</x:v>
+      </x:c>
+      <x:c r="J17" s="28"/>
+      <x:c r="K17" s="28"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="17" t="str">
@@ -1920,76 +1956,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月14日-9月16日</x:v>
+        <x:v>9月14日-9月17日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3867.02</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3895.51</x:v>
+        <x:v>3898.84</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>3842.72</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3891.6</x:v>
+        <x:v>3875.6</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>3.5</x:v>
+        <x:v>-12.5</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.0008976083495579879</x:v>
+        <x:v>-0.0032175015624558156</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>52.8</x:v>
+        <x:v>56.1</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="32" t="n">
+      <x:c r="C24" s="28"/>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>238.9</x:v>
-      </x:c>
-      <x:c r="J24" s="30"/>
-      <x:c r="K24" s="30"/>
+        <x:v>242.2</x:v>
+      </x:c>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="31" t="str">
+      <x:c r="A25" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="30"/>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="34" t="n">
+      <x:c r="B25" s="28"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>79.6</x:v>
-      </x:c>
-      <x:c r="J25" s="30"/>
-      <x:c r="K25" s="30"/>
+        <x:v>80.7</x:v>
+      </x:c>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
@@ -2130,7 +2166,7 @@
       <x:c r="F31" s="23" t="n">
         <x:v>7593</x:v>
       </x:c>
-      <x:c r="G31" s="28" t="n">
+      <x:c r="G31" s="34" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
         <x:v>177.8</x:v>
       </x:c>
@@ -2150,42 +2186,42 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="31" t="str">
+      <x:c r="A32" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="30" t="n">
+      <x:c r="B32" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="30"/>
-      <x:c r="E32" s="30"/>
-      <x:c r="F32" s="30"/>
-      <x:c r="G32" s="30"/>
-      <x:c r="H32" s="30"/>
-      <x:c r="I32" s="32" t="n">
+      <x:c r="C32" s="28"/>
+      <x:c r="D32" s="28"/>
+      <x:c r="E32" s="28"/>
+      <x:c r="F32" s="28"/>
+      <x:c r="G32" s="28"/>
+      <x:c r="H32" s="28"/>
+      <x:c r="I32" s="30" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
         <x:v>1084.4</x:v>
       </x:c>
-      <x:c r="J32" s="30"/>
-      <x:c r="K32" s="30"/>
+      <x:c r="J32" s="28"/>
+      <x:c r="K32" s="28"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="31" t="str">
+      <x:c r="A33" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="30"/>
-      <x:c r="C33" s="30"/>
-      <x:c r="D33" s="30"/>
-      <x:c r="E33" s="30"/>
-      <x:c r="F33" s="30"/>
-      <x:c r="G33" s="30"/>
-      <x:c r="H33" s="30"/>
-      <x:c r="I33" s="34" t="n">
+      <x:c r="B33" s="28"/>
+      <x:c r="C33" s="28"/>
+      <x:c r="D33" s="28"/>
+      <x:c r="E33" s="28"/>
+      <x:c r="F33" s="28"/>
+      <x:c r="G33" s="28"/>
+      <x:c r="H33" s="28"/>
+      <x:c r="I33" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
         <x:v>361.5</x:v>
       </x:c>
-      <x:c r="J33" s="30"/>
-      <x:c r="K33" s="30"/>
+      <x:c r="J33" s="28"/>
+      <x:c r="K33" s="28"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="17" t="str">
@@ -2346,42 +2382,42 @@
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="31" t="str">
+      <x:c r="A40" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="30" t="n">
+      <x:c r="B40" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="30"/>
-      <x:c r="H40" s="30"/>
-      <x:c r="I40" s="32" t="n">
+      <x:c r="C40" s="28"/>
+      <x:c r="D40" s="28"/>
+      <x:c r="E40" s="28"/>
+      <x:c r="F40" s="28"/>
+      <x:c r="G40" s="28"/>
+      <x:c r="H40" s="28"/>
+      <x:c r="I40" s="30" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
         <x:v>991.2</x:v>
       </x:c>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="30"/>
+      <x:c r="J40" s="28"/>
+      <x:c r="K40" s="28"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="31" t="str">
+      <x:c r="A41" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="30"/>
-      <x:c r="H41" s="30"/>
-      <x:c r="I41" s="34" t="n">
+      <x:c r="B41" s="28"/>
+      <x:c r="C41" s="28"/>
+      <x:c r="D41" s="28"/>
+      <x:c r="E41" s="28"/>
+      <x:c r="F41" s="28"/>
+      <x:c r="G41" s="28"/>
+      <x:c r="H41" s="28"/>
+      <x:c r="I41" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
         <x:v>330.4</x:v>
       </x:c>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="30"/>
+      <x:c r="J41" s="28"/>
+      <x:c r="K41" s="28"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="17" t="str">
@@ -2542,42 +2578,42 @@
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="31" t="str">
+      <x:c r="A48" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="30" t="n">
+      <x:c r="B48" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C48" s="30"/>
-      <x:c r="D48" s="30"/>
-      <x:c r="E48" s="30"/>
-      <x:c r="F48" s="30"/>
-      <x:c r="G48" s="30"/>
-      <x:c r="H48" s="30"/>
-      <x:c r="I48" s="32" t="n">
+      <x:c r="C48" s="28"/>
+      <x:c r="D48" s="28"/>
+      <x:c r="E48" s="28"/>
+      <x:c r="F48" s="28"/>
+      <x:c r="G48" s="28"/>
+      <x:c r="H48" s="28"/>
+      <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
         <x:v>341</x:v>
       </x:c>
-      <x:c r="J48" s="30"/>
-      <x:c r="K48" s="30"/>
+      <x:c r="J48" s="28"/>
+      <x:c r="K48" s="28"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="31" t="str">
+      <x:c r="A49" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="30"/>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="34" t="n">
+      <x:c r="B49" s="28"/>
+      <x:c r="C49" s="28"/>
+      <x:c r="D49" s="28"/>
+      <x:c r="E49" s="28"/>
+      <x:c r="F49" s="28"/>
+      <x:c r="G49" s="28"/>
+      <x:c r="H49" s="28"/>
+      <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
         <x:v>113.7</x:v>
       </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
+      <x:c r="J49" s="28"/>
+      <x:c r="K49" s="28"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="17" t="str">
@@ -2738,42 +2774,42 @@
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="31" t="str">
+      <x:c r="A56" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B56" s="30" t="n">
+      <x:c r="B56" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
+      <x:c r="C56" s="28"/>
+      <x:c r="D56" s="28"/>
+      <x:c r="E56" s="28"/>
+      <x:c r="F56" s="28"/>
+      <x:c r="G56" s="28"/>
+      <x:c r="H56" s="28"/>
+      <x:c r="I56" s="30" t="n">
         <x:f>ROUND(SUM(I53:I55),1)</x:f>
         <x:v>206.4</x:v>
       </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
+      <x:c r="J56" s="28"/>
+      <x:c r="K56" s="28"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="31" t="str">
+      <x:c r="A57" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
+      <x:c r="B57" s="28"/>
+      <x:c r="C57" s="28"/>
+      <x:c r="D57" s="28"/>
+      <x:c r="E57" s="28"/>
+      <x:c r="F57" s="28"/>
+      <x:c r="G57" s="28"/>
+      <x:c r="H57" s="28"/>
+      <x:c r="I57" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
         <x:v>68.8</x:v>
       </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
+      <x:c r="J57" s="28"/>
+      <x:c r="K57" s="28"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="17" t="str">
@@ -2876,7 +2912,7 @@
       <x:c r="F62" s="23" t="n">
         <x:v>134340</x:v>
       </x:c>
-      <x:c r="G62" s="28" t="n">
+      <x:c r="G62" s="34" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
         <x:v>-7660</x:v>
       </x:c>
@@ -2900,7 +2936,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>9月14日-9月16日</x:v>
+        <x:v>9月14日-9月17日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
         <x:v>133600</x:v>
@@ -2912,15 +2948,15 @@
         <x:v>126200</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
-        <x:v>127460</x:v>
-      </x:c>
-      <x:c r="G63" s="28" t="n">
+        <x:v>132280</x:v>
+      </x:c>
+      <x:c r="G63" s="34" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-6880</x:v>
+        <x:v>-2060</x:v>
       </x:c>
       <x:c r="H63" s="24" t="n">
         <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.051213339288372794</x:v>
+        <x:v>-0.015334226589251099</x:v>
       </x:c>
       <x:c r="I63" s="26" t="n">
         <x:f>ROUND(D63-E63,1)</x:f>
@@ -2930,46 +2966,46 @@
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K63" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B64" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B64" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="32" t="n">
+      <x:c r="C64" s="28"/>
+      <x:c r="D64" s="28"/>
+      <x:c r="E64" s="28"/>
+      <x:c r="F64" s="28"/>
+      <x:c r="G64" s="28"/>
+      <x:c r="H64" s="28"/>
+      <x:c r="I64" s="30" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
         <x:v>46120</x:v>
       </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
+      <x:c r="J64" s="28"/>
+      <x:c r="K64" s="28"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="31" t="str">
+      <x:c r="A65" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B65" s="30"/>
-      <x:c r="C65" s="30"/>
-      <x:c r="D65" s="30"/>
-      <x:c r="E65" s="30"/>
-      <x:c r="F65" s="30"/>
-      <x:c r="G65" s="30"/>
-      <x:c r="H65" s="30"/>
-      <x:c r="I65" s="34" t="n">
+      <x:c r="B65" s="28"/>
+      <x:c r="C65" s="28"/>
+      <x:c r="D65" s="28"/>
+      <x:c r="E65" s="28"/>
+      <x:c r="F65" s="28"/>
+      <x:c r="G65" s="28"/>
+      <x:c r="H65" s="28"/>
+      <x:c r="I65" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
         <x:v>15373.3</x:v>
       </x:c>
-      <x:c r="J65" s="30"/>
-      <x:c r="K65" s="30"/>
+      <x:c r="J65" s="28"/>
+      <x:c r="K65" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3354,7 +3390,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7427.24</x:v>
       </x:c>
-      <x:c r="H12" s="28" t="n">
+      <x:c r="H12" s="34" t="n">
         <x:v>-160.5</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -3476,43 +3512,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>9月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>7555.79</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7632.53</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7522.77</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>7548.82</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-38.6</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.005088679566071841</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>109.8</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1687.3</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B19" s="28" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="30" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>1797.1</x:v>
+      </x:c>
+      <x:c r="K19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>140.6</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="B20" s="28"/>
+      <x:c r="C20" s="28"/>
+      <x:c r="D20" s="28"/>
+      <x:c r="E20" s="28"/>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28"/>
+      <x:c r="H20" s="28"/>
+      <x:c r="I20" s="28"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>138.2</x:v>
+      </x:c>
+      <x:c r="K20" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4011,43 +4083,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>9月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>7651.46</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7738.03</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7622.55</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>7654.98</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-28.5</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.0037079600753305852</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>115.5</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1502.0999999999997</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B19" s="28" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="30" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>1617.5999999999997</x:v>
+      </x:c>
+      <x:c r="K19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>125.2</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="B20" s="28"/>
+      <x:c r="C20" s="28"/>
+      <x:c r="D20" s="28"/>
+      <x:c r="E20" s="28"/>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28"/>
+      <x:c r="H20" s="28"/>
+      <x:c r="I20" s="28"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>124.4</x:v>
+      </x:c>
+      <x:c r="K20" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4546,43 +4654,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>9月17日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>3877</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>3898.84</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>3866.89</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>3875.6</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-16</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.004111419467571209</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>433.29999999999995</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B19" s="28" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="30" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>465.29999999999995</x:v>
+      </x:c>
+      <x:c r="K19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>36.1</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="B20" s="28"/>
+      <x:c r="C20" s="28"/>
+      <x:c r="D20" s="28"/>
+      <x:c r="E20" s="28"/>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28"/>
+      <x:c r="H20" s="28"/>
+      <x:c r="I20" s="28"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>35.8</x:v>
+      </x:c>
+      <x:c r="K20" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4959,7 +5103,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7415.2</x:v>
       </x:c>
-      <x:c r="H12" s="28" t="n">
+      <x:c r="H12" s="34" t="n">
         <x:v>-158.8</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -5082,42 +5226,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
+      <x:c r="B18" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="30" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>1888.6</x:v>
       </x:c>
-      <x:c r="K18" s="30"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>157.4</x:v>
       </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="K19" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5617,42 +5761,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
+      <x:c r="B18" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="30" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>1774.3999999999999</x:v>
       </x:c>
-      <x:c r="K18" s="30"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>147.9</x:v>
       </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="K19" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6152,42 +6296,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
+      <x:c r="B18" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="30" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>648.9999999999999</x:v>
       </x:c>
-      <x:c r="K18" s="30"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>54.1</x:v>
       </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="K19" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6687,42 +6831,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
+      <x:c r="B18" s="28" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="30" t="n">
         <x:f>SUM(J4:J15)</x:f>
         <x:v>381</x:v>
       </x:c>
-      <x:c r="K18" s="30"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
         <x:v>31.8</x:v>
       </x:c>
-      <x:c r="K19" s="30"/>
+      <x:c r="K19" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-18
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra6e0ce2a73814e16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R42fba0f6c3e34506"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Re47ba9afd89645aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rfdabc5d71ce44d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7debc316274542ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R4340d72de10846ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R0de631513e7e4c05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb13776be04d74d1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R51f6757a8d404630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R9aa2f499f2f442c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2fd3dfa04f6c4b93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R04dc1601788e4a30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6505f23d53944571"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re2bd729993784b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3914b76009e34b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R3a859c9491794691"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1800ddbfcaa443c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6e921edc3b474a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R21ad533024f74b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R13125ff48490491c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -77,8 +77,14 @@
       <x:color rgb="FF1D4ED8"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -108,6 +114,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFBFDBFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -145,7 +156,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -201,6 +212,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -217,12 +234,6 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -231,6 +242,24 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
@@ -485,25 +514,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7632.53</x:v>
+        <x:v>7706.9</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7522.77</x:v>
+        <x:v>7603.37</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>109.8</x:v>
+        <x:v>103.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1797.1</x:v>
+        <x:v>1900.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>138.2</x:v>
+        <x:v>135.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +543,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7738.03</x:v>
+        <x:v>7819.98</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7622.55</x:v>
+        <x:v>7710.24</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>115.5</x:v>
+        <x:v>109.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1617.6</x:v>
+        <x:v>1727.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>124.4</x:v>
+        <x:v>123.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +572,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3898.84</x:v>
+        <x:v>3919.67</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3866.89</x:v>
+        <x:v>3888.5</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>32</x:v>
+        <x:v>31.2</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>465.3</x:v>
+        <x:v>496.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.8</x:v>
+        <x:v>35.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +601,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7648</x:v>
+        <x:v>7712.4</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7522.2</x:v>
+        <x:v>7606.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>125.8</x:v>
+        <x:v>105.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2014.4</x:v>
+        <x:v>2120.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>155</x:v>
+        <x:v>151.4</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -601,25 +630,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7754</x:v>
+        <x:v>7820</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7617.2</x:v>
+        <x:v>7709.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>136.8</x:v>
+        <x:v>110.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1911.2</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>147</x:v>
+        <x:v>144.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -720,7 +749,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +954,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>156920</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-2360</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +990,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>153680</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>-3240</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +1026,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>149080</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>-4600</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1062,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>142000</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="n">
+      <x:c r="H7" s="28" t="n">
         <x:v>-7080</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1069,7 +1098,7 @@
       <x:c r="G8" s="23" t="n">
         <x:v>141140</x:v>
       </x:c>
-      <x:c r="H8" s="34" t="n">
+      <x:c r="H8" s="28" t="n">
         <x:v>-860</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
@@ -1105,7 +1134,7 @@
       <x:c r="G9" s="23" t="n">
         <x:v>142640</x:v>
       </x:c>
-      <x:c r="H9" s="34" t="n">
+      <x:c r="H9" s="28" t="n">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="I9" s="24" t="n">
@@ -1141,7 +1170,7 @@
       <x:c r="G10" s="23" t="n">
         <x:v>141140</x:v>
       </x:c>
-      <x:c r="H10" s="34" t="n">
+      <x:c r="H10" s="28" t="n">
         <x:v>-1500</x:v>
       </x:c>
       <x:c r="I10" s="24" t="n">
@@ -1177,7 +1206,7 @@
       <x:c r="G11" s="23" t="n">
         <x:v>140960</x:v>
       </x:c>
-      <x:c r="H11" s="34" t="n">
+      <x:c r="H11" s="28" t="n">
         <x:v>-180</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
@@ -1213,7 +1242,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>134340</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-6620</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -1249,7 +1278,7 @@
       <x:c r="G13" s="23" t="n">
         <x:v>132580</x:v>
       </x:c>
-      <x:c r="H13" s="34" t="n">
+      <x:c r="H13" s="28" t="n">
         <x:v>-1760</x:v>
       </x:c>
       <x:c r="I13" s="24" t="n">
@@ -1285,7 +1314,7 @@
       <x:c r="G14" s="23" t="n">
         <x:v>130000</x:v>
       </x:c>
-      <x:c r="H14" s="34" t="n">
+      <x:c r="H14" s="28" t="n">
         <x:v>-2580</x:v>
       </x:c>
       <x:c r="I14" s="24" t="n">
@@ -1321,7 +1350,7 @@
       <x:c r="G15" s="23" t="n">
         <x:v>127460</x:v>
       </x:c>
-      <x:c r="H15" s="34" t="n">
+      <x:c r="H15" s="28" t="n">
         <x:v>-2540</x:v>
       </x:c>
       <x:c r="I15" s="24" t="n">
@@ -1357,7 +1386,7 @@
       <x:c r="G16" s="23" t="n">
         <x:v>132280</x:v>
       </x:c>
-      <x:c r="H16" s="34" t="n">
+      <x:c r="H16" s="28" t="n">
         <x:v>4820</x:v>
       </x:c>
       <x:c r="I16" s="24" t="n">
@@ -1372,42 +1401,42 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="A19" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
+      <x:c r="B19" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>SUM(J4:J16)</x:f>
         <x:v>73220</x:v>
       </x:c>
-      <x:c r="K19" s="28"/>
+      <x:c r="K19" s="30"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="A20" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
         <x:v>5632.3</x:v>
       </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1564,76 +1593,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>7363.42</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>7632.53</x:v>
+        <x:v>7706.9</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>7329.6</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>7548.82</x:v>
-      </x:c>
-      <x:c r="G7" s="23" t="n">
+        <x:v>7687.59</x:v>
+      </x:c>
+      <x:c r="G7" s="28" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>121.6</x:v>
+        <x:v>260.4</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.01636947237466413</x:v>
+        <x:v>0.03505339803210883</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>302.9</x:v>
+        <x:v>377.3</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="A8" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B8" s="28" t="n">
+      <x:c r="B8" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="30" t="n">
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="30"/>
+      <x:c r="E8" s="30"/>
+      <x:c r="F8" s="30"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1051.4</x:v>
-      </x:c>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="28"/>
+        <x:v>1125.8</x:v>
+      </x:c>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="str">
+      <x:c r="A9" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B9" s="28"/>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="32" t="n">
+      <x:c r="B9" s="30"/>
+      <x:c r="C9" s="30"/>
+      <x:c r="D9" s="30"/>
+      <x:c r="E9" s="30"/>
+      <x:c r="F9" s="30"/>
+      <x:c r="G9" s="30"/>
+      <x:c r="H9" s="30"/>
+      <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>350.5</x:v>
-      </x:c>
-      <x:c r="J9" s="28"/>
-      <x:c r="K9" s="28"/>
+        <x:v>375.3</x:v>
+      </x:c>
+      <x:c r="J9" s="30"/>
+      <x:c r="K9" s="30"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="17" t="str">
@@ -1760,76 +1789,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>7511.04</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7738.03</x:v>
+        <x:v>7819.98</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>7487.46</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7654.98</x:v>
-      </x:c>
-      <x:c r="G15" s="23" t="n">
+        <x:v>7799.61</x:v>
+      </x:c>
+      <x:c r="G15" s="28" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>74.4</x:v>
+        <x:v>219.1</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.009819880905581835</x:v>
+        <x:v>0.028898996641400165</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>250.6</x:v>
+        <x:v>332.5</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="28" t="n">
+      <x:c r="B16" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="28"/>
-      <x:c r="E16" s="28"/>
-      <x:c r="F16" s="28"/>
-      <x:c r="G16" s="28"/>
-      <x:c r="H16" s="28"/>
-      <x:c r="I16" s="30" t="n">
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>974.6</x:v>
-      </x:c>
-      <x:c r="J16" s="28"/>
-      <x:c r="K16" s="28"/>
+        <x:v>1056.5</x:v>
+      </x:c>
+      <x:c r="J16" s="30"/>
+      <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="28"/>
-      <x:c r="E17" s="28"/>
-      <x:c r="F17" s="28"/>
-      <x:c r="G17" s="28"/>
-      <x:c r="H17" s="28"/>
-      <x:c r="I17" s="32" t="n">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>324.9</x:v>
-      </x:c>
-      <x:c r="J17" s="28"/>
-      <x:c r="K17" s="28"/>
+        <x:v>352.2</x:v>
+      </x:c>
+      <x:c r="J17" s="30"/>
+      <x:c r="K17" s="30"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="17" t="str">
@@ -1956,76 +1985,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3867.02</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3898.84</x:v>
+        <x:v>3919.67</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
         <x:v>3842.72</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3875.6</x:v>
+        <x:v>3911.87</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-12.5</x:v>
+        <x:v>23.8</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.0032175015624558156</x:v>
+        <x:v>0.0061109382193405</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>56.1</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+      <x:c r="A24" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
+      <x:c r="B24" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="28"/>
-      <x:c r="E24" s="28"/>
-      <x:c r="F24" s="28"/>
-      <x:c r="G24" s="28"/>
-      <x:c r="H24" s="28"/>
-      <x:c r="I24" s="30" t="n">
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>242.2</x:v>
-      </x:c>
-      <x:c r="J24" s="28"/>
-      <x:c r="K24" s="28"/>
+        <x:v>263.1</x:v>
+      </x:c>
+      <x:c r="J24" s="30"/>
+      <x:c r="K24" s="30"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="29" t="str">
+      <x:c r="A25" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="28"/>
-      <x:c r="E25" s="28"/>
-      <x:c r="F25" s="28"/>
-      <x:c r="G25" s="28"/>
-      <x:c r="H25" s="28"/>
-      <x:c r="I25" s="32" t="n">
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>80.7</x:v>
-      </x:c>
-      <x:c r="J25" s="28"/>
-      <x:c r="K25" s="28"/>
+        <x:v>87.7</x:v>
+      </x:c>
+      <x:c r="J25" s="30"/>
+      <x:c r="K25" s="30"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
@@ -2152,76 +2181,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>7312</x:v>
       </x:c>
       <x:c r="D31" s="23" t="n">
-        <x:v>7648</x:v>
+        <x:v>7712.4</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
         <x:v>7283.4</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>7559.8</x:v>
-      </x:c>
-      <x:c r="G31" s="23" t="n">
+        <x:v>7679.2</x:v>
+      </x:c>
+      <x:c r="G31" s="28" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>144.6</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.019500485489265307</x:v>
+        <x:v>0.03560254612148017</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>364.6</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="29" t="str">
+      <x:c r="A32" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="28" t="n">
+      <x:c r="B32" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="28"/>
-      <x:c r="D32" s="28"/>
-      <x:c r="E32" s="28"/>
-      <x:c r="F32" s="28"/>
-      <x:c r="G32" s="28"/>
-      <x:c r="H32" s="28"/>
-      <x:c r="I32" s="30" t="n">
+      <x:c r="C32" s="30"/>
+      <x:c r="D32" s="30"/>
+      <x:c r="E32" s="30"/>
+      <x:c r="F32" s="30"/>
+      <x:c r="G32" s="30"/>
+      <x:c r="H32" s="30"/>
+      <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1108.8</x:v>
-      </x:c>
-      <x:c r="J32" s="28"/>
-      <x:c r="K32" s="28"/>
+        <x:v>1173.2</x:v>
+      </x:c>
+      <x:c r="J32" s="30"/>
+      <x:c r="K32" s="30"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="29" t="str">
+      <x:c r="A33" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="28"/>
-      <x:c r="C33" s="28"/>
-      <x:c r="D33" s="28"/>
-      <x:c r="E33" s="28"/>
-      <x:c r="F33" s="28"/>
-      <x:c r="G33" s="28"/>
-      <x:c r="H33" s="28"/>
-      <x:c r="I33" s="32" t="n">
+      <x:c r="B33" s="30"/>
+      <x:c r="C33" s="30"/>
+      <x:c r="D33" s="30"/>
+      <x:c r="E33" s="30"/>
+      <x:c r="F33" s="30"/>
+      <x:c r="G33" s="30"/>
+      <x:c r="H33" s="30"/>
+      <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>369.6</x:v>
-      </x:c>
-      <x:c r="J33" s="28"/>
-      <x:c r="K33" s="28"/>
+        <x:v>391.1</x:v>
+      </x:c>
+      <x:c r="J33" s="30"/>
+      <x:c r="K33" s="30"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="17" t="str">
@@ -2348,76 +2377,76 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7482.2</x:v>
       </x:c>
       <x:c r="D39" s="23" t="n">
-        <x:v>7754</x:v>
+        <x:v>7820</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
         <x:v>7452.2</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>7664.6</x:v>
-      </x:c>
-      <x:c r="G39" s="23" t="n">
+        <x:v>7789.8</x:v>
+      </x:c>
+      <x:c r="G39" s="28" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>95.6</x:v>
+        <x:v>220.8</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.01263046637600751</x:v>
+        <x:v>0.02917162108600868</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>301.8</x:v>
+        <x:v>367.8</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="29" t="str">
+      <x:c r="A40" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="28" t="n">
+      <x:c r="B40" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C40" s="28"/>
-      <x:c r="D40" s="28"/>
-      <x:c r="E40" s="28"/>
-      <x:c r="F40" s="28"/>
-      <x:c r="G40" s="28"/>
-      <x:c r="H40" s="28"/>
-      <x:c r="I40" s="30" t="n">
+      <x:c r="C40" s="30"/>
+      <x:c r="D40" s="30"/>
+      <x:c r="E40" s="30"/>
+      <x:c r="F40" s="30"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1035.2</x:v>
-      </x:c>
-      <x:c r="J40" s="28"/>
-      <x:c r="K40" s="28"/>
+        <x:v>1101.2</x:v>
+      </x:c>
+      <x:c r="J40" s="30"/>
+      <x:c r="K40" s="30"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="29" t="str">
+      <x:c r="A41" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="28"/>
-      <x:c r="C41" s="28"/>
-      <x:c r="D41" s="28"/>
-      <x:c r="E41" s="28"/>
-      <x:c r="F41" s="28"/>
-      <x:c r="G41" s="28"/>
-      <x:c r="H41" s="28"/>
-      <x:c r="I41" s="32" t="n">
+      <x:c r="B41" s="30"/>
+      <x:c r="C41" s="30"/>
+      <x:c r="D41" s="30"/>
+      <x:c r="E41" s="30"/>
+      <x:c r="F41" s="30"/>
+      <x:c r="G41" s="30"/>
+      <x:c r="H41" s="30"/>
+      <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>345.1</x:v>
-      </x:c>
-      <x:c r="J41" s="28"/>
-      <x:c r="K41" s="28"/>
+        <x:v>367.1</x:v>
+      </x:c>
+      <x:c r="J41" s="30"/>
+      <x:c r="K41" s="30"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="17" t="str">
@@ -2578,42 +2607,42 @@
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="29" t="str">
+      <x:c r="A48" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="28" t="n">
+      <x:c r="B48" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C48" s="28"/>
-      <x:c r="D48" s="28"/>
-      <x:c r="E48" s="28"/>
-      <x:c r="F48" s="28"/>
-      <x:c r="G48" s="28"/>
-      <x:c r="H48" s="28"/>
-      <x:c r="I48" s="30" t="n">
+      <x:c r="C48" s="30"/>
+      <x:c r="D48" s="30"/>
+      <x:c r="E48" s="30"/>
+      <x:c r="F48" s="30"/>
+      <x:c r="G48" s="30"/>
+      <x:c r="H48" s="30"/>
+      <x:c r="I48" s="32" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
         <x:v>341</x:v>
       </x:c>
-      <x:c r="J48" s="28"/>
-      <x:c r="K48" s="28"/>
+      <x:c r="J48" s="30"/>
+      <x:c r="K48" s="30"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29" t="str">
+      <x:c r="A49" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="28"/>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="32" t="n">
+      <x:c r="B49" s="30"/>
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
         <x:v>113.7</x:v>
       </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="17" t="str">
@@ -2774,42 +2803,42 @@
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="29" t="str">
+      <x:c r="A56" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B56" s="28" t="n">
+      <x:c r="B56" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C56" s="28"/>
-      <x:c r="D56" s="28"/>
-      <x:c r="E56" s="28"/>
-      <x:c r="F56" s="28"/>
-      <x:c r="G56" s="28"/>
-      <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
+      <x:c r="C56" s="30"/>
+      <x:c r="D56" s="30"/>
+      <x:c r="E56" s="30"/>
+      <x:c r="F56" s="30"/>
+      <x:c r="G56" s="30"/>
+      <x:c r="H56" s="30"/>
+      <x:c r="I56" s="32" t="n">
         <x:f>ROUND(SUM(I53:I55),1)</x:f>
         <x:v>206.4</x:v>
       </x:c>
-      <x:c r="J56" s="28"/>
-      <x:c r="K56" s="28"/>
+      <x:c r="J56" s="30"/>
+      <x:c r="K56" s="30"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29" t="str">
+      <x:c r="A57" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
+      <x:c r="B57" s="30"/>
+      <x:c r="C57" s="30"/>
+      <x:c r="D57" s="30"/>
+      <x:c r="E57" s="30"/>
+      <x:c r="F57" s="30"/>
+      <x:c r="G57" s="30"/>
+      <x:c r="H57" s="30"/>
+      <x:c r="I57" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
         <x:v>68.8</x:v>
       </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+      <x:c r="J57" s="30"/>
+      <x:c r="K57" s="30"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="17" t="str">
@@ -2912,7 +2941,7 @@
       <x:c r="F62" s="23" t="n">
         <x:v>134340</x:v>
       </x:c>
-      <x:c r="G62" s="34" t="n">
+      <x:c r="G62" s="28" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
         <x:v>-7660</x:v>
       </x:c>
@@ -2950,7 +2979,7 @@
       <x:c r="F63" s="23" t="n">
         <x:v>132280</x:v>
       </x:c>
-      <x:c r="G63" s="34" t="n">
+      <x:c r="G63" s="28" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
         <x:v>-2060</x:v>
       </x:c>
@@ -2970,42 +2999,42 @@
       </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="29" t="str">
+      <x:c r="A64" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B64" s="28" t="n">
+      <x:c r="B64" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C64" s="28"/>
-      <x:c r="D64" s="28"/>
-      <x:c r="E64" s="28"/>
-      <x:c r="F64" s="28"/>
-      <x:c r="G64" s="28"/>
-      <x:c r="H64" s="28"/>
-      <x:c r="I64" s="30" t="n">
+      <x:c r="C64" s="30"/>
+      <x:c r="D64" s="30"/>
+      <x:c r="E64" s="30"/>
+      <x:c r="F64" s="30"/>
+      <x:c r="G64" s="30"/>
+      <x:c r="H64" s="30"/>
+      <x:c r="I64" s="32" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
         <x:v>46120</x:v>
       </x:c>
-      <x:c r="J64" s="28"/>
-      <x:c r="K64" s="28"/>
+      <x:c r="J64" s="30"/>
+      <x:c r="K64" s="30"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="29" t="str">
+      <x:c r="A65" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B65" s="28"/>
-      <x:c r="C65" s="28"/>
-      <x:c r="D65" s="28"/>
-      <x:c r="E65" s="28"/>
-      <x:c r="F65" s="28"/>
-      <x:c r="G65" s="28"/>
-      <x:c r="H65" s="28"/>
-      <x:c r="I65" s="32" t="n">
+      <x:c r="B65" s="30"/>
+      <x:c r="C65" s="30"/>
+      <x:c r="D65" s="30"/>
+      <x:c r="E65" s="30"/>
+      <x:c r="F65" s="30"/>
+      <x:c r="G65" s="30"/>
+      <x:c r="H65" s="30"/>
+      <x:c r="I65" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
         <x:v>15373.3</x:v>
       </x:c>
-      <x:c r="J65" s="28"/>
-      <x:c r="K65" s="28"/>
+      <x:c r="J65" s="30"/>
+      <x:c r="K65" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3390,7 +3419,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7427.24</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-160.5</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -3548,43 +3577,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>7621.24</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>7706.9</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>7603.37</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>7687.59</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>138.8</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.018383005555835386</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>103.5</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>1797.1</x:v>
-      </x:c>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>1900.6</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>138.2</x:v>
-      </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>135.8</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4119,43 +4184,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>7731.07</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>7819.98</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>7710.24</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>7799.61</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>144.6</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.018893583000870073</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>109.7</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>1617.5999999999997</x:v>
-      </x:c>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>1727.2999999999997</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>124.4</x:v>
-      </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>123.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4690,43 +4791,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>3891.96</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>3919.67</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>3888.5</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>3911.87</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>36.3</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.009358550934049026</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>31.2</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>465.29999999999995</x:v>
-      </x:c>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>496.49999999999994</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>35.8</x:v>
-      </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>35.5</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5103,7 +5240,7 @@
       <x:c r="G12" s="23" t="n">
         <x:v>7415.2</x:v>
       </x:c>
-      <x:c r="H12" s="34" t="n">
+      <x:c r="H12" s="28" t="n">
         <x:v>-158.8</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
@@ -5261,43 +5398,79 @@
         <x:v>IM2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>7626.6</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>7712.4</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>7606.6</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>7679.2</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>119.4</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.01579406862615418</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>105.8</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2014.3999999999999</x:v>
-      </x:c>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2120.2</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>151.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5832,43 +6005,79 @@
         <x:v>IC2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>7723</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>7820</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>7709.2</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>7789.8</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>125.2</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.016334838086788483</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>110.8</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>1911.1999999999998</x:v>
-      </x:c>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2021.9999999999998</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>144.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6404,42 +6613,42 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="A19" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
+      <x:c r="B19" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>SUM(J4:J16)</x:f>
         <x:v>697.3999999999999</x:v>
       </x:c>
-      <x:c r="K19" s="28"/>
+      <x:c r="K19" s="30"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="A20" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
         <x:v>53.6</x:v>
       </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6975,42 +7184,42 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="A19" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="n">
+      <x:c r="B19" s="30" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="28"/>
-      <x:c r="J19" s="30" t="n">
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="32" t="n">
         <x:f>SUM(J4:J16)</x:f>
         <x:v>415</x:v>
       </x:c>
-      <x:c r="K19" s="28"/>
+      <x:c r="K19" s="30"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="29" t="str">
+      <x:c r="A20" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="28"/>
-      <x:c r="E20" s="28"/>
-      <x:c r="F20" s="28"/>
-      <x:c r="G20" s="28"/>
-      <x:c r="H20" s="28"/>
-      <x:c r="I20" s="28"/>
-      <x:c r="J20" s="32" t="n">
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
         <x:v>31.9</x:v>
       </x:c>
-      <x:c r="K20" s="28"/>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-21
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R2fd3dfa04f6c4b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R04dc1601788e4a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6505f23d53944571"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re2bd729993784b8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R3914b76009e34b7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R3a859c9491794691"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1800ddbfcaa443c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6e921edc3b474a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R21ad533024f74b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R13125ff48490491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra19fc4aa5e884359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R606d2e9edec5419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R8cc5011706954b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4016840a39de42ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9c4e61e4cb7f48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5cbd679f42df44a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R207048fcaa414741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R8dac8869aa744cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rd39ff3cd26014f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R2a1b2802326246a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -156,7 +156,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -262,6 +262,12 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -514,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7706.9</x:v>
+        <x:v>7777.91</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7603.37</x:v>
+        <x:v>7723.68</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>103.5</x:v>
+        <x:v>54.2</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1900.6</x:v>
+        <x:v>1954.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>135.8</x:v>
+        <x:v>130.3</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -543,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7819.98</x:v>
+        <x:v>7869.35</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7710.24</x:v>
+        <x:v>7809.59</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>109.7</x:v>
+        <x:v>59.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1727.3</x:v>
+        <x:v>1787.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>123.4</x:v>
+        <x:v>119.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -572,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3919.67</x:v>
+        <x:v>3950.94</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3888.5</x:v>
+        <x:v>3918.13</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>31.2</x:v>
+        <x:v>32.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>496.5</x:v>
+        <x:v>529.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.5</x:v>
+        <x:v>35.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -659,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4500.6</x:v>
+        <x:v>4520.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4452.2</x:v>
+        <x:v>4481</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>48.4</x:v>
+        <x:v>39.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>697.4</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>53.6</x:v>
+        <x:v>52.6</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -688,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2872.4</x:v>
+        <x:v>2870.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2838.4</x:v>
+        <x:v>2853.4</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>34</x:v>
+        <x:v>17.4</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>415</x:v>
+        <x:v>432.4</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>31.9</x:v>
+        <x:v>30.9</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -717,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-17</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>133760</x:v>
+        <x:v>134800</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>127900</x:v>
+        <x:v>127100</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>5860</x:v>
+        <x:v>7700</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>73220</x:v>
+        <x:v>89880</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5632.3</x:v>
+        <x:v>5992</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -749,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1400,43 +1406,115 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>135900</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>135900</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>126940</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>128580</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>-3700</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>-0.02797097066827936</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>8960</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>128500</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>134800</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>127100</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>133500</x:v>
+      </x:c>
+      <x:c r="H18" s="28" t="n">
+        <x:v>4920</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.038264115725618275</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>7700</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>73220</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>89880</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B20" s="30"/>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>5632.3</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>5992</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1627,193 +1705,193 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="30"/>
-      <x:c r="E8" s="30"/>
-      <x:c r="F8" s="30"/>
-      <x:c r="G8" s="30"/>
-      <x:c r="H8" s="30"/>
-      <x:c r="I8" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1125.8</x:v>
-      </x:c>
-      <x:c r="J8" s="30"/>
-      <x:c r="K8" s="30"/>
+      <x:c r="A8" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="n">
+        <x:v>7723.68</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7777.91</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7723.68</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>7766.33</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:f>ROUND(F8-F7,1)</x:f>
+        <x:v>78.7</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="n">
+        <x:f>IFERROR(F8/F7-1,"")</x:f>
+        <x:v>0.01024248171403519</x:v>
+      </x:c>
+      <x:c r="I8" s="23" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>54.2</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C9" s="30"/>
       <x:c r="D9" s="30"/>
       <x:c r="E9" s="30"/>
       <x:c r="F9" s="30"/>
       <x:c r="G9" s="30"/>
       <x:c r="H9" s="30"/>
-      <x:c r="I9" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>375.3</x:v>
+      <x:c r="I9" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I8),1)</x:f>
+        <x:v>1180</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="17" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="J10" s="30"/>
+      <x:c r="K10" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B11" s="17"/>
-      <x:c r="C11" s="17"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="17"/>
-      <x:c r="F11" s="17"/>
-      <x:c r="G11" s="17"/>
-      <x:c r="H11" s="17"/>
-      <x:c r="I11" s="17"/>
-      <x:c r="J11" s="17"/>
-      <x:c r="K11" s="17"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="20" t="str">
+      <x:c r="B12" s="17"/>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
+      <x:c r="H12" s="17"/>
+      <x:c r="I12" s="17"/>
+      <x:c r="J12" s="17"/>
+      <x:c r="K12" s="17"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="str">
+      <x:c r="B13" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="str">
+      <x:c r="C13" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D12" s="20" t="str">
+      <x:c r="D13" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E12" s="20" t="str">
+      <x:c r="E13" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="str">
+      <x:c r="F13" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G12" s="20" t="str">
+      <x:c r="G13" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H12" s="20" t="str">
+      <x:c r="H13" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I12" s="20" t="str">
+      <x:c r="I13" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J12" s="20" t="str">
+      <x:c r="J13" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K12" s="20" t="str">
+      <x:c r="K13" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B13" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C13" s="23" t="n">
-        <x:v>7944.29</x:v>
-      </x:c>
-      <x:c r="D13" s="23" t="n">
-        <x:v>7955.57</x:v>
-      </x:c>
-      <x:c r="E13" s="23" t="n">
-        <x:v>7610.58</x:v>
-      </x:c>
-      <x:c r="F13" s="23" t="n">
-        <x:v>7652.69</x:v>
-      </x:c>
-      <x:c r="G13" s="23"/>
-      <x:c r="H13" s="24"/>
-      <x:c r="I13" s="26" t="n">
-        <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="J13" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K13" s="22" t="n">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C14" s="23" t="n">
-        <x:v>7687.47</x:v>
+        <x:v>7944.29</x:v>
       </x:c>
       <x:c r="D14" s="23" t="n">
-        <x:v>7830.16</x:v>
+        <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E14" s="23" t="n">
-        <x:v>7451.12</x:v>
+        <x:v>7610.58</x:v>
       </x:c>
       <x:c r="F14" s="23" t="n">
-        <x:v>7580.54</x:v>
-      </x:c>
-      <x:c r="G14" s="23" t="n">
-        <x:f>ROUND(F14-F13,1)</x:f>
-        <x:v>-72.1</x:v>
-      </x:c>
-      <x:c r="H14" s="24" t="n">
-        <x:f>IFERROR(F14/F13-1,"")</x:f>
-        <x:v>-0.009428057323633832</x:v>
-      </x:c>
+        <x:v>7652.69</x:v>
+      </x:c>
+      <x:c r="G14" s="23"/>
+      <x:c r="H14" s="24"/>
       <x:c r="I14" s="26" t="n">
         <x:f>ROUND(D14-E14,1)</x:f>
-        <x:v>379</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J14" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K14" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
-        <x:v>7511.04</x:v>
+        <x:v>7687.47</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7819.98</x:v>
+        <x:v>7830.16</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7487.46</x:v>
+        <x:v>7451.12</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7799.61</x:v>
-      </x:c>
-      <x:c r="G15" s="28" t="n">
+        <x:v>7580.54</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>219.1</x:v>
+        <x:v>-72.1</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.028898996641400165</x:v>
+        <x:v>-0.009428057323633832</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>332.5</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
@@ -1823,1230 +1901,1382 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="31" t="str">
+      <x:c r="A16" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="n">
+        <x:v>7511.04</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>7819.98</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>7487.46</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>7799.61</x:v>
+      </x:c>
+      <x:c r="G16" s="28" t="n">
+        <x:f>ROUND(F16-F15,1)</x:f>
+        <x:v>219.1</x:v>
+      </x:c>
+      <x:c r="H16" s="24" t="n">
+        <x:f>IFERROR(F16/F15-1,"")</x:f>
+        <x:v>0.028898996641400165</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="n">
+        <x:f>ROUND(D16-E16,1)</x:f>
+        <x:v>332.5</x:v>
+      </x:c>
+      <x:c r="J16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="n">
+        <x:v>7829.82</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>7869.35</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>7809.59</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>7850.48</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:f>ROUND(F17-F16,1)</x:f>
+        <x:v>50.9</x:v>
+      </x:c>
+      <x:c r="H17" s="24" t="n">
+        <x:f>IFERROR(F17/F16-1,"")</x:f>
+        <x:v>0.0065221209778436595</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:f>ROUND(D17-E17,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="J17" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="32" t="n">
-        <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1056.5</x:v>
-      </x:c>
-      <x:c r="J16" s="30"/>
-      <x:c r="K16" s="30"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="32" t="n">
+        <x:f>ROUND(SUM(I14:I17),1)</x:f>
+        <x:v>1116.3</x:v>
+      </x:c>
+      <x:c r="J18" s="30"/>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>352.2</x:v>
-      </x:c>
-      <x:c r="J17" s="30"/>
-      <x:c r="K17" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="17" t="str">
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="J19" s="30"/>
+      <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B19" s="17"/>
-      <x:c r="C19" s="17"/>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="17"/>
-      <x:c r="F19" s="17"/>
-      <x:c r="G19" s="17"/>
-      <x:c r="H19" s="17"/>
-      <x:c r="I19" s="17"/>
-      <x:c r="J19" s="17"/>
-      <x:c r="K19" s="17"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="20" t="str">
+      <x:c r="B21" s="17"/>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="17"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="17"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B20" s="20" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D20" s="20" t="str">
+      <x:c r="D22" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="str">
+      <x:c r="E22" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
+      <x:c r="F22" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="str">
+      <x:c r="G22" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H20" s="20" t="str">
+      <x:c r="H22" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I20" s="20" t="str">
+      <x:c r="I22" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J20" s="20" t="str">
+      <x:c r="J22" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K20" s="20" t="str">
+      <x:c r="K22" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B21" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C21" s="23" t="n">
-        <x:v>3979.88</x:v>
-      </x:c>
-      <x:c r="D21" s="23" t="n">
-        <x:v>3995.18</x:v>
-      </x:c>
-      <x:c r="E21" s="23" t="n">
-        <x:v>3915.22</x:v>
-      </x:c>
-      <x:c r="F21" s="23" t="n">
-        <x:v>3930.12</x:v>
-      </x:c>
-      <x:c r="G21" s="23"/>
-      <x:c r="H21" s="24"/>
-      <x:c r="I21" s="26" t="n">
-        <x:f>ROUND(D21-E21,1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J21" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K21" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B22" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C22" s="23" t="n">
-        <x:v>3942.51</x:v>
-      </x:c>
-      <x:c r="D22" s="23" t="n">
-        <x:v>3958.12</x:v>
-      </x:c>
-      <x:c r="E22" s="23" t="n">
-        <x:v>3852.03</x:v>
-      </x:c>
-      <x:c r="F22" s="23" t="n">
-        <x:v>3888.11</x:v>
-      </x:c>
-      <x:c r="G22" s="23" t="n">
-        <x:f>ROUND(F22-F21,1)</x:f>
-        <x:v>-42</x:v>
-      </x:c>
-      <x:c r="H22" s="24" t="n">
-        <x:f>IFERROR(F22/F21-1,"")</x:f>
-        <x:v>-0.010689241040986008</x:v>
-      </x:c>
-      <x:c r="I22" s="26" t="n">
-        <x:f>ROUND(D22-E22,1)</x:f>
-        <x:v>106.1</x:v>
-      </x:c>
-      <x:c r="J22" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K22" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
-        <x:v>3867.02</x:v>
+        <x:v>3979.88</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3919.67</x:v>
+        <x:v>3995.18</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3842.72</x:v>
+        <x:v>3915.22</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3911.87</x:v>
-      </x:c>
-      <x:c r="G23" s="23" t="n">
-        <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>23.8</x:v>
-      </x:c>
-      <x:c r="H23" s="24" t="n">
-        <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.0061109382193405</x:v>
-      </x:c>
+        <x:v>3930.12</x:v>
+      </x:c>
+      <x:c r="G23" s="23"/>
+      <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="n">
+        <x:v>3942.51</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>3958.12</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>3852.03</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>3888.11</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:f>ROUND(F24-F23,1)</x:f>
+        <x:v>-42</x:v>
+      </x:c>
+      <x:c r="H24" s="24" t="n">
+        <x:f>IFERROR(F24/F23-1,"")</x:f>
+        <x:v>-0.010689241040986008</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="n">
+        <x:f>ROUND(D24-E24,1)</x:f>
+        <x:v>106.1</x:v>
+      </x:c>
+      <x:c r="J24" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
+    <x:row r="25">
+      <x:c r="A25" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="n">
+        <x:v>3919.67</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="n">
+        <x:v>3842.72</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="n">
+        <x:v>3911.87</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="n">
+        <x:f>ROUND(F25-F24,1)</x:f>
+        <x:v>23.8</x:v>
+      </x:c>
+      <x:c r="H25" s="24" t="n">
+        <x:f>IFERROR(F25/F24-1,"")</x:f>
+        <x:v>0.0061109382193405</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="n">
+        <x:f>ROUND(D25-E25,1)</x:f>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J25" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K25" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="n">
+        <x:v>3920.27</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>3950.94</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>3918.13</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>3949.91</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="n">
+        <x:f>ROUND(F26-F25,1)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H26" s="24" t="n">
+        <x:f>IFERROR(F26/F25-1,"")</x:f>
+        <x:v>0.009724249527719442</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="30" t="n">
+      <x:c r="B27" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="32" t="n">
+        <x:f>ROUND(SUM(I23:I26),1)</x:f>
+        <x:v>295.9</x:v>
+      </x:c>
+      <x:c r="J27" s="30"/>
+      <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="J28" s="30"/>
+      <x:c r="K28" s="30"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B30" s="17"/>
+      <x:c r="C30" s="17"/>
+      <x:c r="D30" s="17"/>
+      <x:c r="E30" s="17"/>
+      <x:c r="F30" s="17"/>
+      <x:c r="G30" s="17"/>
+      <x:c r="H30" s="17"/>
+      <x:c r="I30" s="17"/>
+      <x:c r="J30" s="17"/>
+      <x:c r="K30" s="17"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F31" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G31" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I31" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J31" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K31" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B32" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C32" s="23" t="n">
+        <x:v>7713.4</x:v>
+      </x:c>
+      <x:c r="D32" s="23" t="n">
+        <x:v>7721</x:v>
+      </x:c>
+      <x:c r="E32" s="23" t="n">
+        <x:v>7432</x:v>
+      </x:c>
+      <x:c r="F32" s="23" t="n">
+        <x:v>7468.2</x:v>
+      </x:c>
+      <x:c r="G32" s="23"/>
+      <x:c r="H32" s="24"/>
+      <x:c r="I32" s="26" t="n">
+        <x:f>ROUND(D32-E32,1)</x:f>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="J32" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K32" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7527.2</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7714.6</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>7259.4</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>7415.2</x:v>
+      </x:c>
+      <x:c r="G33" s="23" t="n">
+        <x:f>ROUND(F33-F32,1)</x:f>
+        <x:v>-53</x:v>
+      </x:c>
+      <x:c r="H33" s="24" t="n">
+        <x:f>IFERROR(F33/F32-1,"")</x:f>
+        <x:v>-0.007096756915990432</x:v>
+      </x:c>
+      <x:c r="I33" s="26" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>455.2</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="32" t="n">
-        <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>263.1</x:v>
-      </x:c>
-      <x:c r="J24" s="30"/>
-      <x:c r="K24" s="30"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
+      <x:c r="B34" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C34" s="23" t="n">
+        <x:v>7312</x:v>
+      </x:c>
+      <x:c r="D34" s="23" t="n">
+        <x:v>7712.4</x:v>
+      </x:c>
+      <x:c r="E34" s="23" t="n">
+        <x:v>7283.4</x:v>
+      </x:c>
+      <x:c r="F34" s="23" t="n">
+        <x:v>7679.2</x:v>
+      </x:c>
+      <x:c r="G34" s="28" t="n">
+        <x:f>ROUND(F34-F33,1)</x:f>
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="H34" s="24" t="n">
+        <x:f>IFERROR(F34/F33-1,"")</x:f>
+        <x:v>0.03560254612148017</x:v>
+      </x:c>
+      <x:c r="I34" s="26" t="n">
+        <x:f>ROUND(D34-E34,1)</x:f>
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="J34" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K34" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B35" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C35" s="30"/>
+      <x:c r="D35" s="30"/>
+      <x:c r="E35" s="30"/>
+      <x:c r="F35" s="30"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(SUM(I32:I34),1)</x:f>
+        <x:v>1173.2</x:v>
+      </x:c>
+      <x:c r="J35" s="30"/>
+      <x:c r="K35" s="30"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="30"/>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>87.7</x:v>
-      </x:c>
-      <x:c r="J25" s="30"/>
-      <x:c r="K25" s="30"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
+      <x:c r="B36" s="30"/>
+      <x:c r="C36" s="30"/>
+      <x:c r="D36" s="30"/>
+      <x:c r="E36" s="30"/>
+      <x:c r="F36" s="30"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I32:I34),0),1)</x:f>
+        <x:v>391.1</x:v>
+      </x:c>
+      <x:c r="J36" s="30"/>
+      <x:c r="K36" s="30"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B38" s="17"/>
+      <x:c r="C38" s="17"/>
+      <x:c r="D38" s="17"/>
+      <x:c r="E38" s="17"/>
+      <x:c r="F38" s="17"/>
+      <x:c r="G38" s="17"/>
+      <x:c r="H38" s="17"/>
+      <x:c r="I38" s="17"/>
+      <x:c r="J38" s="17"/>
+      <x:c r="K38" s="17"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B28" s="20" t="str">
+      <x:c r="B39" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C28" s="20" t="str">
+      <x:c r="C39" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D28" s="20" t="str">
+      <x:c r="D39" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E28" s="20" t="str">
+      <x:c r="E39" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F28" s="20" t="str">
+      <x:c r="F39" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G28" s="20" t="str">
+      <x:c r="G39" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H28" s="20" t="str">
+      <x:c r="H39" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I28" s="20" t="str">
+      <x:c r="I39" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J28" s="20" t="str">
+      <x:c r="J39" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K28" s="20" t="str">
+      <x:c r="K39" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
+    <x:row r="40">
+      <x:c r="A40" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="22" t="str">
+      <x:c r="B40" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7713.4</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7721</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>7432</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7468.2</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
+      <x:c r="C40" s="23" t="n">
+        <x:v>7880.8</x:v>
+      </x:c>
+      <x:c r="D40" s="23" t="n">
+        <x:v>7903</x:v>
+      </x:c>
+      <x:c r="E40" s="23" t="n">
+        <x:v>7568</x:v>
+      </x:c>
+      <x:c r="F40" s="23" t="n">
+        <x:v>7608</x:v>
+      </x:c>
+      <x:c r="G40" s="23"/>
+      <x:c r="H40" s="24"/>
+      <x:c r="I40" s="26" t="n">
+        <x:f>ROUND(D40-E40,1)</x:f>
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="J40" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K40" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="22" t="n">
+    <x:row r="41">
+      <x:c r="A41" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B30" s="22" t="str">
+      <x:c r="B41" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C30" s="23" t="n">
-        <x:v>7527.2</x:v>
-      </x:c>
-      <x:c r="D30" s="23" t="n">
-        <x:v>7714.6</x:v>
-      </x:c>
-      <x:c r="E30" s="23" t="n">
-        <x:v>7259.4</x:v>
-      </x:c>
-      <x:c r="F30" s="23" t="n">
-        <x:v>7415.2</x:v>
-      </x:c>
-      <x:c r="G30" s="23" t="n">
-        <x:f>ROUND(F30-F29,1)</x:f>
-        <x:v>-53</x:v>
-      </x:c>
-      <x:c r="H30" s="24" t="n">
-        <x:f>IFERROR(F30/F29-1,"")</x:f>
-        <x:v>-0.007096756915990432</x:v>
-      </x:c>
-      <x:c r="I30" s="26" t="n">
-        <x:f>ROUND(D30-E30,1)</x:f>
-        <x:v>455.2</x:v>
-      </x:c>
-      <x:c r="J30" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K30" s="22" t="n">
+      <x:c r="C41" s="23" t="n">
+        <x:v>7665.6</x:v>
+      </x:c>
+      <x:c r="D41" s="23" t="n">
+        <x:v>7817.2</x:v>
+      </x:c>
+      <x:c r="E41" s="23" t="n">
+        <x:v>7418.8</x:v>
+      </x:c>
+      <x:c r="F41" s="23" t="n">
+        <x:v>7569</x:v>
+      </x:c>
+      <x:c r="G41" s="23" t="n">
+        <x:f>ROUND(F41-F40,1)</x:f>
+        <x:v>-39</x:v>
+      </x:c>
+      <x:c r="H41" s="24" t="n">
+        <x:f>IFERROR(F41/F40-1,"")</x:f>
+        <x:v>-0.005126182965299653</x:v>
+      </x:c>
+      <x:c r="I41" s="26" t="n">
+        <x:f>ROUND(D41-E41,1)</x:f>
+        <x:v>398.4</x:v>
+      </x:c>
+      <x:c r="J41" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K41" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="22" t="n">
+    <x:row r="42">
+      <x:c r="A42" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B31" s="22" t="str">
+      <x:c r="B42" s="22" t="str">
         <x:v>9月14日-9月18日</x:v>
       </x:c>
-      <x:c r="C31" s="23" t="n">
-        <x:v>7312</x:v>
-      </x:c>
-      <x:c r="D31" s="23" t="n">
-        <x:v>7712.4</x:v>
-      </x:c>
-      <x:c r="E31" s="23" t="n">
-        <x:v>7283.4</x:v>
-      </x:c>
-      <x:c r="F31" s="23" t="n">
-        <x:v>7679.2</x:v>
-      </x:c>
-      <x:c r="G31" s="28" t="n">
-        <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>264</x:v>
-      </x:c>
-      <x:c r="H31" s="24" t="n">
-        <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.03560254612148017</x:v>
-      </x:c>
-      <x:c r="I31" s="26" t="n">
-        <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="J31" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K31" s="22" t="n">
+      <x:c r="C42" s="23" t="n">
+        <x:v>7482.2</x:v>
+      </x:c>
+      <x:c r="D42" s="23" t="n">
+        <x:v>7820</x:v>
+      </x:c>
+      <x:c r="E42" s="23" t="n">
+        <x:v>7452.2</x:v>
+      </x:c>
+      <x:c r="F42" s="23" t="n">
+        <x:v>7789.8</x:v>
+      </x:c>
+      <x:c r="G42" s="28" t="n">
+        <x:f>ROUND(F42-F41,1)</x:f>
+        <x:v>220.8</x:v>
+      </x:c>
+      <x:c r="H42" s="24" t="n">
+        <x:f>IFERROR(F42/F41-1,"")</x:f>
+        <x:v>0.02917162108600868</x:v>
+      </x:c>
+      <x:c r="I42" s="26" t="n">
+        <x:f>ROUND(D42-E42,1)</x:f>
+        <x:v>367.8</x:v>
+      </x:c>
+      <x:c r="J42" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K42" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="31" t="str">
+    <x:row r="43">
+      <x:c r="A43" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="30" t="n">
+      <x:c r="B43" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="30"/>
-      <x:c r="E32" s="30"/>
-      <x:c r="F32" s="30"/>
-      <x:c r="G32" s="30"/>
-      <x:c r="H32" s="30"/>
-      <x:c r="I32" s="32" t="n">
-        <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1173.2</x:v>
-      </x:c>
-      <x:c r="J32" s="30"/>
-      <x:c r="K32" s="30"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="31" t="str">
+      <x:c r="C43" s="30"/>
+      <x:c r="D43" s="30"/>
+      <x:c r="E43" s="30"/>
+      <x:c r="F43" s="30"/>
+      <x:c r="G43" s="30"/>
+      <x:c r="H43" s="30"/>
+      <x:c r="I43" s="32" t="n">
+        <x:f>ROUND(SUM(I40:I42),1)</x:f>
+        <x:v>1101.2</x:v>
+      </x:c>
+      <x:c r="J43" s="30"/>
+      <x:c r="K43" s="30"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="30"/>
-      <x:c r="C33" s="30"/>
-      <x:c r="D33" s="30"/>
-      <x:c r="E33" s="30"/>
-      <x:c r="F33" s="30"/>
-      <x:c r="G33" s="30"/>
-      <x:c r="H33" s="30"/>
-      <x:c r="I33" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>391.1</x:v>
-      </x:c>
-      <x:c r="J33" s="30"/>
-      <x:c r="K33" s="30"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B35" s="17"/>
-      <x:c r="C35" s="17"/>
-      <x:c r="D35" s="17"/>
-      <x:c r="E35" s="17"/>
-      <x:c r="F35" s="17"/>
-      <x:c r="G35" s="17"/>
-      <x:c r="H35" s="17"/>
-      <x:c r="I35" s="17"/>
-      <x:c r="J35" s="17"/>
-      <x:c r="K35" s="17"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="20" t="str">
+      <x:c r="B44" s="30"/>
+      <x:c r="C44" s="30"/>
+      <x:c r="D44" s="30"/>
+      <x:c r="E44" s="30"/>
+      <x:c r="F44" s="30"/>
+      <x:c r="G44" s="30"/>
+      <x:c r="H44" s="30"/>
+      <x:c r="I44" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I40:I42),0),1)</x:f>
+        <x:v>367.1</x:v>
+      </x:c>
+      <x:c r="J44" s="30"/>
+      <x:c r="K44" s="30"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B46" s="17"/>
+      <x:c r="C46" s="17"/>
+      <x:c r="D46" s="17"/>
+      <x:c r="E46" s="17"/>
+      <x:c r="F46" s="17"/>
+      <x:c r="G46" s="17"/>
+      <x:c r="H46" s="17"/>
+      <x:c r="I46" s="17"/>
+      <x:c r="J46" s="17"/>
+      <x:c r="K46" s="17"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B36" s="20" t="str">
+      <x:c r="B47" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C36" s="20" t="str">
+      <x:c r="C47" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D36" s="20" t="str">
+      <x:c r="D47" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E36" s="20" t="str">
+      <x:c r="E47" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F36" s="20" t="str">
+      <x:c r="F47" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G36" s="20" t="str">
+      <x:c r="G47" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H36" s="20" t="str">
+      <x:c r="H47" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I36" s="20" t="str">
+      <x:c r="I47" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J36" s="20" t="str">
+      <x:c r="J47" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K36" s="20" t="str">
+      <x:c r="K47" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="22" t="n">
+    <x:row r="48">
+      <x:c r="A48" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B37" s="22" t="str">
+      <x:c r="B48" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C37" s="23" t="n">
-        <x:v>7880.8</x:v>
-      </x:c>
-      <x:c r="D37" s="23" t="n">
-        <x:v>7903</x:v>
-      </x:c>
-      <x:c r="E37" s="23" t="n">
-        <x:v>7568</x:v>
-      </x:c>
-      <x:c r="F37" s="23" t="n">
-        <x:v>7608</x:v>
-      </x:c>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="24"/>
-      <x:c r="I37" s="26" t="n">
-        <x:f>ROUND(D37-E37,1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J37" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K37" s="22" t="n">
+      <x:c r="C48" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="D48" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="E48" s="23" t="n">
+        <x:v>4497.6</x:v>
+      </x:c>
+      <x:c r="F48" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="G48" s="23"/>
+      <x:c r="H48" s="24"/>
+      <x:c r="I48" s="26" t="n">
+        <x:f>ROUND(D48-E48,1)</x:f>
+        <x:v>120.2</x:v>
+      </x:c>
+      <x:c r="J48" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K48" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="22" t="n">
+    <x:row r="49">
+      <x:c r="A49" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B38" s="22" t="str">
+      <x:c r="B49" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C38" s="23" t="n">
-        <x:v>7665.6</x:v>
-      </x:c>
-      <x:c r="D38" s="23" t="n">
-        <x:v>7817.2</x:v>
-      </x:c>
-      <x:c r="E38" s="23" t="n">
-        <x:v>7418.8</x:v>
-      </x:c>
-      <x:c r="F38" s="23" t="n">
-        <x:v>7569</x:v>
-      </x:c>
-      <x:c r="G38" s="23" t="n">
-        <x:f>ROUND(F38-F37,1)</x:f>
-        <x:v>-39</x:v>
-      </x:c>
-      <x:c r="H38" s="24" t="n">
-        <x:f>IFERROR(F38/F37-1,"")</x:f>
-        <x:v>-0.005126182965299653</x:v>
-      </x:c>
-      <x:c r="I38" s="26" t="n">
-        <x:f>ROUND(D38-E38,1)</x:f>
-        <x:v>398.4</x:v>
-      </x:c>
-      <x:c r="J38" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K38" s="22" t="n">
+      <x:c r="C49" s="23" t="n">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="D49" s="23" t="n">
+        <x:v>4584</x:v>
+      </x:c>
+      <x:c r="E49" s="23" t="n">
+        <x:v>4451.6</x:v>
+      </x:c>
+      <x:c r="F49" s="23" t="n">
+        <x:v>4503.4</x:v>
+      </x:c>
+      <x:c r="G49" s="23" t="n">
+        <x:f>ROUND(F49-F48,1)</x:f>
+        <x:v>-34</x:v>
+      </x:c>
+      <x:c r="H49" s="24" t="n">
+        <x:f>IFERROR(F49/F48-1,"")</x:f>
+        <x:v>-0.007493278088773314</x:v>
+      </x:c>
+      <x:c r="I49" s="26" t="n">
+        <x:f>ROUND(D49-E49,1)</x:f>
+        <x:v>132.4</x:v>
+      </x:c>
+      <x:c r="J49" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K49" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="22" t="n">
+    <x:row r="50">
+      <x:c r="A50" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B39" s="22" t="str">
+      <x:c r="B50" s="22" t="str">
         <x:v>9月14日-9月18日</x:v>
       </x:c>
-      <x:c r="C39" s="23" t="n">
-        <x:v>7482.2</x:v>
-      </x:c>
-      <x:c r="D39" s="23" t="n">
-        <x:v>7820</x:v>
-      </x:c>
-      <x:c r="E39" s="23" t="n">
-        <x:v>7452.2</x:v>
-      </x:c>
-      <x:c r="F39" s="23" t="n">
-        <x:v>7789.8</x:v>
-      </x:c>
-      <x:c r="G39" s="28" t="n">
-        <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>220.8</x:v>
-      </x:c>
-      <x:c r="H39" s="24" t="n">
-        <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.02917162108600868</x:v>
-      </x:c>
-      <x:c r="I39" s="26" t="n">
-        <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>367.8</x:v>
-      </x:c>
-      <x:c r="J39" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K39" s="22" t="n">
+      <x:c r="C50" s="23" t="n">
+        <x:v>4468</x:v>
+      </x:c>
+      <x:c r="D50" s="23" t="n">
+        <x:v>4520.6</x:v>
+      </x:c>
+      <x:c r="E50" s="23" t="n">
+        <x:v>4412.2</x:v>
+      </x:c>
+      <x:c r="F50" s="23" t="n">
+        <x:v>4508</x:v>
+      </x:c>
+      <x:c r="G50" s="23" t="n">
+        <x:f>ROUND(F50-F49,1)</x:f>
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="H50" s="24" t="n">
+        <x:f>IFERROR(F50/F49-1,"")</x:f>
+        <x:v>0.0010214504596528506</x:v>
+      </x:c>
+      <x:c r="I50" s="26" t="n">
+        <x:f>ROUND(D50-E50,1)</x:f>
+        <x:v>108.4</x:v>
+      </x:c>
+      <x:c r="J50" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K50" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="31" t="str">
+    <x:row r="51">
+      <x:c r="A51" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="30" t="n">
+      <x:c r="B51" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="30"/>
-      <x:c r="H40" s="30"/>
-      <x:c r="I40" s="32" t="n">
-        <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1101.2</x:v>
-      </x:c>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="30"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="31" t="str">
+      <x:c r="C51" s="30"/>
+      <x:c r="D51" s="30"/>
+      <x:c r="E51" s="30"/>
+      <x:c r="F51" s="30"/>
+      <x:c r="G51" s="30"/>
+      <x:c r="H51" s="30"/>
+      <x:c r="I51" s="32" t="n">
+        <x:f>ROUND(SUM(I48:I50),1)</x:f>
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="J51" s="30"/>
+      <x:c r="K51" s="30"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="30"/>
-      <x:c r="H41" s="30"/>
-      <x:c r="I41" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>367.1</x:v>
-      </x:c>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="30"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B43" s="17"/>
-      <x:c r="C43" s="17"/>
-      <x:c r="D43" s="17"/>
-      <x:c r="E43" s="17"/>
-      <x:c r="F43" s="17"/>
-      <x:c r="G43" s="17"/>
-      <x:c r="H43" s="17"/>
-      <x:c r="I43" s="17"/>
-      <x:c r="J43" s="17"/>
-      <x:c r="K43" s="17"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="20" t="str">
+      <x:c r="B52" s="30"/>
+      <x:c r="C52" s="30"/>
+      <x:c r="D52" s="30"/>
+      <x:c r="E52" s="30"/>
+      <x:c r="F52" s="30"/>
+      <x:c r="G52" s="30"/>
+      <x:c r="H52" s="30"/>
+      <x:c r="I52" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I48:I50),0),1)</x:f>
+        <x:v>120.3</x:v>
+      </x:c>
+      <x:c r="J52" s="30"/>
+      <x:c r="K52" s="30"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B54" s="17"/>
+      <x:c r="C54" s="17"/>
+      <x:c r="D54" s="17"/>
+      <x:c r="E54" s="17"/>
+      <x:c r="F54" s="17"/>
+      <x:c r="G54" s="17"/>
+      <x:c r="H54" s="17"/>
+      <x:c r="I54" s="17"/>
+      <x:c r="J54" s="17"/>
+      <x:c r="K54" s="17"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B44" s="20" t="str">
+      <x:c r="B55" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C44" s="20" t="str">
+      <x:c r="C55" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D44" s="20" t="str">
+      <x:c r="D55" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E44" s="20" t="str">
+      <x:c r="E55" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F44" s="20" t="str">
+      <x:c r="F55" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G44" s="20" t="str">
+      <x:c r="G55" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H44" s="20" t="str">
+      <x:c r="H55" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I44" s="20" t="str">
+      <x:c r="I55" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J44" s="20" t="str">
+      <x:c r="J55" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K44" s="20" t="str">
+      <x:c r="K55" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="22" t="n">
+    <x:row r="56">
+      <x:c r="A56" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B45" s="22" t="str">
+      <x:c r="B56" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C45" s="23" t="n">
-        <x:v>4602</x:v>
-      </x:c>
-      <x:c r="D45" s="23" t="n">
-        <x:v>4617.8</x:v>
-      </x:c>
-      <x:c r="E45" s="23" t="n">
-        <x:v>4497.6</x:v>
-      </x:c>
-      <x:c r="F45" s="23" t="n">
-        <x:v>4537.4</x:v>
-      </x:c>
-      <x:c r="G45" s="23"/>
-      <x:c r="H45" s="24"/>
-      <x:c r="I45" s="26" t="n">
-        <x:f>ROUND(D45-E45,1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J45" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K45" s="22" t="n">
+      <x:c r="C56" s="23" t="n">
+        <x:v>2913</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="n">
+        <x:v>2949.4</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="n">
+        <x:v>2881.4</x:v>
+      </x:c>
+      <x:c r="F56" s="23" t="n">
+        <x:v>2915.8</x:v>
+      </x:c>
+      <x:c r="G56" s="23"/>
+      <x:c r="H56" s="24"/>
+      <x:c r="I56" s="26" t="n">
+        <x:f>ROUND(D56-E56,1)</x:f>
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="J56" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K56" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="22" t="n">
+    <x:row r="57">
+      <x:c r="A57" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B46" s="22" t="str">
+      <x:c r="B57" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C46" s="23" t="n">
-        <x:v>4562</x:v>
-      </x:c>
-      <x:c r="D46" s="23" t="n">
-        <x:v>4584</x:v>
-      </x:c>
-      <x:c r="E46" s="23" t="n">
-        <x:v>4451.6</x:v>
-      </x:c>
-      <x:c r="F46" s="23" t="n">
-        <x:v>4503.4</x:v>
-      </x:c>
-      <x:c r="G46" s="23" t="n">
-        <x:f>ROUND(F46-F45,1)</x:f>
-        <x:v>-34</x:v>
-      </x:c>
-      <x:c r="H46" s="24" t="n">
-        <x:f>IFERROR(F46/F45-1,"")</x:f>
-        <x:v>-0.007493278088773314</x:v>
-      </x:c>
-      <x:c r="I46" s="26" t="n">
-        <x:f>ROUND(D46-E46,1)</x:f>
-        <x:v>132.4</x:v>
-      </x:c>
-      <x:c r="J46" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K46" s="22" t="n">
+      <x:c r="C57" s="23" t="n">
+        <x:v>2923.2</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="n">
+        <x:v>2931.4</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="n">
+        <x:v>2836.8</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="n">
+        <x:v>2867</x:v>
+      </x:c>
+      <x:c r="G57" s="23" t="n">
+        <x:f>ROUND(F57-F56,1)</x:f>
+        <x:v>-48.8</x:v>
+      </x:c>
+      <x:c r="H57" s="24" t="n">
+        <x:f>IFERROR(F57/F56-1,"")</x:f>
+        <x:v>-0.01673640167364021</x:v>
+      </x:c>
+      <x:c r="I57" s="26" t="n">
+        <x:f>ROUND(D57-E57,1)</x:f>
+        <x:v>94.6</x:v>
+      </x:c>
+      <x:c r="J57" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K57" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
+    <x:row r="58">
+      <x:c r="A58" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>4468</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>4500.6</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>4412.2</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>4460.2</x:v>
-      </x:c>
-      <x:c r="G47" s="23" t="n">
-        <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>-43.2</x:v>
-      </x:c>
-      <x:c r="H47" s="24" t="n">
-        <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>-0.0095927521428254</x:v>
-      </x:c>
-      <x:c r="I47" s="23" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>88.4</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
+      <x:c r="B58" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C58" s="23" t="n">
+        <x:v>2849.2</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="n">
+        <x:v>2873.2</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="n">
+        <x:v>2829.4</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="n">
+        <x:v>2862.2</x:v>
+      </x:c>
+      <x:c r="G58" s="23" t="n">
+        <x:f>ROUND(F58-F57,1)</x:f>
+        <x:v>-4.8</x:v>
+      </x:c>
+      <x:c r="H58" s="24" t="n">
+        <x:f>IFERROR(F58/F57-1,"")</x:f>
+        <x:v>-0.0016742239274503135</x:v>
+      </x:c>
+      <x:c r="I58" s="23" t="n">
+        <x:f>ROUND(D58-E58,1)</x:f>
+        <x:v>43.8</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K58" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B59" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C59" s="30"/>
+      <x:c r="D59" s="30"/>
+      <x:c r="E59" s="30"/>
+      <x:c r="F59" s="30"/>
+      <x:c r="G59" s="30"/>
+      <x:c r="H59" s="30"/>
+      <x:c r="I59" s="32" t="n">
+        <x:f>ROUND(SUM(I56:I58),1)</x:f>
+        <x:v>206.4</x:v>
+      </x:c>
+      <x:c r="J59" s="30"/>
+      <x:c r="K59" s="30"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B60" s="30"/>
+      <x:c r="C60" s="30"/>
+      <x:c r="D60" s="30"/>
+      <x:c r="E60" s="30"/>
+      <x:c r="F60" s="30"/>
+      <x:c r="G60" s="30"/>
+      <x:c r="H60" s="30"/>
+      <x:c r="I60" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I56:I58),0),1)</x:f>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="J60" s="30"/>
+      <x:c r="K60" s="30"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="17" t="str">
+        <x:v>碳酸锂2610</x:v>
+      </x:c>
+      <x:c r="B62" s="17"/>
+      <x:c r="C62" s="17"/>
+      <x:c r="D62" s="17"/>
+      <x:c r="E62" s="17"/>
+      <x:c r="F62" s="17"/>
+      <x:c r="G62" s="17"/>
+      <x:c r="H62" s="17"/>
+      <x:c r="I62" s="17"/>
+      <x:c r="J62" s="17"/>
+      <x:c r="K62" s="17"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B63" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C63" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D63" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E63" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F63" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G63" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H63" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I63" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J63" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K63" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B64" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C64" s="23" t="n">
+        <x:v>159280</x:v>
+      </x:c>
+      <x:c r="D64" s="23" t="n">
+        <x:v>161280</x:v>
+      </x:c>
+      <x:c r="E64" s="23" t="n">
+        <x:v>140220</x:v>
+      </x:c>
+      <x:c r="F64" s="23" t="n">
+        <x:v>142000</x:v>
+      </x:c>
+      <x:c r="G64" s="23"/>
+      <x:c r="H64" s="24"/>
+      <x:c r="I64" s="26" t="n">
+        <x:f>ROUND(D64-E64,1)</x:f>
+        <x:v>21060</x:v>
+      </x:c>
+      <x:c r="J64" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K64" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="31" t="str">
+    <x:row r="65">
+      <x:c r="A65" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B65" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C65" s="23" t="n">
+        <x:v>141000</x:v>
+      </x:c>
+      <x:c r="D65" s="23" t="n">
+        <x:v>143540</x:v>
+      </x:c>
+      <x:c r="E65" s="23" t="n">
+        <x:v>127120</x:v>
+      </x:c>
+      <x:c r="F65" s="23" t="n">
+        <x:v>134340</x:v>
+      </x:c>
+      <x:c r="G65" s="28" t="n">
+        <x:f>ROUND(F65-F64,1)</x:f>
+        <x:v>-7660</x:v>
+      </x:c>
+      <x:c r="H65" s="24" t="n">
+        <x:f>IFERROR(F65/F64-1,"")</x:f>
+        <x:v>-0.05394366197183098</x:v>
+      </x:c>
+      <x:c r="I65" s="26" t="n">
+        <x:f>ROUND(D65-E65,1)</x:f>
+        <x:v>16420</x:v>
+      </x:c>
+      <x:c r="J65" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K65" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B66" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C66" s="23" t="n">
+        <x:v>133600</x:v>
+      </x:c>
+      <x:c r="D66" s="23" t="n">
+        <x:v>135900</x:v>
+      </x:c>
+      <x:c r="E66" s="23" t="n">
+        <x:v>126200</x:v>
+      </x:c>
+      <x:c r="F66" s="23" t="n">
+        <x:v>128580</x:v>
+      </x:c>
+      <x:c r="G66" s="28" t="n">
+        <x:f>ROUND(F66-F65,1)</x:f>
+        <x:v>-5760</x:v>
+      </x:c>
+      <x:c r="H66" s="24" t="n">
+        <x:f>IFERROR(F66/F65-1,"")</x:f>
+        <x:v>-0.04287628405538191</x:v>
+      </x:c>
+      <x:c r="I66" s="26" t="n">
+        <x:f>ROUND(D66-E66,1)</x:f>
+        <x:v>9700</x:v>
+      </x:c>
+      <x:c r="J66" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K66" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B67" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="C67" s="23" t="n">
+        <x:v>128500</x:v>
+      </x:c>
+      <x:c r="D67" s="23" t="n">
+        <x:v>134800</x:v>
+      </x:c>
+      <x:c r="E67" s="23" t="n">
+        <x:v>127100</x:v>
+      </x:c>
+      <x:c r="F67" s="23" t="n">
+        <x:v>133500</x:v>
+      </x:c>
+      <x:c r="G67" s="28" t="n">
+        <x:f>ROUND(F67-F66,1)</x:f>
+        <x:v>4920</x:v>
+      </x:c>
+      <x:c r="H67" s="24" t="n">
+        <x:f>IFERROR(F67/F66-1,"")</x:f>
+        <x:v>0.038264115725618275</x:v>
+      </x:c>
+      <x:c r="I67" s="26" t="n">
+        <x:f>ROUND(D67-E67,1)</x:f>
+        <x:v>7700</x:v>
+      </x:c>
+      <x:c r="J67" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K67" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C48" s="30"/>
-      <x:c r="D48" s="30"/>
-      <x:c r="E48" s="30"/>
-      <x:c r="F48" s="30"/>
-      <x:c r="G48" s="30"/>
-      <x:c r="H48" s="30"/>
-      <x:c r="I48" s="32" t="n">
-        <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="J48" s="30"/>
-      <x:c r="K48" s="30"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="31" t="str">
+      <x:c r="B68" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C68" s="30"/>
+      <x:c r="D68" s="30"/>
+      <x:c r="E68" s="30"/>
+      <x:c r="F68" s="30"/>
+      <x:c r="G68" s="30"/>
+      <x:c r="H68" s="30"/>
+      <x:c r="I68" s="32" t="n">
+        <x:f>ROUND(SUM(I64:I67),1)</x:f>
+        <x:v>54880</x:v>
+      </x:c>
+      <x:c r="J68" s="30"/>
+      <x:c r="K68" s="30"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="30"/>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>113.7</x:v>
-      </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B51" s="17"/>
-      <x:c r="C51" s="17"/>
-      <x:c r="D51" s="17"/>
-      <x:c r="E51" s="17"/>
-      <x:c r="F51" s="17"/>
-      <x:c r="G51" s="17"/>
-      <x:c r="H51" s="17"/>
-      <x:c r="I51" s="17"/>
-      <x:c r="J51" s="17"/>
-      <x:c r="K51" s="17"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B52" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C52" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D52" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E52" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F52" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G52" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H52" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I52" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J52" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K52" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B53" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C53" s="23" t="n">
-        <x:v>2913</x:v>
-      </x:c>
-      <x:c r="D53" s="23" t="n">
-        <x:v>2949.4</x:v>
-      </x:c>
-      <x:c r="E53" s="23" t="n">
-        <x:v>2881.4</x:v>
-      </x:c>
-      <x:c r="F53" s="23" t="n">
-        <x:v>2915.8</x:v>
-      </x:c>
-      <x:c r="G53" s="23"/>
-      <x:c r="H53" s="24"/>
-      <x:c r="I53" s="26" t="n">
-        <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="J53" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K53" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>2923.2</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>2931.4</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>2836.8</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>2867</x:v>
-      </x:c>
-      <x:c r="G54" s="23" t="n">
-        <x:f>ROUND(F54-F53,1)</x:f>
-        <x:v>-48.8</x:v>
-      </x:c>
-      <x:c r="H54" s="24" t="n">
-        <x:f>IFERROR(F54/F53-1,"")</x:f>
-        <x:v>-0.01673640167364021</x:v>
-      </x:c>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>94.6</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>2849.2</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>2873.2</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>2829.4</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>2845.8</x:v>
-      </x:c>
-      <x:c r="G55" s="23" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-21.2</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.007394489012905403</x:v>
-      </x:c>
-      <x:c r="I55" s="23" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
-        <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>206.4</x:v>
-      </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>68.8</x:v>
-      </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="17" t="str">
-        <x:v>碳酸锂2610</x:v>
-      </x:c>
-      <x:c r="B59" s="17"/>
-      <x:c r="C59" s="17"/>
-      <x:c r="D59" s="17"/>
-      <x:c r="E59" s="17"/>
-      <x:c r="F59" s="17"/>
-      <x:c r="G59" s="17"/>
-      <x:c r="H59" s="17"/>
-      <x:c r="I59" s="17"/>
-      <x:c r="J59" s="17"/>
-      <x:c r="K59" s="17"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B60" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C60" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D60" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E60" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F60" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G60" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H60" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I60" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J60" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K60" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B61" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C61" s="23" t="n">
-        <x:v>159280</x:v>
-      </x:c>
-      <x:c r="D61" s="23" t="n">
-        <x:v>161280</x:v>
-      </x:c>
-      <x:c r="E61" s="23" t="n">
-        <x:v>140220</x:v>
-      </x:c>
-      <x:c r="F61" s="23" t="n">
-        <x:v>142000</x:v>
-      </x:c>
-      <x:c r="G61" s="23"/>
-      <x:c r="H61" s="24"/>
-      <x:c r="I61" s="26" t="n">
-        <x:f>ROUND(D61-E61,1)</x:f>
-        <x:v>21060</x:v>
-      </x:c>
-      <x:c r="J61" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K61" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B62" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C62" s="23" t="n">
-        <x:v>141000</x:v>
-      </x:c>
-      <x:c r="D62" s="23" t="n">
-        <x:v>143540</x:v>
-      </x:c>
-      <x:c r="E62" s="23" t="n">
-        <x:v>127120</x:v>
-      </x:c>
-      <x:c r="F62" s="23" t="n">
-        <x:v>134340</x:v>
-      </x:c>
-      <x:c r="G62" s="28" t="n">
-        <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>-7660</x:v>
-      </x:c>
-      <x:c r="H62" s="24" t="n">
-        <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>-0.05394366197183098</x:v>
-      </x:c>
-      <x:c r="I62" s="26" t="n">
-        <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>16420</x:v>
-      </x:c>
-      <x:c r="J62" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K62" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B63" s="22" t="str">
-        <x:v>9月14日-9月17日</x:v>
-      </x:c>
-      <x:c r="C63" s="23" t="n">
-        <x:v>133600</x:v>
-      </x:c>
-      <x:c r="D63" s="23" t="n">
-        <x:v>134840</x:v>
-      </x:c>
-      <x:c r="E63" s="23" t="n">
-        <x:v>126200</x:v>
-      </x:c>
-      <x:c r="F63" s="23" t="n">
-        <x:v>132280</x:v>
-      </x:c>
-      <x:c r="G63" s="28" t="n">
-        <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-2060</x:v>
-      </x:c>
-      <x:c r="H63" s="24" t="n">
-        <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.015334226589251099</x:v>
-      </x:c>
-      <x:c r="I63" s="26" t="n">
-        <x:f>ROUND(D63-E63,1)</x:f>
-        <x:v>8640</x:v>
-      </x:c>
-      <x:c r="J63" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K63" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B64" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="32" t="n">
-        <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>46120</x:v>
-      </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B65" s="30"/>
-      <x:c r="C65" s="30"/>
-      <x:c r="D65" s="30"/>
-      <x:c r="E65" s="30"/>
-      <x:c r="F65" s="30"/>
-      <x:c r="G65" s="30"/>
-      <x:c r="H65" s="30"/>
-      <x:c r="I65" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
-        <x:v>15373.3</x:v>
-      </x:c>
-      <x:c r="J65" s="30"/>
-      <x:c r="K65" s="30"/>
+      <x:c r="B69" s="30"/>
+      <x:c r="C69" s="30"/>
+      <x:c r="D69" s="30"/>
+      <x:c r="E69" s="30"/>
+      <x:c r="F69" s="30"/>
+      <x:c r="G69" s="30"/>
+      <x:c r="H69" s="30"/>
+      <x:c r="I69" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I64:I67),0),1)</x:f>
+        <x:v>13720</x:v>
+      </x:c>
+      <x:c r="J69" s="30"/>
+      <x:c r="K69" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A11:K11"/>
-    <x:mergeCell ref="A19:K19"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A35:K35"/>
-    <x:mergeCell ref="A43:K43"/>
-    <x:mergeCell ref="A51:K51"/>
-    <x:mergeCell ref="A59:K59"/>
+    <x:mergeCell ref="A12:K12"/>
+    <x:mergeCell ref="A21:K21"/>
+    <x:mergeCell ref="A30:K30"/>
+    <x:mergeCell ref="A38:K38"/>
+    <x:mergeCell ref="A46:K46"/>
+    <x:mergeCell ref="A54:K54"/>
+    <x:mergeCell ref="A62:K62"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3613,31 +3843,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>1900.6</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>7723.68</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>7777.91</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>7723.68</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>7766.33</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="n">
+        <x:v>78.7</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.01024248171403519</x:v>
+      </x:c>
+      <x:c r="J18" s="23" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>54.2</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -3645,11 +3893,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>135.8</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>1954.8</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>130.3</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4220,31 +4486,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>1727.2999999999997</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>7829.82</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>7869.35</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>7809.59</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>7850.48</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="n">
+        <x:v>50.9</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.0065221209778436595</x:v>
+      </x:c>
+      <x:c r="J18" s="23" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -4252,11 +4536,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>123.4</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>1787.0999999999997</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>119.1</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4827,31 +5129,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>496.49999999999994</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>9月21日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>3920.27</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>3950.94</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>3918.13</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>3949.91</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.009724249527719442</x:v>
+      </x:c>
+      <x:c r="J18" s="23" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -4859,11 +5179,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>35.5</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>529.3</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>35.3</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6612,31 +6950,49 @@
         <x:v>IF2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>697.3999999999999</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>4486</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>4520.6</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>4481</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>4508</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>47.8</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.010717008205910039</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -6644,11 +7000,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>53.6</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>736.9999999999999</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>52.6</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7183,31 +7557,49 @@
         <x:v>IH2609</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="41" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>9月18日</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="n">
+        <x:v>2856.4</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="n">
+        <x:v>2870.8</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="n">
+        <x:v>2853.4</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="n">
+        <x:v>2862.2</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="n">
+        <x:v>16.4</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="n">
+        <x:v>0.0057628786281536115</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>17.4</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -7215,11 +7607,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>31.9</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>432.4</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>30.9</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-22
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R9a3c3f1d677e4f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rd1cc03d6886d4424"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9bf5d91f434f4119"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rd7fffb31a6b748b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re165c48dff9548c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R31fe2982e1504c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Radc10241dd2543af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb9b29311feea4aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R72694fe6b8a94b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rabf1671d1f7644a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Re117c37c08d94898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8521a711c6cb4803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf911a28356a04619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re99c05918f7f4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf388897026fe46c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R42b44684c68844d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R3578579d14524bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rc973f1b08f0447c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rd3fa9ec1aa0f42f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf3042c11e16646c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7777.91</x:v>
+        <x:v>7852.23</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7723.68</x:v>
+        <x:v>7734.35</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>54.2</x:v>
+        <x:v>117.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1954.8</x:v>
+        <x:v>2072.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>130.3</x:v>
+        <x:v>129.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7869.35</x:v>
+        <x:v>7922.62</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7809.59</x:v>
+        <x:v>7808.98</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>59.8</x:v>
+        <x:v>113.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1787.1</x:v>
+        <x:v>1900.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>119.1</x:v>
+        <x:v>118.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3950.94</x:v>
+        <x:v>3967.68</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3918.13</x:v>
+        <x:v>3945.42</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>32.8</x:v>
+        <x:v>22.3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>529.3</x:v>
+        <x:v>551.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.3</x:v>
+        <x:v>34.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7599</x:v>
+        <x:v>7687</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7527</x:v>
+        <x:v>7563</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>72</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2192.2</x:v>
+        <x:v>2316.2</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>146.1</x:v>
+        <x:v>144.8</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>134800</x:v>
+        <x:v>136560</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>127100</x:v>
+        <x:v>131400</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>7700</x:v>
+        <x:v>5160</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>89880</x:v>
+        <x:v>95040</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5992</x:v>
+        <x:v>5940</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1478,31 +1478,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>89880</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>9月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>133040</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>136560</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>131400</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>135480</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="n">
+        <x:v>1980</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>0.014831460674157304</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>5160</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -1510,11 +1528,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>5992</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>95040</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>5940</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1709,37 +1745,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>9月21日</x:v>
+        <x:v>9月21日-9月22日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7723.68</x:v>
       </x:c>
       <x:c r="D8" s="23" t="n">
-        <x:v>7777.91</x:v>
+        <x:v>7852.23</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
         <x:v>7723.68</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7766.33</x:v>
+        <x:v>7759.03</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>78.7</x:v>
+        <x:v>71.4</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>0.01024248171403519</x:v>
+        <x:v>0.009292899335162197</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>54.2</x:v>
+        <x:v>128.5</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1757,7 +1793,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1180</x:v>
+        <x:v>1254.3</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1775,7 +1811,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>295</x:v>
+        <x:v>313.6</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -1943,37 +1979,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月21日</x:v>
+        <x:v>9月21日-9月22日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7829.82</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>7869.35</x:v>
+        <x:v>7922.62</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7809.59</x:v>
+        <x:v>7808.98</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7850.48</x:v>
+        <x:v>7828.94</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>50.9</x:v>
+        <x:v>29.3</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>0.0065221209778436595</x:v>
+        <x:v>0.0037604444324779163</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>59.8</x:v>
+        <x:v>113.6</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1991,7 +2027,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1116.3</x:v>
+        <x:v>1170.1</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2009,7 +2045,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>279.1</x:v>
+        <x:v>292.5</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2177,37 +2213,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>9月21日</x:v>
+        <x:v>9月21日-9月22日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3920.27</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3950.94</x:v>
+        <x:v>3967.68</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
         <x:v>3918.13</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3949.91</x:v>
+        <x:v>3952.13</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>38</x:v>
+        <x:v>40.3</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.009724249527719442</x:v>
+        <x:v>0.010291753049053387</x:v>
       </x:c>
       <x:c r="I26" s="23" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>32.8</x:v>
+        <x:v>49.5</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2225,7 +2261,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>295.9</x:v>
+        <x:v>312.6</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2243,7 +2279,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>74</x:v>
+        <x:v>78.2</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2411,37 +2447,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>9月21日</x:v>
+        <x:v>9月21日-9月22日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>7549</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>7599</x:v>
+        <x:v>7687</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
         <x:v>7527</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>7560.6</x:v>
+        <x:v>7580.2</x:v>
       </x:c>
       <x:c r="G35" s="23" t="n">
         <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>-118.6</x:v>
+        <x:v>-99</x:v>
       </x:c>
       <x:c r="H35" s="24" t="n">
         <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>-0.01544431711636618</x:v>
+        <x:v>-0.012891967913324254</x:v>
       </x:c>
       <x:c r="I35" s="23" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>72</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2459,7 +2495,7 @@
       <x:c r="H36" s="30"/>
       <x:c r="I36" s="32" t="n">
         <x:f>ROUND(SUM(I32:I35),1)</x:f>
-        <x:v>1245.2</x:v>
+        <x:v>1333.2</x:v>
       </x:c>
       <x:c r="J36" s="30"/>
       <x:c r="K36" s="30"/>
@@ -2477,7 +2513,7 @@
       <x:c r="H37" s="30"/>
       <x:c r="I37" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I32:I35),0),1)</x:f>
-        <x:v>311.3</x:v>
+        <x:v>333.3</x:v>
       </x:c>
       <x:c r="J37" s="30"/>
       <x:c r="K37" s="30"/>
@@ -3347,37 +3383,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>9月21日</x:v>
+        <x:v>9月21日-9月22日</x:v>
       </x:c>
       <x:c r="C71" s="23" t="n">
         <x:v>128500</x:v>
       </x:c>
       <x:c r="D71" s="23" t="n">
-        <x:v>134800</x:v>
+        <x:v>136560</x:v>
       </x:c>
       <x:c r="E71" s="23" t="n">
         <x:v>127100</x:v>
       </x:c>
       <x:c r="F71" s="23" t="n">
-        <x:v>133500</x:v>
+        <x:v>135480</x:v>
       </x:c>
       <x:c r="G71" s="28" t="n">
         <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>4920</x:v>
+        <x:v>6900</x:v>
       </x:c>
       <x:c r="H71" s="24" t="n">
         <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>0.038264115725618275</x:v>
+        <x:v>0.05366308912739148</x:v>
       </x:c>
       <x:c r="I71" s="26" t="n">
         <x:f>ROUND(D71-E71,1)</x:f>
-        <x:v>7700</x:v>
+        <x:v>9460</x:v>
       </x:c>
       <x:c r="J71" s="22" t="str">
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K71" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3395,7 +3431,7 @@
       <x:c r="H72" s="30"/>
       <x:c r="I72" s="32" t="n">
         <x:f>ROUND(SUM(I68:I71),1)</x:f>
-        <x:v>54880</x:v>
+        <x:v>56640</x:v>
       </x:c>
       <x:c r="J72" s="30"/>
       <x:c r="K72" s="30"/>
@@ -3413,7 +3449,7 @@
       <x:c r="H73" s="30"/>
       <x:c r="I73" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I68:I71),0),1)</x:f>
-        <x:v>13720</x:v>
+        <x:v>14160</x:v>
       </x:c>
       <x:c r="J73" s="30"/>
       <x:c r="K73" s="30"/>
@@ -4031,31 +4067,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>1954.8</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>9月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7819.62</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7852.23</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7734.35</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7759.03</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-7.3</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.0009399549079166514</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>117.9</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -4063,11 +4117,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>130.3</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>2072.7</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>129.5</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4674,31 +4746,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>1787.0999999999997</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>9月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7911.64</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7922.62</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7808.98</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7828.94</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-21.5</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.002743781271973167</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>113.6</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -4706,11 +4796,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>119.1</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>1900.6999999999996</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>118.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5317,31 +5425,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>529.3</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>9月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3963.81</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3967.68</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3945.42</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>3952.13</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>0.0005620381223876425</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>22.3</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -5349,11 +5475,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>35.3</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>551.5999999999999</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>34.5</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5960,31 +6104,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>2192.2</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>9月22日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7638.2</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7687</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7563</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>7580.2</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>19.6</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>0.002592386847604544</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -5992,11 +6154,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>146.1</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>2316.2</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>144.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-23
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc324215572de48c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R84c00860ce8643ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R42216eee8d894e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R7af804bae13945a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R328fe406866b4b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rf70a446e2fde41ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5d99927c4b9e4016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R0517e1a6d5c34ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R131fef15569e4d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rc0f98bfd20104498"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc7ca47cf28d24e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rbf42fea0385f418d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Redfc00dbcaf74d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Re3026e2984134efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf4eb5e71301f478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Ra5472b5c5a794595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R171e029cf16a455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R67e57d09bc734e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R11d64c6663694b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rfedbe1af1c5e465f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7852.23</x:v>
+        <x:v>7769.96</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7734.35</x:v>
+        <x:v>7730.37</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>117.9</x:v>
+        <x:v>39.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2072.7</x:v>
+        <x:v>2112.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>129.5</x:v>
+        <x:v>124.3</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7922.62</x:v>
+        <x:v>7839.94</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7808.98</x:v>
+        <x:v>7781.31</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>113.6</x:v>
+        <x:v>58.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1900.7</x:v>
+        <x:v>1959.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>118.8</x:v>
+        <x:v>115.3</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3967.68</x:v>
+        <x:v>3951.52</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3945.42</x:v>
+        <x:v>3934.46</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>22.3</x:v>
+        <x:v>17.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>551.6</x:v>
+        <x:v>568.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>34.5</x:v>
+        <x:v>33.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7687</x:v>
+        <x:v>7614.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7563</x:v>
+        <x:v>7572.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>124</x:v>
+        <x:v>42.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2316.2</x:v>
+        <x:v>2358.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>144.8</x:v>
+        <x:v>138.7</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4520</x:v>
+        <x:v>4490.4</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4477.6</x:v>
+        <x:v>4457.2</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>42.4</x:v>
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>819.2</x:v>
+        <x:v>852.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>51.2</x:v>
+        <x:v>50.1</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>136560</x:v>
+        <x:v>136000</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>131400</x:v>
+        <x:v>129360</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>5160</x:v>
+        <x:v>6640</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>95040</x:v>
+        <x:v>101680</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5940</x:v>
+        <x:v>5981.2</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1514,31 +1514,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>95040</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>136000</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>136000</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>129360</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>129840</x:v>
+      </x:c>
+      <x:c r="H20" s="28" t="n">
+        <x:v>-5640</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.041629760850310005</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>6640</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -1546,11 +1564,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>5940</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>101680</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>5981.2</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1745,7 +1781,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7723.68</x:v>
@@ -1757,15 +1793,15 @@
         <x:v>7723.68</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7759.03</x:v>
+        <x:v>7745.56</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>71.4</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>0.009292899335162197</x:v>
+        <x:v>0.007540724726474712</x:v>
       </x:c>
       <x:c r="I8" s="23" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
@@ -1775,7 +1811,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1979,7 +2015,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7829.82</x:v>
@@ -1988,28 +2024,28 @@
         <x:v>7922.62</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7808.98</x:v>
+        <x:v>7781.31</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7828.94</x:v>
+        <x:v>7791.82</x:v>
       </x:c>
       <x:c r="G17" s="23" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>29.3</x:v>
+        <x:v>-7.8</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>0.0037604444324779163</x:v>
+        <x:v>-0.000998767887112284</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>113.6</x:v>
+        <x:v>141.3</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2027,7 +2063,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1170.1</x:v>
+        <x:v>1197.8</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2045,7 +2081,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>292.5</x:v>
+        <x:v>299.5</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2213,7 +2249,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3920.27</x:v>
@@ -2225,15 +2261,15 @@
         <x:v>3918.13</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3952.13</x:v>
+        <x:v>3936.52</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>40.3</x:v>
+        <x:v>24.7</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.010291753049053387</x:v>
+        <x:v>0.006301334144539483</x:v>
       </x:c>
       <x:c r="I26" s="23" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
@@ -2243,7 +2279,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2447,7 +2483,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>7549</x:v>
@@ -2459,15 +2495,15 @@
         <x:v>7527</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>7580.2</x:v>
+        <x:v>7578</x:v>
       </x:c>
       <x:c r="G35" s="23" t="n">
         <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>-99</x:v>
+        <x:v>-101.2</x:v>
       </x:c>
       <x:c r="H35" s="24" t="n">
         <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>-0.012891967913324254</x:v>
+        <x:v>-0.013178456089175894</x:v>
       </x:c>
       <x:c r="I35" s="23" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
@@ -2477,7 +2513,7 @@
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2915,7 +2951,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C53" s="23" t="n">
         <x:v>4451</x:v>
@@ -2927,15 +2963,15 @@
         <x:v>4434.8</x:v>
       </x:c>
       <x:c r="F53" s="23" t="n">
-        <x:v>4480.6</x:v>
+        <x:v>4461.8</x:v>
       </x:c>
       <x:c r="G53" s="23" t="n">
         <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>-27.4</x:v>
+        <x:v>-46.2</x:v>
       </x:c>
       <x:c r="H53" s="24" t="n">
         <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>-0.006078083407275892</x:v>
+        <x:v>-0.010248447204968869</x:v>
       </x:c>
       <x:c r="I53" s="23" t="n">
         <x:f>ROUND(D53-E53,1)</x:f>
@@ -2945,7 +2981,7 @@
         <x:v>IF2612</x:v>
       </x:c>
       <x:c r="K53" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3383,7 +3419,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>9月21日-9月22日</x:v>
+        <x:v>9月21日-9月23日</x:v>
       </x:c>
       <x:c r="C71" s="23" t="n">
         <x:v>128500</x:v>
@@ -3395,15 +3431,15 @@
         <x:v>127100</x:v>
       </x:c>
       <x:c r="F71" s="23" t="n">
-        <x:v>135480</x:v>
+        <x:v>129840</x:v>
       </x:c>
       <x:c r="G71" s="28" t="n">
         <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>6900</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="H71" s="24" t="n">
         <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>0.05366308912739148</x:v>
+        <x:v>0.009799346710219314</x:v>
       </x:c>
       <x:c r="I71" s="26" t="n">
         <x:f>ROUND(D71-E71,1)</x:f>
@@ -3413,7 +3449,7 @@
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K71" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -4103,31 +4139,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>2072.7</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>7762.68</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>7769.96</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>7730.37</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>7745.56</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-13.5</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.0017360417474864276</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -4135,11 +4189,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>129.5</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>2112.2999999999997</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>124.3</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4782,31 +4854,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>1900.6999999999996</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>7839.94</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>7839.94</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>7781.31</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>7791.82</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-37.1</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.004741382613738243</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>58.6</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -4814,11 +4904,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>118.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>1959.2999999999995</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>115.3</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5461,31 +5569,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>551.5999999999999</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3951.37</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3951.52</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3934.46</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>3936.52</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-15.6</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.003949768858817926</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>17.1</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -5493,11 +5619,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>34.5</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>568.6999999999999</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>33.5</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6140,31 +6284,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>2316.2</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>7600</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>7614.8</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>7572.6</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>7578</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-2.2</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.0002902298092398725</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>42.2</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -6172,11 +6334,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>144.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>2358.3999999999996</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>138.7</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7498,31 +7678,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>819.1999999999998</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>9月23日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>4485</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>4490.4</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>4457.2</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>4461.8</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-18.8</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.004195866625005595</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -7530,11 +7728,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>51.2</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>852.3999999999999</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>50.1</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-24
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R0c55504763c74278"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R214d132e2605479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6fa300e81a8243d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb9731b97c3514825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc88d8f9769b44cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R3e12dd5784a840e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R986b28b5a1a94b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rbd53ef98571c44bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R8b6734410ab1428f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R785e25bfe5924a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc7733053ed344f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rc2c0a34a8b7b492f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R0460f1f8b767455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4cc03ea0ad084d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R2e20f92ca562404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rbb65aa29c76a4d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc7c748cd77ef4d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R61a6d9d59e604a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R773e5e189b9449c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R15d8a482c35d4183"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7769.96</x:v>
+        <x:v>7725.52</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7730.37</x:v>
+        <x:v>7569.51</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>39.6</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2112.3</x:v>
+        <x:v>2268.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>124.3</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7839.94</x:v>
+        <x:v>7774.22</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7781.31</x:v>
+        <x:v>7624.07</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>58.6</x:v>
+        <x:v>150.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1959.3</x:v>
+        <x:v>2109.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>115.3</x:v>
+        <x:v>117.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3951.52</x:v>
+        <x:v>3930.5</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3934.46</x:v>
+        <x:v>3888.37</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>17.1</x:v>
+        <x:v>42.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>568.7</x:v>
+        <x:v>610.8</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>33.5</x:v>
+        <x:v>33.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2875.6</x:v>
+        <x:v>2850</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2855.2</x:v>
+        <x:v>2798</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>20.4</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>502</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>29.5</x:v>
+        <x:v>30.8</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>136000</x:v>
+        <x:v>131640</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>129360</x:v>
+        <x:v>125000</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
         <x:v>6640</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>101680</x:v>
+        <x:v>108320</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5981.2</x:v>
+        <x:v>6017.8</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-23</x:v>
+        <x:v>2026-09-24</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1550,31 +1550,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>101680</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>9月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>131640</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>131640</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>125980</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="n">
+        <x:v>-3860</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>-0.029728897104128182</x:v>
+      </x:c>
+      <x:c r="J21" s="26" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>6640</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -1582,11 +1600,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>5981.2</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>108320</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>6017.8</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1781,7 +1817,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>9月21日-9月23日</x:v>
+        <x:v>9月21日-9月24日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>7723.68</x:v>
@@ -1790,28 +1826,28 @@
         <x:v>7852.23</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>7723.68</x:v>
+        <x:v>7569.51</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>7745.56</x:v>
+        <x:v>7570.14</x:v>
       </x:c>
       <x:c r="G8" s="23" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>58</x:v>
+        <x:v>-117.4</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>0.007540724726474712</x:v>
-      </x:c>
-      <x:c r="I8" s="23" t="n">
+        <x:v>-0.015277869917620479</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>128.5</x:v>
+        <x:v>282.7</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1829,7 +1865,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1254.3</x:v>
+        <x:v>1408.5</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1847,7 +1883,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>313.6</x:v>
+        <x:v>352.1</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -2015,7 +2051,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月21日-9月23日</x:v>
+        <x:v>9月21日-9月24日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>7829.82</x:v>
@@ -2024,28 +2060,28 @@
         <x:v>7922.62</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7781.31</x:v>
+        <x:v>7624.07</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7791.82</x:v>
-      </x:c>
-      <x:c r="G17" s="23" t="n">
+        <x:v>7624.07</x:v>
+      </x:c>
+      <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-7.8</x:v>
+        <x:v>-175.5</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.000998767887112284</x:v>
-      </x:c>
-      <x:c r="I17" s="23" t="n">
+        <x:v>-0.02250625351780411</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>141.3</x:v>
+        <x:v>298.6</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2063,7 +2099,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1197.8</x:v>
+        <x:v>1355.1</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -2081,7 +2117,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>299.5</x:v>
+        <x:v>338.8</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -2249,7 +2285,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>9月21日-9月23日</x:v>
+        <x:v>9月21日-9月24日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3920.27</x:v>
@@ -2258,28 +2294,28 @@
         <x:v>3967.68</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3918.13</x:v>
+        <x:v>3888.37</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3936.52</x:v>
+        <x:v>3888.37</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>24.7</x:v>
+        <x:v>-23.5</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.006301334144539483</x:v>
-      </x:c>
-      <x:c r="I26" s="23" t="n">
+        <x:v>-0.00600735709519995</x:v>
+      </x:c>
+      <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>49.5</x:v>
+        <x:v>79.3</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2297,7 +2333,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>312.6</x:v>
+        <x:v>342.4</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2315,7 +2351,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>78.2</x:v>
+        <x:v>85.6</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -3185,7 +3221,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>9月21日-9月23日</x:v>
+        <x:v>9月21日-9月24日</x:v>
       </x:c>
       <x:c r="C62" s="23" t="n">
         <x:v>2830</x:v>
@@ -3194,28 +3230,28 @@
         <x:v>2881.2</x:v>
       </x:c>
       <x:c r="E62" s="23" t="n">
-        <x:v>2822</x:v>
+        <x:v>2798</x:v>
       </x:c>
       <x:c r="F62" s="23" t="n">
-        <x:v>2859.4</x:v>
+        <x:v>2804.6</x:v>
       </x:c>
       <x:c r="G62" s="23" t="n">
         <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>-2.8</x:v>
+        <x:v>-57.6</x:v>
       </x:c>
       <x:c r="H62" s="24" t="n">
         <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>-0.000978268464817189</x:v>
-      </x:c>
-      <x:c r="I62" s="23" t="n">
+        <x:v>-0.02012437984766957</x:v>
+      </x:c>
+      <x:c r="I62" s="26" t="n">
         <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>59.2</x:v>
+        <x:v>83.2</x:v>
       </x:c>
       <x:c r="J62" s="22" t="str">
         <x:v>IH2612</x:v>
       </x:c>
       <x:c r="K62" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3233,7 +3269,7 @@
       <x:c r="H63" s="30"/>
       <x:c r="I63" s="32" t="n">
         <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>265.6</x:v>
+        <x:v>289.6</x:v>
       </x:c>
       <x:c r="J63" s="30"/>
       <x:c r="K63" s="30"/>
@@ -3251,7 +3287,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>66.4</x:v>
+        <x:v>72.4</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -3419,7 +3455,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>9月21日-9月23日</x:v>
+        <x:v>9月21日-9月24日</x:v>
       </x:c>
       <x:c r="C71" s="23" t="n">
         <x:v>128500</x:v>
@@ -3428,28 +3464,28 @@
         <x:v>136560</x:v>
       </x:c>
       <x:c r="E71" s="23" t="n">
-        <x:v>127100</x:v>
+        <x:v>125000</x:v>
       </x:c>
       <x:c r="F71" s="23" t="n">
-        <x:v>129840</x:v>
+        <x:v>125980</x:v>
       </x:c>
       <x:c r="G71" s="28" t="n">
         <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>1260</x:v>
+        <x:v>-2600</x:v>
       </x:c>
       <x:c r="H71" s="24" t="n">
         <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>0.009799346710219314</x:v>
+        <x:v>-0.02022087416394458</x:v>
       </x:c>
       <x:c r="I71" s="26" t="n">
         <x:f>ROUND(D71-E71,1)</x:f>
-        <x:v>9460</x:v>
+        <x:v>11560</x:v>
       </x:c>
       <x:c r="J71" s="22" t="str">
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K71" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3467,7 +3503,7 @@
       <x:c r="H72" s="30"/>
       <x:c r="I72" s="32" t="n">
         <x:f>ROUND(SUM(I68:I71),1)</x:f>
-        <x:v>56640</x:v>
+        <x:v>58740</x:v>
       </x:c>
       <x:c r="J72" s="30"/>
       <x:c r="K72" s="30"/>
@@ -3485,7 +3521,7 @@
       <x:c r="H73" s="30"/>
       <x:c r="I73" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I68:I71),0),1)</x:f>
-        <x:v>14160</x:v>
+        <x:v>14685</x:v>
       </x:c>
       <x:c r="J73" s="30"/>
       <x:c r="K73" s="30"/>
@@ -4175,31 +4211,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>2112.2999999999997</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>9月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>7707.87</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>7725.52</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>7569.51</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>7570.14</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="n">
+        <x:v>-175.4</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>-0.022647813715212295</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -4207,11 +4261,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>124.3</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>2268.2999999999997</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4890,31 +4962,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>1959.2999999999995</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>9月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>7763.73</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>7774.22</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>7624.07</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>7624.07</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="n">
+        <x:v>-167.7</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>-0.0215289880926407</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>150.2</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -4922,11 +5012,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>115.3</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>2109.4999999999995</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>117.2</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5605,31 +5713,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>568.6999999999999</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>9月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>3925.32</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>3930.5</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>3888.37</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>3888.37</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>-48.2</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>-0.012231615741822743</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>42.1</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -5637,11 +5763,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>33.5</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>610.8</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8465,31 +8609,49 @@
         <x:v>IH2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B23" s="30" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C23" s="30"/>
-      <x:c r="D23" s="30"/>
-      <x:c r="E23" s="30"/>
-      <x:c r="F23" s="30"/>
-      <x:c r="G23" s="30"/>
-      <x:c r="H23" s="30"/>
-      <x:c r="I23" s="30"/>
-      <x:c r="J23" s="32" t="n">
-        <x:f>SUM(J4:J20)</x:f>
-        <x:v>501.99999999999994</x:v>
-      </x:c>
-      <x:c r="K23" s="30"/>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>9月24日</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>2838</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>2850</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>2798</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="n">
+        <x:v>2804.6</x:v>
+      </x:c>
+      <x:c r="H21" s="23" t="n">
+        <x:v>-54.8</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="n">
+        <x:v>-0.019164859760789077</x:v>
+      </x:c>
+      <x:c r="J21" s="23" t="n">
+        <x:f>ROUND(E21-F21,1)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B24" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C24" s="30"/>
       <x:c r="D24" s="30"/>
       <x:c r="E24" s="30"/>
@@ -8497,11 +8659,29 @@
       <x:c r="G24" s="30"/>
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="30"/>
-      <x:c r="J24" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
-        <x:v>29.5</x:v>
+      <x:c r="J24" s="32" t="n">
+        <x:f>SUM(J4:J21)</x:f>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="30"/>
+      <x:c r="J25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
+        <x:v>30.8</x:v>
+      </x:c>
+      <x:c r="K25" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-25
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R798ac79c3045459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1e32235e70044422"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R0b9589bb1ba14263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R6392955afe0b4682"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7d61c55e94f94707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rbb1f9abae6034c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4fc77a555c104581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Ra6661a5e253e411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb7f814ceaa614b60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R6c6e19d67c184b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R49d235040144420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R7d203501e382466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rd424b2fd1c364419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rcf4a4daa04aa4e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7650a391d6cc43d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rac07a1a53da445cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R82fc29eca17d4650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R1c6245ac7b68435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc3d26f086dc34c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R63bc6d1a53304c62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-25</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-28
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R463e6a4867c040ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R6fdc2d976e564045"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R12111a5293c8425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb622e8704ad347c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R80575efabeef4b91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R7f3721228d904cd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R3d9dc2e6cf4347ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R6849ee60b2ec4de0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb6b56f017e254ba8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rfbb6528943e74a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Ra3af8670887c4877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2d23b30e7aca464f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf446daab0a8745c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rd826316540034287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R39663b978b684a4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Ra434159af3be4b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R0cfdb3ed78de4fac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R0486657de9ee4141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R08f1d3d317f94498"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rb02d022b94aa473d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7725.52</x:v>
+        <x:v>7551.22</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7569.51</x:v>
+        <x:v>7246.61</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>156</x:v>
+        <x:v>304.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2268.3</x:v>
+        <x:v>2572.9</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>126</x:v>
+        <x:v>135.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7774.22</x:v>
+        <x:v>7601.09</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7624.07</x:v>
+        <x:v>7364.43</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>150.2</x:v>
+        <x:v>236.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2109.5</x:v>
+        <x:v>2346.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>117.2</x:v>
+        <x:v>123.5</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3930.5</x:v>
+        <x:v>3878.41</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3888.37</x:v>
+        <x:v>3806.67</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>42.1</x:v>
+        <x:v>71.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>610.8</x:v>
+        <x:v>682.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>33.9</x:v>
+        <x:v>35.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7639.6</x:v>
+        <x:v>7458.4</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7450</x:v>
+        <x:v>7186</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>189.6</x:v>
+        <x:v>272.4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2489.8</x:v>
+        <x:v>2762.2</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>138.3</x:v>
+        <x:v>145.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-25</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1851,193 +1851,193 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="30"/>
-      <x:c r="D9" s="30"/>
-      <x:c r="E9" s="30"/>
-      <x:c r="F9" s="30"/>
-      <x:c r="G9" s="30"/>
-      <x:c r="H9" s="30"/>
-      <x:c r="I9" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1408.5</x:v>
-      </x:c>
-      <x:c r="J9" s="30"/>
-      <x:c r="K9" s="30"/>
+      <x:c r="A9" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="n">
+        <x:v>7551.22</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>7551.22</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>7246.61</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>7294.17</x:v>
+      </x:c>
+      <x:c r="G9" s="28" t="n">
+        <x:f>ROUND(F9-F8,1)</x:f>
+        <x:v>-276</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="n">
+        <x:f>IFERROR(F9/F8-1,"")</x:f>
+        <x:v>-0.0364550721651119</x:v>
+      </x:c>
+      <x:c r="I9" s="26" t="n">
+        <x:f>ROUND(D9-E9,1)</x:f>
+        <x:v>304.6</x:v>
+      </x:c>
+      <x:c r="J9" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="C10" s="30"/>
       <x:c r="D10" s="30"/>
       <x:c r="E10" s="30"/>
       <x:c r="F10" s="30"/>
       <x:c r="G10" s="30"/>
       <x:c r="H10" s="30"/>
-      <x:c r="I10" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>352.1</x:v>
+      <x:c r="I10" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I9),1)</x:f>
+        <x:v>1713.1</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="17" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I9),0),1)</x:f>
+        <x:v>342.6</x:v>
+      </x:c>
+      <x:c r="J11" s="30"/>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B12" s="17"/>
-      <x:c r="C12" s="17"/>
-      <x:c r="D12" s="17"/>
-      <x:c r="E12" s="17"/>
-      <x:c r="F12" s="17"/>
-      <x:c r="G12" s="17"/>
-      <x:c r="H12" s="17"/>
-      <x:c r="I12" s="17"/>
-      <x:c r="J12" s="17"/>
-      <x:c r="K12" s="17"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="20" t="str">
+      <x:c r="B13" s="17"/>
+      <x:c r="C13" s="17"/>
+      <x:c r="D13" s="17"/>
+      <x:c r="E13" s="17"/>
+      <x:c r="F13" s="17"/>
+      <x:c r="G13" s="17"/>
+      <x:c r="H13" s="17"/>
+      <x:c r="I13" s="17"/>
+      <x:c r="J13" s="17"/>
+      <x:c r="K13" s="17"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B13" s="20" t="str">
+      <x:c r="B14" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C13" s="20" t="str">
+      <x:c r="C14" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D13" s="20" t="str">
+      <x:c r="D14" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E13" s="20" t="str">
+      <x:c r="E14" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F13" s="20" t="str">
+      <x:c r="F14" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G13" s="20" t="str">
+      <x:c r="G14" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H13" s="20" t="str">
+      <x:c r="H14" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I13" s="20" t="str">
+      <x:c r="I14" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J13" s="20" t="str">
+      <x:c r="J14" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K13" s="20" t="str">
+      <x:c r="K14" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B14" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C14" s="23" t="n">
-        <x:v>7944.29</x:v>
-      </x:c>
-      <x:c r="D14" s="23" t="n">
-        <x:v>7955.57</x:v>
-      </x:c>
-      <x:c r="E14" s="23" t="n">
-        <x:v>7610.58</x:v>
-      </x:c>
-      <x:c r="F14" s="23" t="n">
-        <x:v>7652.69</x:v>
-      </x:c>
-      <x:c r="G14" s="23"/>
-      <x:c r="H14" s="24"/>
-      <x:c r="I14" s="26" t="n">
-        <x:f>ROUND(D14-E14,1)</x:f>
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="J14" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K14" s="22" t="n">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
-        <x:v>7687.47</x:v>
+        <x:v>7944.29</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>7830.16</x:v>
+        <x:v>7955.57</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>7451.12</x:v>
+        <x:v>7610.58</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>7580.54</x:v>
-      </x:c>
-      <x:c r="G15" s="23" t="n">
-        <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-72.1</x:v>
-      </x:c>
-      <x:c r="H15" s="24" t="n">
-        <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.009428057323633832</x:v>
-      </x:c>
+        <x:v>7652.69</x:v>
+      </x:c>
+      <x:c r="G15" s="23"/>
+      <x:c r="H15" s="24"/>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>379</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C16" s="23" t="n">
-        <x:v>7511.04</x:v>
+        <x:v>7687.47</x:v>
       </x:c>
       <x:c r="D16" s="23" t="n">
-        <x:v>7819.98</x:v>
+        <x:v>7830.16</x:v>
       </x:c>
       <x:c r="E16" s="23" t="n">
-        <x:v>7487.46</x:v>
+        <x:v>7451.12</x:v>
       </x:c>
       <x:c r="F16" s="23" t="n">
-        <x:v>7799.61</x:v>
-      </x:c>
-      <x:c r="G16" s="28" t="n">
+        <x:v>7580.54</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
         <x:f>ROUND(F16-F15,1)</x:f>
-        <x:v>219.1</x:v>
+        <x:v>-72.1</x:v>
       </x:c>
       <x:c r="H16" s="24" t="n">
         <x:f>IFERROR(F16/F15-1,"")</x:f>
-        <x:v>0.028898996641400165</x:v>
+        <x:v>-0.009428057323633832</x:v>
       </x:c>
       <x:c r="I16" s="26" t="n">
         <x:f>ROUND(D16-E16,1)</x:f>
-        <x:v>332.5</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="J16" s="22" t="str">
         <x:v>中证500</x:v>
@@ -2048,1495 +2048,1647 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>9月21日-9月24日</x:v>
+        <x:v>9月14日-9月18日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
-        <x:v>7829.82</x:v>
+        <x:v>7511.04</x:v>
       </x:c>
       <x:c r="D17" s="23" t="n">
-        <x:v>7922.62</x:v>
+        <x:v>7819.98</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>7624.07</x:v>
+        <x:v>7487.46</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>7624.07</x:v>
+        <x:v>7799.61</x:v>
       </x:c>
       <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-175.5</x:v>
+        <x:v>219.1</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.02250625351780411</x:v>
+        <x:v>0.028898996641400165</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>298.6</x:v>
+        <x:v>332.5</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
+      <x:c r="B18" s="22" t="str">
+        <x:v>9月21日-9月24日</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="n">
+        <x:v>7829.82</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>7922.62</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>7624.07</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>7624.07</x:v>
+      </x:c>
+      <x:c r="G18" s="28" t="n">
+        <x:f>ROUND(F18-F17,1)</x:f>
+        <x:v>-175.5</x:v>
+      </x:c>
+      <x:c r="H18" s="24" t="n">
+        <x:f>IFERROR(F18/F17-1,"")</x:f>
+        <x:v>-0.02250625351780411</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="n">
+        <x:f>ROUND(D18-E18,1)</x:f>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="J18" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>7599.2</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>7601.09</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>7364.43</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>7402.3</x:v>
+      </x:c>
+      <x:c r="G19" s="28" t="n">
+        <x:f>ROUND(F19-F18,1)</x:f>
+        <x:v>-221.8</x:v>
+      </x:c>
+      <x:c r="H19" s="24" t="n">
+        <x:f>IFERROR(F19/F18-1,"")</x:f>
+        <x:v>-0.029088137963056426</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="n">
+        <x:f>ROUND(D19-E19,1)</x:f>
+        <x:v>236.7</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="32" t="n">
-        <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1355.1</x:v>
-      </x:c>
-      <x:c r="J18" s="30"/>
-      <x:c r="K18" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
+      <x:c r="B20" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="32" t="n">
+        <x:f>ROUND(SUM(I15:I19),1)</x:f>
+        <x:v>1591.8</x:v>
+      </x:c>
+      <x:c r="J20" s="30"/>
+      <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="30"/>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>338.8</x:v>
-      </x:c>
-      <x:c r="J19" s="30"/>
-      <x:c r="K19" s="30"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I15:I19),0),1)</x:f>
+        <x:v>318.4</x:v>
+      </x:c>
+      <x:c r="J21" s="30"/>
+      <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="17" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B21" s="17"/>
-      <x:c r="C21" s="17"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="17"/>
-      <x:c r="G21" s="17"/>
-      <x:c r="H21" s="17"/>
-      <x:c r="I21" s="17"/>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
+      <x:c r="B23" s="17"/>
+      <x:c r="C23" s="17"/>
+      <x:c r="D23" s="17"/>
+      <x:c r="E23" s="17"/>
+      <x:c r="F23" s="17"/>
+      <x:c r="G23" s="17"/>
+      <x:c r="H23" s="17"/>
+      <x:c r="I23" s="17"/>
+      <x:c r="J23" s="17"/>
+      <x:c r="K23" s="17"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B22" s="20" t="str">
+      <x:c r="B24" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="str">
+      <x:c r="C24" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="str">
+      <x:c r="D24" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="str">
+      <x:c r="E24" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
+      <x:c r="F24" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="str">
+      <x:c r="G24" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H22" s="20" t="str">
+      <x:c r="H24" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I22" s="20" t="str">
+      <x:c r="I24" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J22" s="20" t="str">
+      <x:c r="J24" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K22" s="20" t="str">
+      <x:c r="K24" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B23" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C23" s="23" t="n">
-        <x:v>3979.88</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="n">
-        <x:v>3995.18</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="n">
-        <x:v>3915.22</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="n">
-        <x:v>3930.12</x:v>
-      </x:c>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
-      <x:c r="I23" s="26" t="n">
-        <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J23" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K23" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B24" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C24" s="23" t="n">
-        <x:v>3942.51</x:v>
-      </x:c>
-      <x:c r="D24" s="23" t="n">
-        <x:v>3958.12</x:v>
-      </x:c>
-      <x:c r="E24" s="23" t="n">
-        <x:v>3852.03</x:v>
-      </x:c>
-      <x:c r="F24" s="23" t="n">
-        <x:v>3888.11</x:v>
-      </x:c>
-      <x:c r="G24" s="23" t="n">
-        <x:f>ROUND(F24-F23,1)</x:f>
-        <x:v>-42</x:v>
-      </x:c>
-      <x:c r="H24" s="24" t="n">
-        <x:f>IFERROR(F24/F23-1,"")</x:f>
-        <x:v>-0.010689241040986008</x:v>
-      </x:c>
-      <x:c r="I24" s="26" t="n">
-        <x:f>ROUND(D24-E24,1)</x:f>
-        <x:v>106.1</x:v>
-      </x:c>
-      <x:c r="J24" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K24" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C25" s="23" t="n">
-        <x:v>3867.02</x:v>
+        <x:v>3979.88</x:v>
       </x:c>
       <x:c r="D25" s="23" t="n">
-        <x:v>3919.67</x:v>
+        <x:v>3995.18</x:v>
       </x:c>
       <x:c r="E25" s="23" t="n">
-        <x:v>3842.72</x:v>
+        <x:v>3915.22</x:v>
       </x:c>
       <x:c r="F25" s="23" t="n">
-        <x:v>3911.87</x:v>
-      </x:c>
-      <x:c r="G25" s="23" t="n">
-        <x:f>ROUND(F25-F24,1)</x:f>
-        <x:v>23.8</x:v>
-      </x:c>
-      <x:c r="H25" s="24" t="n">
-        <x:f>IFERROR(F25/F24-1,"")</x:f>
-        <x:v>0.0061109382193405</x:v>
-      </x:c>
+        <x:v>3930.12</x:v>
+      </x:c>
+      <x:c r="G25" s="23"/>
+      <x:c r="H25" s="24"/>
       <x:c r="I25" s="26" t="n">
         <x:f>ROUND(D25-E25,1)</x:f>
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="J25" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K25" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>9月21日-9月24日</x:v>
+        <x:v>9月7日-9月11日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
-        <x:v>3920.27</x:v>
+        <x:v>3942.51</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3967.68</x:v>
+        <x:v>3958.12</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3888.37</x:v>
+        <x:v>3852.03</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3888.37</x:v>
+        <x:v>3888.11</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-23.5</x:v>
+        <x:v>-42</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.00600735709519995</x:v>
+        <x:v>-0.010689241040986008</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>79.3</x:v>
+        <x:v>106.1</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="n">
+        <x:v>3867.02</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="n">
+        <x:v>3919.67</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="n">
+        <x:v>3842.72</x:v>
+      </x:c>
+      <x:c r="F27" s="23" t="n">
+        <x:v>3911.87</x:v>
+      </x:c>
+      <x:c r="G27" s="23" t="n">
+        <x:f>ROUND(F27-F26,1)</x:f>
+        <x:v>23.8</x:v>
+      </x:c>
+      <x:c r="H27" s="24" t="n">
+        <x:f>IFERROR(F27/F26-1,"")</x:f>
+        <x:v>0.0061109382193405</x:v>
+      </x:c>
+      <x:c r="I27" s="26" t="n">
+        <x:f>ROUND(D27-E27,1)</x:f>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J27" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K27" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="31" t="str">
+      <x:c r="B28" s="22" t="str">
+        <x:v>9月21日-9月24日</x:v>
+      </x:c>
+      <x:c r="C28" s="23" t="n">
+        <x:v>3920.27</x:v>
+      </x:c>
+      <x:c r="D28" s="23" t="n">
+        <x:v>3967.68</x:v>
+      </x:c>
+      <x:c r="E28" s="23" t="n">
+        <x:v>3888.37</x:v>
+      </x:c>
+      <x:c r="F28" s="23" t="n">
+        <x:v>3888.37</x:v>
+      </x:c>
+      <x:c r="G28" s="23" t="n">
+        <x:f>ROUND(F28-F27,1)</x:f>
+        <x:v>-23.5</x:v>
+      </x:c>
+      <x:c r="H28" s="24" t="n">
+        <x:f>IFERROR(F28/F27-1,"")</x:f>
+        <x:v>-0.00600735709519995</x:v>
+      </x:c>
+      <x:c r="I28" s="26" t="n">
+        <x:f>ROUND(D28-E28,1)</x:f>
+        <x:v>79.3</x:v>
+      </x:c>
+      <x:c r="J28" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K28" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="n">
+        <x:v>3878.41</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>3878.41</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>3806.67</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>3823.62</x:v>
+      </x:c>
+      <x:c r="G29" s="23" t="n">
+        <x:f>ROUND(F29-F28,1)</x:f>
+        <x:v>-64.7</x:v>
+      </x:c>
+      <x:c r="H29" s="24" t="n">
+        <x:f>IFERROR(F29/F28-1,"")</x:f>
+        <x:v>-0.016652221882176854</x:v>
+      </x:c>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>71.7</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B27" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C27" s="30"/>
-      <x:c r="D27" s="30"/>
-      <x:c r="E27" s="30"/>
-      <x:c r="F27" s="30"/>
-      <x:c r="G27" s="30"/>
-      <x:c r="H27" s="30"/>
-      <x:c r="I27" s="32" t="n">
-        <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>342.4</x:v>
-      </x:c>
-      <x:c r="J27" s="30"/>
-      <x:c r="K27" s="30"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="31" t="str">
+      <x:c r="B30" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C30" s="30"/>
+      <x:c r="D30" s="30"/>
+      <x:c r="E30" s="30"/>
+      <x:c r="F30" s="30"/>
+      <x:c r="G30" s="30"/>
+      <x:c r="H30" s="30"/>
+      <x:c r="I30" s="32" t="n">
+        <x:f>ROUND(SUM(I25:I29),1)</x:f>
+        <x:v>414.1</x:v>
+      </x:c>
+      <x:c r="J30" s="30"/>
+      <x:c r="K30" s="30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B28" s="30"/>
-      <x:c r="C28" s="30"/>
-      <x:c r="D28" s="30"/>
-      <x:c r="E28" s="30"/>
-      <x:c r="F28" s="30"/>
-      <x:c r="G28" s="30"/>
-      <x:c r="H28" s="30"/>
-      <x:c r="I28" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>85.6</x:v>
-      </x:c>
-      <x:c r="J28" s="30"/>
-      <x:c r="K28" s="30"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="17" t="str">
+      <x:c r="B31" s="30"/>
+      <x:c r="C31" s="30"/>
+      <x:c r="D31" s="30"/>
+      <x:c r="E31" s="30"/>
+      <x:c r="F31" s="30"/>
+      <x:c r="G31" s="30"/>
+      <x:c r="H31" s="30"/>
+      <x:c r="I31" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I25:I29),0),1)</x:f>
+        <x:v>82.8</x:v>
+      </x:c>
+      <x:c r="J31" s="30"/>
+      <x:c r="K31" s="30"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="17" t="str">
         <x:v>IM主力</x:v>
       </x:c>
-      <x:c r="B30" s="17"/>
-      <x:c r="C30" s="17"/>
-      <x:c r="D30" s="17"/>
-      <x:c r="E30" s="17"/>
-      <x:c r="F30" s="17"/>
-      <x:c r="G30" s="17"/>
-      <x:c r="H30" s="17"/>
-      <x:c r="I30" s="17"/>
-      <x:c r="J30" s="17"/>
-      <x:c r="K30" s="17"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="20" t="str">
+      <x:c r="B33" s="17"/>
+      <x:c r="C33" s="17"/>
+      <x:c r="D33" s="17"/>
+      <x:c r="E33" s="17"/>
+      <x:c r="F33" s="17"/>
+      <x:c r="G33" s="17"/>
+      <x:c r="H33" s="17"/>
+      <x:c r="I33" s="17"/>
+      <x:c r="J33" s="17"/>
+      <x:c r="K33" s="17"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B31" s="20" t="str">
+      <x:c r="B34" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C31" s="20" t="str">
+      <x:c r="C34" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D31" s="20" t="str">
+      <x:c r="D34" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E31" s="20" t="str">
+      <x:c r="E34" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F31" s="20" t="str">
+      <x:c r="F34" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G31" s="20" t="str">
+      <x:c r="G34" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H31" s="20" t="str">
+      <x:c r="H34" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I31" s="20" t="str">
+      <x:c r="I34" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J31" s="20" t="str">
+      <x:c r="J34" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K31" s="20" t="str">
+      <x:c r="K34" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B32" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C32" s="23" t="n">
-        <x:v>7713.4</x:v>
-      </x:c>
-      <x:c r="D32" s="23" t="n">
-        <x:v>7721</x:v>
-      </x:c>
-      <x:c r="E32" s="23" t="n">
-        <x:v>7432</x:v>
-      </x:c>
-      <x:c r="F32" s="23" t="n">
-        <x:v>7468.2</x:v>
-      </x:c>
-      <x:c r="G32" s="23"/>
-      <x:c r="H32" s="24"/>
-      <x:c r="I32" s="26" t="n">
-        <x:f>ROUND(D32-E32,1)</x:f>
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J32" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K32" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B33" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C33" s="23" t="n">
-        <x:v>7527.2</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="n">
-        <x:v>7714.6</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="n">
-        <x:v>7259.4</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="n">
-        <x:v>7415.2</x:v>
-      </x:c>
-      <x:c r="G33" s="23" t="n">
-        <x:f>ROUND(F33-F32,1)</x:f>
-        <x:v>-53</x:v>
-      </x:c>
-      <x:c r="H33" s="24" t="n">
-        <x:f>IFERROR(F33/F32-1,"")</x:f>
-        <x:v>-0.007096756915990432</x:v>
-      </x:c>
-      <x:c r="I33" s="26" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
-        <x:v>455.2</x:v>
-      </x:c>
-      <x:c r="J33" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K33" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B34" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
-      </x:c>
-      <x:c r="C34" s="23" t="n">
-        <x:v>7312</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="n">
-        <x:v>7712.4</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="n">
-        <x:v>7283.4</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="n">
-        <x:v>7679.2</x:v>
-      </x:c>
-      <x:c r="G34" s="28" t="n">
-        <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>264</x:v>
-      </x:c>
-      <x:c r="H34" s="24" t="n">
-        <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>0.03560254612148017</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="J34" s="22" t="str">
-        <x:v>IM2609</x:v>
-      </x:c>
-      <x:c r="K34" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>9月21日-9月24日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
-        <x:v>7549</x:v>
+        <x:v>7713.4</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>7687</x:v>
+        <x:v>7721</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
-        <x:v>7386</x:v>
+        <x:v>7432</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>7391</x:v>
-      </x:c>
-      <x:c r="G35" s="28" t="n">
-        <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>-288.2</x:v>
-      </x:c>
-      <x:c r="H35" s="24" t="n">
-        <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>-0.03752995103656631</x:v>
-      </x:c>
+        <x:v>7468.2</x:v>
+      </x:c>
+      <x:c r="G35" s="23"/>
+      <x:c r="H35" s="24"/>
       <x:c r="I35" s="26" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>301</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
-        <x:v>IM2612</x:v>
+        <x:v>IM2609</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="31" t="str">
+      <x:c r="A36" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B36" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C36" s="23" t="n">
+        <x:v>7527.2</x:v>
+      </x:c>
+      <x:c r="D36" s="23" t="n">
+        <x:v>7714.6</x:v>
+      </x:c>
+      <x:c r="E36" s="23" t="n">
+        <x:v>7259.4</x:v>
+      </x:c>
+      <x:c r="F36" s="23" t="n">
+        <x:v>7415.2</x:v>
+      </x:c>
+      <x:c r="G36" s="23" t="n">
+        <x:f>ROUND(F36-F35,1)</x:f>
+        <x:v>-53</x:v>
+      </x:c>
+      <x:c r="H36" s="24" t="n">
+        <x:f>IFERROR(F36/F35-1,"")</x:f>
+        <x:v>-0.007096756915990432</x:v>
+      </x:c>
+      <x:c r="I36" s="26" t="n">
+        <x:f>ROUND(D36-E36,1)</x:f>
+        <x:v>455.2</x:v>
+      </x:c>
+      <x:c r="J36" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K36" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C37" s="23" t="n">
+        <x:v>7312</x:v>
+      </x:c>
+      <x:c r="D37" s="23" t="n">
+        <x:v>7712.4</x:v>
+      </x:c>
+      <x:c r="E37" s="23" t="n">
+        <x:v>7283.4</x:v>
+      </x:c>
+      <x:c r="F37" s="23" t="n">
+        <x:v>7679.2</x:v>
+      </x:c>
+      <x:c r="G37" s="28" t="n">
+        <x:f>ROUND(F37-F36,1)</x:f>
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="H37" s="24" t="n">
+        <x:f>IFERROR(F37/F36-1,"")</x:f>
+        <x:v>0.03560254612148017</x:v>
+      </x:c>
+      <x:c r="I37" s="26" t="n">
+        <x:f>ROUND(D37-E37,1)</x:f>
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="J37" s="22" t="str">
+        <x:v>IM2609</x:v>
+      </x:c>
+      <x:c r="K37" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B38" s="22" t="str">
+        <x:v>9月21日-9月24日</x:v>
+      </x:c>
+      <x:c r="C38" s="23" t="n">
+        <x:v>7549</x:v>
+      </x:c>
+      <x:c r="D38" s="23" t="n">
+        <x:v>7687</x:v>
+      </x:c>
+      <x:c r="E38" s="23" t="n">
+        <x:v>7386</x:v>
+      </x:c>
+      <x:c r="F38" s="23" t="n">
+        <x:v>7391</x:v>
+      </x:c>
+      <x:c r="G38" s="28" t="n">
+        <x:f>ROUND(F38-F37,1)</x:f>
+        <x:v>-288.2</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="n">
+        <x:f>IFERROR(F38/F37-1,"")</x:f>
+        <x:v>-0.03752995103656631</x:v>
+      </x:c>
+      <x:c r="I38" s="26" t="n">
+        <x:f>ROUND(D38-E38,1)</x:f>
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="J38" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K38" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B36" s="30" t="n">
+      <x:c r="B39" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="30"/>
-      <x:c r="E36" s="30"/>
-      <x:c r="F36" s="30"/>
-      <x:c r="G36" s="30"/>
-      <x:c r="H36" s="30"/>
-      <x:c r="I36" s="32" t="n">
-        <x:f>ROUND(SUM(I32:I35),1)</x:f>
+      <x:c r="C39" s="30"/>
+      <x:c r="D39" s="30"/>
+      <x:c r="E39" s="30"/>
+      <x:c r="F39" s="30"/>
+      <x:c r="G39" s="30"/>
+      <x:c r="H39" s="30"/>
+      <x:c r="I39" s="32" t="n">
+        <x:f>ROUND(SUM(I35:I38),1)</x:f>
         <x:v>1474.2</x:v>
       </x:c>
-      <x:c r="J36" s="30"/>
-      <x:c r="K36" s="30"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="31" t="str">
+      <x:c r="J39" s="30"/>
+      <x:c r="K39" s="30"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B37" s="30"/>
-      <x:c r="C37" s="30"/>
-      <x:c r="D37" s="30"/>
-      <x:c r="E37" s="30"/>
-      <x:c r="F37" s="30"/>
-      <x:c r="G37" s="30"/>
-      <x:c r="H37" s="30"/>
-      <x:c r="I37" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I32:I35),0),1)</x:f>
+      <x:c r="B40" s="30"/>
+      <x:c r="C40" s="30"/>
+      <x:c r="D40" s="30"/>
+      <x:c r="E40" s="30"/>
+      <x:c r="F40" s="30"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I35:I38),0),1)</x:f>
         <x:v>368.6</x:v>
       </x:c>
-      <x:c r="J37" s="30"/>
-      <x:c r="K37" s="30"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="17" t="str">
+      <x:c r="J40" s="30"/>
+      <x:c r="K40" s="30"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="17" t="str">
         <x:v>IC主力</x:v>
       </x:c>
-      <x:c r="B39" s="17"/>
-      <x:c r="C39" s="17"/>
-      <x:c r="D39" s="17"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="17"/>
-      <x:c r="G39" s="17"/>
-      <x:c r="H39" s="17"/>
-      <x:c r="I39" s="17"/>
-      <x:c r="J39" s="17"/>
-      <x:c r="K39" s="17"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
+      <x:c r="B42" s="17"/>
+      <x:c r="C42" s="17"/>
+      <x:c r="D42" s="17"/>
+      <x:c r="E42" s="17"/>
+      <x:c r="F42" s="17"/>
+      <x:c r="G42" s="17"/>
+      <x:c r="H42" s="17"/>
+      <x:c r="I42" s="17"/>
+      <x:c r="J42" s="17"/>
+      <x:c r="K42" s="17"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B40" s="20" t="str">
+      <x:c r="B43" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C40" s="20" t="str">
+      <x:c r="C43" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D40" s="20" t="str">
+      <x:c r="D43" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E40" s="20" t="str">
+      <x:c r="E43" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F40" s="20" t="str">
+      <x:c r="F43" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G40" s="20" t="str">
+      <x:c r="G43" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H40" s="20" t="str">
+      <x:c r="H43" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I40" s="20" t="str">
+      <x:c r="I43" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J40" s="20" t="str">
+      <x:c r="J43" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K40" s="20" t="str">
+      <x:c r="K43" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>7880.8</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>7903</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>7568</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>7608</x:v>
-      </x:c>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B42" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C42" s="23" t="n">
-        <x:v>7665.6</x:v>
-      </x:c>
-      <x:c r="D42" s="23" t="n">
-        <x:v>7817.2</x:v>
-      </x:c>
-      <x:c r="E42" s="23" t="n">
-        <x:v>7418.8</x:v>
-      </x:c>
-      <x:c r="F42" s="23" t="n">
-        <x:v>7569</x:v>
-      </x:c>
-      <x:c r="G42" s="23" t="n">
-        <x:f>ROUND(F42-F41,1)</x:f>
-        <x:v>-39</x:v>
-      </x:c>
-      <x:c r="H42" s="24" t="n">
-        <x:f>IFERROR(F42/F41-1,"")</x:f>
-        <x:v>-0.005126182965299653</x:v>
-      </x:c>
-      <x:c r="I42" s="26" t="n">
-        <x:f>ROUND(D42-E42,1)</x:f>
-        <x:v>398.4</x:v>
-      </x:c>
-      <x:c r="J42" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K42" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B43" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
-      </x:c>
-      <x:c r="C43" s="23" t="n">
-        <x:v>7482.2</x:v>
-      </x:c>
-      <x:c r="D43" s="23" t="n">
-        <x:v>7820</x:v>
-      </x:c>
-      <x:c r="E43" s="23" t="n">
-        <x:v>7452.2</x:v>
-      </x:c>
-      <x:c r="F43" s="23" t="n">
-        <x:v>7789.8</x:v>
-      </x:c>
-      <x:c r="G43" s="28" t="n">
-        <x:f>ROUND(F43-F42,1)</x:f>
-        <x:v>220.8</x:v>
-      </x:c>
-      <x:c r="H43" s="24" t="n">
-        <x:f>IFERROR(F43/F42-1,"")</x:f>
-        <x:v>0.02917162108600868</x:v>
-      </x:c>
-      <x:c r="I43" s="26" t="n">
-        <x:f>ROUND(D43-E43,1)</x:f>
-        <x:v>367.8</x:v>
-      </x:c>
-      <x:c r="J43" s="22" t="str">
-        <x:v>IC2609</x:v>
-      </x:c>
-      <x:c r="K43" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>9月21日-9月24日</x:v>
+        <x:v>9月1日-9月4日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
-        <x:v>7688</x:v>
+        <x:v>7880.8</x:v>
       </x:c>
       <x:c r="D44" s="23" t="n">
-        <x:v>7780</x:v>
+        <x:v>7903</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
-        <x:v>7450</x:v>
+        <x:v>7568</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>7451.6</x:v>
-      </x:c>
-      <x:c r="G44" s="28" t="n">
-        <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-338.2</x:v>
-      </x:c>
-      <x:c r="H44" s="24" t="n">
-        <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.04341574879971244</x:v>
-      </x:c>
+        <x:v>7608</x:v>
+      </x:c>
+      <x:c r="G44" s="23"/>
+      <x:c r="H44" s="24"/>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>330</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
-        <x:v>IC2612</x:v>
+        <x:v>IC2609</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="31" t="str">
+      <x:c r="A45" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B45" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C45" s="23" t="n">
+        <x:v>7665.6</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="n">
+        <x:v>7817.2</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="n">
+        <x:v>7418.8</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="n">
+        <x:v>7569</x:v>
+      </x:c>
+      <x:c r="G45" s="23" t="n">
+        <x:f>ROUND(F45-F44,1)</x:f>
+        <x:v>-39</x:v>
+      </x:c>
+      <x:c r="H45" s="24" t="n">
+        <x:f>IFERROR(F45/F44-1,"")</x:f>
+        <x:v>-0.005126182965299653</x:v>
+      </x:c>
+      <x:c r="I45" s="26" t="n">
+        <x:f>ROUND(D45-E45,1)</x:f>
+        <x:v>398.4</x:v>
+      </x:c>
+      <x:c r="J45" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K45" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="n">
+        <x:v>7482.2</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="n">
+        <x:v>7820</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="n">
+        <x:v>7452.2</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="n">
+        <x:v>7789.8</x:v>
+      </x:c>
+      <x:c r="G46" s="28" t="n">
+        <x:f>ROUND(F46-F45,1)</x:f>
+        <x:v>220.8</x:v>
+      </x:c>
+      <x:c r="H46" s="24" t="n">
+        <x:f>IFERROR(F46/F45-1,"")</x:f>
+        <x:v>0.02917162108600868</x:v>
+      </x:c>
+      <x:c r="I46" s="26" t="n">
+        <x:f>ROUND(D46-E46,1)</x:f>
+        <x:v>367.8</x:v>
+      </x:c>
+      <x:c r="J46" s="22" t="str">
+        <x:v>IC2609</x:v>
+      </x:c>
+      <x:c r="K46" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>9月21日-9月24日</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="n">
+        <x:v>7688</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="n">
+        <x:v>7780</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="n">
+        <x:v>7450</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="n">
+        <x:v>7451.6</x:v>
+      </x:c>
+      <x:c r="G47" s="28" t="n">
+        <x:f>ROUND(F47-F46,1)</x:f>
+        <x:v>-338.2</x:v>
+      </x:c>
+      <x:c r="H47" s="24" t="n">
+        <x:f>IFERROR(F47/F46-1,"")</x:f>
+        <x:v>-0.04341574879971244</x:v>
+      </x:c>
+      <x:c r="I47" s="26" t="n">
+        <x:f>ROUND(D47-E47,1)</x:f>
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="J47" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K47" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B48" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="C48" s="23" t="n">
+        <x:v>7440.8</x:v>
+      </x:c>
+      <x:c r="D48" s="23" t="n">
+        <x:v>7458.4</x:v>
+      </x:c>
+      <x:c r="E48" s="23" t="n">
+        <x:v>7186</x:v>
+      </x:c>
+      <x:c r="F48" s="23" t="n">
+        <x:v>7270</x:v>
+      </x:c>
+      <x:c r="G48" s="28" t="n">
+        <x:f>ROUND(F48-F47,1)</x:f>
+        <x:v>-181.6</x:v>
+      </x:c>
+      <x:c r="H48" s="24" t="n">
+        <x:f>IFERROR(F48/F47-1,"")</x:f>
+        <x:v>-0.024370604970744614</x:v>
+      </x:c>
+      <x:c r="I48" s="26" t="n">
+        <x:f>ROUND(D48-E48,1)</x:f>
+        <x:v>272.4</x:v>
+      </x:c>
+      <x:c r="J48" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K48" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B45" s="30" t="n">
+      <x:c r="B49" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="32" t="n">
+        <x:f>ROUND(SUM(I44:I48),1)</x:f>
+        <x:v>1703.6</x:v>
+      </x:c>
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B50" s="30"/>
+      <x:c r="C50" s="30"/>
+      <x:c r="D50" s="30"/>
+      <x:c r="E50" s="30"/>
+      <x:c r="F50" s="30"/>
+      <x:c r="G50" s="30"/>
+      <x:c r="H50" s="30"/>
+      <x:c r="I50" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I44:I48),0),1)</x:f>
+        <x:v>340.7</x:v>
+      </x:c>
+      <x:c r="J50" s="30"/>
+      <x:c r="K50" s="30"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B52" s="17"/>
+      <x:c r="C52" s="17"/>
+      <x:c r="D52" s="17"/>
+      <x:c r="E52" s="17"/>
+      <x:c r="F52" s="17"/>
+      <x:c r="G52" s="17"/>
+      <x:c r="H52" s="17"/>
+      <x:c r="I52" s="17"/>
+      <x:c r="J52" s="17"/>
+      <x:c r="K52" s="17"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B53" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C53" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D53" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E53" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F53" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G53" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H53" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I53" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J53" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K53" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B54" s="22" t="str">
+        <x:v>9月1日-9月4日</x:v>
+      </x:c>
+      <x:c r="C54" s="23" t="n">
+        <x:v>4602</x:v>
+      </x:c>
+      <x:c r="D54" s="23" t="n">
+        <x:v>4617.8</x:v>
+      </x:c>
+      <x:c r="E54" s="23" t="n">
+        <x:v>4497.6</x:v>
+      </x:c>
+      <x:c r="F54" s="23" t="n">
+        <x:v>4537.4</x:v>
+      </x:c>
+      <x:c r="G54" s="23"/>
+      <x:c r="H54" s="24"/>
+      <x:c r="I54" s="26" t="n">
+        <x:f>ROUND(D54-E54,1)</x:f>
+        <x:v>120.2</x:v>
+      </x:c>
+      <x:c r="J54" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K54" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C45" s="30"/>
-      <x:c r="D45" s="30"/>
-      <x:c r="E45" s="30"/>
-      <x:c r="F45" s="30"/>
-      <x:c r="G45" s="30"/>
-      <x:c r="H45" s="30"/>
-      <x:c r="I45" s="32" t="n">
-        <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1431.2</x:v>
-      </x:c>
-      <x:c r="J45" s="30"/>
-      <x:c r="K45" s="30"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="31" t="str">
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B55" s="22" t="str">
+        <x:v>9月7日-9月11日</x:v>
+      </x:c>
+      <x:c r="C55" s="23" t="n">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="D55" s="23" t="n">
+        <x:v>4584</x:v>
+      </x:c>
+      <x:c r="E55" s="23" t="n">
+        <x:v>4451.6</x:v>
+      </x:c>
+      <x:c r="F55" s="23" t="n">
+        <x:v>4503.4</x:v>
+      </x:c>
+      <x:c r="G55" s="23" t="n">
+        <x:f>ROUND(F55-F54,1)</x:f>
+        <x:v>-34</x:v>
+      </x:c>
+      <x:c r="H55" s="24" t="n">
+        <x:f>IFERROR(F55/F54-1,"")</x:f>
+        <x:v>-0.007493278088773314</x:v>
+      </x:c>
+      <x:c r="I55" s="26" t="n">
+        <x:f>ROUND(D55-E55,1)</x:f>
+        <x:v>132.4</x:v>
+      </x:c>
+      <x:c r="J55" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K55" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B56" s="22" t="str">
+        <x:v>9月14日-9月18日</x:v>
+      </x:c>
+      <x:c r="C56" s="23" t="n">
+        <x:v>4468</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="n">
+        <x:v>4520.6</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="n">
+        <x:v>4412.2</x:v>
+      </x:c>
+      <x:c r="F56" s="23" t="n">
+        <x:v>4508</x:v>
+      </x:c>
+      <x:c r="G56" s="23" t="n">
+        <x:f>ROUND(F56-F55,1)</x:f>
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="H56" s="24" t="n">
+        <x:f>IFERROR(F56/F55-1,"")</x:f>
+        <x:v>0.0010214504596528506</x:v>
+      </x:c>
+      <x:c r="I56" s="26" t="n">
+        <x:f>ROUND(D56-E56,1)</x:f>
+        <x:v>108.4</x:v>
+      </x:c>
+      <x:c r="J56" s="22" t="str">
+        <x:v>IF2609</x:v>
+      </x:c>
+      <x:c r="K56" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B57" s="22" t="str">
+        <x:v>9月21日-9月24日</x:v>
+      </x:c>
+      <x:c r="C57" s="23" t="n">
+        <x:v>4451</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="n">
+        <x:v>4520</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="n">
+        <x:v>4367</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="n">
+        <x:v>4375</x:v>
+      </x:c>
+      <x:c r="G57" s="23" t="n">
+        <x:f>ROUND(F57-F56,1)</x:f>
+        <x:v>-133</x:v>
+      </x:c>
+      <x:c r="H57" s="24" t="n">
+        <x:f>IFERROR(F57/F56-1,"")</x:f>
+        <x:v>-0.029503105590062084</x:v>
+      </x:c>
+      <x:c r="I57" s="26" t="n">
+        <x:f>ROUND(D57-E57,1)</x:f>
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="J57" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K57" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B58" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C58" s="30"/>
+      <x:c r="D58" s="30"/>
+      <x:c r="E58" s="30"/>
+      <x:c r="F58" s="30"/>
+      <x:c r="G58" s="30"/>
+      <x:c r="H58" s="30"/>
+      <x:c r="I58" s="32" t="n">
+        <x:f>ROUND(SUM(I54:I57),1)</x:f>
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="J58" s="30"/>
+      <x:c r="K58" s="30"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B46" s="30"/>
-      <x:c r="C46" s="30"/>
-      <x:c r="D46" s="30"/>
-      <x:c r="E46" s="30"/>
-      <x:c r="F46" s="30"/>
-      <x:c r="G46" s="30"/>
-      <x:c r="H46" s="30"/>
-      <x:c r="I46" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>357.8</x:v>
-      </x:c>
-      <x:c r="J46" s="30"/>
-      <x:c r="K46" s="30"/>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B48" s="17"/>
-      <x:c r="C48" s="17"/>
-      <x:c r="D48" s="17"/>
-      <x:c r="E48" s="17"/>
-      <x:c r="F48" s="17"/>
-      <x:c r="G48" s="17"/>
-      <x:c r="H48" s="17"/>
-      <x:c r="I48" s="17"/>
-      <x:c r="J48" s="17"/>
-      <x:c r="K48" s="17"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="20" t="str">
+      <x:c r="B59" s="30"/>
+      <x:c r="C59" s="30"/>
+      <x:c r="D59" s="30"/>
+      <x:c r="E59" s="30"/>
+      <x:c r="F59" s="30"/>
+      <x:c r="G59" s="30"/>
+      <x:c r="H59" s="30"/>
+      <x:c r="I59" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I54:I57),0),1)</x:f>
+        <x:v>128.5</x:v>
+      </x:c>
+      <x:c r="J59" s="30"/>
+      <x:c r="K59" s="30"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B61" s="17"/>
+      <x:c r="C61" s="17"/>
+      <x:c r="D61" s="17"/>
+      <x:c r="E61" s="17"/>
+      <x:c r="F61" s="17"/>
+      <x:c r="G61" s="17"/>
+      <x:c r="H61" s="17"/>
+      <x:c r="I61" s="17"/>
+      <x:c r="J61" s="17"/>
+      <x:c r="K61" s="17"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B49" s="20" t="str">
+      <x:c r="B62" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C49" s="20" t="str">
+      <x:c r="C62" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D49" s="20" t="str">
+      <x:c r="D62" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E49" s="20" t="str">
+      <x:c r="E62" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F49" s="20" t="str">
+      <x:c r="F62" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G49" s="20" t="str">
+      <x:c r="G62" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H49" s="20" t="str">
+      <x:c r="H62" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I49" s="20" t="str">
+      <x:c r="I62" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J49" s="20" t="str">
+      <x:c r="J62" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K49" s="20" t="str">
+      <x:c r="K62" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="22" t="n">
+    <x:row r="63">
+      <x:c r="A63" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B50" s="22" t="str">
+      <x:c r="B63" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C50" s="23" t="n">
-        <x:v>4602</x:v>
-      </x:c>
-      <x:c r="D50" s="23" t="n">
-        <x:v>4617.8</x:v>
-      </x:c>
-      <x:c r="E50" s="23" t="n">
-        <x:v>4497.6</x:v>
-      </x:c>
-      <x:c r="F50" s="23" t="n">
-        <x:v>4537.4</x:v>
-      </x:c>
-      <x:c r="G50" s="23"/>
-      <x:c r="H50" s="24"/>
-      <x:c r="I50" s="26" t="n">
-        <x:f>ROUND(D50-E50,1)</x:f>
-        <x:v>120.2</x:v>
-      </x:c>
-      <x:c r="J50" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K50" s="22" t="n">
+      <x:c r="C63" s="23" t="n">
+        <x:v>2913</x:v>
+      </x:c>
+      <x:c r="D63" s="23" t="n">
+        <x:v>2949.4</x:v>
+      </x:c>
+      <x:c r="E63" s="23" t="n">
+        <x:v>2881.4</x:v>
+      </x:c>
+      <x:c r="F63" s="23" t="n">
+        <x:v>2915.8</x:v>
+      </x:c>
+      <x:c r="G63" s="23"/>
+      <x:c r="H63" s="24"/>
+      <x:c r="I63" s="26" t="n">
+        <x:f>ROUND(D63-E63,1)</x:f>
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="J63" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K63" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="22" t="n">
+    <x:row r="64">
+      <x:c r="A64" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B51" s="22" t="str">
+      <x:c r="B64" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C51" s="23" t="n">
-        <x:v>4562</x:v>
-      </x:c>
-      <x:c r="D51" s="23" t="n">
-        <x:v>4584</x:v>
-      </x:c>
-      <x:c r="E51" s="23" t="n">
-        <x:v>4451.6</x:v>
-      </x:c>
-      <x:c r="F51" s="23" t="n">
-        <x:v>4503.4</x:v>
-      </x:c>
-      <x:c r="G51" s="23" t="n">
-        <x:f>ROUND(F51-F50,1)</x:f>
-        <x:v>-34</x:v>
-      </x:c>
-      <x:c r="H51" s="24" t="n">
-        <x:f>IFERROR(F51/F50-1,"")</x:f>
-        <x:v>-0.007493278088773314</x:v>
-      </x:c>
-      <x:c r="I51" s="26" t="n">
-        <x:f>ROUND(D51-E51,1)</x:f>
-        <x:v>132.4</x:v>
-      </x:c>
-      <x:c r="J51" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K51" s="22" t="n">
+      <x:c r="C64" s="23" t="n">
+        <x:v>2923.2</x:v>
+      </x:c>
+      <x:c r="D64" s="23" t="n">
+        <x:v>2931.4</x:v>
+      </x:c>
+      <x:c r="E64" s="23" t="n">
+        <x:v>2836.8</x:v>
+      </x:c>
+      <x:c r="F64" s="23" t="n">
+        <x:v>2867</x:v>
+      </x:c>
+      <x:c r="G64" s="23" t="n">
+        <x:f>ROUND(F64-F63,1)</x:f>
+        <x:v>-48.8</x:v>
+      </x:c>
+      <x:c r="H64" s="24" t="n">
+        <x:f>IFERROR(F64/F63-1,"")</x:f>
+        <x:v>-0.01673640167364021</x:v>
+      </x:c>
+      <x:c r="I64" s="26" t="n">
+        <x:f>ROUND(D64-E64,1)</x:f>
+        <x:v>94.6</x:v>
+      </x:c>
+      <x:c r="J64" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K64" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="22" t="n">
+    <x:row r="65">
+      <x:c r="A65" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B52" s="22" t="str">
+      <x:c r="B65" s="22" t="str">
         <x:v>9月14日-9月18日</x:v>
       </x:c>
-      <x:c r="C52" s="23" t="n">
-        <x:v>4468</x:v>
-      </x:c>
-      <x:c r="D52" s="23" t="n">
-        <x:v>4520.6</x:v>
-      </x:c>
-      <x:c r="E52" s="23" t="n">
-        <x:v>4412.2</x:v>
-      </x:c>
-      <x:c r="F52" s="23" t="n">
-        <x:v>4508</x:v>
-      </x:c>
-      <x:c r="G52" s="23" t="n">
-        <x:f>ROUND(F52-F51,1)</x:f>
-        <x:v>4.6</x:v>
-      </x:c>
-      <x:c r="H52" s="24" t="n">
-        <x:f>IFERROR(F52/F51-1,"")</x:f>
-        <x:v>0.0010214504596528506</x:v>
-      </x:c>
-      <x:c r="I52" s="26" t="n">
-        <x:f>ROUND(D52-E52,1)</x:f>
-        <x:v>108.4</x:v>
-      </x:c>
-      <x:c r="J52" s="22" t="str">
-        <x:v>IF2609</x:v>
-      </x:c>
-      <x:c r="K52" s="22" t="n">
+      <x:c r="C65" s="23" t="n">
+        <x:v>2849.2</x:v>
+      </x:c>
+      <x:c r="D65" s="23" t="n">
+        <x:v>2873.2</x:v>
+      </x:c>
+      <x:c r="E65" s="23" t="n">
+        <x:v>2829.4</x:v>
+      </x:c>
+      <x:c r="F65" s="23" t="n">
+        <x:v>2862.2</x:v>
+      </x:c>
+      <x:c r="G65" s="23" t="n">
+        <x:f>ROUND(F65-F64,1)</x:f>
+        <x:v>-4.8</x:v>
+      </x:c>
+      <x:c r="H65" s="24" t="n">
+        <x:f>IFERROR(F65/F64-1,"")</x:f>
+        <x:v>-0.0016742239274503135</x:v>
+      </x:c>
+      <x:c r="I65" s="23" t="n">
+        <x:f>ROUND(D65-E65,1)</x:f>
+        <x:v>43.8</x:v>
+      </x:c>
+      <x:c r="J65" s="22" t="str">
+        <x:v>IH2609</x:v>
+      </x:c>
+      <x:c r="K65" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="22" t="n">
+    <x:row r="66">
+      <x:c r="A66" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B53" s="22" t="str">
+      <x:c r="B66" s="22" t="str">
         <x:v>9月21日-9月24日</x:v>
       </x:c>
-      <x:c r="C53" s="23" t="n">
-        <x:v>4451</x:v>
-      </x:c>
-      <x:c r="D53" s="23" t="n">
-        <x:v>4520</x:v>
-      </x:c>
-      <x:c r="E53" s="23" t="n">
-        <x:v>4367</x:v>
-      </x:c>
-      <x:c r="F53" s="23" t="n">
-        <x:v>4375</x:v>
-      </x:c>
-      <x:c r="G53" s="23" t="n">
-        <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>-133</x:v>
-      </x:c>
-      <x:c r="H53" s="24" t="n">
-        <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>-0.029503105590062084</x:v>
-      </x:c>
-      <x:c r="I53" s="26" t="n">
-        <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="J53" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K53" s="22" t="n">
+      <x:c r="C66" s="23" t="n">
+        <x:v>2830</x:v>
+      </x:c>
+      <x:c r="D66" s="23" t="n">
+        <x:v>2881.2</x:v>
+      </x:c>
+      <x:c r="E66" s="23" t="n">
+        <x:v>2798</x:v>
+      </x:c>
+      <x:c r="F66" s="23" t="n">
+        <x:v>2804.6</x:v>
+      </x:c>
+      <x:c r="G66" s="23" t="n">
+        <x:f>ROUND(F66-F65,1)</x:f>
+        <x:v>-57.6</x:v>
+      </x:c>
+      <x:c r="H66" s="24" t="n">
+        <x:f>IFERROR(F66/F65-1,"")</x:f>
+        <x:v>-0.02012437984766957</x:v>
+      </x:c>
+      <x:c r="I66" s="26" t="n">
+        <x:f>ROUND(D66-E66,1)</x:f>
+        <x:v>83.2</x:v>
+      </x:c>
+      <x:c r="J66" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K66" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="31" t="str">
+    <x:row r="67">
+      <x:c r="A67" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B54" s="30" t="n">
+      <x:c r="B67" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C54" s="30"/>
-      <x:c r="D54" s="30"/>
-      <x:c r="E54" s="30"/>
-      <x:c r="F54" s="30"/>
-      <x:c r="G54" s="30"/>
-      <x:c r="H54" s="30"/>
-      <x:c r="I54" s="32" t="n">
-        <x:f>ROUND(SUM(I50:I53),1)</x:f>
-        <x:v>514</x:v>
-      </x:c>
-      <x:c r="J54" s="30"/>
-      <x:c r="K54" s="30"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="31" t="str">
+      <x:c r="C67" s="30"/>
+      <x:c r="D67" s="30"/>
+      <x:c r="E67" s="30"/>
+      <x:c r="F67" s="30"/>
+      <x:c r="G67" s="30"/>
+      <x:c r="H67" s="30"/>
+      <x:c r="I67" s="32" t="n">
+        <x:f>ROUND(SUM(I63:I66),1)</x:f>
+        <x:v>289.6</x:v>
+      </x:c>
+      <x:c r="J67" s="30"/>
+      <x:c r="K67" s="30"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B55" s="30"/>
-      <x:c r="C55" s="30"/>
-      <x:c r="D55" s="30"/>
-      <x:c r="E55" s="30"/>
-      <x:c r="F55" s="30"/>
-      <x:c r="G55" s="30"/>
-      <x:c r="H55" s="30"/>
-      <x:c r="I55" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I50:I53),0),1)</x:f>
-        <x:v>128.5</x:v>
-      </x:c>
-      <x:c r="J55" s="30"/>
-      <x:c r="K55" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B57" s="17"/>
-      <x:c r="C57" s="17"/>
-      <x:c r="D57" s="17"/>
-      <x:c r="E57" s="17"/>
-      <x:c r="F57" s="17"/>
-      <x:c r="G57" s="17"/>
-      <x:c r="H57" s="17"/>
-      <x:c r="I57" s="17"/>
-      <x:c r="J57" s="17"/>
-      <x:c r="K57" s="17"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="20" t="str">
+      <x:c r="B68" s="30"/>
+      <x:c r="C68" s="30"/>
+      <x:c r="D68" s="30"/>
+      <x:c r="E68" s="30"/>
+      <x:c r="F68" s="30"/>
+      <x:c r="G68" s="30"/>
+      <x:c r="H68" s="30"/>
+      <x:c r="I68" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I63:I66),0),1)</x:f>
+        <x:v>72.4</x:v>
+      </x:c>
+      <x:c r="J68" s="30"/>
+      <x:c r="K68" s="30"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="17" t="str">
+        <x:v>碳酸锂2610</x:v>
+      </x:c>
+      <x:c r="B70" s="17"/>
+      <x:c r="C70" s="17"/>
+      <x:c r="D70" s="17"/>
+      <x:c r="E70" s="17"/>
+      <x:c r="F70" s="17"/>
+      <x:c r="G70" s="17"/>
+      <x:c r="H70" s="17"/>
+      <x:c r="I70" s="17"/>
+      <x:c r="J70" s="17"/>
+      <x:c r="K70" s="17"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B58" s="20" t="str">
+      <x:c r="B71" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C58" s="20" t="str">
+      <x:c r="C71" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D58" s="20" t="str">
+      <x:c r="D71" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E58" s="20" t="str">
+      <x:c r="E71" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F58" s="20" t="str">
+      <x:c r="F71" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G58" s="20" t="str">
+      <x:c r="G71" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H58" s="20" t="str">
+      <x:c r="H71" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I58" s="20" t="str">
+      <x:c r="I71" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J58" s="20" t="str">
+      <x:c r="J71" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K58" s="20" t="str">
+      <x:c r="K71" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="22" t="n">
+    <x:row r="72">
+      <x:c r="A72" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B59" s="22" t="str">
+      <x:c r="B72" s="22" t="str">
         <x:v>9月1日-9月4日</x:v>
       </x:c>
-      <x:c r="C59" s="23" t="n">
-        <x:v>2913</x:v>
-      </x:c>
-      <x:c r="D59" s="23" t="n">
-        <x:v>2949.4</x:v>
-      </x:c>
-      <x:c r="E59" s="23" t="n">
-        <x:v>2881.4</x:v>
-      </x:c>
-      <x:c r="F59" s="23" t="n">
-        <x:v>2915.8</x:v>
-      </x:c>
-      <x:c r="G59" s="23"/>
-      <x:c r="H59" s="24"/>
-      <x:c r="I59" s="26" t="n">
-        <x:f>ROUND(D59-E59,1)</x:f>
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="J59" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K59" s="22" t="n">
+      <x:c r="C72" s="23" t="n">
+        <x:v>159280</x:v>
+      </x:c>
+      <x:c r="D72" s="23" t="n">
+        <x:v>161280</x:v>
+      </x:c>
+      <x:c r="E72" s="23" t="n">
+        <x:v>140220</x:v>
+      </x:c>
+      <x:c r="F72" s="23" t="n">
+        <x:v>142000</x:v>
+      </x:c>
+      <x:c r="G72" s="23"/>
+      <x:c r="H72" s="24"/>
+      <x:c r="I72" s="26" t="n">
+        <x:f>ROUND(D72-E72,1)</x:f>
+        <x:v>21060</x:v>
+      </x:c>
+      <x:c r="J72" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K72" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="22" t="n">
+    <x:row r="73">
+      <x:c r="A73" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B60" s="22" t="str">
+      <x:c r="B73" s="22" t="str">
         <x:v>9月7日-9月11日</x:v>
       </x:c>
-      <x:c r="C60" s="23" t="n">
-        <x:v>2923.2</x:v>
-      </x:c>
-      <x:c r="D60" s="23" t="n">
-        <x:v>2931.4</x:v>
-      </x:c>
-      <x:c r="E60" s="23" t="n">
-        <x:v>2836.8</x:v>
-      </x:c>
-      <x:c r="F60" s="23" t="n">
-        <x:v>2867</x:v>
-      </x:c>
-      <x:c r="G60" s="23" t="n">
-        <x:f>ROUND(F60-F59,1)</x:f>
-        <x:v>-48.8</x:v>
-      </x:c>
-      <x:c r="H60" s="24" t="n">
-        <x:f>IFERROR(F60/F59-1,"")</x:f>
-        <x:v>-0.01673640167364021</x:v>
-      </x:c>
-      <x:c r="I60" s="26" t="n">
-        <x:f>ROUND(D60-E60,1)</x:f>
-        <x:v>94.6</x:v>
-      </x:c>
-      <x:c r="J60" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K60" s="22" t="n">
+      <x:c r="C73" s="23" t="n">
+        <x:v>141000</x:v>
+      </x:c>
+      <x:c r="D73" s="23" t="n">
+        <x:v>143540</x:v>
+      </x:c>
+      <x:c r="E73" s="23" t="n">
+        <x:v>127120</x:v>
+      </x:c>
+      <x:c r="F73" s="23" t="n">
+        <x:v>134340</x:v>
+      </x:c>
+      <x:c r="G73" s="28" t="n">
+        <x:f>ROUND(F73-F72,1)</x:f>
+        <x:v>-7660</x:v>
+      </x:c>
+      <x:c r="H73" s="24" t="n">
+        <x:f>IFERROR(F73/F72-1,"")</x:f>
+        <x:v>-0.05394366197183098</x:v>
+      </x:c>
+      <x:c r="I73" s="26" t="n">
+        <x:f>ROUND(D73-E73,1)</x:f>
+        <x:v>16420</x:v>
+      </x:c>
+      <x:c r="J73" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K73" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="22" t="n">
+    <x:row r="74">
+      <x:c r="A74" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B61" s="22" t="str">
+      <x:c r="B74" s="22" t="str">
         <x:v>9月14日-9月18日</x:v>
       </x:c>
-      <x:c r="C61" s="23" t="n">
-        <x:v>2849.2</x:v>
-      </x:c>
-      <x:c r="D61" s="23" t="n">
-        <x:v>2873.2</x:v>
-      </x:c>
-      <x:c r="E61" s="23" t="n">
-        <x:v>2829.4</x:v>
-      </x:c>
-      <x:c r="F61" s="23" t="n">
-        <x:v>2862.2</x:v>
-      </x:c>
-      <x:c r="G61" s="23" t="n">
-        <x:f>ROUND(F61-F60,1)</x:f>
-        <x:v>-4.8</x:v>
-      </x:c>
-      <x:c r="H61" s="24" t="n">
-        <x:f>IFERROR(F61/F60-1,"")</x:f>
-        <x:v>-0.0016742239274503135</x:v>
-      </x:c>
-      <x:c r="I61" s="23" t="n">
-        <x:f>ROUND(D61-E61,1)</x:f>
-        <x:v>43.8</x:v>
-      </x:c>
-      <x:c r="J61" s="22" t="str">
-        <x:v>IH2609</x:v>
-      </x:c>
-      <x:c r="K61" s="22" t="n">
+      <x:c r="C74" s="23" t="n">
+        <x:v>133600</x:v>
+      </x:c>
+      <x:c r="D74" s="23" t="n">
+        <x:v>135900</x:v>
+      </x:c>
+      <x:c r="E74" s="23" t="n">
+        <x:v>126200</x:v>
+      </x:c>
+      <x:c r="F74" s="23" t="n">
+        <x:v>128580</x:v>
+      </x:c>
+      <x:c r="G74" s="28" t="n">
+        <x:f>ROUND(F74-F73,1)</x:f>
+        <x:v>-5760</x:v>
+      </x:c>
+      <x:c r="H74" s="24" t="n">
+        <x:f>IFERROR(F74/F73-1,"")</x:f>
+        <x:v>-0.04287628405538191</x:v>
+      </x:c>
+      <x:c r="I74" s="26" t="n">
+        <x:f>ROUND(D74-E74,1)</x:f>
+        <x:v>9700</x:v>
+      </x:c>
+      <x:c r="J74" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K74" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="22" t="n">
+    <x:row r="75">
+      <x:c r="A75" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B62" s="22" t="str">
+      <x:c r="B75" s="22" t="str">
         <x:v>9月21日-9月24日</x:v>
       </x:c>
-      <x:c r="C62" s="23" t="n">
-        <x:v>2830</x:v>
-      </x:c>
-      <x:c r="D62" s="23" t="n">
-        <x:v>2881.2</x:v>
-      </x:c>
-      <x:c r="E62" s="23" t="n">
-        <x:v>2798</x:v>
-      </x:c>
-      <x:c r="F62" s="23" t="n">
-        <x:v>2804.6</x:v>
-      </x:c>
-      <x:c r="G62" s="23" t="n">
-        <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>-57.6</x:v>
-      </x:c>
-      <x:c r="H62" s="24" t="n">
-        <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>-0.02012437984766957</x:v>
-      </x:c>
-      <x:c r="I62" s="26" t="n">
-        <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>83.2</x:v>
-      </x:c>
-      <x:c r="J62" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K62" s="22" t="n">
+      <x:c r="C75" s="23" t="n">
+        <x:v>128500</x:v>
+      </x:c>
+      <x:c r="D75" s="23" t="n">
+        <x:v>136560</x:v>
+      </x:c>
+      <x:c r="E75" s="23" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="F75" s="23" t="n">
+        <x:v>125980</x:v>
+      </x:c>
+      <x:c r="G75" s="28" t="n">
+        <x:f>ROUND(F75-F74,1)</x:f>
+        <x:v>-2600</x:v>
+      </x:c>
+      <x:c r="H75" s="24" t="n">
+        <x:f>IFERROR(F75/F74-1,"")</x:f>
+        <x:v>-0.02022087416394458</x:v>
+      </x:c>
+      <x:c r="I75" s="26" t="n">
+        <x:f>ROUND(D75-E75,1)</x:f>
+        <x:v>11560</x:v>
+      </x:c>
+      <x:c r="J75" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K75" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="31" t="str">
+    <x:row r="76">
+      <x:c r="A76" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B63" s="30" t="n">
+      <x:c r="B76" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C63" s="30"/>
-      <x:c r="D63" s="30"/>
-      <x:c r="E63" s="30"/>
-      <x:c r="F63" s="30"/>
-      <x:c r="G63" s="30"/>
-      <x:c r="H63" s="30"/>
-      <x:c r="I63" s="32" t="n">
-        <x:f>ROUND(SUM(I59:I62),1)</x:f>
-        <x:v>289.6</x:v>
-      </x:c>
-      <x:c r="J63" s="30"/>
-      <x:c r="K63" s="30"/>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
+      <x:c r="C76" s="30"/>
+      <x:c r="D76" s="30"/>
+      <x:c r="E76" s="30"/>
+      <x:c r="F76" s="30"/>
+      <x:c r="G76" s="30"/>
+      <x:c r="H76" s="30"/>
+      <x:c r="I76" s="32" t="n">
+        <x:f>ROUND(SUM(I72:I75),1)</x:f>
+        <x:v>58740</x:v>
+      </x:c>
+      <x:c r="J76" s="30"/>
+      <x:c r="K76" s="30"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B64" s="30"/>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I59:I62),0),1)</x:f>
-        <x:v>72.4</x:v>
-      </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66" s="17" t="str">
-        <x:v>碳酸锂2610</x:v>
-      </x:c>
-      <x:c r="B66" s="17"/>
-      <x:c r="C66" s="17"/>
-      <x:c r="D66" s="17"/>
-      <x:c r="E66" s="17"/>
-      <x:c r="F66" s="17"/>
-      <x:c r="G66" s="17"/>
-      <x:c r="H66" s="17"/>
-      <x:c r="I66" s="17"/>
-      <x:c r="J66" s="17"/>
-      <x:c r="K66" s="17"/>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B67" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C67" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D67" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E67" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F67" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G67" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H67" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I67" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J67" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K67" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B68" s="22" t="str">
-        <x:v>9月1日-9月4日</x:v>
-      </x:c>
-      <x:c r="C68" s="23" t="n">
-        <x:v>159280</x:v>
-      </x:c>
-      <x:c r="D68" s="23" t="n">
-        <x:v>161280</x:v>
-      </x:c>
-      <x:c r="E68" s="23" t="n">
-        <x:v>140220</x:v>
-      </x:c>
-      <x:c r="F68" s="23" t="n">
-        <x:v>142000</x:v>
-      </x:c>
-      <x:c r="G68" s="23"/>
-      <x:c r="H68" s="24"/>
-      <x:c r="I68" s="26" t="n">
-        <x:f>ROUND(D68-E68,1)</x:f>
-        <x:v>21060</x:v>
-      </x:c>
-      <x:c r="J68" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K68" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B69" s="22" t="str">
-        <x:v>9月7日-9月11日</x:v>
-      </x:c>
-      <x:c r="C69" s="23" t="n">
-        <x:v>141000</x:v>
-      </x:c>
-      <x:c r="D69" s="23" t="n">
-        <x:v>143540</x:v>
-      </x:c>
-      <x:c r="E69" s="23" t="n">
-        <x:v>127120</x:v>
-      </x:c>
-      <x:c r="F69" s="23" t="n">
-        <x:v>134340</x:v>
-      </x:c>
-      <x:c r="G69" s="28" t="n">
-        <x:f>ROUND(F69-F68,1)</x:f>
-        <x:v>-7660</x:v>
-      </x:c>
-      <x:c r="H69" s="24" t="n">
-        <x:f>IFERROR(F69/F68-1,"")</x:f>
-        <x:v>-0.05394366197183098</x:v>
-      </x:c>
-      <x:c r="I69" s="26" t="n">
-        <x:f>ROUND(D69-E69,1)</x:f>
-        <x:v>16420</x:v>
-      </x:c>
-      <x:c r="J69" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K69" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B70" s="22" t="str">
-        <x:v>9月14日-9月18日</x:v>
-      </x:c>
-      <x:c r="C70" s="23" t="n">
-        <x:v>133600</x:v>
-      </x:c>
-      <x:c r="D70" s="23" t="n">
-        <x:v>135900</x:v>
-      </x:c>
-      <x:c r="E70" s="23" t="n">
-        <x:v>126200</x:v>
-      </x:c>
-      <x:c r="F70" s="23" t="n">
-        <x:v>128580</x:v>
-      </x:c>
-      <x:c r="G70" s="28" t="n">
-        <x:f>ROUND(F70-F69,1)</x:f>
-        <x:v>-5760</x:v>
-      </x:c>
-      <x:c r="H70" s="24" t="n">
-        <x:f>IFERROR(F70/F69-1,"")</x:f>
-        <x:v>-0.04287628405538191</x:v>
-      </x:c>
-      <x:c r="I70" s="26" t="n">
-        <x:f>ROUND(D70-E70,1)</x:f>
-        <x:v>9700</x:v>
-      </x:c>
-      <x:c r="J70" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K70" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B71" s="22" t="str">
-        <x:v>9月21日-9月24日</x:v>
-      </x:c>
-      <x:c r="C71" s="23" t="n">
-        <x:v>128500</x:v>
-      </x:c>
-      <x:c r="D71" s="23" t="n">
-        <x:v>136560</x:v>
-      </x:c>
-      <x:c r="E71" s="23" t="n">
-        <x:v>125000</x:v>
-      </x:c>
-      <x:c r="F71" s="23" t="n">
-        <x:v>125980</x:v>
-      </x:c>
-      <x:c r="G71" s="28" t="n">
-        <x:f>ROUND(F71-F70,1)</x:f>
-        <x:v>-2600</x:v>
-      </x:c>
-      <x:c r="H71" s="24" t="n">
-        <x:f>IFERROR(F71/F70-1,"")</x:f>
-        <x:v>-0.02022087416394458</x:v>
-      </x:c>
-      <x:c r="I71" s="26" t="n">
-        <x:f>ROUND(D71-E71,1)</x:f>
-        <x:v>11560</x:v>
-      </x:c>
-      <x:c r="J71" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K71" s="22" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B72" s="30" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C72" s="30"/>
-      <x:c r="D72" s="30"/>
-      <x:c r="E72" s="30"/>
-      <x:c r="F72" s="30"/>
-      <x:c r="G72" s="30"/>
-      <x:c r="H72" s="30"/>
-      <x:c r="I72" s="32" t="n">
-        <x:f>ROUND(SUM(I68:I71),1)</x:f>
-        <x:v>58740</x:v>
-      </x:c>
-      <x:c r="J72" s="30"/>
-      <x:c r="K72" s="30"/>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B73" s="30"/>
-      <x:c r="C73" s="30"/>
-      <x:c r="D73" s="30"/>
-      <x:c r="E73" s="30"/>
-      <x:c r="F73" s="30"/>
-      <x:c r="G73" s="30"/>
-      <x:c r="H73" s="30"/>
-      <x:c r="I73" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I68:I71),0),1)</x:f>
+      <x:c r="B77" s="30"/>
+      <x:c r="C77" s="30"/>
+      <x:c r="D77" s="30"/>
+      <x:c r="E77" s="30"/>
+      <x:c r="F77" s="30"/>
+      <x:c r="G77" s="30"/>
+      <x:c r="H77" s="30"/>
+      <x:c r="I77" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I72:I75),0),1)</x:f>
         <x:v>14685</x:v>
       </x:c>
-      <x:c r="J73" s="30"/>
-      <x:c r="K73" s="30"/>
+      <x:c r="J77" s="30"/>
+      <x:c r="K77" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A12:K12"/>
-    <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A30:K30"/>
-    <x:mergeCell ref="A39:K39"/>
-    <x:mergeCell ref="A48:K48"/>
-    <x:mergeCell ref="A57:K57"/>
-    <x:mergeCell ref="A66:K66"/>
+    <x:mergeCell ref="A13:K13"/>
+    <x:mergeCell ref="A23:K23"/>
+    <x:mergeCell ref="A33:K33"/>
+    <x:mergeCell ref="A42:K42"/>
+    <x:mergeCell ref="A52:K52"/>
+    <x:mergeCell ref="A61:K61"/>
+    <x:mergeCell ref="A70:K70"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4247,31 +4399,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>2268.2999999999997</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7551.22</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7551.22</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7246.61</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7294.17</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>-276</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>-0.0364550721651119</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>304.6</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -4279,11 +4449,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>126</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>2572.8999999999996</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>135.4</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4998,31 +5186,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>2109.4999999999995</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7599.2</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7601.09</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7364.43</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7402.3</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>-221.8</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>-0.029088137963056426</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>236.7</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -5030,11 +5236,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>117.2</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>2346.1999999999994</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>123.5</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5749,31 +5973,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>610.8</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>3878.41</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>3878.41</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>3806.67</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>3823.62</x:v>
+      </x:c>
+      <x:c r="H22" s="23" t="n">
+        <x:v>-64.7</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>-0.016652221882176854</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>71.7</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -5781,11 +6023,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>33.9</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>682.5</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>35.9</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7251,31 +7511,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B24" s="30" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="30"/>
-      <x:c r="J24" s="32" t="n">
-        <x:f>SUM(J4:J21)</x:f>
-        <x:v>2489.7999999999997</x:v>
-      </x:c>
-      <x:c r="K24" s="30"/>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>9月28日</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>7440.8</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>7458.4</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>7186</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:v>7270</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="n">
+        <x:v>-181.6</x:v>
+      </x:c>
+      <x:c r="I22" s="24" t="n">
+        <x:v>-0.024370604970744614</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:f>ROUND(E22-F22,1)</x:f>
+        <x:v>272.4</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="C25" s="30"/>
       <x:c r="D25" s="30"/>
       <x:c r="E25" s="30"/>
@@ -7283,11 +7561,29 @@
       <x:c r="G25" s="30"/>
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="30"/>
-      <x:c r="J25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J21),0),1)</x:f>
-        <x:v>138.3</x:v>
+      <x:c r="J25" s="32" t="n">
+        <x:f>SUM(J4:J22)</x:f>
+        <x:v>2762.2</x:v>
       </x:c>
       <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="30"/>
+      <x:c r="E26" s="30"/>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="30"/>
+      <x:c r="J26" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
+        <x:v>145.4</x:v>
+      </x:c>
+      <x:c r="K26" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-29
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R99cde11241914ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R6e6a7e2534a54181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R70feb0f629cb4cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4db30590b0e24236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R26ead102c51f49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R95af62df664c4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R7922d33b85f840d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rf09ba78d12a3473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R624aceea07ac44b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rfc342d3861224624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc1db95b85da34bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R1004d6b96a614b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R83cc833a508b4acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rae6d53544b8d40b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rd4cbc922460146cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re2a160e2b23248a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R70fbd403646c48ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R7ebbf7f55cbe4f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R72e25a6e90364fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R0085b5f451ff4e49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7551.22</x:v>
+        <x:v>7357.03</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7246.61</x:v>
+        <x:v>7256.25</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>304.6</x:v>
+        <x:v>100.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2572.9</x:v>
+        <x:v>2673.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>135.4</x:v>
+        <x:v>133.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7601.09</x:v>
+        <x:v>7473.7</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7364.43</x:v>
+        <x:v>7386.14</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>236.7</x:v>
+        <x:v>87.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2346.2</x:v>
+        <x:v>2433.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>123.5</x:v>
+        <x:v>121.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3878.41</x:v>
+        <x:v>3843.84</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3806.67</x:v>
+        <x:v>3810.81</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>71.7</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>682.5</x:v>
+        <x:v>715.5</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.9</x:v>
+        <x:v>35.8</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>124660</x:v>
+        <x:v>122480</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>119520</x:v>
+        <x:v>118100</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>5140</x:v>
+        <x:v>4380</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>113460</x:v>
+        <x:v>117840</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>5971.6</x:v>
+        <x:v>5892</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1622,31 +1622,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>113460</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>9月29日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>119080</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>122480</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>118100</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>0.00016669444907480013</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>4380</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -1654,11 +1672,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>5971.6</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>117840</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>5892</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1891,7 +1927,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>9月28日</x:v>
+        <x:v>9月28日-9月29日</x:v>
       </x:c>
       <x:c r="C9" s="23" t="n">
         <x:v>7551.22</x:v>
@@ -1903,15 +1939,15 @@
         <x:v>7246.61</x:v>
       </x:c>
       <x:c r="F9" s="23" t="n">
-        <x:v>7294.17</x:v>
+        <x:v>7325.35</x:v>
       </x:c>
       <x:c r="G9" s="28" t="n">
         <x:f>ROUND(F9-F8,1)</x:f>
-        <x:v>-276</x:v>
+        <x:v>-244.8</x:v>
       </x:c>
       <x:c r="H9" s="24" t="n">
         <x:f>IFERROR(F9/F8-1,"")</x:f>
-        <x:v>-0.0364550721651119</x:v>
+        <x:v>-0.03233625798201878</x:v>
       </x:c>
       <x:c r="I9" s="26" t="n">
         <x:f>ROUND(D9-E9,1)</x:f>
@@ -1921,7 +1957,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K9" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2163,7 +2199,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>9月28日</x:v>
+        <x:v>9月28日-9月29日</x:v>
       </x:c>
       <x:c r="C19" s="23" t="n">
         <x:v>7599.2</x:v>
@@ -2175,15 +2211,15 @@
         <x:v>7364.43</x:v>
       </x:c>
       <x:c r="F19" s="23" t="n">
-        <x:v>7402.3</x:v>
+        <x:v>7439.63</x:v>
       </x:c>
       <x:c r="G19" s="28" t="n">
         <x:f>ROUND(F19-F18,1)</x:f>
-        <x:v>-221.8</x:v>
+        <x:v>-184.4</x:v>
       </x:c>
       <x:c r="H19" s="24" t="n">
         <x:f>IFERROR(F19/F18-1,"")</x:f>
-        <x:v>-0.029088137963056426</x:v>
+        <x:v>-0.024191803065816475</x:v>
       </x:c>
       <x:c r="I19" s="26" t="n">
         <x:f>ROUND(D19-E19,1)</x:f>
@@ -2193,7 +2229,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K19" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2435,7 +2471,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>9月28日</x:v>
+        <x:v>9月28日-9月29日</x:v>
       </x:c>
       <x:c r="C29" s="23" t="n">
         <x:v>3878.41</x:v>
@@ -2447,15 +2483,15 @@
         <x:v>3806.67</x:v>
       </x:c>
       <x:c r="F29" s="23" t="n">
-        <x:v>3823.62</x:v>
+        <x:v>3830.45</x:v>
       </x:c>
       <x:c r="G29" s="23" t="n">
         <x:f>ROUND(F29-F28,1)</x:f>
-        <x:v>-64.7</x:v>
+        <x:v>-57.9</x:v>
       </x:c>
       <x:c r="H29" s="24" t="n">
         <x:f>IFERROR(F29/F28-1,"")</x:f>
-        <x:v>-0.016652221882176854</x:v>
+        <x:v>-0.014895701797925653</x:v>
       </x:c>
       <x:c r="I29" s="26" t="n">
         <x:f>ROUND(D29-E29,1)</x:f>
@@ -2465,7 +2501,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K29" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -3795,7 +3831,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B79" s="22" t="str">
-        <x:v>9月28日</x:v>
+        <x:v>9月28日-9月29日</x:v>
       </x:c>
       <x:c r="C79" s="23" t="n">
         <x:v>124280</x:v>
@@ -3804,28 +3840,28 @@
         <x:v>124660</x:v>
       </x:c>
       <x:c r="E79" s="23" t="n">
-        <x:v>119520</x:v>
+        <x:v>118100</x:v>
       </x:c>
       <x:c r="F79" s="23" t="n">
-        <x:v>119980</x:v>
+        <x:v>120000</x:v>
       </x:c>
       <x:c r="G79" s="28" t="n">
         <x:f>ROUND(F79-F78,1)</x:f>
-        <x:v>-6000</x:v>
+        <x:v>-5980</x:v>
       </x:c>
       <x:c r="H79" s="24" t="n">
         <x:f>IFERROR(F79/F78-1,"")</x:f>
-        <x:v>-0.04762660739799973</x:v>
-      </x:c>
-      <x:c r="I79" s="23" t="n">
+        <x:v>-0.047467852040006364</x:v>
+      </x:c>
+      <x:c r="I79" s="26" t="n">
         <x:f>ROUND(D79-E79,1)</x:f>
-        <x:v>5140</x:v>
+        <x:v>6560</x:v>
       </x:c>
       <x:c r="J79" s="22" t="str">
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K79" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3843,7 +3879,7 @@
       <x:c r="H80" s="30"/>
       <x:c r="I80" s="32" t="n">
         <x:f>ROUND(SUM(I75:I79),1)</x:f>
-        <x:v>63880</x:v>
+        <x:v>65300</x:v>
       </x:c>
       <x:c r="J80" s="30"/>
       <x:c r="K80" s="30"/>
@@ -3861,7 +3897,7 @@
       <x:c r="H81" s="30"/>
       <x:c r="I81" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I75:I79),0),1)</x:f>
-        <x:v>12776</x:v>
+        <x:v>13060</x:v>
       </x:c>
       <x:c r="J81" s="30"/>
       <x:c r="K81" s="30"/>
@@ -4623,31 +4659,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>2572.8999999999996</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>9月29日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7265.51</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>7357.03</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7256.25</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>7325.35</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>31.2</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>0.004274646738422705</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>100.8</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -4655,11 +4709,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>135.4</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>2673.7</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>133.7</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5410,31 +5482,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>2346.1999999999994</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>9月29日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7388.11</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>7473.7</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7386.14</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>7439.63</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>37.3</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>0.005043027167231706</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>87.6</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -5442,11 +5532,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>123.5</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>2433.7999999999993</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>121.7</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6197,31 +6305,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B25" s="30" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="30"/>
-      <x:c r="J25" s="32" t="n">
-        <x:f>SUM(J4:J22)</x:f>
-        <x:v>682.5</x:v>
-      </x:c>
-      <x:c r="K25" s="30"/>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>9月29日</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>3816.15</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>3843.84</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>3810.81</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:v>3830.45</x:v>
+      </x:c>
+      <x:c r="H23" s="23" t="n">
+        <x:v>6.8</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="n">
+        <x:v>0.0017862653715587928</x:v>
+      </x:c>
+      <x:c r="J23" s="23" t="n">
+        <x:f>ROUND(E23-F23,1)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B26" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="C26" s="30"/>
       <x:c r="D26" s="30"/>
       <x:c r="E26" s="30"/>
@@ -6229,11 +6355,29 @@
       <x:c r="G26" s="30"/>
       <x:c r="H26" s="30"/>
       <x:c r="I26" s="30"/>
-      <x:c r="J26" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J22),0),1)</x:f>
-        <x:v>35.9</x:v>
+      <x:c r="J26" s="32" t="n">
+        <x:f>SUM(J4:J23)</x:f>
+        <x:v>715.5</x:v>
       </x:c>
       <x:c r="K26" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="30"/>
+      <x:c r="J27" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
+        <x:v>35.8</x:v>
+      </x:c>
+      <x:c r="K27" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-09-30
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rda40fa45999e468d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rf2c7ebd4555845f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdc4704ad74fb4342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R2ad581b18bc545e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R27e71e30e7fd4178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R181475442dc54c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9d92942dcefd4673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Raf01773fa0ab4f40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc4e0559725ea4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R2d713a5fe4c1412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rbeb99358909e4470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rab4098f4a80c46cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R69789068a91d4475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R72b6a386f42347dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rd02a9c305cf64837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R0aace50fe9a5411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd6f3951509a244f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Red87e8a83e134046"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf636a6311d77490a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rcf686a871c8842d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7357.03</x:v>
+        <x:v>7375.44</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7256.25</x:v>
+        <x:v>7288.98</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>100.8</x:v>
+        <x:v>86.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2673.7</x:v>
+        <x:v>2760.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>133.7</x:v>
+        <x:v>131.4</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7473.7</x:v>
+        <x:v>7485.11</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7386.14</x:v>
+        <x:v>7417.49</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>87.6</x:v>
+        <x:v>67.6</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2433.8</x:v>
+        <x:v>2501.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>121.7</x:v>
+        <x:v>119.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3843.84</x:v>
+        <x:v>3851.22</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3810.81</x:v>
+        <x:v>3833.09</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>33</x:v>
+        <x:v>18.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>715.5</x:v>
+        <x:v>733.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>35.8</x:v>
+        <x:v>34.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7226.4</x:v>
+        <x:v>7232</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>7123</x:v>
+        <x:v>7153</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>103.4</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2970.6</x:v>
+        <x:v>3049.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>148.5</x:v>
+        <x:v>145.2</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>7352.8</x:v>
+        <x:v>7344</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>7238</x:v>
+        <x:v>7282</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>114.8</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2877</x:v>
+        <x:v>2939</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>143.9</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2777.8</x:v>
+        <x:v>2782.2</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2752</x:v>
+        <x:v>2762</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>25.8</x:v>
+        <x:v>20.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>637.6</x:v>
+        <x:v>657.8</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>31.9</x:v>
+        <x:v>31.3</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-09-29</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1927,7 +1927,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C9" s="23" t="n">
         <x:v>7551.22</x:v>
@@ -1939,15 +1939,15 @@
         <x:v>7246.61</x:v>
       </x:c>
       <x:c r="F9" s="23" t="n">
-        <x:v>7325.35</x:v>
+        <x:v>7298.82</x:v>
       </x:c>
       <x:c r="G9" s="28" t="n">
         <x:f>ROUND(F9-F8,1)</x:f>
-        <x:v>-244.8</x:v>
+        <x:v>-271.3</x:v>
       </x:c>
       <x:c r="H9" s="24" t="n">
         <x:f>IFERROR(F9/F8-1,"")</x:f>
-        <x:v>-0.03233625798201878</x:v>
+        <x:v>-0.03584081668238637</x:v>
       </x:c>
       <x:c r="I9" s="26" t="n">
         <x:f>ROUND(D9-E9,1)</x:f>
@@ -1957,7 +1957,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K9" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2199,7 +2199,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C19" s="23" t="n">
         <x:v>7599.2</x:v>
@@ -2211,15 +2211,15 @@
         <x:v>7364.43</x:v>
       </x:c>
       <x:c r="F19" s="23" t="n">
-        <x:v>7439.63</x:v>
+        <x:v>7435.16</x:v>
       </x:c>
       <x:c r="G19" s="28" t="n">
         <x:f>ROUND(F19-F18,1)</x:f>
-        <x:v>-184.4</x:v>
+        <x:v>-188.9</x:v>
       </x:c>
       <x:c r="H19" s="24" t="n">
         <x:f>IFERROR(F19/F18-1,"")</x:f>
-        <x:v>-0.024191803065816475</x:v>
+        <x:v>-0.02477810408351444</x:v>
       </x:c>
       <x:c r="I19" s="26" t="n">
         <x:f>ROUND(D19-E19,1)</x:f>
@@ -2229,7 +2229,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K19" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2471,7 +2471,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C29" s="23" t="n">
         <x:v>3878.41</x:v>
@@ -2483,15 +2483,15 @@
         <x:v>3806.67</x:v>
       </x:c>
       <x:c r="F29" s="23" t="n">
-        <x:v>3830.45</x:v>
+        <x:v>3842.19</x:v>
       </x:c>
       <x:c r="G29" s="23" t="n">
         <x:f>ROUND(F29-F28,1)</x:f>
-        <x:v>-57.9</x:v>
+        <x:v>-46.2</x:v>
       </x:c>
       <x:c r="H29" s="24" t="n">
         <x:f>IFERROR(F29/F28-1,"")</x:f>
-        <x:v>-0.014895701797925653</x:v>
+        <x:v>-0.011876441799520077</x:v>
       </x:c>
       <x:c r="I29" s="26" t="n">
         <x:f>ROUND(D29-E29,1)</x:f>
@@ -2501,7 +2501,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K29" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2743,7 +2743,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>7390</x:v>
@@ -2755,15 +2755,15 @@
         <x:v>7076.2</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>7191.2</x:v>
+        <x:v>7168.8</x:v>
       </x:c>
       <x:c r="G39" s="28" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>-199.8</x:v>
+        <x:v>-222.2</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>-0.02703287782438102</x:v>
+        <x:v>-0.030063590853740996</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
@@ -2773,7 +2773,7 @@
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3015,7 +3015,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B49" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C49" s="23" t="n">
         <x:v>7440.8</x:v>
@@ -3027,15 +3027,15 @@
         <x:v>7186</x:v>
       </x:c>
       <x:c r="F49" s="23" t="n">
-        <x:v>7309.6</x:v>
+        <x:v>7310.2</x:v>
       </x:c>
       <x:c r="G49" s="23" t="n">
         <x:f>ROUND(F49-F48,1)</x:f>
-        <x:v>-142</x:v>
+        <x:v>-141.4</x:v>
       </x:c>
       <x:c r="H49" s="24" t="n">
         <x:f>IFERROR(F49/F48-1,"")</x:f>
-        <x:v>-0.019056310054216596</x:v>
+        <x:v>-0.018975790434269224</x:v>
       </x:c>
       <x:c r="I49" s="26" t="n">
         <x:f>ROUND(D49-E49,1)</x:f>
@@ -3045,7 +3045,7 @@
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K49" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3559,7 +3559,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B69" s="22" t="str">
-        <x:v>9月28日-9月29日</x:v>
+        <x:v>9月28日-9月30日</x:v>
       </x:c>
       <x:c r="C69" s="23" t="n">
         <x:v>2802</x:v>
@@ -3571,15 +3571,15 @@
         <x:v>2746</x:v>
       </x:c>
       <x:c r="F69" s="23" t="n">
-        <x:v>2763.6</x:v>
+        <x:v>2778.8</x:v>
       </x:c>
       <x:c r="G69" s="23" t="n">
         <x:f>ROUND(F69-F68,1)</x:f>
-        <x:v>-41</x:v>
+        <x:v>-25.8</x:v>
       </x:c>
       <x:c r="H69" s="24" t="n">
         <x:f>IFERROR(F69/F68-1,"")</x:f>
-        <x:v>-0.014618840476360306</x:v>
+        <x:v>-0.009199172787563215</x:v>
       </x:c>
       <x:c r="I69" s="23" t="n">
         <x:f>ROUND(D69-E69,1)</x:f>
@@ -3589,7 +3589,7 @@
         <x:v>IH2612</x:v>
       </x:c>
       <x:c r="K69" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4695,31 +4695,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>2673.7</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7361.14</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7375.44</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7288.98</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7298.82</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>-26.5</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>-0.0036216699543367703</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>86.5</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -4727,11 +4745,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>133.7</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>2760.2</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>131.4</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5518,31 +5554,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>2433.7999999999993</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7469.05</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7485.11</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7417.49</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7435.16</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>-4.5</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>-0.0006008363319144339</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>67.6</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -5550,11 +5604,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>121.7</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>2501.399999999999</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>119.1</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6341,31 +6413,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>715.5</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>3839.25</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>3851.22</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>3833.09</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>3842.19</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>11.7</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.0030649140440419664</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>18.1</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -6373,11 +6463,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>35.8</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>733.6</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>34.9</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7164,31 +7272,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>2970.6</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7223.6</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7232</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7153</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7168.8</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>-22.4</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>-0.003114918233396269</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -7196,11 +7322,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>148.5</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>3049.6</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>145.2</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7987,31 +8131,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>2877</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>7332</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>7344</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>7282</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>7310.2</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.00008208383495666993</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -8019,11 +8181,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>143.9</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>2939</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9633,31 +9813,49 @@
         <x:v>IH2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B26" s="30" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="30"/>
-      <x:c r="E26" s="30"/>
-      <x:c r="F26" s="30"/>
-      <x:c r="G26" s="30"/>
-      <x:c r="H26" s="30"/>
-      <x:c r="I26" s="30"/>
-      <x:c r="J26" s="32" t="n">
-        <x:f>SUM(J4:J23)</x:f>
-        <x:v>637.5999999999999</x:v>
-      </x:c>
-      <x:c r="K26" s="30"/>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>9月30日</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>2769.6</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>2782.2</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:v>2778.8</x:v>
+      </x:c>
+      <x:c r="H24" s="23" t="n">
+        <x:v>15.2</x:v>
+      </x:c>
+      <x:c r="I24" s="24" t="n">
+        <x:v>0.005500072369373443</x:v>
+      </x:c>
+      <x:c r="J24" s="23" t="n">
+        <x:f>ROUND(E24-F24,1)</x:f>
+        <x:v>20.2</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B27" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="C27" s="30"/>
       <x:c r="D27" s="30"/>
       <x:c r="E27" s="30"/>
@@ -9665,11 +9863,29 @@
       <x:c r="G27" s="30"/>
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="30"/>
-      <x:c r="J27" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J23),0),1)</x:f>
-        <x:v>31.9</x:v>
+      <x:c r="J27" s="32" t="n">
+        <x:f>SUM(J4:J24)</x:f>
+        <x:v>657.8</x:v>
       </x:c>
       <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="30"/>
+      <x:c r="J28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J24),0),1)</x:f>
+        <x:v>31.3</x:v>
+      </x:c>
+      <x:c r="K28" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-01
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rbfd9b54494214b3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rf8b611efafa64b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R141a444e9c984089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R41c591ae61c34592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rb67e48140e47440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R4c134df6310c4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R6e4761f2d02248b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rfcdd827fd2f94826"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R882c7efcf6964597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R0c7d1339dc444fd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R25e2f40fbd4943ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rc20e95cac2e14bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R74feed225d0d4fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R0b84cb61de1441c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R974d89fb255b4ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re82d3e485bd54e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9dc51fbc76e64e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rf3da90fc811048b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rce90ed79318c4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf137b4663d9a4579"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-02
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R25e2f40fbd4943ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rc20e95cac2e14bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R74feed225d0d4fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R0b84cb61de1441c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R974d89fb255b4ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re82d3e485bd54e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9dc51fbc76e64e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rf3da90fc811048b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rce90ed79318c4945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf137b4663d9a4579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rfb8360900c0c42cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Ra005a4adb7114b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R24174142ebae43ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4d9cd30c0fec415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9655c29dcc974f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R47b313dc76294218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R7ee756a70d2f4c57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd55d1571f60c4f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rcbd8ebca814e41df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rfa935d0be38e4902"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -617,7 +617,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-01</x:v>
+        <x:v>2026-10-02</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-05
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rba2b838a769347b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rcc3c710350c2443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R87b43001949d4274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R924d2d9755b3428f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Raeba3ee1a0af4638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb9e954b4d4c349bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9d9cad8fd3024877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R553f8372dde54871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R2d82f40f8a6c43ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R3f2166ae16cb4486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rf1c82e9090d64f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R635eb18d88414b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9080be732e414d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R37acd4e8539a445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Ree052e8fcea34b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R81481d8c1ef748cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R22791ebc6fff465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd96b6a63e06b44da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R4c0dae1fe8d84dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R223312e103784969"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -617,7 +617,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-02</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-06
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7212f5ad82ba4355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfd85d03257754909"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R7db24a98a7e940b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R3eddee4293bc4b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R59e00a39ff634b1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R1ed18c00f0714b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rd66f3fa4c95e46a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rff8fba5ed43f4915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R7f72ae2e43234f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R70f32d65bf394c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R8a5c9d3d7af14f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R636bdf70ef714a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R898f710c4d924065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R4a42911139ab447c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rad1586e6d8e84d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Redb57152e75445b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R383adcc3550947bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rec8875c05a3f4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf145ca43a6924a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R772388493ede436c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -617,7 +617,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-07
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R13e8096c3579475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R4bc10fdd06b34d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6fa23374e285490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R224dc67ed491409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc4f878d035a34ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Ra5593a2d85c54338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R1c290005fc654807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Raed6623edd8a4715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R43f71d88b7924b7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rb70188d1b0d74cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc87fc52944ad475e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re1cde86c6807486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1b7f9bda1f034e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R9d4d060bd1744b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7a1c9b18af294a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R29be668a4e274da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rff171a81bb3b498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R391ac9f442a94316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R34e505d38bc146fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R268b253728d84899"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -617,7 +617,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-06</x:v>
+        <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-08
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R33f6abaf4e8a4c94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re71ea2363f2747c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf8a62df4a74d45b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rc9ef972bc261484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R36d0976a5f2f4a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd402681128954469"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R83c1fdbf64d743d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Raa4f61ecb1154a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R334786c2a62f4b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R5d8d7b648a784887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R9018d3343e6d474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8ed67dba783241ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R2bbae6a86abc4d56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R72e236accdf94641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R63e1868cc9b04243"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rc47f1ed6d0f74a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re417c1eca8fd418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Ra41650a730c44954"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rc81bb19f2f8a41b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rab4edee0959546b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,8 +71,14 @@
       <x:color rgb="FFE11D48"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D4ED8"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +103,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFDBFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -134,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -172,6 +183,40 @@
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -184,32 +229,13 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -461,17 +487,27 @@
       <x:c r="A4" s="9" t="str">
         <x:v>中证1000</x:v>
       </x:c>
-      <x:c r="B4" s="9" t="str"/>
-      <x:c r="C4" s="10" t="str"/>
-      <x:c r="D4" s="10" t="str"/>
-      <x:c r="E4" s="12" t="str"/>
+      <x:c r="B4" s="9" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="n">
+        <x:v>7366.86</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="n">
+        <x:v>7087.8</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:v>279.1</x:v>
+      </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="10" t="str"/>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="H4" s="10" t="n">
+        <x:v>279.1</x:v>
+      </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
       </x:c>
@@ -480,17 +516,27 @@
       <x:c r="A5" s="9" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B5" s="9" t="str"/>
-      <x:c r="C5" s="10" t="str"/>
-      <x:c r="D5" s="10" t="str"/>
-      <x:c r="E5" s="12" t="str"/>
+      <x:c r="B5" s="9" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="n">
+        <x:v>7461.24</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="n">
+        <x:v>7206.06</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>255.2</x:v>
+      </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H5" s="10" t="str"/>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="n">
+        <x:v>255.2</x:v>
+      </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
       </x:c>
@@ -499,17 +545,27 @@
       <x:c r="A6" s="9" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B6" s="9" t="str"/>
-      <x:c r="C6" s="10" t="str"/>
-      <x:c r="D6" s="10" t="str"/>
-      <x:c r="E6" s="12" t="str"/>
+      <x:c r="B6" s="9" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="n">
+        <x:v>3864.12</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="n">
+        <x:v>3795.37</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>68.8</x:v>
+      </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="10" t="str"/>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="H6" s="10" t="n">
+        <x:v>68.8</x:v>
+      </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
       </x:c>
@@ -518,17 +574,27 @@
       <x:c r="A7" s="9" t="str">
         <x:v>IM主力</x:v>
       </x:c>
-      <x:c r="B7" s="9" t="str"/>
-      <x:c r="C7" s="10" t="str"/>
-      <x:c r="D7" s="10" t="str"/>
-      <x:c r="E7" s="12" t="str"/>
+      <x:c r="B7" s="9" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="n">
+        <x:v>6948.2</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:v>303.6</x:v>
+      </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H7" s="10" t="str"/>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="n">
+        <x:v>303.6</x:v>
+      </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
       </x:c>
@@ -537,17 +603,27 @@
       <x:c r="A8" s="9" t="str">
         <x:v>IC主力</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="str"/>
-      <x:c r="C8" s="10" t="str"/>
-      <x:c r="D8" s="10" t="str"/>
-      <x:c r="E8" s="12" t="str"/>
+      <x:c r="B8" s="9" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="n">
+        <x:v>7056.4</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:v>298.6</x:v>
+      </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="10" t="str"/>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="H8" s="10" t="n">
+        <x:v>298.6</x:v>
+      </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
       </x:c>
@@ -617,7 +693,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-07</x:v>
+        <x:v>2026-10-08</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -801,55 +877,55 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22"/>
+      <x:c r="B4" s="22"/>
+      <x:c r="C4" s="22"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="24"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="22"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
+      <x:c r="B7" s="28" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="31"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="31"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -932,153 +1008,198 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B5" s="21"/>
-      <x:c r="C5" s="21"/>
-      <x:c r="D5" s="21"/>
-      <x:c r="E5" s="21"/>
-      <x:c r="F5" s="21"/>
-      <x:c r="G5" s="21"/>
-      <x:c r="H5" s="21"/>
-      <x:c r="I5" s="21"/>
-      <x:c r="J5" s="21"/>
-      <x:c r="K5" s="21"/>
+      <x:c r="A5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="n">
+        <x:v>7306.74</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7366.86</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7087.8</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7138.58</x:v>
+      </x:c>
+      <x:c r="G5" s="23"/>
+      <x:c r="H5" s="24"/>
+      <x:c r="I5" s="26" t="n">
+        <x:f>ROUND(D5-E5,1)</x:f>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="J5" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B6" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="28"/>
+      <x:c r="D6" s="28"/>
+      <x:c r="E6" s="28"/>
+      <x:c r="F6" s="28"/>
+      <x:c r="G6" s="28"/>
+      <x:c r="H6" s="28"/>
+      <x:c r="I6" s="30" t="n">
+        <x:f>ROUND(SUM(I5:I5),1)</x:f>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="J6" s="28"/>
+      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="17" t="str">
+      <x:c r="A7" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B7" s="28"/>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="J7" s="28"/>
+      <x:c r="K7" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B7" s="17"/>
-      <x:c r="C7" s="17"/>
-      <x:c r="D7" s="17"/>
-      <x:c r="E7" s="17"/>
-      <x:c r="F7" s="17"/>
-      <x:c r="G7" s="17"/>
-      <x:c r="H7" s="17"/>
-      <x:c r="I7" s="17"/>
-      <x:c r="J7" s="17"/>
-      <x:c r="K7" s="17"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="20" t="str">
+      <x:c r="B9" s="17"/>
+      <x:c r="C9" s="17"/>
+      <x:c r="D9" s="17"/>
+      <x:c r="E9" s="17"/>
+      <x:c r="F9" s="17"/>
+      <x:c r="G9" s="17"/>
+      <x:c r="H9" s="17"/>
+      <x:c r="I9" s="17"/>
+      <x:c r="J9" s="17"/>
+      <x:c r="K9" s="17"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B8" s="20" t="str">
+      <x:c r="B10" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C8" s="20" t="str">
+      <x:c r="C10" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D8" s="20" t="str">
+      <x:c r="D10" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E8" s="20" t="str">
+      <x:c r="E10" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F8" s="20" t="str">
+      <x:c r="F10" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G8" s="20" t="str">
+      <x:c r="G10" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H8" s="20" t="str">
+      <x:c r="H10" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I8" s="20" t="str">
+      <x:c r="I10" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J8" s="20" t="str">
+      <x:c r="J10" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K8" s="20" t="str">
+      <x:c r="K10" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B9" s="21"/>
-      <x:c r="C9" s="21"/>
-      <x:c r="D9" s="21"/>
-      <x:c r="E9" s="21"/>
-      <x:c r="F9" s="21"/>
-      <x:c r="G9" s="21"/>
-      <x:c r="H9" s="21"/>
-      <x:c r="I9" s="21"/>
-      <x:c r="J9" s="21"/>
-      <x:c r="K9" s="21"/>
-    </x:row>
     <x:row r="11">
-      <x:c r="A11" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B11" s="17"/>
-      <x:c r="C11" s="17"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="17"/>
-      <x:c r="F11" s="17"/>
-      <x:c r="G11" s="17"/>
-      <x:c r="H11" s="17"/>
-      <x:c r="I11" s="17"/>
-      <x:c r="J11" s="17"/>
-      <x:c r="K11" s="17"/>
+      <x:c r="A11" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="n">
+        <x:v>7420.44</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>7461.24</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>7206.06</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>7248.43</x:v>
+      </x:c>
+      <x:c r="G11" s="23"/>
+      <x:c r="H11" s="24"/>
+      <x:c r="I11" s="26" t="n">
+        <x:f>ROUND(D11-E11,1)</x:f>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="J11" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B12" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C12" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D12" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E12" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F12" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G12" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H12" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I12" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J12" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K12" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
+      <x:c r="A12" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="30" t="n">
+        <x:f>ROUND(SUM(I11:I11),1)</x:f>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="J12" s="28"/>
+      <x:c r="K12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B13" s="21"/>
-      <x:c r="C13" s="21"/>
-      <x:c r="D13" s="21"/>
-      <x:c r="E13" s="21"/>
-      <x:c r="F13" s="21"/>
-      <x:c r="G13" s="21"/>
-      <x:c r="H13" s="21"/>
-      <x:c r="I13" s="21"/>
-      <x:c r="J13" s="21"/>
-      <x:c r="K13" s="21"/>
+      <x:c r="A13" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="28"/>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="J13" s="28"/>
+      <x:c r="K13" s="28"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="17" t="str">
-        <x:v>IM主力</x:v>
+        <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B15" s="17"/>
       <x:c r="C15" s="17"/>
@@ -1127,153 +1248,198 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B17" s="21"/>
-      <x:c r="C17" s="21"/>
-      <x:c r="D17" s="21"/>
-      <x:c r="E17" s="21"/>
-      <x:c r="F17" s="21"/>
-      <x:c r="G17" s="21"/>
-      <x:c r="H17" s="21"/>
-      <x:c r="I17" s="21"/>
-      <x:c r="J17" s="21"/>
-      <x:c r="K17" s="21"/>
+      <x:c r="A17" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="n">
+        <x:v>3838.98</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>3864.12</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>3795.37</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>3811.9</x:v>
+      </x:c>
+      <x:c r="G17" s="23"/>
+      <x:c r="H17" s="24"/>
+      <x:c r="I17" s="26" t="n">
+        <x:f>ROUND(D17-E17,1)</x:f>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="J17" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="30" t="n">
+        <x:f>ROUND(SUM(I17:I17),1)</x:f>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="J18" s="28"/>
+      <x:c r="K18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B19" s="17"/>
-      <x:c r="C19" s="17"/>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="17"/>
-      <x:c r="F19" s="17"/>
-      <x:c r="G19" s="17"/>
-      <x:c r="H19" s="17"/>
-      <x:c r="I19" s="17"/>
-      <x:c r="J19" s="17"/>
-      <x:c r="K19" s="17"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="20" t="str">
+      <x:c r="A19" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="28"/>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="J19" s="28"/>
+      <x:c r="K19" s="28"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B21" s="17"/>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="17"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="17"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B20" s="20" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D20" s="20" t="str">
+      <x:c r="D22" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="str">
+      <x:c r="E22" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
+      <x:c r="F22" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="str">
+      <x:c r="G22" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H20" s="20" t="str">
+      <x:c r="H22" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I20" s="20" t="str">
+      <x:c r="I22" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J20" s="20" t="str">
+      <x:c r="J22" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K20" s="20" t="str">
+      <x:c r="K22" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B21" s="21"/>
-      <x:c r="C21" s="21"/>
-      <x:c r="D21" s="21"/>
-      <x:c r="E21" s="21"/>
-      <x:c r="F21" s="21"/>
-      <x:c r="G21" s="21"/>
-      <x:c r="H21" s="21"/>
-      <x:c r="I21" s="21"/>
-      <x:c r="J21" s="21"/>
-      <x:c r="K21" s="21"/>
-    </x:row>
     <x:row r="23">
-      <x:c r="A23" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B23" s="17"/>
-      <x:c r="C23" s="17"/>
-      <x:c r="D23" s="17"/>
-      <x:c r="E23" s="17"/>
-      <x:c r="F23" s="17"/>
-      <x:c r="G23" s="17"/>
-      <x:c r="H23" s="17"/>
-      <x:c r="I23" s="17"/>
-      <x:c r="J23" s="17"/>
-      <x:c r="K23" s="17"/>
+      <x:c r="A23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="n">
+        <x:v>7182.8</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>6948.2</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>7022.2</x:v>
+      </x:c>
+      <x:c r="G23" s="23"/>
+      <x:c r="H23" s="24"/>
+      <x:c r="I23" s="26" t="n">
+        <x:f>ROUND(D23-E23,1)</x:f>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B24" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C24" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D24" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E24" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F24" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G24" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H24" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I24" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J24" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K24" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
+      <x:c r="A24" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C24" s="28"/>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="30" t="n">
+        <x:f>ROUND(SUM(I23:I23),1)</x:f>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="21" t="str">
-        <x:v>暂无数据</x:v>
-      </x:c>
-      <x:c r="B25" s="21"/>
-      <x:c r="C25" s="21"/>
-      <x:c r="D25" s="21"/>
-      <x:c r="E25" s="21"/>
-      <x:c r="F25" s="21"/>
-      <x:c r="G25" s="21"/>
-      <x:c r="H25" s="21"/>
-      <x:c r="I25" s="21"/>
-      <x:c r="J25" s="21"/>
-      <x:c r="K25" s="21"/>
+      <x:c r="A25" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B25" s="28"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str">
-        <x:v>IH主力</x:v>
+        <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B27" s="17"/>
       <x:c r="C27" s="17"/>
@@ -1322,104 +1488,284 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="21" t="str">
+      <x:c r="A29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="n">
+        <x:v>7295</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>7056.4</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>7122.8</x:v>
+      </x:c>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C30" s="28"/>
+      <x:c r="D30" s="28"/>
+      <x:c r="E30" s="28"/>
+      <x:c r="F30" s="28"/>
+      <x:c r="G30" s="28"/>
+      <x:c r="H30" s="28"/>
+      <x:c r="I30" s="30" t="n">
+        <x:f>ROUND(SUM(I29:I29),1)</x:f>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="J30" s="28"/>
+      <x:c r="K30" s="28"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B31" s="28"/>
+      <x:c r="C31" s="28"/>
+      <x:c r="D31" s="28"/>
+      <x:c r="E31" s="28"/>
+      <x:c r="F31" s="28"/>
+      <x:c r="G31" s="28"/>
+      <x:c r="H31" s="28"/>
+      <x:c r="I31" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="J31" s="28"/>
+      <x:c r="K31" s="28"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B33" s="17"/>
+      <x:c r="C33" s="17"/>
+      <x:c r="D33" s="17"/>
+      <x:c r="E33" s="17"/>
+      <x:c r="F33" s="17"/>
+      <x:c r="G33" s="17"/>
+      <x:c r="H33" s="17"/>
+      <x:c r="I33" s="17"/>
+      <x:c r="J33" s="17"/>
+      <x:c r="K33" s="17"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C34" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E34" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F34" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G34" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H34" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I34" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J34" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K34" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="33" t="str">
         <x:v>暂无数据</x:v>
       </x:c>
-      <x:c r="B29" s="21"/>
-      <x:c r="C29" s="21"/>
-      <x:c r="D29" s="21"/>
-      <x:c r="E29" s="21"/>
-      <x:c r="F29" s="21"/>
-      <x:c r="G29" s="21"/>
-      <x:c r="H29" s="21"/>
-      <x:c r="I29" s="21"/>
-      <x:c r="J29" s="21"/>
-      <x:c r="K29" s="21"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="17" t="str">
+      <x:c r="B35" s="33"/>
+      <x:c r="C35" s="33"/>
+      <x:c r="D35" s="33"/>
+      <x:c r="E35" s="33"/>
+      <x:c r="F35" s="33"/>
+      <x:c r="G35" s="33"/>
+      <x:c r="H35" s="33"/>
+      <x:c r="I35" s="33"/>
+      <x:c r="J35" s="33"/>
+      <x:c r="K35" s="33"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B37" s="17"/>
+      <x:c r="C37" s="17"/>
+      <x:c r="D37" s="17"/>
+      <x:c r="E37" s="17"/>
+      <x:c r="F37" s="17"/>
+      <x:c r="G37" s="17"/>
+      <x:c r="H37" s="17"/>
+      <x:c r="I37" s="17"/>
+      <x:c r="J37" s="17"/>
+      <x:c r="K37" s="17"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B38" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C38" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D38" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E38" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F38" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G38" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H38" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I38" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J38" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K38" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="33" t="str">
+        <x:v>暂无数据</x:v>
+      </x:c>
+      <x:c r="B39" s="33"/>
+      <x:c r="C39" s="33"/>
+      <x:c r="D39" s="33"/>
+      <x:c r="E39" s="33"/>
+      <x:c r="F39" s="33"/>
+      <x:c r="G39" s="33"/>
+      <x:c r="H39" s="33"/>
+      <x:c r="I39" s="33"/>
+      <x:c r="J39" s="33"/>
+      <x:c r="K39" s="33"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="17" t="str">
         <x:v>碳酸锂2610</x:v>
       </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
+      <x:c r="B41" s="17"/>
+      <x:c r="C41" s="17"/>
+      <x:c r="D41" s="17"/>
+      <x:c r="E41" s="17"/>
+      <x:c r="F41" s="17"/>
+      <x:c r="G41" s="17"/>
+      <x:c r="H41" s="17"/>
+      <x:c r="I41" s="17"/>
+      <x:c r="J41" s="17"/>
+      <x:c r="K41" s="17"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B32" s="20" t="str">
+      <x:c r="B42" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C32" s="20" t="str">
+      <x:c r="C42" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D32" s="20" t="str">
+      <x:c r="D42" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E32" s="20" t="str">
+      <x:c r="E42" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
+      <x:c r="F42" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G32" s="20" t="str">
+      <x:c r="G42" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="str">
+      <x:c r="H42" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I32" s="20" t="str">
+      <x:c r="I42" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J32" s="20" t="str">
+      <x:c r="J42" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K32" s="20" t="str">
+      <x:c r="K42" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="21" t="str">
+    <x:row r="43">
+      <x:c r="A43" s="33" t="str">
         <x:v>暂无数据</x:v>
       </x:c>
-      <x:c r="B33" s="21"/>
-      <x:c r="C33" s="21"/>
-      <x:c r="D33" s="21"/>
-      <x:c r="E33" s="21"/>
-      <x:c r="F33" s="21"/>
-      <x:c r="G33" s="21"/>
-      <x:c r="H33" s="21"/>
-      <x:c r="I33" s="21"/>
-      <x:c r="J33" s="21"/>
-      <x:c r="K33" s="21"/>
+      <x:c r="B43" s="33"/>
+      <x:c r="C43" s="33"/>
+      <x:c r="D43" s="33"/>
+      <x:c r="E43" s="33"/>
+      <x:c r="F43" s="33"/>
+      <x:c r="G43" s="33"/>
+      <x:c r="H43" s="33"/>
+      <x:c r="I43" s="33"/>
+      <x:c r="J43" s="33"/>
+      <x:c r="K43" s="33"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A5:K5"/>
-    <x:mergeCell ref="A7:K7"/>
     <x:mergeCell ref="A9:K9"/>
-    <x:mergeCell ref="A11:K11"/>
-    <x:mergeCell ref="A13:K13"/>
     <x:mergeCell ref="A15:K15"/>
-    <x:mergeCell ref="A17:K17"/>
-    <x:mergeCell ref="A19:K19"/>
     <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A23:K23"/>
-    <x:mergeCell ref="A25:K25"/>
     <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A29:K29"/>
-    <x:mergeCell ref="A31:K31"/>
     <x:mergeCell ref="A33:K33"/>
+    <x:mergeCell ref="A35:K35"/>
+    <x:mergeCell ref="A37:K37"/>
+    <x:mergeCell ref="A39:K39"/>
+    <x:mergeCell ref="A41:K41"/>
+    <x:mergeCell ref="A43:K43"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1483,55 +1829,78 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7306.74</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7366.86</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>7087.8</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7138.58</x:v>
+      </x:c>
+      <x:c r="H4" s="38" t="n">
+        <x:v>-160.2</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.02195423369804983</x:v>
+      </x:c>
+      <x:c r="J4" s="26" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="31"/>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="31"/>
+        <x:v>279.1</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1599,55 +1968,78 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7420.44</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7461.24</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>7206.06</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7248.43</x:v>
+      </x:c>
+      <x:c r="H4" s="38" t="n">
+        <x:v>-186.7</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.025114456178481626</x:v>
+      </x:c>
+      <x:c r="J4" s="26" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="31"/>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="31"/>
+        <x:v>255.2</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1715,55 +2107,78 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>3838.98</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>3864.12</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>3795.37</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>3811.9</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-30.3</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.007883524760618266</x:v>
+      </x:c>
+      <x:c r="J4" s="26" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="31"/>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="31"/>
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1831,55 +2246,78 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7182.8</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>6948.2</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7022.2</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="n">
+        <x:v>-146.6</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.02044972659301425</x:v>
+      </x:c>
+      <x:c r="J4" s="26" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="31"/>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="31"/>
+        <x:v>303.6</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1947,55 +2385,78 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>10月8日</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="n">
+        <x:v>7295</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="n">
+        <x:v>7056.4</x:v>
+      </x:c>
+      <x:c r="G4" s="23" t="n">
+        <x:v>7122.8</x:v>
+      </x:c>
+      <x:c r="H4" s="38" t="n">
+        <x:v>-187.4</x:v>
+      </x:c>
+      <x:c r="I4" s="24" t="n">
+        <x:v>-0.02563541353177745</x:v>
+      </x:c>
+      <x:c r="J4" s="26" t="n">
+        <x:f>ROUND(E4-F4,1)</x:f>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="B7" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="31"/>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="31"/>
+        <x:v>298.6</x:v>
+      </x:c>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2063,55 +2524,55 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22"/>
+      <x:c r="B4" s="22"/>
+      <x:c r="C4" s="22"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="24"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="22"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
+      <x:c r="B7" s="28" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="31"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="31"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2179,55 +2640,55 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="25"/>
-      <x:c r="B4" s="25"/>
-      <x:c r="C4" s="25"/>
-      <x:c r="D4" s="26"/>
-      <x:c r="E4" s="26"/>
-      <x:c r="F4" s="26"/>
-      <x:c r="G4" s="26"/>
-      <x:c r="H4" s="26"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="26"/>
-      <x:c r="K4" s="25"/>
+      <x:c r="A4" s="22"/>
+      <x:c r="B4" s="22"/>
+      <x:c r="C4" s="22"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="24"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="22"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B7" s="31" t="n">
+      <x:c r="B7" s="28" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="31"/>
-      <x:c r="J7" s="32" t="n">
+      <x:c r="C7" s="28"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="28"/>
+      <x:c r="F7" s="28"/>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="30" t="n">
         <x:f>SUM(J4:J4)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="31"/>
+      <x:c r="K7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="30" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="31"/>
-      <x:c r="C8" s="31"/>
-      <x:c r="D8" s="31"/>
-      <x:c r="E8" s="31"/>
-      <x:c r="F8" s="31"/>
-      <x:c r="G8" s="31"/>
-      <x:c r="H8" s="31"/>
-      <x:c r="I8" s="31"/>
-      <x:c r="J8" s="34" t="n">
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="31"/>
+      <x:c r="K8" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-09
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R85f1825adb8e4791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R7ddf818262574301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R92fd78210e324623"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R9442735c7f584913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rcf33dbc244a34dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd33f7caf6dce4b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R063de2fa309a40e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R3577d9704b814ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R42fe9f161a4547bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R7fdcacf3e03445c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5f2b9e143a4043ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8feb8bc1f46a460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ree38798f50e24ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R1f9c9f975c324bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R6bdc263c88bc494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rd6417a3e3d6c4990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R180915db7e714188"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R28bf4aff52d14d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf2a7e2d4905d43ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R753bed1ae8de403a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7366.86</x:v>
+        <x:v>7175.33</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7087.8</x:v>
+        <x:v>6925.42</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>279.1</x:v>
+        <x:v>249.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>279.1</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>279.1</x:v>
+        <x:v>264.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7461.24</x:v>
+        <x:v>7277.14</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7206.06</x:v>
+        <x:v>7048.45</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>255.2</x:v>
+        <x:v>228.7</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>255.2</x:v>
+        <x:v>483.9</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>255.2</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3864.12</x:v>
+        <x:v>3824.71</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3795.37</x:v>
+        <x:v>3754.14</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>68.8</x:v>
+        <x:v>70.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>68.8</x:v>
+        <x:v>139.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>68.8</x:v>
+        <x:v>69.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7251.8</x:v>
+        <x:v>7049</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6948.2</x:v>
+        <x:v>6819.2</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>303.6</x:v>
+        <x:v>229.8</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>303.6</x:v>
+        <x:v>533.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>303.6</x:v>
+        <x:v>266.7</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>126800</x:v>
+        <x:v>123200</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>120000</x:v>
+        <x:v>119000</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>6800</x:v>
+        <x:v>4200</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>6800</x:v>
+        <x:v>11000</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>6800</x:v>
+        <x:v>5500</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -939,31 +939,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="30" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>6800</x:v>
-      </x:c>
-      <x:c r="K7" s="28"/>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>10月9日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>122300</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>123200</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>119000</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>121000</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.008333333333333304</x:v>
+      </x:c>
+      <x:c r="J5" s="23" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>4200</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
@@ -971,11 +989,29 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="28"/>
-      <x:c r="J8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>6800</x:v>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>11000</x:v>
       </x:c>
       <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>5500</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1062,7 +1098,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>10月8日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C5" s="23" t="n">
         <x:v>7306.74</x:v>
@@ -1071,22 +1107,22 @@
         <x:v>7366.86</x:v>
       </x:c>
       <x:c r="E5" s="23" t="n">
-        <x:v>7087.8</x:v>
+        <x:v>6925.42</x:v>
       </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>7138.58</x:v>
+        <x:v>7155.91</x:v>
       </x:c>
       <x:c r="G5" s="23"/>
       <x:c r="H5" s="24"/>
       <x:c r="I5" s="26" t="n">
         <x:f>ROUND(D5-E5,1)</x:f>
-        <x:v>279.1</x:v>
+        <x:v>441.4</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K5" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1104,7 +1140,7 @@
       <x:c r="H6" s="28"/>
       <x:c r="I6" s="30" t="n">
         <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>279.1</x:v>
+        <x:v>441.4</x:v>
       </x:c>
       <x:c r="J6" s="28"/>
       <x:c r="K6" s="28"/>
@@ -1122,7 +1158,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>279.1</x:v>
+        <x:v>441.4</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1182,7 +1218,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>10月8日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C11" s="23" t="n">
         <x:v>7420.44</x:v>
@@ -1191,22 +1227,22 @@
         <x:v>7461.24</x:v>
       </x:c>
       <x:c r="E11" s="23" t="n">
-        <x:v>7206.06</x:v>
+        <x:v>7048.45</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n">
-        <x:v>7248.43</x:v>
+        <x:v>7251.01</x:v>
       </x:c>
       <x:c r="G11" s="23"/>
       <x:c r="H11" s="24"/>
       <x:c r="I11" s="26" t="n">
         <x:f>ROUND(D11-E11,1)</x:f>
-        <x:v>255.2</x:v>
+        <x:v>412.8</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K11" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1224,7 +1260,7 @@
       <x:c r="H12" s="28"/>
       <x:c r="I12" s="30" t="n">
         <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>255.2</x:v>
+        <x:v>412.8</x:v>
       </x:c>
       <x:c r="J12" s="28"/>
       <x:c r="K12" s="28"/>
@@ -1242,7 +1278,7 @@
       <x:c r="H13" s="28"/>
       <x:c r="I13" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>255.2</x:v>
+        <x:v>412.8</x:v>
       </x:c>
       <x:c r="J13" s="28"/>
       <x:c r="K13" s="28"/>
@@ -1302,7 +1338,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>10月8日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>3838.98</x:v>
@@ -1311,22 +1347,22 @@
         <x:v>3864.12</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>3795.37</x:v>
+        <x:v>3754.14</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>3811.9</x:v>
+        <x:v>3813.79</x:v>
       </x:c>
       <x:c r="G17" s="23"/>
       <x:c r="H17" s="24"/>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>68.8</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1344,7 +1380,7 @@
       <x:c r="H18" s="28"/>
       <x:c r="I18" s="30" t="n">
         <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>68.8</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J18" s="28"/>
       <x:c r="K18" s="28"/>
@@ -1362,7 +1398,7 @@
       <x:c r="H19" s="28"/>
       <x:c r="I19" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>68.8</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J19" s="28"/>
       <x:c r="K19" s="28"/>
@@ -1422,7 +1458,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月8日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>7182.8</x:v>
@@ -1431,22 +1467,22 @@
         <x:v>7251.8</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>6948.2</x:v>
+        <x:v>6819.2</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>7022.2</x:v>
+        <x:v>7015.8</x:v>
       </x:c>
       <x:c r="G23" s="23"/>
       <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>303.6</x:v>
+        <x:v>432.6</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1464,7 +1500,7 @@
       <x:c r="H24" s="28"/>
       <x:c r="I24" s="30" t="n">
         <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>303.6</x:v>
+        <x:v>432.6</x:v>
       </x:c>
       <x:c r="J24" s="28"/>
       <x:c r="K24" s="28"/>
@@ -1482,7 +1518,7 @@
       <x:c r="H25" s="28"/>
       <x:c r="I25" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>303.6</x:v>
+        <x:v>432.6</x:v>
       </x:c>
       <x:c r="J25" s="28"/>
       <x:c r="K25" s="28"/>
@@ -1902,7 +1938,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>10月8日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>120020</x:v>
@@ -1911,22 +1947,22 @@
         <x:v>126800</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>120000</x:v>
+        <x:v>119000</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>120000</x:v>
+        <x:v>121000</x:v>
       </x:c>
       <x:c r="G47" s="23"/>
       <x:c r="H47" s="24"/>
       <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>6800</x:v>
+        <x:v>7800</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1944,7 +1980,7 @@
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
         <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>6800</x:v>
+        <x:v>7800</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -1962,7 +1998,7 @@
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>6800</x:v>
+        <x:v>7800</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
@@ -2076,31 +2112,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="30" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>279.1</x:v>
-      </x:c>
-      <x:c r="K7" s="28"/>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>10月9日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7107.54</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7175.33</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>6925.42</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7155.91</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>17.3</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.0024276536790230896</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>249.9</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
@@ -2108,11 +2162,29 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="28"/>
-      <x:c r="J8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>279.1</x:v>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>264.5</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2215,31 +2287,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="30" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>255.2</x:v>
-      </x:c>
-      <x:c r="K7" s="28"/>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>10月9日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7209.86</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7277.14</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>7048.45</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7251.01</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>2.6</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.000355939148201756</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>228.7</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
@@ -2247,11 +2337,29 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="28"/>
-      <x:c r="J8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>255.2</x:v>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>483.9</x:v>
       </x:c>
       <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2354,31 +2462,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="30" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>68.8</x:v>
-      </x:c>
-      <x:c r="K7" s="28"/>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>10月9日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>3804.09</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>3824.71</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>3754.14</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>3813.79</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>0.0004958157349352899</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>70.6</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
@@ -2386,11 +2512,29 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="28"/>
-      <x:c r="J8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>68.8</x:v>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>139.39999999999998</x:v>
       </x:c>
       <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>69.7</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2493,31 +2637,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="30" t="n">
-        <x:f>SUM(J4:J4)</x:f>
-        <x:v>303.6</x:v>
-      </x:c>
-      <x:c r="K7" s="28"/>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>10月9日</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="n">
+        <x:v>7001.4</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>7049</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="n">
+        <x:v>6819.2</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="n">
+        <x:v>7015.8</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>-6.4</x:v>
+      </x:c>
+      <x:c r="I5" s="24" t="n">
+        <x:v>-0.0009113952892255694</x:v>
+      </x:c>
+      <x:c r="J5" s="26" t="n">
+        <x:f>ROUND(E5-F5,1)</x:f>
+        <x:v>229.8</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28"/>
       <x:c r="E8" s="28"/>
@@ -2525,11 +2687,29 @@
       <x:c r="G8" s="28"/>
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="28"/>
-      <x:c r="J8" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J4),0),1)</x:f>
-        <x:v>303.6</x:v>
+      <x:c r="J8" s="30" t="n">
+        <x:f>SUM(J4:J5)</x:f>
+        <x:v>533.4000000000001</x:v>
       </x:c>
       <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
+        <x:v>266.7</x:v>
+      </x:c>
+      <x:c r="K9" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-12
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7b1742cae7194261"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rfd4878d882a14c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R327a61cc12ab4611"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rde40584e08394134"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R547594f7b6244ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R8b1c2f0db59b4d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R7e1800a95ffd44da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rdbdc358b5a694969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R0cc4e1156797417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rc6c4d5b4e00a4255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R998584401f894a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R15011e453f45439b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1e62f5d1263647dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Ra5f545b31e0e4ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R6e01058089c94c9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb940b55884824437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4f24abca041f4398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rdbd614f5820c4d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9630211abb7140d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf53979a5f5b54cdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -217,6 +217,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -225,12 +231,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7175.33</x:v>
+        <x:v>7145.06</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6925.42</x:v>
+        <x:v>7014.37</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>249.9</x:v>
+        <x:v>130.7</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>529</x:v>
+        <x:v>659.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>264.5</x:v>
+        <x:v>219.9</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7277.14</x:v>
+        <x:v>7236.78</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7048.45</x:v>
+        <x:v>7085.92</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>228.7</x:v>
+        <x:v>150.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>483.9</x:v>
+        <x:v>634.8</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>242</x:v>
+        <x:v>211.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3824.71</x:v>
+        <x:v>3828.22</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3754.14</x:v>
+        <x:v>3791</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>70.6</x:v>
+        <x:v>37.2</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>139.4</x:v>
+        <x:v>176.6</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>69.7</x:v>
+        <x:v>58.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>7049</x:v>
+        <x:v>7031.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6819.2</x:v>
+        <x:v>6886.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>229.8</x:v>
+        <x:v>144.6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>533.4</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>266.7</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4264.6</x:v>
+        <x:v>4273.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4180.4</x:v>
+        <x:v>4213.8</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>84.2</x:v>
+        <x:v>59.8</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>197.2</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>98.6</x:v>
+        <x:v>85.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2778.6</x:v>
+        <x:v>2794</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2735</x:v>
+        <x:v>2761.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>43.6</x:v>
+        <x:v>32.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>94.6</x:v>
+        <x:v>127.4</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>47.3</x:v>
+        <x:v>42.5</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>120000</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>220</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>121000</x:v>
       </x:c>
-      <x:c r="H5" s="37" t="n">
+      <x:c r="H5" s="34" t="n">
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -1126,843 +1126,951 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B6" s="28" t="n">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="n">
+        <x:v>7132.68</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7145.06</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7014.37</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7021.47</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:f>ROUND(F6-F5,1)</x:f>
+        <x:v>-134.4</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="n">
+        <x:f>IFERROR(F6/F5-1,"")</x:f>
+        <x:v>-0.018787268146189584</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="n">
+        <x:f>ROUND(D6-E6,1)</x:f>
+        <x:v>130.7</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="28"/>
-      <x:c r="D6" s="28"/>
-      <x:c r="E6" s="28"/>
-      <x:c r="F6" s="28"/>
-      <x:c r="G6" s="28"/>
-      <x:c r="H6" s="28"/>
-      <x:c r="I6" s="30" t="n">
-        <x:f>ROUND(SUM(I5:I5),1)</x:f>
-        <x:v>441.4</x:v>
-      </x:c>
-      <x:c r="J6" s="28"/>
-      <x:c r="K6" s="28"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B7" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="C7" s="28"/>
       <x:c r="D7" s="28"/>
       <x:c r="E7" s="28"/>
       <x:c r="F7" s="28"/>
       <x:c r="G7" s="28"/>
       <x:c r="H7" s="28"/>
-      <x:c r="I7" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I5),0),1)</x:f>
-        <x:v>441.4</x:v>
+      <x:c r="I7" s="30" t="n">
+        <x:f>ROUND(SUM(I5:I6),1)</x:f>
+        <x:v>572.1</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="17" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B8" s="28"/>
+      <x:c r="C8" s="28"/>
+      <x:c r="D8" s="28"/>
+      <x:c r="E8" s="28"/>
+      <x:c r="F8" s="28"/>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B9" s="17"/>
-      <x:c r="C9" s="17"/>
-      <x:c r="D9" s="17"/>
-      <x:c r="E9" s="17"/>
-      <x:c r="F9" s="17"/>
-      <x:c r="G9" s="17"/>
-      <x:c r="H9" s="17"/>
-      <x:c r="I9" s="17"/>
-      <x:c r="J9" s="17"/>
-      <x:c r="K9" s="17"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="20" t="str">
+      <x:c r="B10" s="17"/>
+      <x:c r="C10" s="17"/>
+      <x:c r="D10" s="17"/>
+      <x:c r="E10" s="17"/>
+      <x:c r="F10" s="17"/>
+      <x:c r="G10" s="17"/>
+      <x:c r="H10" s="17"/>
+      <x:c r="I10" s="17"/>
+      <x:c r="J10" s="17"/>
+      <x:c r="K10" s="17"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B10" s="20" t="str">
+      <x:c r="B11" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C10" s="20" t="str">
+      <x:c r="C11" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D10" s="20" t="str">
+      <x:c r="D11" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E10" s="20" t="str">
+      <x:c r="E11" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F10" s="20" t="str">
+      <x:c r="F11" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G10" s="20" t="str">
+      <x:c r="G11" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H10" s="20" t="str">
+      <x:c r="H11" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I10" s="20" t="str">
+      <x:c r="I11" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J10" s="20" t="str">
+      <x:c r="J11" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K10" s="20" t="str">
+      <x:c r="K11" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="22" t="n">
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B11" s="22" t="str">
+      <x:c r="B12" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C11" s="23" t="n">
+      <x:c r="C12" s="23" t="n">
         <x:v>7420.44</x:v>
       </x:c>
-      <x:c r="D11" s="23" t="n">
+      <x:c r="D12" s="23" t="n">
         <x:v>7461.24</x:v>
       </x:c>
-      <x:c r="E11" s="23" t="n">
+      <x:c r="E12" s="23" t="n">
         <x:v>7048.45</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="n">
+      <x:c r="F12" s="23" t="n">
         <x:v>7251.01</x:v>
       </x:c>
-      <x:c r="G11" s="23"/>
-      <x:c r="H11" s="24"/>
-      <x:c r="I11" s="26" t="n">
-        <x:f>ROUND(D11-E11,1)</x:f>
+      <x:c r="G12" s="23"/>
+      <x:c r="H12" s="24"/>
+      <x:c r="I12" s="26" t="n">
+        <x:f>ROUND(D12-E12,1)</x:f>
         <x:v>412.8</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="str">
+      <x:c r="J12" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="K11" s="22" t="n">
+      <x:c r="K12" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="29" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="n">
+        <x:v>7226.07</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>7236.78</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>7085.92</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>7093.02</x:v>
+      </x:c>
+      <x:c r="G13" s="34" t="n">
+        <x:f>ROUND(F13-F12,1)</x:f>
+        <x:v>-158</x:v>
+      </x:c>
+      <x:c r="H13" s="24" t="n">
+        <x:f>IFERROR(F13/F12-1,"")</x:f>
+        <x:v>-0.02178868874818818</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="n">
+        <x:f>ROUND(D13-E13,1)</x:f>
+        <x:v>150.9</x:v>
+      </x:c>
+      <x:c r="J13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="n">
+      <x:c r="B14" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="30" t="n">
+        <x:f>ROUND(SUM(I12:I13),1)</x:f>
+        <x:v>563.7</x:v>
+      </x:c>
+      <x:c r="J14" s="28"/>
+      <x:c r="K14" s="28"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="28"/>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
+        <x:v>281.9</x:v>
+      </x:c>
+      <x:c r="J15" s="28"/>
+      <x:c r="K15" s="28"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B17" s="17"/>
+      <x:c r="C17" s="17"/>
+      <x:c r="D17" s="17"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="17"/>
+      <x:c r="G17" s="17"/>
+      <x:c r="H17" s="17"/>
+      <x:c r="I17" s="17"/>
+      <x:c r="J17" s="17"/>
+      <x:c r="K17" s="17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J18" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K18" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="28"/>
-      <x:c r="E12" s="28"/>
-      <x:c r="F12" s="28"/>
-      <x:c r="G12" s="28"/>
-      <x:c r="H12" s="28"/>
-      <x:c r="I12" s="30" t="n">
-        <x:f>ROUND(SUM(I11:I11),1)</x:f>
-        <x:v>412.8</x:v>
-      </x:c>
-      <x:c r="J12" s="28"/>
-      <x:c r="K12" s="28"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
+      <x:c r="B19" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="n">
+        <x:v>3838.98</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3864.12</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3754.14</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3813.79</x:v>
+      </x:c>
+      <x:c r="G19" s="23"/>
+      <x:c r="H19" s="24"/>
+      <x:c r="I19" s="26" t="n">
+        <x:f>ROUND(D19-E19,1)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="n">
+        <x:v>3806.98</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3828.22</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3791</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3797.24</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:f>ROUND(F20-F19,1)</x:f>
+        <x:v>-16.6</x:v>
+      </x:c>
+      <x:c r="H20" s="24" t="n">
+        <x:f>IFERROR(F20/F19-1,"")</x:f>
+        <x:v>-0.00433951528531995</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="n">
+        <x:f>ROUND(D20-E20,1)</x:f>
+        <x:v>37.2</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
+      <x:c r="E21" s="28"/>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28"/>
+      <x:c r="H21" s="28"/>
+      <x:c r="I21" s="30" t="n">
+        <x:f>ROUND(SUM(I19:I20),1)</x:f>
+        <x:v>147.2</x:v>
+      </x:c>
+      <x:c r="J21" s="28"/>
+      <x:c r="K21" s="28"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B13" s="28"/>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="28"/>
-      <x:c r="E13" s="28"/>
-      <x:c r="F13" s="28"/>
-      <x:c r="G13" s="28"/>
-      <x:c r="H13" s="28"/>
-      <x:c r="I13" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I11:I11),0),1)</x:f>
-        <x:v>412.8</x:v>
-      </x:c>
-      <x:c r="J13" s="28"/>
-      <x:c r="K13" s="28"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B15" s="17"/>
-      <x:c r="C15" s="17"/>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="17"/>
-      <x:c r="F15" s="17"/>
-      <x:c r="G15" s="17"/>
-      <x:c r="H15" s="17"/>
-      <x:c r="I15" s="17"/>
-      <x:c r="J15" s="17"/>
-      <x:c r="K15" s="17"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="20" t="str">
+      <x:c r="B22" s="28"/>
+      <x:c r="C22" s="28"/>
+      <x:c r="D22" s="28"/>
+      <x:c r="E22" s="28"/>
+      <x:c r="F22" s="28"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
+        <x:v>73.6</x:v>
+      </x:c>
+      <x:c r="J22" s="28"/>
+      <x:c r="K22" s="28"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B24" s="17"/>
+      <x:c r="C24" s="17"/>
+      <x:c r="D24" s="17"/>
+      <x:c r="E24" s="17"/>
+      <x:c r="F24" s="17"/>
+      <x:c r="G24" s="17"/>
+      <x:c r="H24" s="17"/>
+      <x:c r="I24" s="17"/>
+      <x:c r="J24" s="17"/>
+      <x:c r="K24" s="17"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B16" s="20" t="str">
+      <x:c r="B25" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C16" s="20" t="str">
+      <x:c r="C25" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D16" s="20" t="str">
+      <x:c r="D25" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E16" s="20" t="str">
+      <x:c r="E25" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F16" s="20" t="str">
+      <x:c r="F25" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G16" s="20" t="str">
+      <x:c r="G25" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H16" s="20" t="str">
+      <x:c r="H25" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I16" s="20" t="str">
+      <x:c r="I25" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J16" s="20" t="str">
+      <x:c r="J25" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K16" s="20" t="str">
+      <x:c r="K25" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="22" t="n">
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B17" s="22" t="str">
+      <x:c r="B26" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C17" s="23" t="n">
-        <x:v>3838.98</x:v>
-      </x:c>
-      <x:c r="D17" s="23" t="n">
-        <x:v>3864.12</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="n">
-        <x:v>3754.14</x:v>
-      </x:c>
-      <x:c r="F17" s="23" t="n">
-        <x:v>3813.79</x:v>
-      </x:c>
-      <x:c r="G17" s="23"/>
-      <x:c r="H17" s="24"/>
-      <x:c r="I17" s="26" t="n">
-        <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="J17" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K17" s="22" t="n">
+      <x:c r="C26" s="23" t="n">
+        <x:v>7182.8</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>6819.2</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>7015.8</x:v>
+      </x:c>
+      <x:c r="G26" s="23"/>
+      <x:c r="H26" s="24"/>
+      <x:c r="I26" s="26" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>432.6</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
+    <x:row r="27">
+      <x:c r="A27" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D27" s="23" t="n">
+        <x:v>7031.2</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="n">
+        <x:v>6886.6</x:v>
+      </x:c>
+      <x:c r="F27" s="23" t="n">
+        <x:v>6921</x:v>
+      </x:c>
+      <x:c r="G27" s="23" t="n">
+        <x:f>ROUND(F27-F26,1)</x:f>
+        <x:v>-94.8</x:v>
+      </x:c>
+      <x:c r="H27" s="24" t="n">
+        <x:f>IFERROR(F27/F26-1,"")</x:f>
+        <x:v>-0.01351235782091853</x:v>
+      </x:c>
+      <x:c r="I27" s="23" t="n">
+        <x:f>ROUND(D27-E27,1)</x:f>
+        <x:v>144.6</x:v>
+      </x:c>
+      <x:c r="J27" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K27" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B18" s="28" t="n">
+      <x:c r="B28" s="28" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="28"/>
+      <x:c r="E28" s="28"/>
+      <x:c r="F28" s="28"/>
+      <x:c r="G28" s="28"/>
+      <x:c r="H28" s="28"/>
+      <x:c r="I28" s="30" t="n">
+        <x:f>ROUND(SUM(I26:I27),1)</x:f>
+        <x:v>577.2</x:v>
+      </x:c>
+      <x:c r="J28" s="28"/>
+      <x:c r="K28" s="28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B29" s="28"/>
+      <x:c r="C29" s="28"/>
+      <x:c r="D29" s="28"/>
+      <x:c r="E29" s="28"/>
+      <x:c r="F29" s="28"/>
+      <x:c r="G29" s="28"/>
+      <x:c r="H29" s="28"/>
+      <x:c r="I29" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
+        <x:v>288.6</x:v>
+      </x:c>
+      <x:c r="J29" s="28"/>
+      <x:c r="K29" s="28"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B31" s="17"/>
+      <x:c r="C31" s="17"/>
+      <x:c r="D31" s="17"/>
+      <x:c r="E31" s="17"/>
+      <x:c r="F31" s="17"/>
+      <x:c r="G31" s="17"/>
+      <x:c r="H31" s="17"/>
+      <x:c r="I31" s="17"/>
+      <x:c r="J31" s="17"/>
+      <x:c r="K31" s="17"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C32" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E32" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F32" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G32" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I32" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J32" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K32" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-      <x:c r="I18" s="30" t="n">
-        <x:f>ROUND(SUM(I17:I17),1)</x:f>
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="J18" s="28"/>
-      <x:c r="K18" s="28"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
+      <x:c r="B33" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7295</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>6932</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>7111</x:v>
+      </x:c>
+      <x:c r="G33" s="23"/>
+      <x:c r="H33" s="24"/>
+      <x:c r="I33" s="26" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B34" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C34" s="28"/>
+      <x:c r="D34" s="28"/>
+      <x:c r="E34" s="28"/>
+      <x:c r="F34" s="28"/>
+      <x:c r="G34" s="28"/>
+      <x:c r="H34" s="28"/>
+      <x:c r="I34" s="30" t="n">
+        <x:f>ROUND(SUM(I33:I33),1)</x:f>
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="J34" s="28"/>
+      <x:c r="K34" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="29" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B19" s="28"/>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="28"/>
-      <x:c r="E19" s="28"/>
-      <x:c r="F19" s="28"/>
-      <x:c r="G19" s="28"/>
-      <x:c r="H19" s="28"/>
-      <x:c r="I19" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I17:I17),0),1)</x:f>
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="J19" s="28"/>
-      <x:c r="K19" s="28"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B21" s="17"/>
-      <x:c r="C21" s="17"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="17"/>
-      <x:c r="F21" s="17"/>
-      <x:c r="G21" s="17"/>
-      <x:c r="H21" s="17"/>
-      <x:c r="I21" s="17"/>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="20" t="str">
+      <x:c r="B35" s="28"/>
+      <x:c r="C35" s="28"/>
+      <x:c r="D35" s="28"/>
+      <x:c r="E35" s="28"/>
+      <x:c r="F35" s="28"/>
+      <x:c r="G35" s="28"/>
+      <x:c r="H35" s="28"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I33:I33),0),1)</x:f>
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="J35" s="28"/>
+      <x:c r="K35" s="28"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B37" s="17"/>
+      <x:c r="C37" s="17"/>
+      <x:c r="D37" s="17"/>
+      <x:c r="E37" s="17"/>
+      <x:c r="F37" s="17"/>
+      <x:c r="G37" s="17"/>
+      <x:c r="H37" s="17"/>
+      <x:c r="I37" s="17"/>
+      <x:c r="J37" s="17"/>
+      <x:c r="K37" s="17"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B22" s="20" t="str">
+      <x:c r="B38" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C22" s="20" t="str">
+      <x:c r="C38" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D22" s="20" t="str">
+      <x:c r="D38" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E22" s="20" t="str">
+      <x:c r="E38" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
+      <x:c r="F38" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G22" s="20" t="str">
+      <x:c r="G38" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H22" s="20" t="str">
+      <x:c r="H38" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I22" s="20" t="str">
+      <x:c r="I38" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J22" s="20" t="str">
+      <x:c r="J38" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K22" s="20" t="str">
+      <x:c r="K38" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="22" t="n">
+    <x:row r="39">
+      <x:c r="A39" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B23" s="22" t="str">
+      <x:c r="B39" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C23" s="23" t="n">
-        <x:v>7182.8</x:v>
-      </x:c>
-      <x:c r="D23" s="23" t="n">
-        <x:v>7251.8</x:v>
-      </x:c>
-      <x:c r="E23" s="23" t="n">
-        <x:v>6819.2</x:v>
-      </x:c>
-      <x:c r="F23" s="23" t="n">
-        <x:v>7015.8</x:v>
-      </x:c>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
-      <x:c r="I23" s="26" t="n">
-        <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>432.6</x:v>
-      </x:c>
-      <x:c r="J23" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K23" s="22" t="n">
+      <x:c r="C39" s="23" t="n">
+        <x:v>4300.8</x:v>
+      </x:c>
+      <x:c r="D39" s="23" t="n">
+        <x:v>4331.6</x:v>
+      </x:c>
+      <x:c r="E39" s="23" t="n">
+        <x:v>4180.4</x:v>
+      </x:c>
+      <x:c r="F39" s="23" t="n">
+        <x:v>4244.8</x:v>
+      </x:c>
+      <x:c r="G39" s="23"/>
+      <x:c r="H39" s="24"/>
+      <x:c r="I39" s="26" t="n">
+        <x:f>ROUND(D39-E39,1)</x:f>
+        <x:v>151.2</x:v>
+      </x:c>
+      <x:c r="J39" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K39" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="29" t="str">
+    <x:row r="40">
+      <x:c r="A40" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B40" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C40" s="23" t="n">
+        <x:v>4240.4</x:v>
+      </x:c>
+      <x:c r="D40" s="23" t="n">
+        <x:v>4273.6</x:v>
+      </x:c>
+      <x:c r="E40" s="23" t="n">
+        <x:v>4213.8</x:v>
+      </x:c>
+      <x:c r="F40" s="23" t="n">
+        <x:v>4233.6</x:v>
+      </x:c>
+      <x:c r="G40" s="23" t="n">
+        <x:f>ROUND(F40-F39,1)</x:f>
+        <x:v>-11.2</x:v>
+      </x:c>
+      <x:c r="H40" s="24" t="n">
+        <x:f>IFERROR(F40/F39-1,"")</x:f>
+        <x:v>-0.0026385224274405594</x:v>
+      </x:c>
+      <x:c r="I40" s="23" t="n">
+        <x:f>ROUND(D40-E40,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="J40" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K40" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="29" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="28"/>
-      <x:c r="E24" s="28"/>
-      <x:c r="F24" s="28"/>
-      <x:c r="G24" s="28"/>
-      <x:c r="H24" s="28"/>
-      <x:c r="I24" s="30" t="n">
-        <x:f>ROUND(SUM(I23:I23),1)</x:f>
-        <x:v>432.6</x:v>
-      </x:c>
-      <x:c r="J24" s="28"/>
-      <x:c r="K24" s="28"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="28"/>
-      <x:c r="E25" s="28"/>
-      <x:c r="F25" s="28"/>
-      <x:c r="G25" s="28"/>
-      <x:c r="H25" s="28"/>
-      <x:c r="I25" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I23:I23),0),1)</x:f>
-        <x:v>432.6</x:v>
-      </x:c>
-      <x:c r="J25" s="28"/>
-      <x:c r="K25" s="28"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B28" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C28" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D28" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E28" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F28" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G28" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H28" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I28" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J28" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K28" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B29" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7295</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7355</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>6932</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7111</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
+      <x:c r="B41" s="28" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B30" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C30" s="28"/>
-      <x:c r="D30" s="28"/>
-      <x:c r="E30" s="28"/>
-      <x:c r="F30" s="28"/>
-      <x:c r="G30" s="28"/>
-      <x:c r="H30" s="28"/>
-      <x:c r="I30" s="30" t="n">
-        <x:f>ROUND(SUM(I29:I29),1)</x:f>
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="J30" s="28"/>
-      <x:c r="K30" s="28"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B31" s="28"/>
-      <x:c r="C31" s="28"/>
-      <x:c r="D31" s="28"/>
-      <x:c r="E31" s="28"/>
-      <x:c r="F31" s="28"/>
-      <x:c r="G31" s="28"/>
-      <x:c r="H31" s="28"/>
-      <x:c r="I31" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I29),0),1)</x:f>
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="J31" s="28"/>
-      <x:c r="K31" s="28"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B33" s="17"/>
-      <x:c r="C33" s="17"/>
-      <x:c r="D33" s="17"/>
-      <x:c r="E33" s="17"/>
-      <x:c r="F33" s="17"/>
-      <x:c r="G33" s="17"/>
-      <x:c r="H33" s="17"/>
-      <x:c r="I33" s="17"/>
-      <x:c r="J33" s="17"/>
-      <x:c r="K33" s="17"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B34" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C34" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D34" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E34" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F34" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G34" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H34" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I34" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J34" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K34" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B35" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C35" s="23" t="n">
-        <x:v>4300.8</x:v>
-      </x:c>
-      <x:c r="D35" s="23" t="n">
-        <x:v>4331.6</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="n">
-        <x:v>4180.4</x:v>
-      </x:c>
-      <x:c r="F35" s="23" t="n">
-        <x:v>4244.8</x:v>
-      </x:c>
-      <x:c r="G35" s="23"/>
-      <x:c r="H35" s="24"/>
-      <x:c r="I35" s="26" t="n">
-        <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>151.2</x:v>
-      </x:c>
-      <x:c r="J35" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K35" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B36" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="30" t="n">
-        <x:f>ROUND(SUM(I35:I35),1)</x:f>
-        <x:v>151.2</x:v>
-      </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B37" s="28"/>
-      <x:c r="C37" s="28"/>
-      <x:c r="D37" s="28"/>
-      <x:c r="E37" s="28"/>
-      <x:c r="F37" s="28"/>
-      <x:c r="G37" s="28"/>
-      <x:c r="H37" s="28"/>
-      <x:c r="I37" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I35:I35),0),1)</x:f>
-        <x:v>151.2</x:v>
-      </x:c>
-      <x:c r="J37" s="28"/>
-      <x:c r="K37" s="28"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B39" s="17"/>
-      <x:c r="C39" s="17"/>
-      <x:c r="D39" s="17"/>
-      <x:c r="E39" s="17"/>
-      <x:c r="F39" s="17"/>
-      <x:c r="G39" s="17"/>
-      <x:c r="H39" s="17"/>
-      <x:c r="I39" s="17"/>
-      <x:c r="J39" s="17"/>
-      <x:c r="K39" s="17"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B40" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C40" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D40" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E40" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F40" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G40" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H40" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I40" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J40" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K40" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>2798.4</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>2735</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>63.4</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="C41" s="28"/>
+      <x:c r="D41" s="28"/>
+      <x:c r="E41" s="28"/>
+      <x:c r="F41" s="28"/>
+      <x:c r="G41" s="28"/>
+      <x:c r="H41" s="28"/>
+      <x:c r="I41" s="30" t="n">
+        <x:f>ROUND(SUM(I39:I40),1)</x:f>
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="J41" s="28"/>
+      <x:c r="K41" s="28"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B42" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B42" s="28"/>
       <x:c r="C42" s="28"/>
       <x:c r="D42" s="28"/>
       <x:c r="E42" s="28"/>
       <x:c r="F42" s="28"/>
       <x:c r="G42" s="28"/>
       <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
-        <x:f>ROUND(SUM(I41:I41),1)</x:f>
-        <x:v>63.4</x:v>
+      <x:c r="I42" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I39:I40),0),1)</x:f>
+        <x:v>105.5</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
     </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I41:I41),0),1)</x:f>
+    <x:row r="44">
+      <x:c r="A44" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B44" s="17"/>
+      <x:c r="C44" s="17"/>
+      <x:c r="D44" s="17"/>
+      <x:c r="E44" s="17"/>
+      <x:c r="F44" s="17"/>
+      <x:c r="G44" s="17"/>
+      <x:c r="H44" s="17"/>
+      <x:c r="I44" s="17"/>
+      <x:c r="J44" s="17"/>
+      <x:c r="K44" s="17"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B45" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C45" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E45" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F45" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G45" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I45" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J45" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K45" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C46" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="D46" s="23" t="n">
+        <x:v>2798.4</x:v>
+      </x:c>
+      <x:c r="E46" s="23" t="n">
+        <x:v>2735</x:v>
+      </x:c>
+      <x:c r="F46" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="G46" s="23"/>
+      <x:c r="H46" s="24"/>
+      <x:c r="I46" s="26" t="n">
+        <x:f>ROUND(D46-E46,1)</x:f>
         <x:v>63.4</x:v>
       </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>碳酸锂2610</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C46" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E46" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F46" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I46" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J46" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str">
-        <x:v>交易日</x:v>
+      <x:c r="J46" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K46" s="22" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="C47" s="23" t="n">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="D47" s="23" t="n">
+        <x:v>2794</x:v>
+      </x:c>
+      <x:c r="E47" s="23" t="n">
+        <x:v>2761.2</x:v>
+      </x:c>
+      <x:c r="F47" s="23" t="n">
+        <x:v>2779</x:v>
+      </x:c>
+      <x:c r="G47" s="23" t="n">
+        <x:f>ROUND(F47-F46,1)</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H47" s="24" t="n">
+        <x:f>IFERROR(F47/F46-1,"")</x:f>
+        <x:v>0.00542691751085389</x:v>
+      </x:c>
+      <x:c r="I47" s="23" t="n">
+        <x:f>ROUND(D47-E47,1)</x:f>
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="J47" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K47" s="22" t="n">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>120020</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>126800</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>119000</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>121000</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>7800</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1970,7 +2078,7 @@
         <x:v>合计</x:v>
       </x:c>
       <x:c r="B48" s="28" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="28"/>
       <x:c r="D48" s="28"/>
@@ -1979,8 +2087,8 @@
       <x:c r="G48" s="28"/>
       <x:c r="H48" s="28"/>
       <x:c r="I48" s="30" t="n">
-        <x:f>ROUND(SUM(I47:I47),1)</x:f>
-        <x:v>7800</x:v>
+        <x:f>ROUND(SUM(I46:I47),1)</x:f>
+        <x:v>96.2</x:v>
       </x:c>
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
@@ -1997,23 +2105,143 @@
       <x:c r="G49" s="28"/>
       <x:c r="H49" s="28"/>
       <x:c r="I49" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I47),0),1)</x:f>
-        <x:v>7800</x:v>
+        <x:f>ROUND(IFERROR(AVERAGE(I46:I47),0),1)</x:f>
+        <x:v>48.1</x:v>
       </x:c>
       <x:c r="J49" s="28"/>
       <x:c r="K49" s="28"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="17" t="str">
+        <x:v>碳酸锂2610</x:v>
+      </x:c>
+      <x:c r="B51" s="17"/>
+      <x:c r="C51" s="17"/>
+      <x:c r="D51" s="17"/>
+      <x:c r="E51" s="17"/>
+      <x:c r="F51" s="17"/>
+      <x:c r="G51" s="17"/>
+      <x:c r="H51" s="17"/>
+      <x:c r="I51" s="17"/>
+      <x:c r="J51" s="17"/>
+      <x:c r="K51" s="17"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B52" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C52" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D52" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E52" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F52" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G52" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H52" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I52" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J52" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K52" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B53" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C53" s="23" t="n">
+        <x:v>120020</x:v>
+      </x:c>
+      <x:c r="D53" s="23" t="n">
+        <x:v>126800</x:v>
+      </x:c>
+      <x:c r="E53" s="23" t="n">
+        <x:v>119000</x:v>
+      </x:c>
+      <x:c r="F53" s="23" t="n">
+        <x:v>121000</x:v>
+      </x:c>
+      <x:c r="G53" s="23"/>
+      <x:c r="H53" s="24"/>
+      <x:c r="I53" s="26" t="n">
+        <x:f>ROUND(D53-E53,1)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="J53" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K53" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="29" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B54" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C54" s="28"/>
+      <x:c r="D54" s="28"/>
+      <x:c r="E54" s="28"/>
+      <x:c r="F54" s="28"/>
+      <x:c r="G54" s="28"/>
+      <x:c r="H54" s="28"/>
+      <x:c r="I54" s="30" t="n">
+        <x:f>ROUND(SUM(I53:I53),1)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="J54" s="28"/>
+      <x:c r="K54" s="28"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B55" s="28"/>
+      <x:c r="C55" s="28"/>
+      <x:c r="D55" s="28"/>
+      <x:c r="E55" s="28"/>
+      <x:c r="F55" s="28"/>
+      <x:c r="G55" s="28"/>
+      <x:c r="H55" s="28"/>
+      <x:c r="I55" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I53:I53),0),1)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="J55" s="28"/>
+      <x:c r="K55" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A9:K9"/>
-    <x:mergeCell ref="A15:K15"/>
-    <x:mergeCell ref="A21:K21"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A33:K33"/>
-    <x:mergeCell ref="A39:K39"/>
-    <x:mergeCell ref="A45:K45"/>
+    <x:mergeCell ref="A10:K10"/>
+    <x:mergeCell ref="A17:K17"/>
+    <x:mergeCell ref="A24:K24"/>
+    <x:mergeCell ref="A31:K31"/>
+    <x:mergeCell ref="A37:K37"/>
+    <x:mergeCell ref="A44:K44"/>
+    <x:mergeCell ref="A51:K51"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2098,7 +2326,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7138.58</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>-160.2</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -2148,31 +2376,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>529</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7132.68</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7145.06</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7014.37</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7021.47</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>-134.4</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.018787268146189584</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>130.7</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2180,11 +2426,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>264.5</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>659.7</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>219.9</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2273,7 +2537,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7248.43</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>-186.7</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -2323,31 +2587,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>483.9</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7226.07</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7236.78</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>7085.92</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>7093.02</x:v>
+      </x:c>
+      <x:c r="H6" s="34" t="n">
+        <x:v>-158</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.02178868874818818</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>150.9</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2355,11 +2637,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>242</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>634.8</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>211.6</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2498,31 +2798,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>139.39999999999998</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>3806.98</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>3828.22</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>3791</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>3797.24</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>-16.6</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.00433951528531995</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>37.2</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2530,11 +2848,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>69.7</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>176.59999999999997</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>58.9</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2673,31 +3009,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>533.4000000000001</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>7031.2</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>6886.6</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>6921</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>-94.8</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.01351235782091853</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>144.6</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2705,11 +3059,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>266.7</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>678.0000000000001</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2798,7 +3170,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7122.8</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="n">
+      <x:c r="H4" s="34" t="n">
         <x:v>-187.4</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -3023,31 +3395,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>197.2</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>4240.4</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>4273.6</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>4213.8</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>4233.6</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>-11.2</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>-0.0026385224274405594</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>59.8</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -3055,11 +3445,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>98.6</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>85.7</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3198,31 +3606,49 @@
         <x:v>IH2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="30" t="n">
-        <x:f>SUM(J4:J5)</x:f>
-        <x:v>94.6</x:v>
-      </x:c>
-      <x:c r="K8" s="28"/>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>10月12日</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="n">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="n">
+        <x:v>2794</x:v>
+      </x:c>
+      <x:c r="F6" s="23" t="n">
+        <x:v>2761.2</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="n">
+        <x:v>2779</x:v>
+      </x:c>
+      <x:c r="H6" s="23" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="n">
+        <x:v>0.00542691751085389</x:v>
+      </x:c>
+      <x:c r="J6" s="23" t="n">
+        <x:f>ROUND(E6-F6,1)</x:f>
+        <x:v>32.8</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C9" s="28"/>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -3230,11 +3656,29 @@
       <x:c r="G9" s="28"/>
       <x:c r="H9" s="28"/>
       <x:c r="I9" s="28"/>
-      <x:c r="J9" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J5),0),1)</x:f>
-        <x:v>47.3</x:v>
+      <x:c r="J9" s="30" t="n">
+        <x:f>SUM(J4:J6)</x:f>
+        <x:v>127.39999999999999</x:v>
       </x:c>
       <x:c r="K9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
+        <x:v>42.5</x:v>
+      </x:c>
+      <x:c r="K10" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-13
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R27e250ea3f9c4c9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R433ce4d67b5a4684"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R2188f34d2db04945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R0daecf9607a142a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rc88c5f856d2e4417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rf76cef010dc84479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rf19f0aba53994194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rdc822ae1d9f34e77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R7d718ae58f124b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R778f353ac0c54d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd2176c0bffe64a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R8ac4bbb7e4a8413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R61fc72bc222c4228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rd95dbd63524042b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R24e70d3428014361"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rdbfc95f0c66741a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rf7c70449dd11423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb35d7eca6e3241d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R7e4fbe6a6f0b4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R3ee24bdd66c64c37"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-13</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7145.06</x:v>
+        <x:v>7087.89</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>7014.37</x:v>
+        <x:v>6796.58</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>130.7</x:v>
+        <x:v>291.3</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>659.7</x:v>
+        <x:v>951</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>219.9</x:v>
+        <x:v>237.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-13</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7236.78</x:v>
+        <x:v>7152.45</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>7085.92</x:v>
+        <x:v>6904.6</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>150.9</x:v>
+        <x:v>247.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>634.8</x:v>
+        <x:v>882.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>211.6</x:v>
+        <x:v>220.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-13</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3828.22</x:v>
+        <x:v>3822.11</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3791</x:v>
+        <x:v>3741.53</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>37.2</x:v>
+        <x:v>80.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>176.6</x:v>
+        <x:v>257.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>58.9</x:v>
+        <x:v>64.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -630,25 +630,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-13</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4273.6</x:v>
+        <x:v>4257.4</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4213.8</x:v>
+        <x:v>4151</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>59.8</x:v>
+        <x:v>106.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>257</x:v>
+        <x:v>363.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>85.7</x:v>
+        <x:v>90.9</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-13</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1166,7 +1166,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>10月12日</x:v>
+        <x:v>10月12日-10月13日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7132.68</x:v>
@@ -1175,28 +1175,28 @@
         <x:v>7145.06</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
-        <x:v>7014.37</x:v>
+        <x:v>6796.58</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7021.47</x:v>
+        <x:v>7023.22</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>-134.4</x:v>
+        <x:v>-132.7</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>-0.018787268146189584</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="n">
+        <x:v>-0.018542715042531244</x:v>
+      </x:c>
+      <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>130.7</x:v>
+        <x:v>348.5</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1214,7 +1214,7 @@
       <x:c r="H7" s="28"/>
       <x:c r="I7" s="30" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>572.1</x:v>
+        <x:v>789.9</x:v>
       </x:c>
       <x:c r="J7" s="28"/>
       <x:c r="K7" s="28"/>
@@ -1232,7 +1232,7 @@
       <x:c r="H8" s="28"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>286</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="J8" s="28"/>
       <x:c r="K8" s="28"/>
@@ -1324,7 +1324,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>10月12日</x:v>
+        <x:v>10月12日-10月13日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7226.07</x:v>
@@ -1333,28 +1333,28 @@
         <x:v>7236.78</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>7085.92</x:v>
+        <x:v>6904.6</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7093.02</x:v>
+        <x:v>7085.09</x:v>
       </x:c>
       <x:c r="G13" s="34" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-158</x:v>
+        <x:v>-165.9</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.02178868874818818</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="n">
+        <x:v>-0.022882329496166753</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>150.9</x:v>
+        <x:v>332.2</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1372,7 +1372,7 @@
       <x:c r="H14" s="28"/>
       <x:c r="I14" s="30" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>563.7</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="J14" s="28"/>
       <x:c r="K14" s="28"/>
@@ -1390,7 +1390,7 @@
       <x:c r="H15" s="28"/>
       <x:c r="I15" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>281.9</x:v>
+        <x:v>372.5</x:v>
       </x:c>
       <x:c r="J15" s="28"/>
       <x:c r="K15" s="28"/>
@@ -1482,7 +1482,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>10月12日</x:v>
+        <x:v>10月12日-10月13日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3806.98</x:v>
@@ -1491,28 +1491,28 @@
         <x:v>3828.22</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3791</x:v>
+        <x:v>3741.53</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3797.24</x:v>
+        <x:v>3800.86</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-16.6</x:v>
+        <x:v>-12.9</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.00433951528531995</x:v>
-      </x:c>
-      <x:c r="I20" s="23" t="n">
+        <x:v>-0.0033903282561441594</x:v>
+      </x:c>
+      <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>37.2</x:v>
+        <x:v>86.7</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1530,7 +1530,7 @@
       <x:c r="H21" s="28"/>
       <x:c r="I21" s="30" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>147.2</x:v>
+        <x:v>196.7</x:v>
       </x:c>
       <x:c r="J21" s="28"/>
       <x:c r="K21" s="28"/>
@@ -1548,7 +1548,7 @@
       <x:c r="H22" s="28"/>
       <x:c r="I22" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>73.6</x:v>
+        <x:v>98.4</x:v>
       </x:c>
       <x:c r="J22" s="28"/>
       <x:c r="K22" s="28"/>
@@ -1956,7 +1956,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>10月12日</x:v>
+        <x:v>10月12日-10月13日</x:v>
       </x:c>
       <x:c r="C41" s="23" t="n">
         <x:v>4240.4</x:v>
@@ -1965,28 +1965,28 @@
         <x:v>4273.6</x:v>
       </x:c>
       <x:c r="E41" s="23" t="n">
-        <x:v>4213.8</x:v>
+        <x:v>4151</x:v>
       </x:c>
       <x:c r="F41" s="23" t="n">
-        <x:v>4233.6</x:v>
+        <x:v>4217.6</x:v>
       </x:c>
       <x:c r="G41" s="23" t="n">
         <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>-11.2</x:v>
+        <x:v>-27.2</x:v>
       </x:c>
       <x:c r="H41" s="24" t="n">
         <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>-0.0026385224274405594</x:v>
-      </x:c>
-      <x:c r="I41" s="23" t="n">
+        <x:v>-0.006407840180927216</x:v>
+      </x:c>
+      <x:c r="I41" s="26" t="n">
         <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>59.8</x:v>
+        <x:v>122.6</x:v>
       </x:c>
       <x:c r="J41" s="22" t="str">
         <x:v>IF2612</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2004,7 +2004,7 @@
       <x:c r="H42" s="28"/>
       <x:c r="I42" s="30" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>211</x:v>
+        <x:v>273.8</x:v>
       </x:c>
       <x:c r="J42" s="28"/>
       <x:c r="K42" s="28"/>
@@ -2022,7 +2022,7 @@
       <x:c r="H43" s="28"/>
       <x:c r="I43" s="32" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>105.5</x:v>
+        <x:v>136.9</x:v>
       </x:c>
       <x:c r="J43" s="28"/>
       <x:c r="K43" s="28"/>
@@ -2524,31 +2524,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>659.7</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>10月13日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>6894.6</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7087.89</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>6796.58</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7023.22</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.0002492355589356343</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>291.3</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2556,11 +2574,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>219.9</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>951</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>237.8</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2735,31 +2771,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>634.8</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>10月13日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>6976.63</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>7152.45</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>6904.6</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>7085.09</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-7.9</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.0011180005131805615</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>247.8</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2767,11 +2821,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>211.6</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>882.5999999999999</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>220.7</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2946,31 +3018,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>176.59999999999997</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>10月13日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>3760.8</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>3822.11</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>3741.53</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>3800.86</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>0.0009533239932162374</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>80.6</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -2978,11 +3068,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>58.9</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>257.19999999999993</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>64.3</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3579,31 +3687,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B9" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="30" t="n">
-        <x:f>SUM(J4:J6)</x:f>
-        <x:v>257</x:v>
-      </x:c>
-      <x:c r="K9" s="28"/>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>10月13日</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>4183.2</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>4257.4</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>4151</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:v>4217.6</x:v>
+      </x:c>
+      <x:c r="H7" s="23" t="n">
+        <x:v>-16</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="n">
+        <x:v>-0.0037792894935751997</x:v>
+      </x:c>
+      <x:c r="J7" s="26" t="n">
+        <x:f>ROUND(E7-F7,1)</x:f>
+        <x:v>106.4</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B10" s="28"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C10" s="28"/>
       <x:c r="D10" s="28"/>
       <x:c r="E10" s="28"/>
@@ -3611,11 +3737,29 @@
       <x:c r="G10" s="28"/>
       <x:c r="H10" s="28"/>
       <x:c r="I10" s="28"/>
-      <x:c r="J10" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J6),0),1)</x:f>
-        <x:v>85.7</x:v>
+      <x:c r="J10" s="30" t="n">
+        <x:f>SUM(J4:J7)</x:f>
+        <x:v>363.4</x:v>
       </x:c>
       <x:c r="K10" s="28"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B11" s="28"/>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
+      <x:c r="E11" s="28"/>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28"/>
+      <x:c r="H11" s="28"/>
+      <x:c r="I11" s="28"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
+        <x:v>90.9</x:v>
+      </x:c>
+      <x:c r="K11" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-14
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rf9ecc966a6754092"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re13ad99ac5c04d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9bb186c20a464d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbcdc6dad17124e93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re2b6498de3f1483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R532d55d27f22493d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R943bfa7204e14ba2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rcd8be6849a964954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R05bbcb41cd654a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Raaa2b0782d404b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R036351c657a34ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R83210437c84444be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Ra0d0120bf45b46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R289ed1c24db349c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R9cb17991936949c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2fd04bb8000c4389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R7bc4049044074f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R68fd2ce804474335"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rb8d18c2cf79f4e6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf7dce820d8104cc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -201,6 +201,12 @@
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -216,12 +222,6 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7087.89</x:v>
+        <x:v>7035.18</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6796.58</x:v>
+        <x:v>6891.6</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>291.3</x:v>
+        <x:v>143.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>951</x:v>
+        <x:v>1094.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>237.8</x:v>
+        <x:v>218.9</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7152.45</x:v>
+        <x:v>7120.11</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6904.6</x:v>
+        <x:v>6969.02</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>247.8</x:v>
+        <x:v>151.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>882.6</x:v>
+        <x:v>1033.7</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>220.7</x:v>
+        <x:v>206.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3822.11</x:v>
+        <x:v>3811.81</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3741.53</x:v>
+        <x:v>3761.96</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>80.6</x:v>
+        <x:v>49.8</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>257.2</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>64.3</x:v>
+        <x:v>61.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6971.6</x:v>
+        <x:v>6925.2</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6680</x:v>
+        <x:v>6761</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>291.6</x:v>
+        <x:v>164.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>969.6</x:v>
+        <x:v>1133.8</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>242.4</x:v>
+        <x:v>226.8</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>111320</x:v>
+        <x:v>108380</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>101000</x:v>
+        <x:v>103000</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>10320</x:v>
+        <x:v>5380</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>40180</x:v>
+        <x:v>45560</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>10045</x:v>
+        <x:v>9112</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -925,7 +925,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>120000</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>220</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -961,7 +961,7 @@
       <x:c r="G5" s="23" t="n">
         <x:v>121000</x:v>
       </x:c>
-      <x:c r="H5" s="34" t="n">
+      <x:c r="H5" s="28" t="n">
         <x:v>1000</x:v>
       </x:c>
       <x:c r="I5" s="24" t="n">
@@ -997,7 +997,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>107100</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>-13900</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -1033,7 +1033,7 @@
       <x:c r="G7" s="23" t="n">
         <x:v>109500</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="n">
+      <x:c r="H7" s="28" t="n">
         <x:v>2400</x:v>
       </x:c>
       <x:c r="I7" s="24" t="n">
@@ -1047,43 +1047,79 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>10月14日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>108380</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>108380</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>103000</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>103000</x:v>
+      </x:c>
+      <x:c r="H8" s="28" t="n">
+        <x:v>-6500</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.05936073059360736</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>5380</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>40180</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="B11" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>45560</x:v>
+      </x:c>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>10045</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>9112</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1202,7 +1238,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>10月12日-10月13日</x:v>
+        <x:v>10月12日-10月14日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7132.68</x:v>
@@ -1214,15 +1250,15 @@
         <x:v>6796.58</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>7023.22</x:v>
-      </x:c>
-      <x:c r="G6" s="23" t="n">
+        <x:v>6905.17</x:v>
+      </x:c>
+      <x:c r="G6" s="28" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>-132.7</x:v>
+        <x:v>-250.7</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>-0.018542715042531244</x:v>
+        <x:v>-0.03503956869217184</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
@@ -1232,46 +1268,46 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="30" t="n">
+      <x:c r="C7" s="30"/>
+      <x:c r="D7" s="30"/>
+      <x:c r="E7" s="30"/>
+      <x:c r="F7" s="30"/>
+      <x:c r="G7" s="30"/>
+      <x:c r="H7" s="30"/>
+      <x:c r="I7" s="32" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
         <x:v>789.9</x:v>
       </x:c>
-      <x:c r="J7" s="28"/>
-      <x:c r="K7" s="28"/>
+      <x:c r="J7" s="30"/>
+      <x:c r="K7" s="30"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="A8" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B8" s="28"/>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="32" t="n">
+      <x:c r="B8" s="30"/>
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="30"/>
+      <x:c r="E8" s="30"/>
+      <x:c r="F8" s="30"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
         <x:v>395</x:v>
       </x:c>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="28"/>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
@@ -1360,7 +1396,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>10月12日-10月13日</x:v>
+        <x:v>10月12日-10月14日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7226.07</x:v>
@@ -1372,15 +1408,15 @@
         <x:v>6904.6</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>7085.09</x:v>
-      </x:c>
-      <x:c r="G13" s="34" t="n">
+        <x:v>6980.11</x:v>
+      </x:c>
+      <x:c r="G13" s="28" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-165.9</x:v>
+        <x:v>-270.9</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.022882329496166753</x:v>
+        <x:v>-0.03736031256335337</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
@@ -1390,46 +1426,46 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="28"/>
-      <x:c r="E14" s="28"/>
-      <x:c r="F14" s="28"/>
-      <x:c r="G14" s="28"/>
-      <x:c r="H14" s="28"/>
-      <x:c r="I14" s="30" t="n">
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="32" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
         <x:v>745</x:v>
       </x:c>
-      <x:c r="J14" s="28"/>
-      <x:c r="K14" s="28"/>
+      <x:c r="J14" s="30"/>
+      <x:c r="K14" s="30"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="A15" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="28"/>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="28"/>
-      <x:c r="E15" s="28"/>
-      <x:c r="F15" s="28"/>
-      <x:c r="G15" s="28"/>
-      <x:c r="H15" s="28"/>
-      <x:c r="I15" s="32" t="n">
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
         <x:v>372.5</x:v>
       </x:c>
-      <x:c r="J15" s="28"/>
-      <x:c r="K15" s="28"/>
+      <x:c r="J15" s="30"/>
+      <x:c r="K15" s="30"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="17" t="str">
@@ -1518,7 +1554,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>10月12日-10月13日</x:v>
+        <x:v>10月12日-10月14日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3806.98</x:v>
@@ -1530,15 +1566,15 @@
         <x:v>3741.53</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3800.86</x:v>
+        <x:v>3767.23</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-12.9</x:v>
+        <x:v>-46.6</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.0033903282561441594</x:v>
+        <x:v>-0.01220832819845874</x:v>
       </x:c>
       <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
@@ -1548,46 +1584,46 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C21" s="28"/>
-      <x:c r="D21" s="28"/>
-      <x:c r="E21" s="28"/>
-      <x:c r="F21" s="28"/>
-      <x:c r="G21" s="28"/>
-      <x:c r="H21" s="28"/>
-      <x:c r="I21" s="30" t="n">
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="32" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
         <x:v>196.7</x:v>
       </x:c>
-      <x:c r="J21" s="28"/>
-      <x:c r="K21" s="28"/>
+      <x:c r="J21" s="30"/>
+      <x:c r="K21" s="30"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="29" t="str">
+      <x:c r="A22" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="28"/>
-      <x:c r="C22" s="28"/>
-      <x:c r="D22" s="28"/>
-      <x:c r="E22" s="28"/>
-      <x:c r="F22" s="28"/>
-      <x:c r="G22" s="28"/>
-      <x:c r="H22" s="28"/>
-      <x:c r="I22" s="32" t="n">
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
         <x:v>98.4</x:v>
       </x:c>
-      <x:c r="J22" s="28"/>
-      <x:c r="K22" s="28"/>
+      <x:c r="J22" s="30"/>
+      <x:c r="K22" s="30"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="17" t="str">
@@ -1676,7 +1712,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>10月12日-10月13日</x:v>
+        <x:v>10月12日-10月14日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7000</x:v>
@@ -1688,15 +1724,15 @@
         <x:v>6680</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>6901.8</x:v>
-      </x:c>
-      <x:c r="G27" s="23" t="n">
+        <x:v>6805.8</x:v>
+      </x:c>
+      <x:c r="G27" s="28" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>-114</x:v>
+        <x:v>-210</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>-0.016249037885914697</x:v>
+        <x:v>-0.029932438210895418</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
@@ -1706,46 +1742,46 @@
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B28" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B28" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C28" s="28"/>
-      <x:c r="D28" s="28"/>
-      <x:c r="E28" s="28"/>
-      <x:c r="F28" s="28"/>
-      <x:c r="G28" s="28"/>
-      <x:c r="H28" s="28"/>
-      <x:c r="I28" s="30" t="n">
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="32" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
         <x:v>783.8</x:v>
       </x:c>
-      <x:c r="J28" s="28"/>
-      <x:c r="K28" s="28"/>
+      <x:c r="J28" s="30"/>
+      <x:c r="K28" s="30"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="29" t="str">
+      <x:c r="A29" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="28"/>
-      <x:c r="C29" s="28"/>
-      <x:c r="D29" s="28"/>
-      <x:c r="E29" s="28"/>
-      <x:c r="F29" s="28"/>
-      <x:c r="G29" s="28"/>
-      <x:c r="H29" s="28"/>
-      <x:c r="I29" s="32" t="n">
+      <x:c r="B29" s="30"/>
+      <x:c r="C29" s="30"/>
+      <x:c r="D29" s="30"/>
+      <x:c r="E29" s="30"/>
+      <x:c r="F29" s="30"/>
+      <x:c r="G29" s="30"/>
+      <x:c r="H29" s="30"/>
+      <x:c r="I29" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
         <x:v>391.9</x:v>
       </x:c>
-      <x:c r="J29" s="28"/>
-      <x:c r="K29" s="28"/>
+      <x:c r="J29" s="30"/>
+      <x:c r="K29" s="30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="17" t="str">
@@ -1868,42 +1904,42 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="29" t="str">
+      <x:c r="A35" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B35" s="28" t="n">
+      <x:c r="B35" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C35" s="28"/>
-      <x:c r="D35" s="28"/>
-      <x:c r="E35" s="28"/>
-      <x:c r="F35" s="28"/>
-      <x:c r="G35" s="28"/>
-      <x:c r="H35" s="28"/>
-      <x:c r="I35" s="30" t="n">
+      <x:c r="C35" s="30"/>
+      <x:c r="D35" s="30"/>
+      <x:c r="E35" s="30"/>
+      <x:c r="F35" s="30"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="32" t="n">
         <x:f>ROUND(SUM(I33:I34),1)</x:f>
         <x:v>760.2</x:v>
       </x:c>
-      <x:c r="J35" s="28"/>
-      <x:c r="K35" s="28"/>
+      <x:c r="J35" s="30"/>
+      <x:c r="K35" s="30"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="29" t="str">
+      <x:c r="A36" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B36" s="28"/>
-      <x:c r="C36" s="28"/>
-      <x:c r="D36" s="28"/>
-      <x:c r="E36" s="28"/>
-      <x:c r="F36" s="28"/>
-      <x:c r="G36" s="28"/>
-      <x:c r="H36" s="28"/>
-      <x:c r="I36" s="32" t="n">
+      <x:c r="B36" s="30"/>
+      <x:c r="C36" s="30"/>
+      <x:c r="D36" s="30"/>
+      <x:c r="E36" s="30"/>
+      <x:c r="F36" s="30"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
         <x:v>380.1</x:v>
       </x:c>
-      <x:c r="J36" s="28"/>
-      <x:c r="K36" s="28"/>
+      <x:c r="J36" s="30"/>
+      <x:c r="K36" s="30"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="17" t="str">
@@ -2026,42 +2062,42 @@
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="29" t="str">
+      <x:c r="A42" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B42" s="28" t="n">
+      <x:c r="B42" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C42" s="28"/>
-      <x:c r="D42" s="28"/>
-      <x:c r="E42" s="28"/>
-      <x:c r="F42" s="28"/>
-      <x:c r="G42" s="28"/>
-      <x:c r="H42" s="28"/>
-      <x:c r="I42" s="30" t="n">
+      <x:c r="C42" s="30"/>
+      <x:c r="D42" s="30"/>
+      <x:c r="E42" s="30"/>
+      <x:c r="F42" s="30"/>
+      <x:c r="G42" s="30"/>
+      <x:c r="H42" s="30"/>
+      <x:c r="I42" s="32" t="n">
         <x:f>ROUND(SUM(I40:I41),1)</x:f>
         <x:v>273.8</x:v>
       </x:c>
-      <x:c r="J42" s="28"/>
-      <x:c r="K42" s="28"/>
+      <x:c r="J42" s="30"/>
+      <x:c r="K42" s="30"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="29" t="str">
+      <x:c r="A43" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="28"/>
-      <x:c r="C43" s="28"/>
-      <x:c r="D43" s="28"/>
-      <x:c r="E43" s="28"/>
-      <x:c r="F43" s="28"/>
-      <x:c r="G43" s="28"/>
-      <x:c r="H43" s="28"/>
-      <x:c r="I43" s="32" t="n">
+      <x:c r="B43" s="30"/>
+      <x:c r="C43" s="30"/>
+      <x:c r="D43" s="30"/>
+      <x:c r="E43" s="30"/>
+      <x:c r="F43" s="30"/>
+      <x:c r="G43" s="30"/>
+      <x:c r="H43" s="30"/>
+      <x:c r="I43" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
         <x:v>136.9</x:v>
       </x:c>
-      <x:c r="J43" s="28"/>
-      <x:c r="K43" s="28"/>
+      <x:c r="J43" s="30"/>
+      <x:c r="K43" s="30"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="17" t="str">
@@ -2184,42 +2220,42 @@
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="29" t="str">
+      <x:c r="A49" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B49" s="28" t="n">
+      <x:c r="B49" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C49" s="28"/>
-      <x:c r="D49" s="28"/>
-      <x:c r="E49" s="28"/>
-      <x:c r="F49" s="28"/>
-      <x:c r="G49" s="28"/>
-      <x:c r="H49" s="28"/>
-      <x:c r="I49" s="30" t="n">
+      <x:c r="C49" s="30"/>
+      <x:c r="D49" s="30"/>
+      <x:c r="E49" s="30"/>
+      <x:c r="F49" s="30"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="32" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
         <x:v>123.6</x:v>
       </x:c>
-      <x:c r="J49" s="28"/>
-      <x:c r="K49" s="28"/>
+      <x:c r="J49" s="30"/>
+      <x:c r="K49" s="30"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="29" t="str">
+      <x:c r="A50" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B50" s="28"/>
-      <x:c r="C50" s="28"/>
-      <x:c r="D50" s="28"/>
-      <x:c r="E50" s="28"/>
-      <x:c r="F50" s="28"/>
-      <x:c r="G50" s="28"/>
-      <x:c r="H50" s="28"/>
-      <x:c r="I50" s="32" t="n">
+      <x:c r="B50" s="30"/>
+      <x:c r="C50" s="30"/>
+      <x:c r="D50" s="30"/>
+      <x:c r="E50" s="30"/>
+      <x:c r="F50" s="30"/>
+      <x:c r="G50" s="30"/>
+      <x:c r="H50" s="30"/>
+      <x:c r="I50" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
         <x:v>61.8</x:v>
       </x:c>
-      <x:c r="J50" s="28"/>
-      <x:c r="K50" s="28"/>
+      <x:c r="J50" s="30"/>
+      <x:c r="K50" s="30"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="17" t="str">
@@ -2308,7 +2344,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>10月12日-10月13日</x:v>
+        <x:v>10月12日-10月14日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>125960</x:v>
@@ -2320,15 +2356,15 @@
         <x:v>101000</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>109500</x:v>
-      </x:c>
-      <x:c r="G55" s="34" t="n">
+        <x:v>103000</x:v>
+      </x:c>
+      <x:c r="G55" s="28" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-11500</x:v>
+        <x:v>-18000</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.0950413223140496</x:v>
+        <x:v>-0.14876033057851235</x:v>
       </x:c>
       <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
@@ -2338,46 +2374,46 @@
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B56" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="29" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C56" s="28"/>
-      <x:c r="D56" s="28"/>
-      <x:c r="E56" s="28"/>
-      <x:c r="F56" s="28"/>
-      <x:c r="G56" s="28"/>
-      <x:c r="H56" s="28"/>
-      <x:c r="I56" s="30" t="n">
+      <x:c r="C56" s="30"/>
+      <x:c r="D56" s="30"/>
+      <x:c r="E56" s="30"/>
+      <x:c r="F56" s="30"/>
+      <x:c r="G56" s="30"/>
+      <x:c r="H56" s="30"/>
+      <x:c r="I56" s="32" t="n">
         <x:f>ROUND(SUM(I54:I55),1)</x:f>
         <x:v>32760</x:v>
       </x:c>
-      <x:c r="J56" s="28"/>
-      <x:c r="K56" s="28"/>
+      <x:c r="J56" s="30"/>
+      <x:c r="K56" s="30"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="29" t="str">
+      <x:c r="A57" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B57" s="28"/>
-      <x:c r="C57" s="28"/>
-      <x:c r="D57" s="28"/>
-      <x:c r="E57" s="28"/>
-      <x:c r="F57" s="28"/>
-      <x:c r="G57" s="28"/>
-      <x:c r="H57" s="28"/>
-      <x:c r="I57" s="32" t="n">
+      <x:c r="B57" s="30"/>
+      <x:c r="C57" s="30"/>
+      <x:c r="D57" s="30"/>
+      <x:c r="E57" s="30"/>
+      <x:c r="F57" s="30"/>
+      <x:c r="G57" s="30"/>
+      <x:c r="H57" s="30"/>
+      <x:c r="I57" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
         <x:v>16380</x:v>
       </x:c>
-      <x:c r="J57" s="28"/>
-      <x:c r="K57" s="28"/>
+      <x:c r="J57" s="30"/>
+      <x:c r="K57" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2474,7 +2510,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7138.58</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-160.2</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -2596,43 +2632,79 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>10月14日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7001.91</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7035.18</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>6891.6</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>6905.17</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-118.1</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.01680852942097788</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>143.6</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>951</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="B11" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>1094.6</x:v>
+      </x:c>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>237.8</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>218.9</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2721,7 +2793,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7248.43</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-186.7</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -2793,7 +2865,7 @@
       <x:c r="G6" s="23" t="n">
         <x:v>7093.02</x:v>
       </x:c>
-      <x:c r="H6" s="34" t="n">
+      <x:c r="H6" s="28" t="n">
         <x:v>-158</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
@@ -2843,43 +2915,79 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>10月14日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>7066.73</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>7120.11</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>6969.02</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>6980.11</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-105</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.014817031258600899</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>151.1</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>882.5999999999999</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="B11" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>1033.6999999999998</x:v>
+      </x:c>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>220.7</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>206.7</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3090,43 +3198,79 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>10月14日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>3790.63</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>3811.81</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>3761.96</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>3767.23</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-33.6</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.00884799755844734</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>49.8</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>257.19999999999993</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="B11" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>306.99999999999994</x:v>
+      </x:c>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>64.3</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>61.4</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3337,43 +3481,79 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>10月14日</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>6895</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>6925.2</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>6761</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:v>6805.8</x:v>
+      </x:c>
+      <x:c r="H8" s="23" t="n">
+        <x:v>-96</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="n">
+        <x:v>-0.013909414935234232</x:v>
+      </x:c>
+      <x:c r="J8" s="23" t="n">
+        <x:f>ROUND(E8-F8,1)</x:f>
+        <x:v>164.2</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
-        <x:f>SUM(J4:J7)</x:f>
-        <x:v>969.6000000000001</x:v>
-      </x:c>
-      <x:c r="K10" s="28"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="B11" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="32" t="n">
+        <x:f>SUM(J4:J8)</x:f>
+        <x:v>1133.8000000000002</x:v>
+      </x:c>
+      <x:c r="K11" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
-        <x:v>242.4</x:v>
-      </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="30"/>
+      <x:c r="E12" s="30"/>
+      <x:c r="F12" s="30"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="30"/>
+      <x:c r="J12" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
+        <x:v>226.8</x:v>
+      </x:c>
+      <x:c r="K12" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3462,7 +3642,7 @@
       <x:c r="G4" s="23" t="n">
         <x:v>7122.8</x:v>
       </x:c>
-      <x:c r="H4" s="34" t="n">
+      <x:c r="H4" s="28" t="n">
         <x:v>-187.4</x:v>
       </x:c>
       <x:c r="I4" s="24" t="n">
@@ -3585,42 +3765,42 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+      <x:c r="A10" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
+      <x:c r="B10" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="30"/>
+      <x:c r="J10" s="32" t="n">
         <x:f>SUM(J4:J7)</x:f>
         <x:v>937.4000000000001</x:v>
       </x:c>
-      <x:c r="K10" s="28"/>
+      <x:c r="K10" s="30"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
         <x:v>234.4</x:v>
       </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="K11" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3832,42 +4012,42 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+      <x:c r="A10" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
+      <x:c r="B10" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="30"/>
+      <x:c r="J10" s="32" t="n">
         <x:f>SUM(J4:J7)</x:f>
         <x:v>363.4</x:v>
       </x:c>
-      <x:c r="K10" s="28"/>
+      <x:c r="K10" s="30"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
         <x:v>90.9</x:v>
       </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="K11" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4079,42 +4259,42 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="29" t="str">
+      <x:c r="A10" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="n">
+      <x:c r="B10" s="30" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="28"/>
-      <x:c r="E10" s="28"/>
-      <x:c r="F10" s="28"/>
-      <x:c r="G10" s="28"/>
-      <x:c r="H10" s="28"/>
-      <x:c r="I10" s="28"/>
-      <x:c r="J10" s="30" t="n">
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="30"/>
+      <x:c r="J10" s="32" t="n">
         <x:f>SUM(J4:J7)</x:f>
         <x:v>179</x:v>
       </x:c>
-      <x:c r="K10" s="28"/>
+      <x:c r="K10" s="30"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="28"/>
-      <x:c r="E11" s="28"/>
-      <x:c r="F11" s="28"/>
-      <x:c r="G11" s="28"/>
-      <x:c r="H11" s="28"/>
-      <x:c r="I11" s="28"/>
-      <x:c r="J11" s="32" t="n">
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="30"/>
+      <x:c r="E11" s="30"/>
+      <x:c r="F11" s="30"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="30"/>
+      <x:c r="J11" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(J4:J7),0),1)</x:f>
         <x:v>44.8</x:v>
       </x:c>
-      <x:c r="K11" s="28"/>
+      <x:c r="K11" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-15
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc3008a43fada41a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Racc1ac8f5aaf4df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9a488111f77849c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R69cf06c4303c40c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R265d9fa69d4f4b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R5fac79b30b834061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R5ae4b3d85fb64066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R928ac4cd6c3f4dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R98d9e91143804c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R81b239f5959e4821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R148f89910c824b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rd0aee85c2a2f4fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R12d4154117994afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb0c236f0956240ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rcc8e13d97d8e4242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R742f4380623c4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc8f7bd3c6ff946a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R638833992ffc4ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3e9c3e94fa0b41c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R461e53fccac24321"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,25 +485,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>7035.18</x:v>
+        <x:v>6805.19</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6891.6</x:v>
+        <x:v>6652.55</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>143.6</x:v>
+        <x:v>152.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1094.6</x:v>
+        <x:v>1247.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>218.9</x:v>
+        <x:v>207.9</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -514,25 +514,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>7120.11</x:v>
+        <x:v>6870.95</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6969.02</x:v>
+        <x:v>6725.59</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>151.1</x:v>
+        <x:v>145.4</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1033.7</x:v>
+        <x:v>1179.1</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>206.7</x:v>
+        <x:v>196.5</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +543,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3811.81</x:v>
+        <x:v>3724.56</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3761.96</x:v>
+        <x:v>3674.82</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>49.8</x:v>
+        <x:v>49.7</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>307</x:v>
+        <x:v>356.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>61.4</x:v>
+        <x:v>59.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +572,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6925.2</x:v>
+        <x:v>6706.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6761</x:v>
+        <x:v>6532.4</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>164.2</x:v>
+        <x:v>174.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1133.8</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>226.8</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -659,25 +659,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2760.8</x:v>
+        <x:v>2719.8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2722.4</x:v>
+        <x:v>2677.6</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>38.4</x:v>
+        <x:v>42.2</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>217.4</x:v>
+        <x:v>259.6</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>43.5</x:v>
+        <x:v>43.3</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -688,25 +688,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>108380</x:v>
+        <x:v>103400</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>103000</x:v>
+        <x:v>102000</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>5380</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>45560</x:v>
+        <x:v>46960</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>9112</x:v>
+        <x:v>7826.7</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -720,7 +720,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1083,31 +1083,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>45560</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>103000</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>103400</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>102000</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>102000</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="n">
+        <x:v>-1000</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.009708737864077666</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -1115,11 +1133,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>9112</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>46960</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>7826.7</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1238,7 +1274,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7132.68</x:v>
@@ -1247,28 +1283,28 @@
         <x:v>7145.06</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
-        <x:v>6796.58</x:v>
+        <x:v>6652.55</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>6905.17</x:v>
+        <x:v>6678.65</x:v>
       </x:c>
       <x:c r="G6" s="28" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>-250.7</x:v>
+        <x:v>-477.3</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>-0.03503956869217184</x:v>
+        <x:v>-0.06669452242971197</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>348.5</x:v>
+        <x:v>492.5</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1286,7 +1322,7 @@
       <x:c r="H7" s="30"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>789.9</x:v>
+        <x:v>933.9</x:v>
       </x:c>
       <x:c r="J7" s="30"/>
       <x:c r="K7" s="30"/>
@@ -1304,7 +1340,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>395</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1396,7 +1432,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7226.07</x:v>
@@ -1405,28 +1441,28 @@
         <x:v>7236.78</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>6904.6</x:v>
+        <x:v>6725.59</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>6980.11</x:v>
+        <x:v>6769.25</x:v>
       </x:c>
       <x:c r="G13" s="28" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-270.9</x:v>
+        <x:v>-481.8</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.03736031256335337</x:v>
+        <x:v>-0.06644039933747159</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>332.2</x:v>
+        <x:v>511.2</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1444,7 +1480,7 @@
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="32" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>745</x:v>
+        <x:v>924</x:v>
       </x:c>
       <x:c r="J14" s="30"/>
       <x:c r="K14" s="30"/>
@@ -1462,7 +1498,7 @@
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>372.5</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="J15" s="30"/>
       <x:c r="K15" s="30"/>
@@ -1554,7 +1590,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3806.98</x:v>
@@ -1563,28 +1599,28 @@
         <x:v>3828.22</x:v>
       </x:c>
       <x:c r="E20" s="23" t="n">
-        <x:v>3741.53</x:v>
+        <x:v>3674.82</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3767.23</x:v>
+        <x:v>3707.48</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-46.6</x:v>
+        <x:v>-106.3</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.01220832819845874</x:v>
+        <x:v>-0.027875158307090864</x:v>
       </x:c>
       <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>86.7</x:v>
+        <x:v>153.4</x:v>
       </x:c>
       <x:c r="J20" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1602,7 +1638,7 @@
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="32" t="n">
         <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>196.7</x:v>
+        <x:v>263.4</x:v>
       </x:c>
       <x:c r="J21" s="30"/>
       <x:c r="K21" s="30"/>
@@ -1620,7 +1656,7 @@
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>98.4</x:v>
+        <x:v>131.7</x:v>
       </x:c>
       <x:c r="J22" s="30"/>
       <x:c r="K22" s="30"/>
@@ -1712,7 +1748,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7000</x:v>
@@ -1721,28 +1757,28 @@
         <x:v>7031.2</x:v>
       </x:c>
       <x:c r="E27" s="23" t="n">
-        <x:v>6680</x:v>
+        <x:v>6532.4</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>6805.8</x:v>
+        <x:v>6553.6</x:v>
       </x:c>
       <x:c r="G27" s="28" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>-210</x:v>
+        <x:v>-462.2</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>-0.029932438210895418</x:v>
+        <x:v>-0.06587987114798022</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>351.2</x:v>
+        <x:v>498.8</x:v>
       </x:c>
       <x:c r="J27" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1760,7 +1796,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="32" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>783.8</x:v>
+        <x:v>931.4</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -1778,7 +1814,7 @@
       <x:c r="H29" s="30"/>
       <x:c r="I29" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>391.9</x:v>
+        <x:v>465.7</x:v>
       </x:c>
       <x:c r="J29" s="30"/>
       <x:c r="K29" s="30"/>
@@ -2186,7 +2222,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C48" s="23" t="n">
         <x:v>2762</x:v>
@@ -2195,28 +2231,28 @@
         <x:v>2794</x:v>
       </x:c>
       <x:c r="E48" s="23" t="n">
-        <x:v>2722.4</x:v>
+        <x:v>2677.6</x:v>
       </x:c>
       <x:c r="F48" s="23" t="n">
-        <x:v>2733.8</x:v>
+        <x:v>2718.6</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-30.2</x:v>
+        <x:v>-45.4</x:v>
       </x:c>
       <x:c r="H48" s="24" t="n">
         <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.010926193921852345</x:v>
+        <x:v>-0.016425470332851022</x:v>
       </x:c>
       <x:c r="I48" s="26" t="n">
         <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>71.6</x:v>
+        <x:v>116.4</x:v>
       </x:c>
       <x:c r="J48" s="22" t="str">
         <x:v>IH2612</x:v>
       </x:c>
       <x:c r="K48" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2234,7 +2270,7 @@
       <x:c r="H49" s="30"/>
       <x:c r="I49" s="32" t="n">
         <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>135</x:v>
+        <x:v>179.8</x:v>
       </x:c>
       <x:c r="J49" s="30"/>
       <x:c r="K49" s="30"/>
@@ -2252,7 +2288,7 @@
       <x:c r="H50" s="30"/>
       <x:c r="I50" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>67.5</x:v>
+        <x:v>89.9</x:v>
       </x:c>
       <x:c r="J50" s="30"/>
       <x:c r="K50" s="30"/>
@@ -2344,7 +2380,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>10月12日-10月14日</x:v>
+        <x:v>10月12日-10月15日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>125960</x:v>
@@ -2356,15 +2392,15 @@
         <x:v>101000</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>103000</x:v>
+        <x:v>102000</x:v>
       </x:c>
       <x:c r="G55" s="28" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-18000</x:v>
+        <x:v>-19000</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.14876033057851235</x:v>
+        <x:v>-0.15702479338842978</x:v>
       </x:c>
       <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
@@ -2374,7 +2410,7 @@
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2668,31 +2704,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>1094.6</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>6734.31</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>6805.19</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>6652.55</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>6678.65</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="n">
+        <x:v>-226.5</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.032804405974074524</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>152.6</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -2700,11 +2754,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>218.9</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1247.1999999999998</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>207.9</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2951,31 +3023,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>1033.6999999999998</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>6809.83</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>6870.95</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>6725.59</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>6769.25</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="n">
+        <x:v>-210.9</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.030208692986213648</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>145.4</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -2983,11 +3073,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>206.7</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1179.1</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>196.5</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3234,31 +3342,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>306.99999999999994</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>3710.7</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>3724.56</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>3674.82</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>3707.48</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-59.7</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.015860459807338523</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>49.7</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -3266,11 +3392,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>61.4</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>356.69999999999993</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>59.4</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3517,31 +3661,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>1133.8000000000002</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>6627</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>6706.6</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>6532.4</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>6553.6</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="n">
+        <x:v>-252.2</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.037056628170090145</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>174.2</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -3549,11 +3711,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>226.8</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>1308.0000000000002</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4366,31 +4546,49 @@
         <x:v>IH2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B11" s="30" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C11" s="30"/>
-      <x:c r="D11" s="30"/>
-      <x:c r="E11" s="30"/>
-      <x:c r="F11" s="30"/>
-      <x:c r="G11" s="30"/>
-      <x:c r="H11" s="30"/>
-      <x:c r="I11" s="30"/>
-      <x:c r="J11" s="32" t="n">
-        <x:f>SUM(J4:J8)</x:f>
-        <x:v>217.4</x:v>
-      </x:c>
-      <x:c r="K11" s="30"/>
+    <x:row r="9">
+      <x:c r="A9" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>10月15日</x:v>
+      </x:c>
+      <x:c r="D9" s="23" t="n">
+        <x:v>2695.6</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>2719.8</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>2677.6</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>2718.6</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>-15.2</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="n">
+        <x:v>-0.00556002633696695</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:f>ROUND(E9-F9,1)</x:f>
+        <x:v>42.2</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B12" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="30"/>
       <x:c r="E12" s="30"/>
@@ -4398,11 +4596,29 @@
       <x:c r="G12" s="30"/>
       <x:c r="H12" s="30"/>
       <x:c r="I12" s="30"/>
-      <x:c r="J12" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J8),0),1)</x:f>
-        <x:v>43.5</x:v>
+      <x:c r="J12" s="32" t="n">
+        <x:f>SUM(J4:J9)</x:f>
+        <x:v>259.6</x:v>
       </x:c>
       <x:c r="K12" s="30"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="30"/>
+      <x:c r="E13" s="30"/>
+      <x:c r="F13" s="30"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="30"/>
+      <x:c r="J13" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+        <x:v>43.3</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-16
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R5450d9c8ae164658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rb79f2b8b9f82465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rfb2333ad697445a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R48097fc073c14c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R1548f0f8129e41b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R4112d5891e5b4f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc665623d394d4e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R093aa4a8b6cd4d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rd60a395ac02346ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rf01c361a6fbc4e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R7fc6c050e45a4bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Raad81cdedebf46c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Re4d2812f58864630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R2b138a8b04ae48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R7507cd6d18334972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R34e4ba02b0054636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R0d47c807d61842a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rbc84aac8789e4ab6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rcf56961b685b403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R6f8597c2c5504609"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="General"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -77,8 +77,14 @@
       <x:color rgb="FF1D4ED8"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -108,6 +114,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFBFDBFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -145,7 +156,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -231,6 +242,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
@@ -485,22 +517,22 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6805.19</x:v>
+        <x:v>6834.45</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6652.55</x:v>
+        <x:v>6626.52</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>152.6</x:v>
+        <x:v>207.9</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1247.2</x:v>
+        <x:v>1455.1</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
         <x:v>207.9</x:v>
@@ -514,25 +546,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6870.95</x:v>
+        <x:v>6907.9</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6725.59</x:v>
+        <x:v>6719.82</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>145.4</x:v>
+        <x:v>188.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1179.1</x:v>
+        <x:v>1367.2</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>196.5</x:v>
+        <x:v>195.3</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -543,25 +575,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3724.56</x:v>
+        <x:v>3750.77</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3674.82</x:v>
+        <x:v>3681.28</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>49.7</x:v>
+        <x:v>69.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>356.7</x:v>
+        <x:v>426.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>59.4</x:v>
+        <x:v>60.9</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -572,25 +604,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6706.6</x:v>
+        <x:v>6748</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6532.4</x:v>
+        <x:v>6519.6</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>174.2</x:v>
+        <x:v>228.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1308</x:v>
+        <x:v>1536.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>218</x:v>
+        <x:v>219.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -720,7 +752,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1274,7 +1306,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>10月12日-10月15日</x:v>
+        <x:v>10月12日-10月16日</x:v>
       </x:c>
       <x:c r="C6" s="23" t="n">
         <x:v>7132.68</x:v>
@@ -1283,28 +1315,28 @@
         <x:v>7145.06</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
-        <x:v>6652.55</x:v>
+        <x:v>6626.52</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
-        <x:v>6678.65</x:v>
+        <x:v>6681.94</x:v>
       </x:c>
       <x:c r="G6" s="28" t="n">
         <x:f>ROUND(F6-F5,1)</x:f>
-        <x:v>-477.3</x:v>
+        <x:v>-474</x:v>
       </x:c>
       <x:c r="H6" s="24" t="n">
         <x:f>IFERROR(F6/F5-1,"")</x:f>
-        <x:v>-0.06669452242971197</x:v>
+        <x:v>-0.06623476259483418</x:v>
       </x:c>
       <x:c r="I6" s="26" t="n">
         <x:f>ROUND(D6-E6,1)</x:f>
-        <x:v>492.5</x:v>
+        <x:v>518.5</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K6" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1322,7 +1354,7 @@
       <x:c r="H7" s="30"/>
       <x:c r="I7" s="32" t="n">
         <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>933.9</x:v>
+        <x:v>959.9</x:v>
       </x:c>
       <x:c r="J7" s="30"/>
       <x:c r="K7" s="30"/>
@@ -1340,7 +1372,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>467</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1432,7 +1464,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>10月12日-10月15日</x:v>
+        <x:v>10月12日-10月16日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:v>7226.07</x:v>
@@ -1441,28 +1473,28 @@
         <x:v>7236.78</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>6725.59</x:v>
+        <x:v>6719.82</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>6769.25</x:v>
+        <x:v>6772.75</x:v>
       </x:c>
       <x:c r="G13" s="28" t="n">
         <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-481.8</x:v>
+        <x:v>-478.3</x:v>
       </x:c>
       <x:c r="H13" s="24" t="n">
         <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.06644039933747159</x:v>
+        <x:v>-0.06595770796068412</x:v>
       </x:c>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>511.2</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1480,7 +1512,7 @@
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="32" t="n">
         <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>924</x:v>
+        <x:v>929.8</x:v>
       </x:c>
       <x:c r="J14" s="30"/>
       <x:c r="K14" s="30"/>
@@ -1498,7 +1530,7 @@
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>462</x:v>
+        <x:v>464.9</x:v>
       </x:c>
       <x:c r="J15" s="30"/>
       <x:c r="K15" s="30"/>
@@ -1590,7 +1622,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>10月12日-10月15日</x:v>
+        <x:v>10月12日-10月16日</x:v>
       </x:c>
       <x:c r="C20" s="23" t="n">
         <x:v>3806.98</x:v>
@@ -1602,15 +1634,15 @@
         <x:v>3674.82</x:v>
       </x:c>
       <x:c r="F20" s="23" t="n">
-        <x:v>3707.48</x:v>
+        <x:v>3716.28</x:v>
       </x:c>
       <x:c r="G20" s="23" t="n">
         <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-106.3</x:v>
+        <x:v>-97.5</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
         <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.027875158307090864</x:v>
+        <x:v>-0.02556774232456427</x:v>
       </x:c>
       <x:c r="I20" s="26" t="n">
         <x:f>ROUND(D20-E20,1)</x:f>
@@ -1620,7 +1652,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K20" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1748,7 +1780,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>10月12日-10月15日</x:v>
+        <x:v>10月12日-10月16日</x:v>
       </x:c>
       <x:c r="C27" s="23" t="n">
         <x:v>7000</x:v>
@@ -1757,28 +1789,28 @@
         <x:v>7031.2</x:v>
       </x:c>
       <x:c r="E27" s="23" t="n">
-        <x:v>6532.4</x:v>
+        <x:v>6519.6</x:v>
       </x:c>
       <x:c r="F27" s="23" t="n">
-        <x:v>6553.6</x:v>
+        <x:v>6583.6</x:v>
       </x:c>
       <x:c r="G27" s="28" t="n">
         <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>-462.2</x:v>
+        <x:v>-432.2</x:v>
       </x:c>
       <x:c r="H27" s="24" t="n">
         <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>-0.06587987114798022</x:v>
+        <x:v>-0.06160380854642378</x:v>
       </x:c>
       <x:c r="I27" s="26" t="n">
         <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>498.8</x:v>
+        <x:v>511.6</x:v>
       </x:c>
       <x:c r="J27" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K27" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1796,7 +1828,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="32" t="n">
         <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>931.4</x:v>
+        <x:v>944.2</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -1814,7 +1846,7 @@
       <x:c r="H29" s="30"/>
       <x:c r="I29" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>465.7</x:v>
+        <x:v>472.1</x:v>
       </x:c>
       <x:c r="J29" s="30"/>
       <x:c r="K29" s="30"/>
@@ -2740,31 +2772,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1247.1999999999998</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>10月16日</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="n">
+        <x:v>6777.39</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="n">
+        <x:v>6834.45</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="n">
+        <x:v>6626.52</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="n">
+        <x:v>6681.94</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="I10" s="43" t="n">
+        <x:v>0.0004926145253905112</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>207.9</x:v>
+      </x:c>
+      <x:c r="K10" s="41" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
       <x:c r="E13" s="30"/>
@@ -2772,11 +2822,29 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
+      <x:c r="J13" s="32" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1455.1</x:v>
+      </x:c>
+      <x:c r="K13" s="30"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="30"/>
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="30"/>
+      <x:c r="J14" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
         <x:v>207.9</x:v>
       </x:c>
-      <x:c r="K13" s="30"/>
+      <x:c r="K14" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3059,31 +3127,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1179.1</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>10月16日</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="n">
+        <x:v>6863.19</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="n">
+        <x:v>6907.9</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="n">
+        <x:v>6719.82</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="n">
+        <x:v>6772.75</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="I10" s="43" t="n">
+        <x:v>0.00051704398567054</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>188.1</x:v>
+      </x:c>
+      <x:c r="K10" s="41" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
       <x:c r="E13" s="30"/>
@@ -3091,11 +3177,29 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>196.5</x:v>
+      <x:c r="J13" s="32" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1367.1999999999998</x:v>
       </x:c>
       <x:c r="K13" s="30"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="30"/>
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="30"/>
+      <x:c r="J14" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>195.3</x:v>
+      </x:c>
+      <x:c r="K14" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3378,31 +3482,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>356.69999999999993</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>10月16日</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="n">
+        <x:v>3723.8</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="n">
+        <x:v>3750.77</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="n">
+        <x:v>3681.28</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="n">
+        <x:v>3716.28</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="n">
+        <x:v>8.8</x:v>
+      </x:c>
+      <x:c r="I10" s="43" t="n">
+        <x:v>0.0023735798979360734</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>69.5</x:v>
+      </x:c>
+      <x:c r="K10" s="41" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
       <x:c r="E13" s="30"/>
@@ -3410,11 +3532,29 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>59.4</x:v>
+      <x:c r="J13" s="32" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>426.19999999999993</x:v>
       </x:c>
       <x:c r="K13" s="30"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="30"/>
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="30"/>
+      <x:c r="J14" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>60.9</x:v>
+      </x:c>
+      <x:c r="K14" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3697,31 +3837,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B12" s="30" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C12" s="30"/>
-      <x:c r="D12" s="30"/>
-      <x:c r="E12" s="30"/>
-      <x:c r="F12" s="30"/>
-      <x:c r="G12" s="30"/>
-      <x:c r="H12" s="30"/>
-      <x:c r="I12" s="30"/>
-      <x:c r="J12" s="32" t="n">
-        <x:f>SUM(J4:J9)</x:f>
-        <x:v>1308.0000000000002</x:v>
-      </x:c>
-      <x:c r="K12" s="30"/>
+    <x:row r="10">
+      <x:c r="A10" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>10月16日</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="n">
+        <x:v>6652</x:v>
+      </x:c>
+      <x:c r="E10" s="42" t="n">
+        <x:v>6748</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="n">
+        <x:v>6519.6</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="n">
+        <x:v>6583.6</x:v>
+      </x:c>
+      <x:c r="H10" s="42" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I10" s="43" t="n">
+        <x:v>0.00457763671875</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:f>ROUND(E10-F10,1)</x:f>
+        <x:v>228.4</x:v>
+      </x:c>
+      <x:c r="K10" s="41" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B13" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
       <x:c r="E13" s="30"/>
@@ -3729,11 +3887,29 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30"/>
-      <x:c r="J13" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J9),0),1)</x:f>
-        <x:v>218</x:v>
+      <x:c r="J13" s="32" t="n">
+        <x:f>SUM(J4:J10)</x:f>
+        <x:v>1536.4000000000003</x:v>
       </x:c>
       <x:c r="K13" s="30"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B14" s="30"/>
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="30"/>
+      <x:c r="E14" s="30"/>
+      <x:c r="F14" s="30"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="30"/>
+      <x:c r="J14" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
+        <x:v>219.5</x:v>
+      </x:c>
+      <x:c r="K14" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-19
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Raf37450212f44a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R2b8b101e1c2a4fd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R8247433566064d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R6a949ea312364e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R0f24de5700e2401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rec68d35ebb2f45e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R47b524d0fd474e84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R87ca9d0aa0b642b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rba5b9b148a704f54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rce77bee9e6f744d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R69b07f83594149cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rb1decc03c8414862"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R4e9578e14483456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R28ebbe6ce1614944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R8cbdde44896049f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb21d6bc8c6924477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc1212e1a0bc04e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re546fc2eab964429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9af04ea328184123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R4b4bfd52efeb4a72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6834.45</x:v>
+        <x:v>6746.32</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6626.52</x:v>
+        <x:v>6578.94</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>207.9</x:v>
+        <x:v>167.4</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1455.1</x:v>
+        <x:v>1622.5</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>207.9</x:v>
+        <x:v>202.8</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6907.9</x:v>
+        <x:v>6848</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6719.82</x:v>
+        <x:v>6692.83</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>188.1</x:v>
+        <x:v>155.2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1367.2</x:v>
+        <x:v>1522.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>195.3</x:v>
+        <x:v>190.3</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3750.77</x:v>
+        <x:v>3743.8</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3681.28</x:v>
+        <x:v>3692.29</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>69.5</x:v>
+        <x:v>51.5</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>426.2</x:v>
+        <x:v>477.7</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>60.9</x:v>
+        <x:v>59.7</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6748</x:v>
+        <x:v>6680</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6519.6</x:v>
+        <x:v>6505</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>228.4</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1536.4</x:v>
+        <x:v>1711.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>219.5</x:v>
+        <x:v>213.9</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>102280</x:v>
+        <x:v>103280</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>99500</x:v>
+        <x:v>99600</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>2780</x:v>
+        <x:v>3680</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>49740</x:v>
+        <x:v>53420</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>7105.7</x:v>
+        <x:v>6677.5</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-16</x:v>
+        <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1190,31 +1190,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="30" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>49740</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>99600</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>103280</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>99600</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>103180</x:v>
+      </x:c>
+      <x:c r="H11" s="28" t="n">
+        <x:v>3680</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.036984924623115534</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>3680</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="30"/>
       <x:c r="D14" s="30"/>
       <x:c r="E14" s="30"/>
@@ -1222,11 +1240,29 @@
       <x:c r="G14" s="30"/>
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="30"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>7105.7</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>53420</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="30"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>6677.5</x:v>
+      </x:c>
+      <x:c r="K15" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1379,1160 +1415,1350 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B7" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C7" s="30"/>
-      <x:c r="D7" s="30"/>
-      <x:c r="E7" s="30"/>
-      <x:c r="F7" s="30"/>
-      <x:c r="G7" s="30"/>
-      <x:c r="H7" s="30"/>
-      <x:c r="I7" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I6),1)</x:f>
-        <x:v>959.9</x:v>
-      </x:c>
-      <x:c r="J7" s="30"/>
-      <x:c r="K7" s="30"/>
+      <x:c r="A7" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="n">
+        <x:v>6639.94</x:v>
+      </x:c>
+      <x:c r="D7" s="23" t="n">
+        <x:v>6746.32</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="n">
+        <x:v>6578.94</x:v>
+      </x:c>
+      <x:c r="F7" s="23" t="n">
+        <x:v>6698.3</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="n">
+        <x:f>ROUND(F7-F6,1)</x:f>
+        <x:v>16.4</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="n">
+        <x:f>IFERROR(F7/F6-1,"")</x:f>
+        <x:v>0.002448390736822015</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="n">
+        <x:f>ROUND(D7-E7,1)</x:f>
+        <x:v>167.4</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B8" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="C8" s="30"/>
       <x:c r="D8" s="30"/>
       <x:c r="E8" s="30"/>
       <x:c r="F8" s="30"/>
       <x:c r="G8" s="30"/>
       <x:c r="H8" s="30"/>
-      <x:c r="I8" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I6),0),1)</x:f>
-        <x:v>480</x:v>
+      <x:c r="I8" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I7),1)</x:f>
+        <x:v>1127.3</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="17" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B9" s="30"/>
+      <x:c r="C9" s="30"/>
+      <x:c r="D9" s="30"/>
+      <x:c r="E9" s="30"/>
+      <x:c r="F9" s="30"/>
+      <x:c r="G9" s="30"/>
+      <x:c r="H9" s="30"/>
+      <x:c r="I9" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
+        <x:v>375.8</x:v>
+      </x:c>
+      <x:c r="J9" s="30"/>
+      <x:c r="K9" s="30"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B10" s="17"/>
-      <x:c r="C10" s="17"/>
-      <x:c r="D10" s="17"/>
-      <x:c r="E10" s="17"/>
-      <x:c r="F10" s="17"/>
-      <x:c r="G10" s="17"/>
-      <x:c r="H10" s="17"/>
-      <x:c r="I10" s="17"/>
-      <x:c r="J10" s="17"/>
-      <x:c r="K10" s="17"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="20" t="str">
+      <x:c r="B11" s="17"/>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="17"/>
+      <x:c r="E11" s="17"/>
+      <x:c r="F11" s="17"/>
+      <x:c r="G11" s="17"/>
+      <x:c r="H11" s="17"/>
+      <x:c r="I11" s="17"/>
+      <x:c r="J11" s="17"/>
+      <x:c r="K11" s="17"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B11" s="20" t="str">
+      <x:c r="B12" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C11" s="20" t="str">
+      <x:c r="C12" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D11" s="20" t="str">
+      <x:c r="D12" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E11" s="20" t="str">
+      <x:c r="E12" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F11" s="20" t="str">
+      <x:c r="F12" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G11" s="20" t="str">
+      <x:c r="G12" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H11" s="20" t="str">
+      <x:c r="H12" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I11" s="20" t="str">
+      <x:c r="I12" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J11" s="20" t="str">
+      <x:c r="J12" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K11" s="20" t="str">
+      <x:c r="K12" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B12" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C12" s="23" t="n">
-        <x:v>7420.44</x:v>
-      </x:c>
-      <x:c r="D12" s="23" t="n">
-        <x:v>7461.24</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="n">
-        <x:v>7048.45</x:v>
-      </x:c>
-      <x:c r="F12" s="23" t="n">
-        <x:v>7251.01</x:v>
-      </x:c>
-      <x:c r="G12" s="23"/>
-      <x:c r="H12" s="24"/>
-      <x:c r="I12" s="26" t="n">
-        <x:f>ROUND(D12-E12,1)</x:f>
-        <x:v>412.8</x:v>
-      </x:c>
-      <x:c r="J12" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K12" s="22" t="n">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
-        <x:v>7226.07</x:v>
+        <x:v>7420.44</x:v>
       </x:c>
       <x:c r="D13" s="23" t="n">
-        <x:v>7236.78</x:v>
+        <x:v>7461.24</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>6719.82</x:v>
+        <x:v>7048.45</x:v>
       </x:c>
       <x:c r="F13" s="23" t="n">
-        <x:v>6772.75</x:v>
-      </x:c>
-      <x:c r="G13" s="28" t="n">
-        <x:f>ROUND(F13-F12,1)</x:f>
-        <x:v>-478.3</x:v>
-      </x:c>
-      <x:c r="H13" s="24" t="n">
-        <x:f>IFERROR(F13/F12-1,"")</x:f>
-        <x:v>-0.06595770796068412</x:v>
-      </x:c>
+        <x:v>7251.01</x:v>
+      </x:c>
+      <x:c r="G13" s="23"/>
+      <x:c r="H13" s="24"/>
       <x:c r="I13" s="26" t="n">
         <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>517</x:v>
+        <x:v>412.8</x:v>
       </x:c>
       <x:c r="J13" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K13" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="n">
+        <x:v>7226.07</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>7236.78</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>6719.82</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>6772.75</x:v>
+      </x:c>
+      <x:c r="G14" s="28" t="n">
+        <x:f>ROUND(F14-F13,1)</x:f>
+        <x:v>-478.3</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="n">
+        <x:f>IFERROR(F14/F13-1,"")</x:f>
+        <x:v>-0.06595770796068412</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="n">
+        <x:f>ROUND(D14-E14,1)</x:f>
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="n">
+        <x:v>6735.53</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>6848</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>6692.83</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>6800.66</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:f>ROUND(F15-F14,1)</x:f>
+        <x:v>27.9</x:v>
+      </x:c>
+      <x:c r="H15" s="24" t="n">
+        <x:f>IFERROR(F15/F14-1,"")</x:f>
+        <x:v>0.004120925768705375</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="n">
+        <x:f>ROUND(D15-E15,1)</x:f>
+        <x:v>155.2</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B14" s="30" t="n">
+      <x:c r="B16" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="32" t="n">
+        <x:f>ROUND(SUM(I13:I15),1)</x:f>
+        <x:v>1085</x:v>
+      </x:c>
+      <x:c r="J16" s="30"/>
+      <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
+        <x:v>361.7</x:v>
+      </x:c>
+      <x:c r="J17" s="30"/>
+      <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="17" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="B19" s="17"/>
+      <x:c r="C19" s="17"/>
+      <x:c r="D19" s="17"/>
+      <x:c r="E19" s="17"/>
+      <x:c r="F19" s="17"/>
+      <x:c r="G19" s="17"/>
+      <x:c r="H19" s="17"/>
+      <x:c r="I19" s="17"/>
+      <x:c r="J19" s="17"/>
+      <x:c r="K19" s="17"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E20" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G20" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J20" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K20" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="n">
+        <x:v>3838.98</x:v>
+      </x:c>
+      <x:c r="D21" s="23" t="n">
+        <x:v>3864.12</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="n">
+        <x:v>3754.14</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="n">
+        <x:v>3813.79</x:v>
+      </x:c>
+      <x:c r="G21" s="23"/>
+      <x:c r="H21" s="24"/>
+      <x:c r="I21" s="26" t="n">
+        <x:f>ROUND(D21-E21,1)</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="32" t="n">
-        <x:f>ROUND(SUM(I12:I13),1)</x:f>
-        <x:v>929.8</x:v>
-      </x:c>
-      <x:c r="J14" s="30"/>
-      <x:c r="K14" s="30"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="n">
+        <x:v>3806.98</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="n">
+        <x:v>3828.22</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="n">
+        <x:v>3674.82</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="n">
+        <x:v>3716.28</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="n">
+        <x:f>ROUND(F22-F21,1)</x:f>
+        <x:v>-97.5</x:v>
+      </x:c>
+      <x:c r="H22" s="24" t="n">
+        <x:f>IFERROR(F22/F21-1,"")</x:f>
+        <x:v>-0.02556774232456427</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="n">
+        <x:f>ROUND(D22-E22,1)</x:f>
+        <x:v>153.4</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="n">
+        <x:v>3694.12</x:v>
+      </x:c>
+      <x:c r="D23" s="23" t="n">
+        <x:v>3743.8</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="n">
+        <x:v>3692.29</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="n">
+        <x:v>3730.92</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="n">
+        <x:f>ROUND(F23-F22,1)</x:f>
+        <x:v>14.6</x:v>
+      </x:c>
+      <x:c r="H23" s="24" t="n">
+        <x:f>IFERROR(F23/F22-1,"")</x:f>
+        <x:v>0.003939423294262001</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="n">
+        <x:f>ROUND(D23-E23,1)</x:f>
+        <x:v>51.5</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="32" t="n">
+        <x:f>ROUND(SUM(I21:I23),1)</x:f>
+        <x:v>314.9</x:v>
+      </x:c>
+      <x:c r="J24" s="30"/>
+      <x:c r="K24" s="30"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B15" s="30"/>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I12:I13),0),1)</x:f>
-        <x:v>464.9</x:v>
-      </x:c>
-      <x:c r="J15" s="30"/>
-      <x:c r="K15" s="30"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="17" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="B17" s="17"/>
-      <x:c r="C17" s="17"/>
-      <x:c r="D17" s="17"/>
-      <x:c r="E17" s="17"/>
-      <x:c r="F17" s="17"/>
-      <x:c r="G17" s="17"/>
-      <x:c r="H17" s="17"/>
-      <x:c r="I17" s="17"/>
-      <x:c r="J17" s="17"/>
-      <x:c r="K17" s="17"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="20" t="str">
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="30"/>
+      <x:c r="E25" s="30"/>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="J25" s="30"/>
+      <x:c r="K25" s="30"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
+      <x:c r="E27" s="17"/>
+      <x:c r="F27" s="17"/>
+      <x:c r="G27" s="17"/>
+      <x:c r="H27" s="17"/>
+      <x:c r="I27" s="17"/>
+      <x:c r="J27" s="17"/>
+      <x:c r="K27" s="17"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B18" s="20" t="str">
+      <x:c r="B28" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C18" s="20" t="str">
+      <x:c r="C28" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D18" s="20" t="str">
+      <x:c r="D28" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E18" s="20" t="str">
+      <x:c r="E28" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F18" s="20" t="str">
+      <x:c r="F28" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G18" s="20" t="str">
+      <x:c r="G28" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H18" s="20" t="str">
+      <x:c r="H28" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I18" s="20" t="str">
+      <x:c r="I28" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J18" s="20" t="str">
+      <x:c r="J28" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K18" s="20" t="str">
+      <x:c r="K28" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="22" t="n">
+    <x:row r="29">
+      <x:c r="A29" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B19" s="22" t="str">
+      <x:c r="B29" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C19" s="23" t="n">
-        <x:v>3838.98</x:v>
-      </x:c>
-      <x:c r="D19" s="23" t="n">
-        <x:v>3864.12</x:v>
-      </x:c>
-      <x:c r="E19" s="23" t="n">
-        <x:v>3754.14</x:v>
-      </x:c>
-      <x:c r="F19" s="23" t="n">
-        <x:v>3813.79</x:v>
-      </x:c>
-      <x:c r="G19" s="23"/>
-      <x:c r="H19" s="24"/>
-      <x:c r="I19" s="26" t="n">
-        <x:f>ROUND(D19-E19,1)</x:f>
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="J19" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K19" s="22" t="n">
+      <x:c r="C29" s="23" t="n">
+        <x:v>7182.8</x:v>
+      </x:c>
+      <x:c r="D29" s="23" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="n">
+        <x:v>6819.2</x:v>
+      </x:c>
+      <x:c r="F29" s="23" t="n">
+        <x:v>7015.8</x:v>
+      </x:c>
+      <x:c r="G29" s="23"/>
+      <x:c r="H29" s="24"/>
+      <x:c r="I29" s="26" t="n">
+        <x:f>ROUND(D29-E29,1)</x:f>
+        <x:v>432.6</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="22" t="n">
+    <x:row r="30">
+      <x:c r="A30" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B20" s="22" t="str">
+      <x:c r="B30" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C20" s="23" t="n">
-        <x:v>3806.98</x:v>
-      </x:c>
-      <x:c r="D20" s="23" t="n">
-        <x:v>3828.22</x:v>
-      </x:c>
-      <x:c r="E20" s="23" t="n">
-        <x:v>3674.82</x:v>
-      </x:c>
-      <x:c r="F20" s="23" t="n">
-        <x:v>3716.28</x:v>
-      </x:c>
-      <x:c r="G20" s="23" t="n">
-        <x:f>ROUND(F20-F19,1)</x:f>
-        <x:v>-97.5</x:v>
-      </x:c>
-      <x:c r="H20" s="24" t="n">
-        <x:f>IFERROR(F20/F19-1,"")</x:f>
-        <x:v>-0.02556774232456427</x:v>
-      </x:c>
-      <x:c r="I20" s="26" t="n">
-        <x:f>ROUND(D20-E20,1)</x:f>
-        <x:v>153.4</x:v>
-      </x:c>
-      <x:c r="J20" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K20" s="22" t="n">
+      <x:c r="C30" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D30" s="23" t="n">
+        <x:v>7031.2</x:v>
+      </x:c>
+      <x:c r="E30" s="23" t="n">
+        <x:v>6519.6</x:v>
+      </x:c>
+      <x:c r="F30" s="23" t="n">
+        <x:v>6583.6</x:v>
+      </x:c>
+      <x:c r="G30" s="28" t="n">
+        <x:f>ROUND(F30-F29,1)</x:f>
+        <x:v>-432.2</x:v>
+      </x:c>
+      <x:c r="H30" s="24" t="n">
+        <x:f>IFERROR(F30/F29-1,"")</x:f>
+        <x:v>-0.06160380854642378</x:v>
+      </x:c>
+      <x:c r="I30" s="26" t="n">
+        <x:f>ROUND(D30-E30,1)</x:f>
+        <x:v>511.6</x:v>
+      </x:c>
+      <x:c r="J30" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K30" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
+    <x:row r="31">
+      <x:c r="A31" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B31" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="C31" s="23" t="n">
+        <x:v>6577.2</x:v>
+      </x:c>
+      <x:c r="D31" s="23" t="n">
+        <x:v>6680</x:v>
+      </x:c>
+      <x:c r="E31" s="23" t="n">
+        <x:v>6505</x:v>
+      </x:c>
+      <x:c r="F31" s="23" t="n">
+        <x:v>6621.8</x:v>
+      </x:c>
+      <x:c r="G31" s="23" t="n">
+        <x:f>ROUND(F31-F30,1)</x:f>
+        <x:v>38.2</x:v>
+      </x:c>
+      <x:c r="H31" s="24" t="n">
+        <x:f>IFERROR(F31/F30-1,"")</x:f>
+        <x:v>0.005802296615833313</x:v>
+      </x:c>
+      <x:c r="I31" s="23" t="n">
+        <x:f>ROUND(D31-E31,1)</x:f>
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="J31" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K31" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B21" s="30" t="n">
+      <x:c r="B32" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C32" s="30"/>
+      <x:c r="D32" s="30"/>
+      <x:c r="E32" s="30"/>
+      <x:c r="F32" s="30"/>
+      <x:c r="G32" s="30"/>
+      <x:c r="H32" s="30"/>
+      <x:c r="I32" s="32" t="n">
+        <x:f>ROUND(SUM(I29:I31),1)</x:f>
+        <x:v>1119.2</x:v>
+      </x:c>
+      <x:c r="J32" s="30"/>
+      <x:c r="K32" s="30"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B33" s="30"/>
+      <x:c r="C33" s="30"/>
+      <x:c r="D33" s="30"/>
+      <x:c r="E33" s="30"/>
+      <x:c r="F33" s="30"/>
+      <x:c r="G33" s="30"/>
+      <x:c r="H33" s="30"/>
+      <x:c r="I33" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
+        <x:v>373.1</x:v>
+      </x:c>
+      <x:c r="J33" s="30"/>
+      <x:c r="K33" s="30"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B35" s="17"/>
+      <x:c r="C35" s="17"/>
+      <x:c r="D35" s="17"/>
+      <x:c r="E35" s="17"/>
+      <x:c r="F35" s="17"/>
+      <x:c r="G35" s="17"/>
+      <x:c r="H35" s="17"/>
+      <x:c r="I35" s="17"/>
+      <x:c r="J35" s="17"/>
+      <x:c r="K35" s="17"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C36" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D36" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E36" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F36" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G36" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H36" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I36" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J36" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K36" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C37" s="23" t="n">
+        <x:v>7295</x:v>
+      </x:c>
+      <x:c r="D37" s="23" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="E37" s="23" t="n">
+        <x:v>6932</x:v>
+      </x:c>
+      <x:c r="F37" s="23" t="n">
+        <x:v>7111</x:v>
+      </x:c>
+      <x:c r="G37" s="23"/>
+      <x:c r="H37" s="24"/>
+      <x:c r="I37" s="26" t="n">
+        <x:f>ROUND(D37-E37,1)</x:f>
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="J37" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K37" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="32" t="n">
-        <x:f>ROUND(SUM(I19:I20),1)</x:f>
-        <x:v>263.4</x:v>
-      </x:c>
-      <x:c r="J21" s="30"/>
-      <x:c r="K21" s="30"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B38" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C38" s="23" t="n">
+        <x:v>7076.6</x:v>
+      </x:c>
+      <x:c r="D38" s="23" t="n">
+        <x:v>7115.6</x:v>
+      </x:c>
+      <x:c r="E38" s="23" t="n">
+        <x:v>6583.2</x:v>
+      </x:c>
+      <x:c r="F38" s="23" t="n">
+        <x:v>6667.8</x:v>
+      </x:c>
+      <x:c r="G38" s="28" t="n">
+        <x:f>ROUND(F38-F37,1)</x:f>
+        <x:v>-443.2</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="n">
+        <x:f>IFERROR(F38/F37-1,"")</x:f>
+        <x:v>-0.062325973843341265</x:v>
+      </x:c>
+      <x:c r="I38" s="26" t="n">
+        <x:f>ROUND(D38-E38,1)</x:f>
+        <x:v>532.4</x:v>
+      </x:c>
+      <x:c r="J38" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K38" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B39" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C39" s="30"/>
+      <x:c r="D39" s="30"/>
+      <x:c r="E39" s="30"/>
+      <x:c r="F39" s="30"/>
+      <x:c r="G39" s="30"/>
+      <x:c r="H39" s="30"/>
+      <x:c r="I39" s="32" t="n">
+        <x:f>ROUND(SUM(I37:I38),1)</x:f>
+        <x:v>955.4</x:v>
+      </x:c>
+      <x:c r="J39" s="30"/>
+      <x:c r="K39" s="30"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B22" s="30"/>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I19:I20),0),1)</x:f>
-        <x:v>131.7</x:v>
-      </x:c>
-      <x:c r="J22" s="30"/>
-      <x:c r="K22" s="30"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B24" s="17"/>
-      <x:c r="C24" s="17"/>
-      <x:c r="D24" s="17"/>
-      <x:c r="E24" s="17"/>
-      <x:c r="F24" s="17"/>
-      <x:c r="G24" s="17"/>
-      <x:c r="H24" s="17"/>
-      <x:c r="I24" s="17"/>
-      <x:c r="J24" s="17"/>
-      <x:c r="K24" s="17"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="20" t="str">
+      <x:c r="B40" s="30"/>
+      <x:c r="C40" s="30"/>
+      <x:c r="D40" s="30"/>
+      <x:c r="E40" s="30"/>
+      <x:c r="F40" s="30"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I37:I38),0),1)</x:f>
+        <x:v>477.7</x:v>
+      </x:c>
+      <x:c r="J40" s="30"/>
+      <x:c r="K40" s="30"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B42" s="17"/>
+      <x:c r="C42" s="17"/>
+      <x:c r="D42" s="17"/>
+      <x:c r="E42" s="17"/>
+      <x:c r="F42" s="17"/>
+      <x:c r="G42" s="17"/>
+      <x:c r="H42" s="17"/>
+      <x:c r="I42" s="17"/>
+      <x:c r="J42" s="17"/>
+      <x:c r="K42" s="17"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B25" s="20" t="str">
+      <x:c r="B43" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C25" s="20" t="str">
+      <x:c r="C43" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D25" s="20" t="str">
+      <x:c r="D43" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E25" s="20" t="str">
+      <x:c r="E43" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F25" s="20" t="str">
+      <x:c r="F43" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G25" s="20" t="str">
+      <x:c r="G43" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H25" s="20" t="str">
+      <x:c r="H43" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I25" s="20" t="str">
+      <x:c r="I43" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J25" s="20" t="str">
+      <x:c r="J43" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K25" s="20" t="str">
+      <x:c r="K43" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="22" t="n">
+    <x:row r="44">
+      <x:c r="A44" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B26" s="22" t="str">
+      <x:c r="B44" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C26" s="23" t="n">
-        <x:v>7182.8</x:v>
-      </x:c>
-      <x:c r="D26" s="23" t="n">
-        <x:v>7251.8</x:v>
-      </x:c>
-      <x:c r="E26" s="23" t="n">
-        <x:v>6819.2</x:v>
-      </x:c>
-      <x:c r="F26" s="23" t="n">
-        <x:v>7015.8</x:v>
-      </x:c>
-      <x:c r="G26" s="23"/>
-      <x:c r="H26" s="24"/>
-      <x:c r="I26" s="26" t="n">
-        <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>432.6</x:v>
-      </x:c>
-      <x:c r="J26" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K26" s="22" t="n">
+      <x:c r="C44" s="23" t="n">
+        <x:v>4300.8</x:v>
+      </x:c>
+      <x:c r="D44" s="23" t="n">
+        <x:v>4331.6</x:v>
+      </x:c>
+      <x:c r="E44" s="23" t="n">
+        <x:v>4180.4</x:v>
+      </x:c>
+      <x:c r="F44" s="23" t="n">
+        <x:v>4244.8</x:v>
+      </x:c>
+      <x:c r="G44" s="23"/>
+      <x:c r="H44" s="24"/>
+      <x:c r="I44" s="26" t="n">
+        <x:f>ROUND(D44-E44,1)</x:f>
+        <x:v>151.2</x:v>
+      </x:c>
+      <x:c r="J44" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K44" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="22" t="n">
+    <x:row r="45">
+      <x:c r="A45" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B27" s="22" t="str">
+      <x:c r="B45" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C27" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D27" s="23" t="n">
-        <x:v>7031.2</x:v>
-      </x:c>
-      <x:c r="E27" s="23" t="n">
-        <x:v>6519.6</x:v>
-      </x:c>
-      <x:c r="F27" s="23" t="n">
-        <x:v>6583.6</x:v>
-      </x:c>
-      <x:c r="G27" s="28" t="n">
-        <x:f>ROUND(F27-F26,1)</x:f>
-        <x:v>-432.2</x:v>
-      </x:c>
-      <x:c r="H27" s="24" t="n">
-        <x:f>IFERROR(F27/F26-1,"")</x:f>
-        <x:v>-0.06160380854642378</x:v>
-      </x:c>
-      <x:c r="I27" s="26" t="n">
-        <x:f>ROUND(D27-E27,1)</x:f>
-        <x:v>511.6</x:v>
-      </x:c>
-      <x:c r="J27" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K27" s="22" t="n">
+      <x:c r="C45" s="23" t="n">
+        <x:v>4240.4</x:v>
+      </x:c>
+      <x:c r="D45" s="23" t="n">
+        <x:v>4273.6</x:v>
+      </x:c>
+      <x:c r="E45" s="23" t="n">
+        <x:v>4045.2</x:v>
+      </x:c>
+      <x:c r="F45" s="23" t="n">
+        <x:v>4088.8</x:v>
+      </x:c>
+      <x:c r="G45" s="28" t="n">
+        <x:f>ROUND(F45-F44,1)</x:f>
+        <x:v>-156</x:v>
+      </x:c>
+      <x:c r="H45" s="24" t="n">
+        <x:f>IFERROR(F45/F44-1,"")</x:f>
+        <x:v>-0.03675084809649454</x:v>
+      </x:c>
+      <x:c r="I45" s="26" t="n">
+        <x:f>ROUND(D45-E45,1)</x:f>
+        <x:v>228.4</x:v>
+      </x:c>
+      <x:c r="J45" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K45" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="31" t="str">
+    <x:row r="46">
+      <x:c r="A46" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B28" s="30" t="n">
+      <x:c r="B46" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C28" s="30"/>
-      <x:c r="D28" s="30"/>
-      <x:c r="E28" s="30"/>
-      <x:c r="F28" s="30"/>
-      <x:c r="G28" s="30"/>
-      <x:c r="H28" s="30"/>
-      <x:c r="I28" s="32" t="n">
-        <x:f>ROUND(SUM(I26:I27),1)</x:f>
-        <x:v>944.2</x:v>
-      </x:c>
-      <x:c r="J28" s="30"/>
-      <x:c r="K28" s="30"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="31" t="str">
+      <x:c r="C46" s="30"/>
+      <x:c r="D46" s="30"/>
+      <x:c r="E46" s="30"/>
+      <x:c r="F46" s="30"/>
+      <x:c r="G46" s="30"/>
+      <x:c r="H46" s="30"/>
+      <x:c r="I46" s="32" t="n">
+        <x:f>ROUND(SUM(I44:I45),1)</x:f>
+        <x:v>379.6</x:v>
+      </x:c>
+      <x:c r="J46" s="30"/>
+      <x:c r="K46" s="30"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B29" s="30"/>
-      <x:c r="C29" s="30"/>
-      <x:c r="D29" s="30"/>
-      <x:c r="E29" s="30"/>
-      <x:c r="F29" s="30"/>
-      <x:c r="G29" s="30"/>
-      <x:c r="H29" s="30"/>
-      <x:c r="I29" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I26:I27),0),1)</x:f>
-        <x:v>472.1</x:v>
-      </x:c>
-      <x:c r="J29" s="30"/>
-      <x:c r="K29" s="30"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B31" s="17"/>
-      <x:c r="C31" s="17"/>
-      <x:c r="D31" s="17"/>
-      <x:c r="E31" s="17"/>
-      <x:c r="F31" s="17"/>
-      <x:c r="G31" s="17"/>
-      <x:c r="H31" s="17"/>
-      <x:c r="I31" s="17"/>
-      <x:c r="J31" s="17"/>
-      <x:c r="K31" s="17"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="20" t="str">
+      <x:c r="B47" s="30"/>
+      <x:c r="C47" s="30"/>
+      <x:c r="D47" s="30"/>
+      <x:c r="E47" s="30"/>
+      <x:c r="F47" s="30"/>
+      <x:c r="G47" s="30"/>
+      <x:c r="H47" s="30"/>
+      <x:c r="I47" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I44:I45),0),1)</x:f>
+        <x:v>189.8</x:v>
+      </x:c>
+      <x:c r="J47" s="30"/>
+      <x:c r="K47" s="30"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B49" s="17"/>
+      <x:c r="C49" s="17"/>
+      <x:c r="D49" s="17"/>
+      <x:c r="E49" s="17"/>
+      <x:c r="F49" s="17"/>
+      <x:c r="G49" s="17"/>
+      <x:c r="H49" s="17"/>
+      <x:c r="I49" s="17"/>
+      <x:c r="J49" s="17"/>
+      <x:c r="K49" s="17"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B32" s="20" t="str">
+      <x:c r="B50" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C32" s="20" t="str">
+      <x:c r="C50" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D32" s="20" t="str">
+      <x:c r="D50" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E32" s="20" t="str">
+      <x:c r="E50" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
+      <x:c r="F50" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G32" s="20" t="str">
+      <x:c r="G50" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="str">
+      <x:c r="H50" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I32" s="20" t="str">
+      <x:c r="I50" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J32" s="20" t="str">
+      <x:c r="J50" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K32" s="20" t="str">
+      <x:c r="K50" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="22" t="n">
+    <x:row r="51">
+      <x:c r="A51" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B33" s="22" t="str">
+      <x:c r="B51" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C33" s="23" t="n">
-        <x:v>7295</x:v>
-      </x:c>
-      <x:c r="D33" s="23" t="n">
-        <x:v>7355</x:v>
-      </x:c>
-      <x:c r="E33" s="23" t="n">
-        <x:v>6932</x:v>
-      </x:c>
-      <x:c r="F33" s="23" t="n">
-        <x:v>7111</x:v>
-      </x:c>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="24"/>
-      <x:c r="I33" s="26" t="n">
-        <x:f>ROUND(D33-E33,1)</x:f>
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="J33" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K33" s="22" t="n">
+      <x:c r="C51" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="n">
+        <x:v>2798.4</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="n">
+        <x:v>2735</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="G51" s="23"/>
+      <x:c r="H51" s="24"/>
+      <x:c r="I51" s="26" t="n">
+        <x:f>ROUND(D51-E51,1)</x:f>
+        <x:v>63.4</x:v>
+      </x:c>
+      <x:c r="J51" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K51" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="22" t="n">
+    <x:row r="52">
+      <x:c r="A52" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B34" s="22" t="str">
+      <x:c r="B52" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C34" s="23" t="n">
-        <x:v>7076.6</x:v>
-      </x:c>
-      <x:c r="D34" s="23" t="n">
-        <x:v>7115.6</x:v>
-      </x:c>
-      <x:c r="E34" s="23" t="n">
-        <x:v>6583.2</x:v>
-      </x:c>
-      <x:c r="F34" s="23" t="n">
-        <x:v>6667.8</x:v>
-      </x:c>
-      <x:c r="G34" s="28" t="n">
-        <x:f>ROUND(F34-F33,1)</x:f>
-        <x:v>-443.2</x:v>
-      </x:c>
-      <x:c r="H34" s="24" t="n">
-        <x:f>IFERROR(F34/F33-1,"")</x:f>
-        <x:v>-0.062325973843341265</x:v>
-      </x:c>
-      <x:c r="I34" s="26" t="n">
-        <x:f>ROUND(D34-E34,1)</x:f>
-        <x:v>532.4</x:v>
-      </x:c>
-      <x:c r="J34" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K34" s="22" t="n">
+      <x:c r="C52" s="23" t="n">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="D52" s="23" t="n">
+        <x:v>2794</x:v>
+      </x:c>
+      <x:c r="E52" s="23" t="n">
+        <x:v>2677.6</x:v>
+      </x:c>
+      <x:c r="F52" s="23" t="n">
+        <x:v>2704.6</x:v>
+      </x:c>
+      <x:c r="G52" s="23" t="n">
+        <x:f>ROUND(F52-F51,1)</x:f>
+        <x:v>-59.4</x:v>
+      </x:c>
+      <x:c r="H52" s="24" t="n">
+        <x:f>IFERROR(F52/F51-1,"")</x:f>
+        <x:v>-0.0214905933429812</x:v>
+      </x:c>
+      <x:c r="I52" s="26" t="n">
+        <x:f>ROUND(D52-E52,1)</x:f>
+        <x:v>116.4</x:v>
+      </x:c>
+      <x:c r="J52" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K52" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="31" t="str">
+    <x:row r="53">
+      <x:c r="A53" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B35" s="30" t="n">
+      <x:c r="B53" s="30" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C35" s="30"/>
-      <x:c r="D35" s="30"/>
-      <x:c r="E35" s="30"/>
-      <x:c r="F35" s="30"/>
-      <x:c r="G35" s="30"/>
-      <x:c r="H35" s="30"/>
-      <x:c r="I35" s="32" t="n">
-        <x:f>ROUND(SUM(I33:I34),1)</x:f>
-        <x:v>955.4</x:v>
-      </x:c>
-      <x:c r="J35" s="30"/>
-      <x:c r="K35" s="30"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="31" t="str">
+      <x:c r="C53" s="30"/>
+      <x:c r="D53" s="30"/>
+      <x:c r="E53" s="30"/>
+      <x:c r="F53" s="30"/>
+      <x:c r="G53" s="30"/>
+      <x:c r="H53" s="30"/>
+      <x:c r="I53" s="32" t="n">
+        <x:f>ROUND(SUM(I51:I52),1)</x:f>
+        <x:v>179.8</x:v>
+      </x:c>
+      <x:c r="J53" s="30"/>
+      <x:c r="K53" s="30"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B36" s="30"/>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="30"/>
-      <x:c r="E36" s="30"/>
-      <x:c r="F36" s="30"/>
-      <x:c r="G36" s="30"/>
-      <x:c r="H36" s="30"/>
-      <x:c r="I36" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I33:I34),0),1)</x:f>
-        <x:v>477.7</x:v>
-      </x:c>
-      <x:c r="J36" s="30"/>
-      <x:c r="K36" s="30"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B38" s="17"/>
-      <x:c r="C38" s="17"/>
-      <x:c r="D38" s="17"/>
-      <x:c r="E38" s="17"/>
-      <x:c r="F38" s="17"/>
-      <x:c r="G38" s="17"/>
-      <x:c r="H38" s="17"/>
-      <x:c r="I38" s="17"/>
-      <x:c r="J38" s="17"/>
-      <x:c r="K38" s="17"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="20" t="str">
+      <x:c r="B54" s="30"/>
+      <x:c r="C54" s="30"/>
+      <x:c r="D54" s="30"/>
+      <x:c r="E54" s="30"/>
+      <x:c r="F54" s="30"/>
+      <x:c r="G54" s="30"/>
+      <x:c r="H54" s="30"/>
+      <x:c r="I54" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I51:I52),0),1)</x:f>
+        <x:v>89.9</x:v>
+      </x:c>
+      <x:c r="J54" s="30"/>
+      <x:c r="K54" s="30"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="17" t="str">
+        <x:v>碳酸锂2610</x:v>
+      </x:c>
+      <x:c r="B56" s="17"/>
+      <x:c r="C56" s="17"/>
+      <x:c r="D56" s="17"/>
+      <x:c r="E56" s="17"/>
+      <x:c r="F56" s="17"/>
+      <x:c r="G56" s="17"/>
+      <x:c r="H56" s="17"/>
+      <x:c r="I56" s="17"/>
+      <x:c r="J56" s="17"/>
+      <x:c r="K56" s="17"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B39" s="20" t="str">
+      <x:c r="B57" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C39" s="20" t="str">
+      <x:c r="C57" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D39" s="20" t="str">
+      <x:c r="D57" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E39" s="20" t="str">
+      <x:c r="E57" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F39" s="20" t="str">
+      <x:c r="F57" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G39" s="20" t="str">
+      <x:c r="G57" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H39" s="20" t="str">
+      <x:c r="H57" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I39" s="20" t="str">
+      <x:c r="I57" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J39" s="20" t="str">
+      <x:c r="J57" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K39" s="20" t="str">
+      <x:c r="K57" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="22" t="n">
+    <x:row r="58">
+      <x:c r="A58" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B40" s="22" t="str">
+      <x:c r="B58" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C40" s="23" t="n">
-        <x:v>4300.8</x:v>
-      </x:c>
-      <x:c r="D40" s="23" t="n">
-        <x:v>4331.6</x:v>
-      </x:c>
-      <x:c r="E40" s="23" t="n">
-        <x:v>4180.4</x:v>
-      </x:c>
-      <x:c r="F40" s="23" t="n">
-        <x:v>4244.8</x:v>
-      </x:c>
-      <x:c r="G40" s="23"/>
-      <x:c r="H40" s="24"/>
-      <x:c r="I40" s="26" t="n">
-        <x:f>ROUND(D40-E40,1)</x:f>
-        <x:v>151.2</x:v>
-      </x:c>
-      <x:c r="J40" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K40" s="22" t="n">
+      <x:c r="C58" s="23" t="n">
+        <x:v>120020</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="n">
+        <x:v>126800</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="n">
+        <x:v>119000</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="n">
+        <x:v>121000</x:v>
+      </x:c>
+      <x:c r="G58" s="23"/>
+      <x:c r="H58" s="24"/>
+      <x:c r="I58" s="26" t="n">
+        <x:f>ROUND(D58-E58,1)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K58" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="22" t="n">
+    <x:row r="59">
+      <x:c r="A59" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B41" s="22" t="str">
+      <x:c r="B59" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C41" s="23" t="n">
-        <x:v>4240.4</x:v>
-      </x:c>
-      <x:c r="D41" s="23" t="n">
-        <x:v>4273.6</x:v>
-      </x:c>
-      <x:c r="E41" s="23" t="n">
-        <x:v>4045.2</x:v>
-      </x:c>
-      <x:c r="F41" s="23" t="n">
-        <x:v>4088.8</x:v>
-      </x:c>
-      <x:c r="G41" s="28" t="n">
-        <x:f>ROUND(F41-F40,1)</x:f>
-        <x:v>-156</x:v>
-      </x:c>
-      <x:c r="H41" s="24" t="n">
-        <x:f>IFERROR(F41/F40-1,"")</x:f>
-        <x:v>-0.03675084809649454</x:v>
-      </x:c>
-      <x:c r="I41" s="26" t="n">
-        <x:f>ROUND(D41-E41,1)</x:f>
-        <x:v>228.4</x:v>
-      </x:c>
-      <x:c r="J41" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K41" s="22" t="n">
+      <x:c r="C59" s="23" t="n">
+        <x:v>125960</x:v>
+      </x:c>
+      <x:c r="D59" s="23" t="n">
+        <x:v>125960</x:v>
+      </x:c>
+      <x:c r="E59" s="23" t="n">
+        <x:v>99500</x:v>
+      </x:c>
+      <x:c r="F59" s="23" t="n">
+        <x:v>99500</x:v>
+      </x:c>
+      <x:c r="G59" s="28" t="n">
+        <x:f>ROUND(F59-F58,1)</x:f>
+        <x:v>-21500</x:v>
+      </x:c>
+      <x:c r="H59" s="24" t="n">
+        <x:f>IFERROR(F59/F58-1,"")</x:f>
+        <x:v>-0.1776859504132231</x:v>
+      </x:c>
+      <x:c r="I59" s="26" t="n">
+        <x:f>ROUND(D59-E59,1)</x:f>
+        <x:v>26460</x:v>
+      </x:c>
+      <x:c r="J59" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K59" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="31" t="str">
+    <x:row r="60">
+      <x:c r="A60" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B60" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="C60" s="23" t="n">
+        <x:v>99600</x:v>
+      </x:c>
+      <x:c r="D60" s="23" t="n">
+        <x:v>103280</x:v>
+      </x:c>
+      <x:c r="E60" s="23" t="n">
+        <x:v>99600</x:v>
+      </x:c>
+      <x:c r="F60" s="23" t="n">
+        <x:v>103180</x:v>
+      </x:c>
+      <x:c r="G60" s="28" t="n">
+        <x:f>ROUND(F60-F59,1)</x:f>
+        <x:v>3680</x:v>
+      </x:c>
+      <x:c r="H60" s="24" t="n">
+        <x:f>IFERROR(F60/F59-1,"")</x:f>
+        <x:v>0.036984924623115534</x:v>
+      </x:c>
+      <x:c r="I60" s="23" t="n">
+        <x:f>ROUND(D60-E60,1)</x:f>
+        <x:v>3680</x:v>
+      </x:c>
+      <x:c r="J60" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K60" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B42" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C42" s="30"/>
-      <x:c r="D42" s="30"/>
-      <x:c r="E42" s="30"/>
-      <x:c r="F42" s="30"/>
-      <x:c r="G42" s="30"/>
-      <x:c r="H42" s="30"/>
-      <x:c r="I42" s="32" t="n">
-        <x:f>ROUND(SUM(I40:I41),1)</x:f>
-        <x:v>379.6</x:v>
-      </x:c>
-      <x:c r="J42" s="30"/>
-      <x:c r="K42" s="30"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="31" t="str">
+      <x:c r="B61" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C61" s="30"/>
+      <x:c r="D61" s="30"/>
+      <x:c r="E61" s="30"/>
+      <x:c r="F61" s="30"/>
+      <x:c r="G61" s="30"/>
+      <x:c r="H61" s="30"/>
+      <x:c r="I61" s="32" t="n">
+        <x:f>ROUND(SUM(I58:I60),1)</x:f>
+        <x:v>37940</x:v>
+      </x:c>
+      <x:c r="J61" s="30"/>
+      <x:c r="K61" s="30"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B43" s="30"/>
-      <x:c r="C43" s="30"/>
-      <x:c r="D43" s="30"/>
-      <x:c r="E43" s="30"/>
-      <x:c r="F43" s="30"/>
-      <x:c r="G43" s="30"/>
-      <x:c r="H43" s="30"/>
-      <x:c r="I43" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I40:I41),0),1)</x:f>
-        <x:v>189.8</x:v>
-      </x:c>
-      <x:c r="J43" s="30"/>
-      <x:c r="K43" s="30"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
-      <x:c r="F45" s="17"/>
-      <x:c r="G45" s="17"/>
-      <x:c r="H45" s="17"/>
-      <x:c r="I45" s="17"/>
-      <x:c r="J45" s="17"/>
-      <x:c r="K45" s="17"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B46" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C46" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E46" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F46" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G46" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H46" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I46" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J46" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>2798.4</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>2735</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>63.4</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B48" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
-      </x:c>
-      <x:c r="C48" s="23" t="n">
-        <x:v>2762</x:v>
-      </x:c>
-      <x:c r="D48" s="23" t="n">
-        <x:v>2794</x:v>
-      </x:c>
-      <x:c r="E48" s="23" t="n">
-        <x:v>2677.6</x:v>
-      </x:c>
-      <x:c r="F48" s="23" t="n">
-        <x:v>2704.6</x:v>
-      </x:c>
-      <x:c r="G48" s="23" t="n">
-        <x:f>ROUND(F48-F47,1)</x:f>
-        <x:v>-59.4</x:v>
-      </x:c>
-      <x:c r="H48" s="24" t="n">
-        <x:f>IFERROR(F48/F47-1,"")</x:f>
-        <x:v>-0.0214905933429812</x:v>
-      </x:c>
-      <x:c r="I48" s="26" t="n">
-        <x:f>ROUND(D48-E48,1)</x:f>
-        <x:v>116.4</x:v>
-      </x:c>
-      <x:c r="J48" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K48" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B49" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="32" t="n">
-        <x:f>ROUND(SUM(I47:I48),1)</x:f>
-        <x:v>179.8</x:v>
-      </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B50" s="30"/>
-      <x:c r="C50" s="30"/>
-      <x:c r="D50" s="30"/>
-      <x:c r="E50" s="30"/>
-      <x:c r="F50" s="30"/>
-      <x:c r="G50" s="30"/>
-      <x:c r="H50" s="30"/>
-      <x:c r="I50" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I47:I48),0),1)</x:f>
-        <x:v>89.9</x:v>
-      </x:c>
-      <x:c r="J50" s="30"/>
-      <x:c r="K50" s="30"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="17" t="str">
-        <x:v>碳酸锂2610</x:v>
-      </x:c>
-      <x:c r="B52" s="17"/>
-      <x:c r="C52" s="17"/>
-      <x:c r="D52" s="17"/>
-      <x:c r="E52" s="17"/>
-      <x:c r="F52" s="17"/>
-      <x:c r="G52" s="17"/>
-      <x:c r="H52" s="17"/>
-      <x:c r="I52" s="17"/>
-      <x:c r="J52" s="17"/>
-      <x:c r="K52" s="17"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B53" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C53" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D53" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E53" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F53" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G53" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H53" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I53" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J53" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K53" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>120020</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>126800</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>119000</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>121000</x:v>
-      </x:c>
-      <x:c r="G54" s="23"/>
-      <x:c r="H54" s="24"/>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>7800</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>125960</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>125960</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>99500</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>99500</x:v>
-      </x:c>
-      <x:c r="G55" s="28" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-21500</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.1776859504132231</x:v>
-      </x:c>
-      <x:c r="I55" s="26" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>26460</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="30" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
-        <x:f>ROUND(SUM(I54:I55),1)</x:f>
-        <x:v>34260</x:v>
-      </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I54:I55),0),1)</x:f>
-        <x:v>17130</x:v>
-      </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
+      <x:c r="B62" s="30"/>
+      <x:c r="C62" s="30"/>
+      <x:c r="D62" s="30"/>
+      <x:c r="E62" s="30"/>
+      <x:c r="F62" s="30"/>
+      <x:c r="G62" s="30"/>
+      <x:c r="H62" s="30"/>
+      <x:c r="I62" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I58:I60),0),1)</x:f>
+        <x:v>12646.7</x:v>
+      </x:c>
+      <x:c r="J62" s="30"/>
+      <x:c r="K62" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A10:K10"/>
-    <x:mergeCell ref="A17:K17"/>
-    <x:mergeCell ref="A24:K24"/>
-    <x:mergeCell ref="A31:K31"/>
-    <x:mergeCell ref="A38:K38"/>
-    <x:mergeCell ref="A45:K45"/>
-    <x:mergeCell ref="A52:K52"/>
+    <x:mergeCell ref="A11:K11"/>
+    <x:mergeCell ref="A19:K19"/>
+    <x:mergeCell ref="A27:K27"/>
+    <x:mergeCell ref="A35:K35"/>
+    <x:mergeCell ref="A42:K42"/>
+    <x:mergeCell ref="A49:K49"/>
+    <x:mergeCell ref="A56:K56"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2847,31 +3073,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="30" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1455.1</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>6639.94</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>6746.32</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>6578.94</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>6698.3</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>16.4</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.002448390736822015</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>167.4</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="30"/>
       <x:c r="D14" s="30"/>
       <x:c r="E14" s="30"/>
@@ -2879,11 +3123,29 @@
       <x:c r="G14" s="30"/>
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="30"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>207.9</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1622.5</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="30"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>202.8</x:v>
+      </x:c>
+      <x:c r="K15" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3202,31 +3464,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="30" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1367.1999999999998</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>6735.53</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>6848</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>6692.83</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>6800.66</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>27.9</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.004120925768705375</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>155.2</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="30"/>
       <x:c r="D14" s="30"/>
       <x:c r="E14" s="30"/>
@@ -3234,11 +3514,29 @@
       <x:c r="G14" s="30"/>
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="30"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>195.3</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1522.3999999999999</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="30"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>190.3</x:v>
+      </x:c>
+      <x:c r="K15" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3557,31 +3855,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="30" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>426.19999999999993</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>3694.12</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>3743.8</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>3692.29</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>3730.92</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>14.6</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.003939423294262001</x:v>
+      </x:c>
+      <x:c r="J11" s="26" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>51.5</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="30"/>
       <x:c r="D14" s="30"/>
       <x:c r="E14" s="30"/>
@@ -3589,11 +3905,29 @@
       <x:c r="G14" s="30"/>
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="30"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>60.9</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>477.69999999999993</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="30"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>59.7</x:v>
+      </x:c>
+      <x:c r="K15" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3912,31 +4246,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B13" s="30" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C13" s="30"/>
-      <x:c r="D13" s="30"/>
-      <x:c r="E13" s="30"/>
-      <x:c r="F13" s="30"/>
-      <x:c r="G13" s="30"/>
-      <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
-      <x:c r="J13" s="32" t="n">
-        <x:f>SUM(J4:J10)</x:f>
-        <x:v>1536.4000000000003</x:v>
-      </x:c>
-      <x:c r="K13" s="30"/>
+    <x:row r="11">
+      <x:c r="A11" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>10月19日</x:v>
+      </x:c>
+      <x:c r="D11" s="23" t="n">
+        <x:v>6577.2</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="n">
+        <x:v>6680</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="n">
+        <x:v>6505</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="n">
+        <x:v>6621.8</x:v>
+      </x:c>
+      <x:c r="H11" s="23" t="n">
+        <x:v>38.2</x:v>
+      </x:c>
+      <x:c r="I11" s="24" t="n">
+        <x:v>0.005802296615833313</x:v>
+      </x:c>
+      <x:c r="J11" s="23" t="n">
+        <x:f>ROUND(E11-F11,1)</x:f>
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B14" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C14" s="30"/>
       <x:c r="D14" s="30"/>
       <x:c r="E14" s="30"/>
@@ -3944,11 +4296,29 @@
       <x:c r="G14" s="30"/>
       <x:c r="H14" s="30"/>
       <x:c r="I14" s="30"/>
-      <x:c r="J14" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J10),0),1)</x:f>
-        <x:v>219.5</x:v>
+      <x:c r="J14" s="32" t="n">
+        <x:f>SUM(J4:J11)</x:f>
+        <x:v>1711.4000000000003</x:v>
       </x:c>
       <x:c r="K14" s="30"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="30"/>
+      <x:c r="E15" s="30"/>
+      <x:c r="F15" s="30"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="30"/>
+      <x:c r="J15" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
+        <x:v>213.9</x:v>
+      </x:c>
+      <x:c r="K15" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-20
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R68f9fba8c3bf468f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R011e076b2fdf42ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rd8db927f29b942c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R44f25684fc8b4073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Re4f98c5183f74387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rbb6df191ad744946"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rbd3abe2343ff429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rbefbf2a21ad7467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf3078214d0514d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R9f04f3a02bc14384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rd4e98b29199f4d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R032375a4523b4336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R93cfd427ce394e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rfdcfbc1b899347b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R5f2c426d4435480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R826753a346614fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Re2b9ecb01af64422"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R40028f112a9c456c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R3bac7d40204b4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R3b4ba42b5a684730"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6746.32</x:v>
+        <x:v>6817.38</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6578.94</x:v>
+        <x:v>6642.3</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>167.4</x:v>
+        <x:v>175.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1622.5</x:v>
+        <x:v>1797.6</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>202.8</x:v>
+        <x:v>199.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6848</x:v>
+        <x:v>6902.09</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6692.83</x:v>
+        <x:v>6745.14</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>155.2</x:v>
+        <x:v>156.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1522.4</x:v>
+        <x:v>1679.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>190.3</x:v>
+        <x:v>186.6</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3743.8</x:v>
+        <x:v>3740.07</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3692.29</x:v>
+        <x:v>3702.44</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>51.5</x:v>
+        <x:v>37.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>477.7</x:v>
+        <x:v>515.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>59.7</x:v>
+        <x:v>57.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6779.4</x:v>
+        <x:v>6828</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6608.2</x:v>
+        <x:v>6645</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>171.2</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1672.4</x:v>
+        <x:v>1855.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>209.1</x:v>
+        <x:v>206.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4140.2</x:v>
+        <x:v>4123.2</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>4082</x:v>
+        <x:v>4049</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>58.2</x:v>
+        <x:v>74.2</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>661</x:v>
+        <x:v>735.2</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>82.6</x:v>
+        <x:v>81.7</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -723,25 +723,25 @@
         <x:v>碳酸锂2610</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:v>103280</x:v>
+        <x:v>103420</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
-        <x:v>99600</x:v>
+        <x:v>101520</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
-        <x:v>3680</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" s="10" t="n">
-        <x:v>53420</x:v>
+        <x:v>55320</x:v>
       </x:c>
       <x:c r="H11" s="10" t="n">
-        <x:v>6677.5</x:v>
+        <x:v>6146.7</x:v>
       </x:c>
       <x:c r="I11" s="10" t="n">
         <x:v>6000</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>2026-10-20</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1226,31 +1226,49 @@
         <x:v>LC2610</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>53420</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>101540</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>103420</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>101520</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>103400</x:v>
+      </x:c>
+      <x:c r="H12" s="28" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.002132196162046851</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>1900</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -1258,11 +1276,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>6677.5</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>55320</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>6146.7</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1419,37 +1455,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>6639.94</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>6746.32</x:v>
+        <x:v>6817.38</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>6578.94</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>6698.3</x:v>
+        <x:v>6766.9</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>16.4</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.002448390736822015</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="n">
+        <x:v>0.012714870232297892</x:v>
+      </x:c>
+      <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>167.4</x:v>
+        <x:v>238.4</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1467,7 +1503,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1127.3</x:v>
+        <x:v>1198.3</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1485,7 +1521,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>375.8</x:v>
+        <x:v>399.4</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1615,37 +1651,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>6735.53</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>6848</x:v>
+        <x:v>6902.09</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>6692.83</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>6800.66</x:v>
+        <x:v>6841.44</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>27.9</x:v>
+        <x:v>68.7</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.004120925768705375</x:v>
-      </x:c>
-      <x:c r="I15" s="23" t="n">
+        <x:v>0.010142113617068294</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>155.2</x:v>
+        <x:v>209.3</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1663,7 +1699,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1085</x:v>
+        <x:v>1139.1</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1681,7 +1717,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>361.7</x:v>
+        <x:v>379.7</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1811,7 +1847,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3694.12</x:v>
@@ -1823,15 +1859,15 @@
         <x:v>3692.29</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3730.92</x:v>
+        <x:v>3735.37</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>14.6</x:v>
+        <x:v>19.1</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.003939423294262001</x:v>
+        <x:v>0.00513685728739488</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
@@ -1841,7 +1877,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2203,37 +2239,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>6670.2</x:v>
       </x:c>
       <x:c r="D39" s="23" t="n">
-        <x:v>6779.4</x:v>
+        <x:v>6828</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
         <x:v>6608.2</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>6719.8</x:v>
+        <x:v>6737.8</x:v>
       </x:c>
       <x:c r="G39" s="23" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>52</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.007798674225381719</x:v>
+        <x:v>0.01049821530339834</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>171.2</x:v>
+        <x:v>219.8</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2251,7 +2287,7 @@
       <x:c r="H40" s="30"/>
       <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1126.6</x:v>
+        <x:v>1175.2</x:v>
       </x:c>
       <x:c r="J40" s="30"/>
       <x:c r="K40" s="30"/>
@@ -2269,7 +2305,7 @@
       <x:c r="H41" s="30"/>
       <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>375.5</x:v>
+        <x:v>391.7</x:v>
       </x:c>
       <x:c r="J41" s="30"/>
       <x:c r="K41" s="30"/>
@@ -2399,7 +2435,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C47" s="23" t="n">
         <x:v>4086.4</x:v>
@@ -2408,28 +2444,28 @@
         <x:v>4140.2</x:v>
       </x:c>
       <x:c r="E47" s="23" t="n">
-        <x:v>4082</x:v>
+        <x:v>4049</x:v>
       </x:c>
       <x:c r="F47" s="23" t="n">
-        <x:v>4110.4</x:v>
+        <x:v>4082.8</x:v>
       </x:c>
       <x:c r="G47" s="23" t="n">
         <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>21.6</x:v>
+        <x:v>-6</x:v>
       </x:c>
       <x:c r="H47" s="24" t="n">
         <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>0.00528272353746817</x:v>
-      </x:c>
-      <x:c r="I47" s="23" t="n">
+        <x:v>-0.0014674232048522695</x:v>
+      </x:c>
+      <x:c r="I47" s="26" t="n">
         <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>58.2</x:v>
+        <x:v>91.2</x:v>
       </x:c>
       <x:c r="J47" s="22" t="str">
         <x:v>IF2612</x:v>
       </x:c>
       <x:c r="K47" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2447,7 +2483,7 @@
       <x:c r="H48" s="30"/>
       <x:c r="I48" s="32" t="n">
         <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>437.8</x:v>
+        <x:v>470.8</x:v>
       </x:c>
       <x:c r="J48" s="30"/>
       <x:c r="K48" s="30"/>
@@ -2465,7 +2501,7 @@
       <x:c r="H49" s="30"/>
       <x:c r="I49" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>145.9</x:v>
+        <x:v>156.9</x:v>
       </x:c>
       <x:c r="J49" s="30"/>
       <x:c r="K49" s="30"/>
@@ -2791,37 +2827,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>10月19日</x:v>
+        <x:v>10月19日-10月20日</x:v>
       </x:c>
       <x:c r="C63" s="23" t="n">
         <x:v>99600</x:v>
       </x:c>
       <x:c r="D63" s="23" t="n">
-        <x:v>103280</x:v>
+        <x:v>103420</x:v>
       </x:c>
       <x:c r="E63" s="23" t="n">
         <x:v>99600</x:v>
       </x:c>
       <x:c r="F63" s="23" t="n">
-        <x:v>103180</x:v>
+        <x:v>103400</x:v>
       </x:c>
       <x:c r="G63" s="28" t="n">
         <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>3680</x:v>
+        <x:v>3900</x:v>
       </x:c>
       <x:c r="H63" s="24" t="n">
         <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>0.036984924623115534</x:v>
+        <x:v>0.03919597989949741</x:v>
       </x:c>
       <x:c r="I63" s="23" t="n">
         <x:f>ROUND(D63-E63,1)</x:f>
-        <x:v>3680</x:v>
+        <x:v>3820</x:v>
       </x:c>
       <x:c r="J63" s="22" t="str">
         <x:v>LC2610</x:v>
       </x:c>
       <x:c r="K63" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -2839,7 +2875,7 @@
       <x:c r="H64" s="30"/>
       <x:c r="I64" s="32" t="n">
         <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>37940</x:v>
+        <x:v>38080</x:v>
       </x:c>
       <x:c r="J64" s="30"/>
       <x:c r="K64" s="30"/>
@@ -2857,7 +2893,7 @@
       <x:c r="H65" s="30"/>
       <x:c r="I65" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
-        <x:v>12646.7</x:v>
+        <x:v>12693.3</x:v>
       </x:c>
       <x:c r="J65" s="30"/>
       <x:c r="K65" s="30"/>
@@ -3223,31 +3259,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1622.5</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>6678.64</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>6817.38</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>6642.3</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>6766.9</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>68.6</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.01024140453547906</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>175.1</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -3255,11 +3309,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>202.8</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1797.6</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>199.7</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3614,31 +3686,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1522.3999999999999</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>6773.45</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>6902.09</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>6745.14</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>6841.44</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>40.8</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.005996476812544671</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>156.9</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -3646,11 +3736,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>190.3</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1679.3</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>186.6</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4005,31 +4113,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>477.69999999999993</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>3718.44</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>3740.07</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>3702.44</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>3735.37</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>4.4</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.0011927353038927446</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>37.6</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -4037,11 +4163,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>59.7</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>515.3</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>57.3</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4787,31 +4931,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>1672.4</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>6666</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>6828</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>6645</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>6737.8</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>0.0026786511503318344</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -4819,11 +4981,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>209.1</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>1855.4</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>206.2</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5178,31 +5358,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B14" s="30" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C14" s="30"/>
-      <x:c r="D14" s="30"/>
-      <x:c r="E14" s="30"/>
-      <x:c r="F14" s="30"/>
-      <x:c r="G14" s="30"/>
-      <x:c r="H14" s="30"/>
-      <x:c r="I14" s="30"/>
-      <x:c r="J14" s="32" t="n">
-        <x:f>SUM(J4:J11)</x:f>
-        <x:v>661</x:v>
-      </x:c>
-      <x:c r="K14" s="30"/>
+    <x:row r="12">
+      <x:c r="A12" s="22" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>10月20日</x:v>
+      </x:c>
+      <x:c r="D12" s="23" t="n">
+        <x:v>4104</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="n">
+        <x:v>4123.2</x:v>
+      </x:c>
+      <x:c r="F12" s="23" t="n">
+        <x:v>4049</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="n">
+        <x:v>4082.8</x:v>
+      </x:c>
+      <x:c r="H12" s="23" t="n">
+        <x:v>-27.6</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="n">
+        <x:v>-0.006714674970805579</x:v>
+      </x:c>
+      <x:c r="J12" s="23" t="n">
+        <x:f>ROUND(E12-F12,1)</x:f>
+        <x:v>74.2</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="C15" s="30"/>
       <x:c r="D15" s="30"/>
       <x:c r="E15" s="30"/>
@@ -5210,11 +5408,29 @@
       <x:c r="G15" s="30"/>
       <x:c r="H15" s="30"/>
       <x:c r="I15" s="30"/>
-      <x:c r="J15" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J11),0),1)</x:f>
-        <x:v>82.6</x:v>
+      <x:c r="J15" s="32" t="n">
+        <x:f>SUM(J4:J12)</x:f>
+        <x:v>735.2</x:v>
       </x:c>
       <x:c r="K15" s="30"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="30"/>
+      <x:c r="E16" s="30"/>
+      <x:c r="F16" s="30"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="30"/>
+      <x:c r="J16" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
+        <x:v>81.7</x:v>
+      </x:c>
+      <x:c r="K16" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-21
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R498b1168de32409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R64a928ad33a84808"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R0944b78d8a954a24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Ra51972fab0b347f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R050b70f25b074a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2f97fd67f4f14486"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R678aba9b2c1e4090"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R7d86a1657d82460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf9772fcbe5964160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rd6f28d6fd18144b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rcb8f84ef15b5403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R67406c5c72f74673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R7a27c73c8c024793"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R6ffeb826dc6345b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R0f40cc9df2c642a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rcb39d0cece19407d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R3acd99b4868c4758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R59ca3723fa374df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R4ba5e433155f4b00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R15d751f6690b4e28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6817.38</x:v>
+        <x:v>6880.55</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6642.3</x:v>
+        <x:v>6763.45</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>175.1</x:v>
+        <x:v>117.1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1797.6</x:v>
+        <x:v>1914.7</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>199.7</x:v>
+        <x:v>191.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6902.09</x:v>
+        <x:v>6941.51</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6745.14</x:v>
+        <x:v>6821.39</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>156.9</x:v>
+        <x:v>120.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1679.3</x:v>
+        <x:v>1799.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>186.6</x:v>
+        <x:v>179.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3740.07</x:v>
+        <x:v>3743.08</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3702.44</x:v>
+        <x:v>3703.12</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>37.6</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>515.3</x:v>
+        <x:v>555.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>57.3</x:v>
+        <x:v>55.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6735.6</x:v>
+        <x:v>6799.6</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6543</x:v>
+        <x:v>6658.2</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>192.6</x:v>
+        <x:v>141.4</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>1904</x:v>
+        <x:v>2045.4</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>211.6</x:v>
+        <x:v>204.5</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1455,37 +1455,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>10月19日-10月20日</x:v>
+        <x:v>10月19日-10月21日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>6639.94</x:v>
       </x:c>
       <x:c r="D7" s="23" t="n">
-        <x:v>6817.38</x:v>
+        <x:v>6880.55</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
         <x:v>6578.94</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>6766.9</x:v>
+        <x:v>6780.26</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>85</x:v>
+        <x:v>98.3</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.012714870232297892</x:v>
+        <x:v>0.014714289562612226</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>238.4</x:v>
+        <x:v>301.6</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1503,7 +1503,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1198.3</x:v>
+        <x:v>1261.5</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1521,7 +1521,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>399.4</x:v>
+        <x:v>420.5</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1651,37 +1651,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>10月19日-10月20日</x:v>
+        <x:v>10月19日-10月21日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>6735.53</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>6902.09</x:v>
+        <x:v>6941.51</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
         <x:v>6692.83</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>6841.44</x:v>
+        <x:v>6840.56</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>68.7</x:v>
+        <x:v>67.8</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.010142113617068294</x:v>
+        <x:v>0.010012181167177392</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>209.3</x:v>
+        <x:v>248.7</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1699,7 +1699,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1139.1</x:v>
+        <x:v>1178.5</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1717,7 +1717,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>379.7</x:v>
+        <x:v>392.8</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1847,7 +1847,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月19日-10月20日</x:v>
+        <x:v>10月19日-10月21日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3694.12</x:v>
@@ -1859,15 +1859,15 @@
         <x:v>3692.29</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3735.37</x:v>
+        <x:v>3713.03</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>19.1</x:v>
+        <x:v>-3.2</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>0.00513685728739488</x:v>
+        <x:v>-0.0008745304444228719</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
@@ -1877,7 +1877,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2043,37 +2043,37 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>10月19日-10月20日</x:v>
+        <x:v>10月19日-10月21日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>6577.2</x:v>
       </x:c>
       <x:c r="D31" s="23" t="n">
-        <x:v>6735.6</x:v>
+        <x:v>6799.6</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
         <x:v>6505</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>6663.8</x:v>
+        <x:v>6659.2</x:v>
       </x:c>
       <x:c r="G31" s="23" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>80.2</x:v>
+        <x:v>75.6</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.012181785041618598</x:v>
+        <x:v>0.011483079166413335</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>230.6</x:v>
+        <x:v>294.6</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2091,7 +2091,7 @@
       <x:c r="H32" s="30"/>
       <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1174.8</x:v>
+        <x:v>1238.8</x:v>
       </x:c>
       <x:c r="J32" s="30"/>
       <x:c r="K32" s="30"/>
@@ -2109,7 +2109,7 @@
       <x:c r="H33" s="30"/>
       <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>391.6</x:v>
+        <x:v>412.9</x:v>
       </x:c>
       <x:c r="J33" s="30"/>
       <x:c r="K33" s="30"/>
@@ -3295,31 +3295,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="30" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="30"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1797.6</x:v>
-      </x:c>
-      <x:c r="K15" s="30"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>10月21日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>6798.97</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>6880.55</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>6763.45</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>6780.26</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>13.4</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>0.0019743161565857203</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>117.1</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="30"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
@@ -3327,11 +3345,29 @@
       <x:c r="G16" s="30"/>
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="30"/>
-      <x:c r="J16" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>199.7</x:v>
+      <x:c r="J16" s="32" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1914.6999999999998</x:v>
       </x:c>
       <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>191.5</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3722,31 +3758,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="30" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="30"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1679.3</x:v>
-      </x:c>
-      <x:c r="K15" s="30"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>10月21日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>6875.71</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>6941.51</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>6821.39</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>6840.56</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-0.9</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.00012862789120404727</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>120.1</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="30"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
@@ -3754,11 +3808,29 @@
       <x:c r="G16" s="30"/>
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="30"/>
-      <x:c r="J16" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>186.6</x:v>
+      <x:c r="J16" s="32" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>1799.3999999999999</x:v>
       </x:c>
       <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>179.9</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4149,31 +4221,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="30" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="30"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>515.3</x:v>
-      </x:c>
-      <x:c r="K15" s="30"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>10月21日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>3740.57</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>3743.08</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>3703.12</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>3713.03</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-22.3</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.00598066590458235</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="30"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
@@ -4181,11 +4271,29 @@
       <x:c r="G16" s="30"/>
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="30"/>
-      <x:c r="J16" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>57.3</x:v>
+      <x:c r="J16" s="32" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>555.3</x:v>
       </x:c>
       <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>55.5</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4576,31 +4684,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B15" s="30" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-      <x:c r="G15" s="30"/>
-      <x:c r="H15" s="30"/>
-      <x:c r="I15" s="30"/>
-      <x:c r="J15" s="32" t="n">
-        <x:f>SUM(J4:J12)</x:f>
-        <x:v>1904.0000000000002</x:v>
-      </x:c>
-      <x:c r="K15" s="30"/>
+    <x:row r="13">
+      <x:c r="A13" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>10月21日</x:v>
+      </x:c>
+      <x:c r="D13" s="23" t="n">
+        <x:v>6722</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="n">
+        <x:v>6799.6</x:v>
+      </x:c>
+      <x:c r="F13" s="23" t="n">
+        <x:v>6658.2</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="n">
+        <x:v>6659.2</x:v>
+      </x:c>
+      <x:c r="H13" s="23" t="n">
+        <x:v>-4.6</x:v>
+      </x:c>
+      <x:c r="I13" s="24" t="n">
+        <x:v>-0.0006902968276358834</x:v>
+      </x:c>
+      <x:c r="J13" s="23" t="n">
+        <x:f>ROUND(E13-F13,1)</x:f>
+        <x:v>141.4</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B16" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="C16" s="30"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
@@ -4608,11 +4734,29 @@
       <x:c r="G16" s="30"/>
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="30"/>
-      <x:c r="J16" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J12),0),1)</x:f>
-        <x:v>211.6</x:v>
+      <x:c r="J16" s="32" t="n">
+        <x:f>SUM(J4:J13)</x:f>
+        <x:v>2045.4000000000003</x:v>
       </x:c>
       <x:c r="K16" s="30"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="30"/>
+      <x:c r="J17" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
+        <x:v>204.5</x:v>
+      </x:c>
+      <x:c r="K17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-22
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rb82b53224a06439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R75b2bd7c38cf43a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R5d9db00902864404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Raf2dc2caa8b1496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R1ca740af0a134493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R99133acb6ea6405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4ce0120c03cf4e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R7d52bef6d82b4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R18f6b5832a8a4aeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R5c496969a70a475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R19edab44772b474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R47112c4d08bc4497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rdf2f93099e9c4aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb7c16bf7bb0d47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R14ad4c6426e94672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re86cf258ffc842e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R9c073d8756964672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R3d6b83e756ca493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9b5f4efa0a724825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R7960880de16347dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6880.55</x:v>
+        <x:v>6782.9</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6763.45</x:v>
+        <x:v>6578.27</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>117.1</x:v>
+        <x:v>204.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>1914.7</x:v>
+        <x:v>2119.3</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>191.5</x:v>
+        <x:v>192.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6941.51</x:v>
+        <x:v>6842.87</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6821.39</x:v>
+        <x:v>6652.78</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>120.1</x:v>
+        <x:v>190.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1799.4</x:v>
+        <x:v>1989.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>179.9</x:v>
+        <x:v>180.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3743.08</x:v>
+        <x:v>3714.48</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3703.12</x:v>
+        <x:v>3649.86</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>40</x:v>
+        <x:v>64.6</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>555.3</x:v>
+        <x:v>619.9</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>55.5</x:v>
+        <x:v>56.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6799.6</x:v>
+        <x:v>6689</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6658.2</x:v>
+        <x:v>6466.8</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>141.4</x:v>
+        <x:v>222.2</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2045.4</x:v>
+        <x:v>2267.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>204.5</x:v>
+        <x:v>206.1</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6864</x:v>
+        <x:v>6753.6</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6726</x:v>
+        <x:v>6543</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>138</x:v>
+        <x:v>210.6</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>1993.4</x:v>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>199.3</x:v>
+        <x:v>200.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -694,25 +694,25 @@
         <x:v>IH主力</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:v>2732</x:v>
+        <x:v>2713</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
-        <x:v>2697</x:v>
+        <x:v>2669.2</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
-        <x:v>35</x:v>
+        <x:v>43.8</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G10" s="10" t="n">
-        <x:v>458.4</x:v>
+        <x:v>502.2</x:v>
       </x:c>
       <x:c r="H10" s="10" t="n">
-        <x:v>45.8</x:v>
+        <x:v>45.7</x:v>
       </x:c>
       <x:c r="I10" s="10" t="n">
         <x:v>60</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1491,7 +1491,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>6639.94</x:v>
@@ -1500,28 +1500,28 @@
         <x:v>6880.55</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>6578.94</x:v>
+        <x:v>6578.27</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>6780.26</x:v>
+        <x:v>6578.27</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>98.3</x:v>
+        <x:v>-103.7</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>0.014714289562612226</x:v>
+        <x:v>-0.015514955237550643</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>301.6</x:v>
+        <x:v>302.3</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1539,7 +1539,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1261.5</x:v>
+        <x:v>1262.2</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1557,7 +1557,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>420.5</x:v>
+        <x:v>420.7</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1687,7 +1687,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>6735.53</x:v>
@@ -1696,28 +1696,28 @@
         <x:v>6941.51</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>6692.83</x:v>
+        <x:v>6652.78</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>6840.56</x:v>
+        <x:v>6655.25</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>67.8</x:v>
+        <x:v>-117.5</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.010012181167177392</x:v>
+        <x:v>-0.017348935070687688</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>248.7</x:v>
+        <x:v>288.7</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1735,7 +1735,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1178.5</x:v>
+        <x:v>1218.5</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1753,7 +1753,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>392.8</x:v>
+        <x:v>406.2</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1883,7 +1883,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3694.12</x:v>
@@ -1892,28 +1892,28 @@
         <x:v>3743.8</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3692.29</x:v>
+        <x:v>3649.86</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3713.03</x:v>
+        <x:v>3658.03</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-3.2</x:v>
+        <x:v>-58.2</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.0008745304444228719</x:v>
+        <x:v>-0.015674276426964617</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>51.5</x:v>
+        <x:v>93.9</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1931,7 +1931,7 @@
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>314.9</x:v>
+        <x:v>357.3</x:v>
       </x:c>
       <x:c r="J24" s="30"/>
       <x:c r="K24" s="30"/>
@@ -1949,7 +1949,7 @@
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>105</x:v>
+        <x:v>119.1</x:v>
       </x:c>
       <x:c r="J25" s="30"/>
       <x:c r="K25" s="30"/>
@@ -2079,7 +2079,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C31" s="23" t="n">
         <x:v>6577.2</x:v>
@@ -2088,28 +2088,28 @@
         <x:v>6799.6</x:v>
       </x:c>
       <x:c r="E31" s="23" t="n">
-        <x:v>6505</x:v>
+        <x:v>6466.8</x:v>
       </x:c>
       <x:c r="F31" s="23" t="n">
-        <x:v>6659.2</x:v>
+        <x:v>6471.6</x:v>
       </x:c>
       <x:c r="G31" s="23" t="n">
         <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>75.6</x:v>
+        <x:v>-112</x:v>
       </x:c>
       <x:c r="H31" s="24" t="n">
         <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.011483079166413335</x:v>
+        <x:v>-0.017011969135427463</x:v>
       </x:c>
       <x:c r="I31" s="26" t="n">
         <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>294.6</x:v>
+        <x:v>332.8</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K31" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2127,7 +2127,7 @@
       <x:c r="H32" s="30"/>
       <x:c r="I32" s="32" t="n">
         <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1238.8</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="J32" s="30"/>
       <x:c r="K32" s="30"/>
@@ -2145,7 +2145,7 @@
       <x:c r="H33" s="30"/>
       <x:c r="I33" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>412.9</x:v>
+        <x:v>425.7</x:v>
       </x:c>
       <x:c r="J33" s="30"/>
       <x:c r="K33" s="30"/>
@@ -2275,7 +2275,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>6670.2</x:v>
@@ -2284,28 +2284,28 @@
         <x:v>6864</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
-        <x:v>6608.2</x:v>
+        <x:v>6543</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>6735</x:v>
+        <x:v>6543</x:v>
       </x:c>
       <x:c r="G39" s="23" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>67.2</x:v>
+        <x:v>-124.8</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.010078286691262539</x:v>
+        <x:v>-0.01871681814091608</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>255.8</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2323,7 +2323,7 @@
       <x:c r="H40" s="30"/>
       <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1211.2</x:v>
+        <x:v>1276.4</x:v>
       </x:c>
       <x:c r="J40" s="30"/>
       <x:c r="K40" s="30"/>
@@ -2341,7 +2341,7 @@
       <x:c r="H41" s="30"/>
       <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>403.7</x:v>
+        <x:v>425.5</x:v>
       </x:c>
       <x:c r="J41" s="30"/>
       <x:c r="K41" s="30"/>
@@ -2667,7 +2667,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
+        <x:v>10月19日-10月22日</x:v>
       </x:c>
       <x:c r="C55" s="23" t="n">
         <x:v>2690</x:v>
@@ -2676,28 +2676,28 @@
         <x:v>2754.6</x:v>
       </x:c>
       <x:c r="E55" s="23" t="n">
-        <x:v>2690</x:v>
+        <x:v>2669.2</x:v>
       </x:c>
       <x:c r="F55" s="23" t="n">
-        <x:v>2701</x:v>
+        <x:v>2679.2</x:v>
       </x:c>
       <x:c r="G55" s="23" t="n">
         <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>-3.6</x:v>
+        <x:v>-25.4</x:v>
       </x:c>
       <x:c r="H55" s="24" t="n">
         <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>-0.0013310655919543946</x:v>
+        <x:v>-0.009391407232123061</x:v>
       </x:c>
       <x:c r="I55" s="26" t="n">
         <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>64.6</x:v>
+        <x:v>85.4</x:v>
       </x:c>
       <x:c r="J55" s="22" t="str">
         <x:v>IH2612</x:v>
       </x:c>
       <x:c r="K55" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2715,7 +2715,7 @@
       <x:c r="H56" s="30"/>
       <x:c r="I56" s="32" t="n">
         <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>244.4</x:v>
+        <x:v>265.2</x:v>
       </x:c>
       <x:c r="J56" s="30"/>
       <x:c r="K56" s="30"/>
@@ -2733,7 +2733,7 @@
       <x:c r="H57" s="30"/>
       <x:c r="I57" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>81.5</x:v>
+        <x:v>88.4</x:v>
       </x:c>
       <x:c r="J57" s="30"/>
       <x:c r="K57" s="30"/>
@@ -3367,31 +3367,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1914.6999999999998</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>6782.28</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>6782.9</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>6578.27</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>6578.27</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>-202</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.029790892974605687</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>204.6</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -3399,11 +3417,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>191.5</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>2119.2999999999997</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>192.7</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3830,31 +3866,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1799.3999999999999</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>6841.53</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>6842.87</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>6652.78</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>6655.25</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>-185.3</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.02708988737764162</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>190.1</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -3862,11 +3916,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>179.9</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>1989.4999999999998</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>180.9</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4293,31 +4365,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>555.3</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>3714.48</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>3714.48</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>3649.86</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>3658.03</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-55</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.014812700139777979</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>64.6</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -4325,11 +4415,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>55.5</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>619.9</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>56.4</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4756,31 +4864,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>2045.4000000000003</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>6670</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>6689</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>6466.8</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>6471.6</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>-187.6</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.02817155213839495</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>222.2</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -4788,11 +4914,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>204.5</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>2267.6000000000004</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>206.1</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5219,31 +5363,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>1993.4</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>6741.8</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>6753.6</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>6543</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>6543</x:v>
+      </x:c>
+      <x:c r="H14" s="28" t="n">
+        <x:v>-192</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.02850779510022272</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>210.6</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -5251,11 +5413,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>199.3</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>2204</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>200.4</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6145,31 +6325,49 @@
         <x:v>IH2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="30"/>
-      <x:c r="J16" s="32" t="n">
-        <x:f>SUM(J4:J13)</x:f>
-        <x:v>458.4000000000001</x:v>
-      </x:c>
-      <x:c r="K16" s="30"/>
+    <x:row r="14">
+      <x:c r="A14" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>10月22日</x:v>
+      </x:c>
+      <x:c r="D14" s="23" t="n">
+        <x:v>2713</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="n">
+        <x:v>2713</x:v>
+      </x:c>
+      <x:c r="F14" s="23" t="n">
+        <x:v>2669.2</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="n">
+        <x:v>2679.2</x:v>
+      </x:c>
+      <x:c r="H14" s="23" t="n">
+        <x:v>-21.8</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>-0.008071084783413562</x:v>
+      </x:c>
+      <x:c r="J14" s="23" t="n">
+        <x:f>ROUND(E14-F14,1)</x:f>
+        <x:v>43.8</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B17" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="C17" s="30"/>
       <x:c r="D17" s="30"/>
       <x:c r="E17" s="30"/>
@@ -6177,11 +6375,29 @@
       <x:c r="G17" s="30"/>
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="30"/>
-      <x:c r="J17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J13),0),1)</x:f>
-        <x:v>45.8</x:v>
+      <x:c r="J17" s="32" t="n">
+        <x:f>SUM(J4:J14)</x:f>
+        <x:v>502.2000000000001</x:v>
       </x:c>
       <x:c r="K17" s="30"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="30"/>
+      <x:c r="J18" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
+        <x:v>45.7</x:v>
+      </x:c>
+      <x:c r="K18" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-23
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R19d73ba89cf5490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R5ed9a77cf9324818"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1115fb31c33a476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rd295f060d8f64c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R04dedf96e42647f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Re289388063584d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra21b4886ce1242ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rbcb40fe721764b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R7fb8860e45584b41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R46a46e88c8e24a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4610d990222c4bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R95dccac45a144845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf6ccca6822164b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rcfdf0405d0944d79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rddaab1f63d05424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2a9dcc36de5e441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R44dd794bd49b4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R19e3f534663645c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R75e18d5d61cc4c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Re4013d0968964329"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-10-23</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6782.9</x:v>
+        <x:v>6753.34</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6578.27</x:v>
+        <x:v>6301.81</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>204.6</x:v>
+        <x:v>451.5</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2119.3</x:v>
+        <x:v>2570.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>192.7</x:v>
+        <x:v>214.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-10-23</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6842.87</x:v>
+        <x:v>6835.39</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6652.78</x:v>
+        <x:v>6440.29</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>190.1</x:v>
+        <x:v>395.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>1989.5</x:v>
+        <x:v>2384.6</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>180.9</x:v>
+        <x:v>198.7</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-10-23</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3714.48</x:v>
+        <x:v>3691.4</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3649.86</x:v>
+        <x:v>3574.27</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>64.6</x:v>
+        <x:v>117.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>619.9</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>56.4</x:v>
+        <x:v>61.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-10-23</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6753.6</x:v>
+        <x:v>6766.6</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6543</x:v>
+        <x:v>6340</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>210.6</x:v>
+        <x:v>426.6</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2204</x:v>
+        <x:v>2630.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>200.4</x:v>
+        <x:v>219.2</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-10-23</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1491,7 +1491,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>10月19日-10月22日</x:v>
+        <x:v>10月19日-10月23日</x:v>
       </x:c>
       <x:c r="C7" s="23" t="n">
         <x:v>6639.94</x:v>
@@ -1500,28 +1500,28 @@
         <x:v>6880.55</x:v>
       </x:c>
       <x:c r="E7" s="23" t="n">
-        <x:v>6578.27</x:v>
+        <x:v>6301.81</x:v>
       </x:c>
       <x:c r="F7" s="23" t="n">
-        <x:v>6578.27</x:v>
+        <x:v>6734.55</x:v>
       </x:c>
       <x:c r="G7" s="23" t="n">
         <x:f>ROUND(F7-F6,1)</x:f>
-        <x:v>-103.7</x:v>
+        <x:v>52.6</x:v>
       </x:c>
       <x:c r="H7" s="24" t="n">
         <x:f>IFERROR(F7/F6-1,"")</x:f>
-        <x:v>-0.015514955237550643</x:v>
+        <x:v>0.007873461898789902</x:v>
       </x:c>
       <x:c r="I7" s="26" t="n">
         <x:f>ROUND(D7-E7,1)</x:f>
-        <x:v>302.3</x:v>
+        <x:v>578.7</x:v>
       </x:c>
       <x:c r="J7" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K7" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1539,7 +1539,7 @@
       <x:c r="H8" s="30"/>
       <x:c r="I8" s="32" t="n">
         <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1262.2</x:v>
+        <x:v>1538.6</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30"/>
@@ -1557,7 +1557,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>420.7</x:v>
+        <x:v>512.9</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1687,7 +1687,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>10月19日-10月22日</x:v>
+        <x:v>10月19日-10月23日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
         <x:v>6735.53</x:v>
@@ -1696,28 +1696,28 @@
         <x:v>6941.51</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>6652.78</x:v>
+        <x:v>6440.29</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>6655.25</x:v>
+        <x:v>6814.44</x:v>
       </x:c>
       <x:c r="G15" s="23" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>-117.5</x:v>
+        <x:v>41.7</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>-0.017348935070687688</x:v>
+        <x:v>0.006155549813591232</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>288.7</x:v>
+        <x:v>501.2</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K15" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1735,7 +1735,7 @@
       <x:c r="H16" s="30"/>
       <x:c r="I16" s="32" t="n">
         <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1218.5</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
@@ -1753,7 +1753,7 @@
       <x:c r="H17" s="30"/>
       <x:c r="I17" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>406.2</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30"/>
@@ -1883,7 +1883,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月19日-10月22日</x:v>
+        <x:v>10月19日-10月23日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
         <x:v>3694.12</x:v>
@@ -1892,28 +1892,28 @@
         <x:v>3743.8</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3649.86</x:v>
+        <x:v>3574.27</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3658.03</x:v>
+        <x:v>3690.48</x:v>
       </x:c>
       <x:c r="G23" s="23" t="n">
         <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-58.2</x:v>
+        <x:v>-25.8</x:v>
       </x:c>
       <x:c r="H23" s="24" t="n">
         <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.015674276426964617</x:v>
+        <x:v>-0.0069424262972650475</x:v>
       </x:c>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>93.9</x:v>
+        <x:v>169.5</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1931,7 +1931,7 @@
       <x:c r="H24" s="30"/>
       <x:c r="I24" s="32" t="n">
         <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>357.3</x:v>
+        <x:v>432.9</x:v>
       </x:c>
       <x:c r="J24" s="30"/>
       <x:c r="K24" s="30"/>
@@ -1949,7 +1949,7 @@
       <x:c r="H25" s="30"/>
       <x:c r="I25" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>119.1</x:v>
+        <x:v>144.3</x:v>
       </x:c>
       <x:c r="J25" s="30"/>
       <x:c r="K25" s="30"/>
@@ -2275,7 +2275,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>10月19日-10月22日</x:v>
+        <x:v>10月19日-10月23日</x:v>
       </x:c>
       <x:c r="C39" s="23" t="n">
         <x:v>6670.2</x:v>
@@ -2284,28 +2284,28 @@
         <x:v>6864</x:v>
       </x:c>
       <x:c r="E39" s="23" t="n">
-        <x:v>6543</x:v>
+        <x:v>6340</x:v>
       </x:c>
       <x:c r="F39" s="23" t="n">
-        <x:v>6543</x:v>
+        <x:v>6742</x:v>
       </x:c>
       <x:c r="G39" s="23" t="n">
         <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>-124.8</x:v>
+        <x:v>74.2</x:v>
       </x:c>
       <x:c r="H39" s="24" t="n">
         <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>-0.01871681814091608</x:v>
+        <x:v>0.011128108221602373</x:v>
       </x:c>
       <x:c r="I39" s="26" t="n">
         <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>321</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="J39" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K39" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2323,7 +2323,7 @@
       <x:c r="H40" s="30"/>
       <x:c r="I40" s="32" t="n">
         <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1276.4</x:v>
+        <x:v>1479.4</x:v>
       </x:c>
       <x:c r="J40" s="30"/>
       <x:c r="K40" s="30"/>
@@ -2341,7 +2341,7 @@
       <x:c r="H41" s="30"/>
       <x:c r="I41" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>425.5</x:v>
+        <x:v>493.1</x:v>
       </x:c>
       <x:c r="J41" s="30"/>
       <x:c r="K41" s="30"/>
@@ -3403,31 +3403,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>2119.2999999999997</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>10月23日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>6480.18</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>6753.34</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>6301.81</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>6734.55</x:v>
+      </x:c>
+      <x:c r="H15" s="28" t="n">
+        <x:v>156.3</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.0237570060213399</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>451.5</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -3435,11 +3453,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>192.7</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2570.7999999999997</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>214.2</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3902,31 +3938,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>1989.4999999999998</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>10月23日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>6559.61</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>6835.39</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>6440.29</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>6814.44</x:v>
+      </x:c>
+      <x:c r="H15" s="28" t="n">
+        <x:v>159.2</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.023919462078809905</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>395.1</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -3934,11 +3988,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>180.9</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2384.6</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>198.7</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4401,31 +4473,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>619.9</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>10月23日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>3623.57</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>3691.4</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>3574.27</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>3690.48</x:v>
+      </x:c>
+      <x:c r="H15" s="23" t="n">
+        <x:v>32.4</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.008870894989926326</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>117.1</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -4433,11 +4523,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>56.4</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>61.4</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5399,31 +5507,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B17" s="30" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="30"/>
-      <x:c r="J17" s="32" t="n">
-        <x:f>SUM(J4:J14)</x:f>
-        <x:v>2204</x:v>
-      </x:c>
-      <x:c r="K17" s="30"/>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>10月23日</x:v>
+      </x:c>
+      <x:c r="D15" s="23" t="n">
+        <x:v>6500</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="n">
+        <x:v>6766.6</x:v>
+      </x:c>
+      <x:c r="F15" s="23" t="n">
+        <x:v>6340</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="n">
+        <x:v>6742</x:v>
+      </x:c>
+      <x:c r="H15" s="28" t="n">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="n">
+        <x:v>0.03041418309643884</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:f>ROUND(E15-F15,1)</x:f>
+        <x:v>426.6</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B18" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="C18" s="30"/>
       <x:c r="D18" s="30"/>
       <x:c r="E18" s="30"/>
@@ -5431,11 +5557,29 @@
       <x:c r="G18" s="30"/>
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="30"/>
-      <x:c r="J18" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J14),0),1)</x:f>
-        <x:v>200.4</x:v>
+      <x:c r="J18" s="32" t="n">
+        <x:f>SUM(J4:J15)</x:f>
+        <x:v>2630.6</x:v>
       </x:c>
       <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="30"/>
+      <x:c r="J19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
+        <x:v>219.2</x:v>
+      </x:c>
+      <x:c r="K19" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-26
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rc739f03ccb114219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rd0588941430c4a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R9bf98215f78440c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rf3e28d41f2f940fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rb28be301d97c4a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R9731da4516c1480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R0ff03a5eb3b74a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R627e7d0b2261488e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Re9182ae7b7734c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R04a965ee4ba84334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R28b344b38b44459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R711cda8eb463459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R1e142a4a35064902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rb836b5fa1e764f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R24376b17c80b419a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rb6fa3dabee2042b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra85b1af222714f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Re49f4f014b0142e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R51337ba6f5234d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R961e34da99e64ab5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6753.34</x:v>
+        <x:v>6704.68</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6301.81</x:v>
+        <x:v>6589.13</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>451.5</x:v>
+        <x:v>115.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2570.8</x:v>
+        <x:v>2686.4</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>214.2</x:v>
+        <x:v>206.6</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6835.39</x:v>
+        <x:v>6787.32</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6440.29</x:v>
+        <x:v>6674.4</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>395.1</x:v>
+        <x:v>112.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2384.6</x:v>
+        <x:v>2497.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>198.7</x:v>
+        <x:v>192.1</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3691.4</x:v>
+        <x:v>3699.01</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3574.27</x:v>
+        <x:v>3664.82</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>117.1</x:v>
+        <x:v>34.2</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>737</x:v>
+        <x:v>771.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>61.4</x:v>
+        <x:v>59.3</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6766.6</x:v>
+        <x:v>6711.4</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6340</x:v>
+        <x:v>6573.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>426.6</x:v>
+        <x:v>137.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2630.6</x:v>
+        <x:v>2768.4</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>219.2</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4063</x:v>
+        <x:v>4049.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>3897.6</x:v>
+        <x:v>3996.4</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>165.4</x:v>
+        <x:v>53.4</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1070.6</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>89.2</x:v>
+        <x:v>86.5</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-26</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1525,193 +1525,193 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B8" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="30"/>
-      <x:c r="D8" s="30"/>
-      <x:c r="E8" s="30"/>
-      <x:c r="F8" s="30"/>
-      <x:c r="G8" s="30"/>
-      <x:c r="H8" s="30"/>
-      <x:c r="I8" s="32" t="n">
-        <x:f>ROUND(SUM(I5:I7),1)</x:f>
-        <x:v>1538.6</x:v>
-      </x:c>
-      <x:c r="J8" s="30"/>
-      <x:c r="K8" s="30"/>
+      <x:c r="A8" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="n">
+        <x:v>6684.93</x:v>
+      </x:c>
+      <x:c r="D8" s="23" t="n">
+        <x:v>6704.68</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="n">
+        <x:v>6589.13</x:v>
+      </x:c>
+      <x:c r="F8" s="23" t="n">
+        <x:v>6630.78</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="n">
+        <x:f>ROUND(F8-F7,1)</x:f>
+        <x:v>-103.8</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="n">
+        <x:f>IFERROR(F8/F7-1,"")</x:f>
+        <x:v>-0.015408601911040876</x:v>
+      </x:c>
+      <x:c r="I8" s="23" t="n">
+        <x:f>ROUND(D8-E8,1)</x:f>
+        <x:v>115.6</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B9" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C9" s="30"/>
       <x:c r="D9" s="30"/>
       <x:c r="E9" s="30"/>
       <x:c r="F9" s="30"/>
       <x:c r="G9" s="30"/>
       <x:c r="H9" s="30"/>
-      <x:c r="I9" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I5:I7),0),1)</x:f>
-        <x:v>512.9</x:v>
+      <x:c r="I9" s="32" t="n">
+        <x:f>ROUND(SUM(I5:I8),1)</x:f>
+        <x:v>1654.2</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="17" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
+      <x:c r="E10" s="30"/>
+      <x:c r="F10" s="30"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
+        <x:v>413.6</x:v>
+      </x:c>
+      <x:c r="J10" s="30"/>
+      <x:c r="K10" s="30"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="17" t="str">
         <x:v>中证500</x:v>
       </x:c>
-      <x:c r="B11" s="17"/>
-      <x:c r="C11" s="17"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="17"/>
-      <x:c r="F11" s="17"/>
-      <x:c r="G11" s="17"/>
-      <x:c r="H11" s="17"/>
-      <x:c r="I11" s="17"/>
-      <x:c r="J11" s="17"/>
-      <x:c r="K11" s="17"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="20" t="str">
+      <x:c r="B12" s="17"/>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
+      <x:c r="H12" s="17"/>
+      <x:c r="I12" s="17"/>
+      <x:c r="J12" s="17"/>
+      <x:c r="K12" s="17"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="str">
+      <x:c r="B13" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="str">
+      <x:c r="C13" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D12" s="20" t="str">
+      <x:c r="D13" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E12" s="20" t="str">
+      <x:c r="E13" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="str">
+      <x:c r="F13" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G12" s="20" t="str">
+      <x:c r="G13" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H12" s="20" t="str">
+      <x:c r="H13" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I12" s="20" t="str">
+      <x:c r="I13" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J12" s="20" t="str">
+      <x:c r="J13" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K12" s="20" t="str">
+      <x:c r="K13" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B13" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C13" s="23" t="n">
-        <x:v>7420.44</x:v>
-      </x:c>
-      <x:c r="D13" s="23" t="n">
-        <x:v>7461.24</x:v>
-      </x:c>
-      <x:c r="E13" s="23" t="n">
-        <x:v>7048.45</x:v>
-      </x:c>
-      <x:c r="F13" s="23" t="n">
-        <x:v>7251.01</x:v>
-      </x:c>
-      <x:c r="G13" s="23"/>
-      <x:c r="H13" s="24"/>
-      <x:c r="I13" s="26" t="n">
-        <x:f>ROUND(D13-E13,1)</x:f>
-        <x:v>412.8</x:v>
-      </x:c>
-      <x:c r="J13" s="22" t="str">
-        <x:v>中证500</x:v>
-      </x:c>
-      <x:c r="K13" s="22" t="n">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C14" s="23" t="n">
-        <x:v>7226.07</x:v>
+        <x:v>7420.44</x:v>
       </x:c>
       <x:c r="D14" s="23" t="n">
-        <x:v>7236.78</x:v>
+        <x:v>7461.24</x:v>
       </x:c>
       <x:c r="E14" s="23" t="n">
-        <x:v>6719.82</x:v>
+        <x:v>7048.45</x:v>
       </x:c>
       <x:c r="F14" s="23" t="n">
-        <x:v>6772.75</x:v>
-      </x:c>
-      <x:c r="G14" s="28" t="n">
-        <x:f>ROUND(F14-F13,1)</x:f>
-        <x:v>-478.3</x:v>
-      </x:c>
-      <x:c r="H14" s="24" t="n">
-        <x:f>IFERROR(F14/F13-1,"")</x:f>
-        <x:v>-0.06595770796068412</x:v>
-      </x:c>
+        <x:v>7251.01</x:v>
+      </x:c>
+      <x:c r="G14" s="23"/>
+      <x:c r="H14" s="24"/>
       <x:c r="I14" s="26" t="n">
         <x:f>ROUND(D14-E14,1)</x:f>
-        <x:v>517</x:v>
+        <x:v>412.8</x:v>
       </x:c>
       <x:c r="J14" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K14" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>10月19日-10月23日</x:v>
+        <x:v>10月12日-10月16日</x:v>
       </x:c>
       <x:c r="C15" s="23" t="n">
-        <x:v>6735.53</x:v>
+        <x:v>7226.07</x:v>
       </x:c>
       <x:c r="D15" s="23" t="n">
-        <x:v>6941.51</x:v>
+        <x:v>7236.78</x:v>
       </x:c>
       <x:c r="E15" s="23" t="n">
-        <x:v>6440.29</x:v>
+        <x:v>6719.82</x:v>
       </x:c>
       <x:c r="F15" s="23" t="n">
-        <x:v>6814.44</x:v>
-      </x:c>
-      <x:c r="G15" s="23" t="n">
+        <x:v>6772.75</x:v>
+      </x:c>
+      <x:c r="G15" s="28" t="n">
         <x:f>ROUND(F15-F14,1)</x:f>
-        <x:v>41.7</x:v>
+        <x:v>-478.3</x:v>
       </x:c>
       <x:c r="H15" s="24" t="n">
         <x:f>IFERROR(F15/F14-1,"")</x:f>
-        <x:v>0.006155549813591232</x:v>
+        <x:v>-0.06595770796068412</x:v>
       </x:c>
       <x:c r="I15" s="26" t="n">
         <x:f>ROUND(D15-E15,1)</x:f>
-        <x:v>501.2</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="J15" s="22" t="str">
         <x:v>中证500</x:v>
@@ -1721,1230 +1721,1420 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="31" t="str">
+      <x:c r="A16" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>10月19日-10月23日</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="n">
+        <x:v>6735.53</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>6941.51</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>6440.29</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>6814.44</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:f>ROUND(F16-F15,1)</x:f>
+        <x:v>41.7</x:v>
+      </x:c>
+      <x:c r="H16" s="24" t="n">
+        <x:f>IFERROR(F16/F15-1,"")</x:f>
+        <x:v>0.006155549813591232</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="n">
+        <x:f>ROUND(D16-E16,1)</x:f>
+        <x:v>501.2</x:v>
+      </x:c>
+      <x:c r="J16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="n">
+        <x:v>6756.46</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>6787.32</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>6674.4</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>6712.73</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:f>ROUND(F17-F16,1)</x:f>
+        <x:v>-101.7</x:v>
+      </x:c>
+      <x:c r="H17" s="24" t="n">
+        <x:f>IFERROR(F17/F16-1,"")</x:f>
+        <x:v>-0.0149256578677045</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="n">
+        <x:f>ROUND(D17-E17,1)</x:f>
+        <x:v>112.9</x:v>
+      </x:c>
+      <x:c r="J17" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B16" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-      <x:c r="G16" s="30"/>
-      <x:c r="H16" s="30"/>
-      <x:c r="I16" s="32" t="n">
-        <x:f>ROUND(SUM(I13:I15),1)</x:f>
-        <x:v>1431</x:v>
-      </x:c>
-      <x:c r="J16" s="30"/>
-      <x:c r="K16" s="30"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="31" t="str">
+      <x:c r="B18" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="32" t="n">
+        <x:f>ROUND(SUM(I14:I17),1)</x:f>
+        <x:v>1543.9</x:v>
+      </x:c>
+      <x:c r="J18" s="30"/>
+      <x:c r="K18" s="30"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
-      <x:c r="G17" s="30"/>
-      <x:c r="H17" s="30"/>
-      <x:c r="I17" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I13:I15),0),1)</x:f>
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="J17" s="30"/>
-      <x:c r="K17" s="30"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="17" t="str">
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="J19" s="30"/>
+      <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
         <x:v>上证指数</x:v>
       </x:c>
-      <x:c r="B19" s="17"/>
-      <x:c r="C19" s="17"/>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="17"/>
-      <x:c r="F19" s="17"/>
-      <x:c r="G19" s="17"/>
-      <x:c r="H19" s="17"/>
-      <x:c r="I19" s="17"/>
-      <x:c r="J19" s="17"/>
-      <x:c r="K19" s="17"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="20" t="str">
+      <x:c r="B21" s="17"/>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="17"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="17"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B20" s="20" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C20" s="20" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D20" s="20" t="str">
+      <x:c r="D22" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E20" s="20" t="str">
+      <x:c r="E22" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
+      <x:c r="F22" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G20" s="20" t="str">
+      <x:c r="G22" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H20" s="20" t="str">
+      <x:c r="H22" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I20" s="20" t="str">
+      <x:c r="I22" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J20" s="20" t="str">
+      <x:c r="J22" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K20" s="20" t="str">
+      <x:c r="K22" s="20" t="str">
         <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B21" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C21" s="23" t="n">
-        <x:v>3838.98</x:v>
-      </x:c>
-      <x:c r="D21" s="23" t="n">
-        <x:v>3864.12</x:v>
-      </x:c>
-      <x:c r="E21" s="23" t="n">
-        <x:v>3754.14</x:v>
-      </x:c>
-      <x:c r="F21" s="23" t="n">
-        <x:v>3813.79</x:v>
-      </x:c>
-      <x:c r="G21" s="23"/>
-      <x:c r="H21" s="24"/>
-      <x:c r="I21" s="26" t="n">
-        <x:f>ROUND(D21-E21,1)</x:f>
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="J21" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K21" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B22" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
-      </x:c>
-      <x:c r="C22" s="23" t="n">
-        <x:v>3806.98</x:v>
-      </x:c>
-      <x:c r="D22" s="23" t="n">
-        <x:v>3828.22</x:v>
-      </x:c>
-      <x:c r="E22" s="23" t="n">
-        <x:v>3674.82</x:v>
-      </x:c>
-      <x:c r="F22" s="23" t="n">
-        <x:v>3716.28</x:v>
-      </x:c>
-      <x:c r="G22" s="23" t="n">
-        <x:f>ROUND(F22-F21,1)</x:f>
-        <x:v>-97.5</x:v>
-      </x:c>
-      <x:c r="H22" s="24" t="n">
-        <x:f>IFERROR(F22/F21-1,"")</x:f>
-        <x:v>-0.02556774232456427</x:v>
-      </x:c>
-      <x:c r="I22" s="26" t="n">
-        <x:f>ROUND(D22-E22,1)</x:f>
-        <x:v>153.4</x:v>
-      </x:c>
-      <x:c r="J22" s="22" t="str">
-        <x:v>上证指数</x:v>
-      </x:c>
-      <x:c r="K22" s="22" t="n">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>10月19日-10月23日</x:v>
+        <x:v>10月8日-10月9日</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n">
-        <x:v>3694.12</x:v>
+        <x:v>3838.98</x:v>
       </x:c>
       <x:c r="D23" s="23" t="n">
-        <x:v>3743.8</x:v>
+        <x:v>3864.12</x:v>
       </x:c>
       <x:c r="E23" s="23" t="n">
-        <x:v>3574.27</x:v>
+        <x:v>3754.14</x:v>
       </x:c>
       <x:c r="F23" s="23" t="n">
-        <x:v>3690.48</x:v>
-      </x:c>
-      <x:c r="G23" s="23" t="n">
-        <x:f>ROUND(F23-F22,1)</x:f>
-        <x:v>-25.8</x:v>
-      </x:c>
-      <x:c r="H23" s="24" t="n">
-        <x:f>IFERROR(F23/F22-1,"")</x:f>
-        <x:v>-0.0069424262972650475</x:v>
-      </x:c>
+        <x:v>3813.79</x:v>
+      </x:c>
+      <x:c r="G23" s="23"/>
+      <x:c r="H23" s="24"/>
       <x:c r="I23" s="26" t="n">
         <x:f>ROUND(D23-E23,1)</x:f>
-        <x:v>169.5</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K23" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="n">
+        <x:v>3806.98</x:v>
+      </x:c>
+      <x:c r="D24" s="23" t="n">
+        <x:v>3828.22</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="n">
+        <x:v>3674.82</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="n">
+        <x:v>3716.28</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="n">
+        <x:f>ROUND(F24-F23,1)</x:f>
+        <x:v>-97.5</x:v>
+      </x:c>
+      <x:c r="H24" s="24" t="n">
+        <x:f>IFERROR(F24/F23-1,"")</x:f>
+        <x:v>-0.02556774232456427</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="n">
+        <x:f>ROUND(D24-E24,1)</x:f>
+        <x:v>153.4</x:v>
+      </x:c>
+      <x:c r="J24" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="31" t="str">
+    <x:row r="25">
+      <x:c r="A25" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>10月19日-10月23日</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="n">
+        <x:v>3694.12</x:v>
+      </x:c>
+      <x:c r="D25" s="23" t="n">
+        <x:v>3743.8</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="n">
+        <x:v>3574.27</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="n">
+        <x:v>3690.48</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="n">
+        <x:f>ROUND(F25-F24,1)</x:f>
+        <x:v>-25.8</x:v>
+      </x:c>
+      <x:c r="H25" s="24" t="n">
+        <x:f>IFERROR(F25/F24-1,"")</x:f>
+        <x:v>-0.0069424262972650475</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="n">
+        <x:f>ROUND(D25-E25,1)</x:f>
+        <x:v>169.5</x:v>
+      </x:c>
+      <x:c r="J25" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K25" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="n">
+        <x:v>3671</x:v>
+      </x:c>
+      <x:c r="D26" s="23" t="n">
+        <x:v>3699.01</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="n">
+        <x:v>3664.82</x:v>
+      </x:c>
+      <x:c r="F26" s="23" t="n">
+        <x:v>3697.52</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="n">
+        <x:f>ROUND(F26-F25,1)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H26" s="24" t="n">
+        <x:f>IFERROR(F26/F25-1,"")</x:f>
+        <x:v>0.0019076109340789849</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="n">
+        <x:f>ROUND(D26-E26,1)</x:f>
+        <x:v>34.2</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B24" s="30" t="n">
+      <x:c r="B27" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="30"/>
+      <x:c r="E27" s="30"/>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="32" t="n">
+        <x:f>ROUND(SUM(I23:I26),1)</x:f>
+        <x:v>467.1</x:v>
+      </x:c>
+      <x:c r="J27" s="30"/>
+      <x:c r="K27" s="30"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="30"/>
+      <x:c r="E28" s="30"/>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
+        <x:v>116.8</x:v>
+      </x:c>
+      <x:c r="J28" s="30"/>
+      <x:c r="K28" s="30"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="17" t="str">
+        <x:v>IM主力</x:v>
+      </x:c>
+      <x:c r="B30" s="17"/>
+      <x:c r="C30" s="17"/>
+      <x:c r="D30" s="17"/>
+      <x:c r="E30" s="17"/>
+      <x:c r="F30" s="17"/>
+      <x:c r="G30" s="17"/>
+      <x:c r="H30" s="17"/>
+      <x:c r="I30" s="17"/>
+      <x:c r="J30" s="17"/>
+      <x:c r="K30" s="17"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C31" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E31" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F31" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G31" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I31" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J31" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K31" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B32" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C32" s="23" t="n">
+        <x:v>7182.8</x:v>
+      </x:c>
+      <x:c r="D32" s="23" t="n">
+        <x:v>7251.8</x:v>
+      </x:c>
+      <x:c r="E32" s="23" t="n">
+        <x:v>6819.2</x:v>
+      </x:c>
+      <x:c r="F32" s="23" t="n">
+        <x:v>7015.8</x:v>
+      </x:c>
+      <x:c r="G32" s="23"/>
+      <x:c r="H32" s="24"/>
+      <x:c r="I32" s="26" t="n">
+        <x:f>ROUND(D32-E32,1)</x:f>
+        <x:v>432.6</x:v>
+      </x:c>
+      <x:c r="J32" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K32" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C33" s="23" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="D33" s="23" t="n">
+        <x:v>7031.2</x:v>
+      </x:c>
+      <x:c r="E33" s="23" t="n">
+        <x:v>6519.6</x:v>
+      </x:c>
+      <x:c r="F33" s="23" t="n">
+        <x:v>6583.6</x:v>
+      </x:c>
+      <x:c r="G33" s="28" t="n">
+        <x:f>ROUND(F33-F32,1)</x:f>
+        <x:v>-432.2</x:v>
+      </x:c>
+      <x:c r="H33" s="24" t="n">
+        <x:f>IFERROR(F33/F32-1,"")</x:f>
+        <x:v>-0.06160380854642378</x:v>
+      </x:c>
+      <x:c r="I33" s="26" t="n">
+        <x:f>ROUND(D33-E33,1)</x:f>
+        <x:v>511.6</x:v>
+      </x:c>
+      <x:c r="J33" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K33" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C24" s="30"/>
-      <x:c r="D24" s="30"/>
-      <x:c r="E24" s="30"/>
-      <x:c r="F24" s="30"/>
-      <x:c r="G24" s="30"/>
-      <x:c r="H24" s="30"/>
-      <x:c r="I24" s="32" t="n">
-        <x:f>ROUND(SUM(I21:I23),1)</x:f>
-        <x:v>432.9</x:v>
-      </x:c>
-      <x:c r="J24" s="30"/>
-      <x:c r="K24" s="30"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="31" t="str">
+      <x:c r="B34" s="22" t="str">
+        <x:v>10月19日-10月23日</x:v>
+      </x:c>
+      <x:c r="C34" s="23" t="n">
+        <x:v>6577.2</x:v>
+      </x:c>
+      <x:c r="D34" s="23" t="n">
+        <x:v>6799.6</x:v>
+      </x:c>
+      <x:c r="E34" s="23" t="n">
+        <x:v>6212.6</x:v>
+      </x:c>
+      <x:c r="F34" s="23" t="n">
+        <x:v>6660</x:v>
+      </x:c>
+      <x:c r="G34" s="23" t="n">
+        <x:f>ROUND(F34-F33,1)</x:f>
+        <x:v>76.4</x:v>
+      </x:c>
+      <x:c r="H34" s="24" t="n">
+        <x:f>IFERROR(F34/F33-1,"")</x:f>
+        <x:v>0.011604593231666405</x:v>
+      </x:c>
+      <x:c r="I34" s="26" t="n">
+        <x:f>ROUND(D34-E34,1)</x:f>
+        <x:v>587</x:v>
+      </x:c>
+      <x:c r="J34" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
+      <x:c r="K34" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B35" s="30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C35" s="30"/>
+      <x:c r="D35" s="30"/>
+      <x:c r="E35" s="30"/>
+      <x:c r="F35" s="30"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="32" t="n">
+        <x:f>ROUND(SUM(I32:I34),1)</x:f>
+        <x:v>1531.2</x:v>
+      </x:c>
+      <x:c r="J35" s="30"/>
+      <x:c r="K35" s="30"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B25" s="30"/>
-      <x:c r="C25" s="30"/>
-      <x:c r="D25" s="30"/>
-      <x:c r="E25" s="30"/>
-      <x:c r="F25" s="30"/>
-      <x:c r="G25" s="30"/>
-      <x:c r="H25" s="30"/>
-      <x:c r="I25" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I21:I23),0),1)</x:f>
-        <x:v>144.3</x:v>
-      </x:c>
-      <x:c r="J25" s="30"/>
-      <x:c r="K25" s="30"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="17" t="str">
-        <x:v>IM主力</x:v>
-      </x:c>
-      <x:c r="B27" s="17"/>
-      <x:c r="C27" s="17"/>
-      <x:c r="D27" s="17"/>
-      <x:c r="E27" s="17"/>
-      <x:c r="F27" s="17"/>
-      <x:c r="G27" s="17"/>
-      <x:c r="H27" s="17"/>
-      <x:c r="I27" s="17"/>
-      <x:c r="J27" s="17"/>
-      <x:c r="K27" s="17"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="20" t="str">
+      <x:c r="B36" s="30"/>
+      <x:c r="C36" s="30"/>
+      <x:c r="D36" s="30"/>
+      <x:c r="E36" s="30"/>
+      <x:c r="F36" s="30"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I32:I34),0),1)</x:f>
+        <x:v>510.4</x:v>
+      </x:c>
+      <x:c r="J36" s="30"/>
+      <x:c r="K36" s="30"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="17" t="str">
+        <x:v>IC主力</x:v>
+      </x:c>
+      <x:c r="B38" s="17"/>
+      <x:c r="C38" s="17"/>
+      <x:c r="D38" s="17"/>
+      <x:c r="E38" s="17"/>
+      <x:c r="F38" s="17"/>
+      <x:c r="G38" s="17"/>
+      <x:c r="H38" s="17"/>
+      <x:c r="I38" s="17"/>
+      <x:c r="J38" s="17"/>
+      <x:c r="K38" s="17"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B28" s="20" t="str">
+      <x:c r="B39" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C28" s="20" t="str">
+      <x:c r="C39" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D28" s="20" t="str">
+      <x:c r="D39" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E28" s="20" t="str">
+      <x:c r="E39" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F28" s="20" t="str">
+      <x:c r="F39" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G28" s="20" t="str">
+      <x:c r="G39" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H28" s="20" t="str">
+      <x:c r="H39" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I28" s="20" t="str">
+      <x:c r="I39" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J28" s="20" t="str">
+      <x:c r="J39" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K28" s="20" t="str">
+      <x:c r="K39" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="22" t="n">
+    <x:row r="40">
+      <x:c r="A40" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B29" s="22" t="str">
+      <x:c r="B40" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C29" s="23" t="n">
-        <x:v>7182.8</x:v>
-      </x:c>
-      <x:c r="D29" s="23" t="n">
-        <x:v>7251.8</x:v>
-      </x:c>
-      <x:c r="E29" s="23" t="n">
-        <x:v>6819.2</x:v>
-      </x:c>
-      <x:c r="F29" s="23" t="n">
-        <x:v>7015.8</x:v>
-      </x:c>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
-      <x:c r="I29" s="26" t="n">
-        <x:f>ROUND(D29-E29,1)</x:f>
-        <x:v>432.6</x:v>
-      </x:c>
-      <x:c r="J29" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K29" s="22" t="n">
+      <x:c r="C40" s="23" t="n">
+        <x:v>7295</x:v>
+      </x:c>
+      <x:c r="D40" s="23" t="n">
+        <x:v>7355</x:v>
+      </x:c>
+      <x:c r="E40" s="23" t="n">
+        <x:v>6932</x:v>
+      </x:c>
+      <x:c r="F40" s="23" t="n">
+        <x:v>7111</x:v>
+      </x:c>
+      <x:c r="G40" s="23"/>
+      <x:c r="H40" s="24"/>
+      <x:c r="I40" s="26" t="n">
+        <x:f>ROUND(D40-E40,1)</x:f>
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="J40" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K40" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="22" t="n">
+    <x:row r="41">
+      <x:c r="A41" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B30" s="22" t="str">
+      <x:c r="B41" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C30" s="23" t="n">
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="D30" s="23" t="n">
-        <x:v>7031.2</x:v>
-      </x:c>
-      <x:c r="E30" s="23" t="n">
-        <x:v>6519.6</x:v>
-      </x:c>
-      <x:c r="F30" s="23" t="n">
-        <x:v>6583.6</x:v>
-      </x:c>
-      <x:c r="G30" s="28" t="n">
-        <x:f>ROUND(F30-F29,1)</x:f>
-        <x:v>-432.2</x:v>
-      </x:c>
-      <x:c r="H30" s="24" t="n">
-        <x:f>IFERROR(F30/F29-1,"")</x:f>
-        <x:v>-0.06160380854642378</x:v>
-      </x:c>
-      <x:c r="I30" s="26" t="n">
-        <x:f>ROUND(D30-E30,1)</x:f>
-        <x:v>511.6</x:v>
-      </x:c>
-      <x:c r="J30" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K30" s="22" t="n">
+      <x:c r="C41" s="23" t="n">
+        <x:v>7076.6</x:v>
+      </x:c>
+      <x:c r="D41" s="23" t="n">
+        <x:v>7115.6</x:v>
+      </x:c>
+      <x:c r="E41" s="23" t="n">
+        <x:v>6583.2</x:v>
+      </x:c>
+      <x:c r="F41" s="23" t="n">
+        <x:v>6667.8</x:v>
+      </x:c>
+      <x:c r="G41" s="28" t="n">
+        <x:f>ROUND(F41-F40,1)</x:f>
+        <x:v>-443.2</x:v>
+      </x:c>
+      <x:c r="H41" s="24" t="n">
+        <x:f>IFERROR(F41/F40-1,"")</x:f>
+        <x:v>-0.062325973843341265</x:v>
+      </x:c>
+      <x:c r="I41" s="26" t="n">
+        <x:f>ROUND(D41-E41,1)</x:f>
+        <x:v>532.4</x:v>
+      </x:c>
+      <x:c r="J41" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K41" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="22" t="n">
+    <x:row r="42">
+      <x:c r="A42" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B31" s="22" t="str">
+      <x:c r="B42" s="22" t="str">
         <x:v>10月19日-10月23日</x:v>
       </x:c>
-      <x:c r="C31" s="23" t="n">
-        <x:v>6577.2</x:v>
-      </x:c>
-      <x:c r="D31" s="23" t="n">
-        <x:v>6799.6</x:v>
-      </x:c>
-      <x:c r="E31" s="23" t="n">
-        <x:v>6212.6</x:v>
-      </x:c>
-      <x:c r="F31" s="23" t="n">
-        <x:v>6660</x:v>
-      </x:c>
-      <x:c r="G31" s="23" t="n">
-        <x:f>ROUND(F31-F30,1)</x:f>
-        <x:v>76.4</x:v>
-      </x:c>
-      <x:c r="H31" s="24" t="n">
-        <x:f>IFERROR(F31/F30-1,"")</x:f>
-        <x:v>0.011604593231666405</x:v>
-      </x:c>
-      <x:c r="I31" s="26" t="n">
-        <x:f>ROUND(D31-E31,1)</x:f>
-        <x:v>587</x:v>
-      </x:c>
-      <x:c r="J31" s="22" t="str">
-        <x:v>IM2612</x:v>
-      </x:c>
-      <x:c r="K31" s="22" t="n">
+      <x:c r="C42" s="23" t="n">
+        <x:v>6670.2</x:v>
+      </x:c>
+      <x:c r="D42" s="23" t="n">
+        <x:v>6864</x:v>
+      </x:c>
+      <x:c r="E42" s="23" t="n">
+        <x:v>6340</x:v>
+      </x:c>
+      <x:c r="F42" s="23" t="n">
+        <x:v>6742</x:v>
+      </x:c>
+      <x:c r="G42" s="23" t="n">
+        <x:f>ROUND(F42-F41,1)</x:f>
+        <x:v>74.2</x:v>
+      </x:c>
+      <x:c r="H42" s="24" t="n">
+        <x:f>IFERROR(F42/F41-1,"")</x:f>
+        <x:v>0.011128108221602373</x:v>
+      </x:c>
+      <x:c r="I42" s="26" t="n">
+        <x:f>ROUND(D42-E42,1)</x:f>
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="J42" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K42" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="31" t="str">
+    <x:row r="43">
+      <x:c r="A43" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B43" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="C43" s="23" t="n">
+        <x:v>6700</x:v>
+      </x:c>
+      <x:c r="D43" s="23" t="n">
+        <x:v>6711.4</x:v>
+      </x:c>
+      <x:c r="E43" s="23" t="n">
+        <x:v>6573.6</x:v>
+      </x:c>
+      <x:c r="F43" s="23" t="n">
+        <x:v>6637</x:v>
+      </x:c>
+      <x:c r="G43" s="23" t="n">
+        <x:f>ROUND(F43-F42,1)</x:f>
+        <x:v>-105</x:v>
+      </x:c>
+      <x:c r="H43" s="24" t="n">
+        <x:f>IFERROR(F43/F42-1,"")</x:f>
+        <x:v>-0.015574013645802465</x:v>
+      </x:c>
+      <x:c r="I43" s="23" t="n">
+        <x:f>ROUND(D43-E43,1)</x:f>
+        <x:v>137.8</x:v>
+      </x:c>
+      <x:c r="J43" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
+      <x:c r="K43" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B32" s="30" t="n">
+      <x:c r="B44" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C44" s="30"/>
+      <x:c r="D44" s="30"/>
+      <x:c r="E44" s="30"/>
+      <x:c r="F44" s="30"/>
+      <x:c r="G44" s="30"/>
+      <x:c r="H44" s="30"/>
+      <x:c r="I44" s="32" t="n">
+        <x:f>ROUND(SUM(I40:I43),1)</x:f>
+        <x:v>1617.2</x:v>
+      </x:c>
+      <x:c r="J44" s="30"/>
+      <x:c r="K44" s="30"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B45" s="30"/>
+      <x:c r="C45" s="30"/>
+      <x:c r="D45" s="30"/>
+      <x:c r="E45" s="30"/>
+      <x:c r="F45" s="30"/>
+      <x:c r="G45" s="30"/>
+      <x:c r="H45" s="30"/>
+      <x:c r="I45" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I40:I43),0),1)</x:f>
+        <x:v>404.3</x:v>
+      </x:c>
+      <x:c r="J45" s="30"/>
+      <x:c r="K45" s="30"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="17" t="str">
+        <x:v>IF主力</x:v>
+      </x:c>
+      <x:c r="B47" s="17"/>
+      <x:c r="C47" s="17"/>
+      <x:c r="D47" s="17"/>
+      <x:c r="E47" s="17"/>
+      <x:c r="F47" s="17"/>
+      <x:c r="G47" s="17"/>
+      <x:c r="H47" s="17"/>
+      <x:c r="I47" s="17"/>
+      <x:c r="J47" s="17"/>
+      <x:c r="K47" s="17"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="20" t="str">
+        <x:v>序号</x:v>
+      </x:c>
+      <x:c r="B48" s="20" t="str">
+        <x:v>周期</x:v>
+      </x:c>
+      <x:c r="C48" s="20" t="str">
+        <x:v>开盘</x:v>
+      </x:c>
+      <x:c r="D48" s="20" t="str">
+        <x:v>高点</x:v>
+      </x:c>
+      <x:c r="E48" s="20" t="str">
+        <x:v>低点</x:v>
+      </x:c>
+      <x:c r="F48" s="20" t="str">
+        <x:v>收盘</x:v>
+      </x:c>
+      <x:c r="G48" s="20" t="str">
+        <x:v>涨跌点数</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="str">
+        <x:v>涨幅</x:v>
+      </x:c>
+      <x:c r="I48" s="20" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="J48" s="20" t="str">
+        <x:v>标的</x:v>
+      </x:c>
+      <x:c r="K48" s="20" t="str">
+        <x:v>交易日</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B49" s="22" t="str">
+        <x:v>10月8日-10月9日</x:v>
+      </x:c>
+      <x:c r="C49" s="23" t="n">
+        <x:v>4300.8</x:v>
+      </x:c>
+      <x:c r="D49" s="23" t="n">
+        <x:v>4331.6</x:v>
+      </x:c>
+      <x:c r="E49" s="23" t="n">
+        <x:v>4180.4</x:v>
+      </x:c>
+      <x:c r="F49" s="23" t="n">
+        <x:v>4244.8</x:v>
+      </x:c>
+      <x:c r="G49" s="23"/>
+      <x:c r="H49" s="24"/>
+      <x:c r="I49" s="26" t="n">
+        <x:f>ROUND(D49-E49,1)</x:f>
+        <x:v>151.2</x:v>
+      </x:c>
+      <x:c r="J49" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K49" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B50" s="22" t="str">
+        <x:v>10月12日-10月16日</x:v>
+      </x:c>
+      <x:c r="C50" s="23" t="n">
+        <x:v>4240.4</x:v>
+      </x:c>
+      <x:c r="D50" s="23" t="n">
+        <x:v>4273.6</x:v>
+      </x:c>
+      <x:c r="E50" s="23" t="n">
+        <x:v>4045.2</x:v>
+      </x:c>
+      <x:c r="F50" s="23" t="n">
+        <x:v>4088.8</x:v>
+      </x:c>
+      <x:c r="G50" s="28" t="n">
+        <x:f>ROUND(F50-F49,1)</x:f>
+        <x:v>-156</x:v>
+      </x:c>
+      <x:c r="H50" s="24" t="n">
+        <x:f>IFERROR(F50/F49-1,"")</x:f>
+        <x:v>-0.03675084809649454</x:v>
+      </x:c>
+      <x:c r="I50" s="26" t="n">
+        <x:f>ROUND(D50-E50,1)</x:f>
+        <x:v>228.4</x:v>
+      </x:c>
+      <x:c r="J50" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K50" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="30"/>
-      <x:c r="E32" s="30"/>
-      <x:c r="F32" s="30"/>
-      <x:c r="G32" s="30"/>
-      <x:c r="H32" s="30"/>
-      <x:c r="I32" s="32" t="n">
-        <x:f>ROUND(SUM(I29:I31),1)</x:f>
-        <x:v>1531.2</x:v>
-      </x:c>
-      <x:c r="J32" s="30"/>
-      <x:c r="K32" s="30"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="31" t="str">
+      <x:c r="B51" s="22" t="str">
+        <x:v>10月19日-10月23日</x:v>
+      </x:c>
+      <x:c r="C51" s="23" t="n">
+        <x:v>4086.4</x:v>
+      </x:c>
+      <x:c r="D51" s="23" t="n">
+        <x:v>4140.2</x:v>
+      </x:c>
+      <x:c r="E51" s="23" t="n">
+        <x:v>3897.6</x:v>
+      </x:c>
+      <x:c r="F51" s="23" t="n">
+        <x:v>4055</x:v>
+      </x:c>
+      <x:c r="G51" s="23" t="n">
+        <x:f>ROUND(F51-F50,1)</x:f>
+        <x:v>-33.8</x:v>
+      </x:c>
+      <x:c r="H51" s="24" t="n">
+        <x:f>IFERROR(F51/F50-1,"")</x:f>
+        <x:v>-0.00826648405400121</x:v>
+      </x:c>
+      <x:c r="I51" s="26" t="n">
+        <x:f>ROUND(D51-E51,1)</x:f>
+        <x:v>242.6</x:v>
+      </x:c>
+      <x:c r="J51" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K51" s="22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B52" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="C52" s="23" t="n">
+        <x:v>4034</x:v>
+      </x:c>
+      <x:c r="D52" s="23" t="n">
+        <x:v>4049.8</x:v>
+      </x:c>
+      <x:c r="E52" s="23" t="n">
+        <x:v>3996.4</x:v>
+      </x:c>
+      <x:c r="F52" s="23" t="n">
+        <x:v>4049</x:v>
+      </x:c>
+      <x:c r="G52" s="23" t="n">
+        <x:f>ROUND(F52-F51,1)</x:f>
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="H52" s="24" t="n">
+        <x:f>IFERROR(F52/F51-1,"")</x:f>
+        <x:v>-0.0014796547472256671</x:v>
+      </x:c>
+      <x:c r="I52" s="23" t="n">
+        <x:f>ROUND(D52-E52,1)</x:f>
+        <x:v>53.4</x:v>
+      </x:c>
+      <x:c r="J52" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
+      <x:c r="K52" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="31" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B53" s="30" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C53" s="30"/>
+      <x:c r="D53" s="30"/>
+      <x:c r="E53" s="30"/>
+      <x:c r="F53" s="30"/>
+      <x:c r="G53" s="30"/>
+      <x:c r="H53" s="30"/>
+      <x:c r="I53" s="32" t="n">
+        <x:f>ROUND(SUM(I49:I52),1)</x:f>
+        <x:v>675.6</x:v>
+      </x:c>
+      <x:c r="J53" s="30"/>
+      <x:c r="K53" s="30"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B33" s="30"/>
-      <x:c r="C33" s="30"/>
-      <x:c r="D33" s="30"/>
-      <x:c r="E33" s="30"/>
-      <x:c r="F33" s="30"/>
-      <x:c r="G33" s="30"/>
-      <x:c r="H33" s="30"/>
-      <x:c r="I33" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I29:I31),0),1)</x:f>
-        <x:v>510.4</x:v>
-      </x:c>
-      <x:c r="J33" s="30"/>
-      <x:c r="K33" s="30"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="17" t="str">
-        <x:v>IC主力</x:v>
-      </x:c>
-      <x:c r="B35" s="17"/>
-      <x:c r="C35" s="17"/>
-      <x:c r="D35" s="17"/>
-      <x:c r="E35" s="17"/>
-      <x:c r="F35" s="17"/>
-      <x:c r="G35" s="17"/>
-      <x:c r="H35" s="17"/>
-      <x:c r="I35" s="17"/>
-      <x:c r="J35" s="17"/>
-      <x:c r="K35" s="17"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="20" t="str">
+      <x:c r="B54" s="30"/>
+      <x:c r="C54" s="30"/>
+      <x:c r="D54" s="30"/>
+      <x:c r="E54" s="30"/>
+      <x:c r="F54" s="30"/>
+      <x:c r="G54" s="30"/>
+      <x:c r="H54" s="30"/>
+      <x:c r="I54" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I49:I52),0),1)</x:f>
+        <x:v>168.9</x:v>
+      </x:c>
+      <x:c r="J54" s="30"/>
+      <x:c r="K54" s="30"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="17" t="str">
+        <x:v>IH主力</x:v>
+      </x:c>
+      <x:c r="B56" s="17"/>
+      <x:c r="C56" s="17"/>
+      <x:c r="D56" s="17"/>
+      <x:c r="E56" s="17"/>
+      <x:c r="F56" s="17"/>
+      <x:c r="G56" s="17"/>
+      <x:c r="H56" s="17"/>
+      <x:c r="I56" s="17"/>
+      <x:c r="J56" s="17"/>
+      <x:c r="K56" s="17"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B36" s="20" t="str">
+      <x:c r="B57" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C36" s="20" t="str">
+      <x:c r="C57" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D36" s="20" t="str">
+      <x:c r="D57" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E36" s="20" t="str">
+      <x:c r="E57" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F36" s="20" t="str">
+      <x:c r="F57" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G36" s="20" t="str">
+      <x:c r="G57" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H36" s="20" t="str">
+      <x:c r="H57" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I36" s="20" t="str">
+      <x:c r="I57" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J36" s="20" t="str">
+      <x:c r="J57" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K36" s="20" t="str">
+      <x:c r="K57" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="22" t="n">
+    <x:row r="58">
+      <x:c r="A58" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B37" s="22" t="str">
+      <x:c r="B58" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C37" s="23" t="n">
-        <x:v>7295</x:v>
-      </x:c>
-      <x:c r="D37" s="23" t="n">
-        <x:v>7355</x:v>
-      </x:c>
-      <x:c r="E37" s="23" t="n">
-        <x:v>6932</x:v>
-      </x:c>
-      <x:c r="F37" s="23" t="n">
-        <x:v>7111</x:v>
-      </x:c>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="24"/>
-      <x:c r="I37" s="26" t="n">
-        <x:f>ROUND(D37-E37,1)</x:f>
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="J37" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K37" s="22" t="n">
+      <x:c r="C58" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="n">
+        <x:v>2798.4</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="n">
+        <x:v>2735</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="n">
+        <x:v>2764</x:v>
+      </x:c>
+      <x:c r="G58" s="23"/>
+      <x:c r="H58" s="24"/>
+      <x:c r="I58" s="26" t="n">
+        <x:f>ROUND(D58-E58,1)</x:f>
+        <x:v>63.4</x:v>
+      </x:c>
+      <x:c r="J58" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K58" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="22" t="n">
+    <x:row r="59">
+      <x:c r="A59" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B38" s="22" t="str">
+      <x:c r="B59" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C38" s="23" t="n">
-        <x:v>7076.6</x:v>
-      </x:c>
-      <x:c r="D38" s="23" t="n">
-        <x:v>7115.6</x:v>
-      </x:c>
-      <x:c r="E38" s="23" t="n">
-        <x:v>6583.2</x:v>
-      </x:c>
-      <x:c r="F38" s="23" t="n">
-        <x:v>6667.8</x:v>
-      </x:c>
-      <x:c r="G38" s="28" t="n">
-        <x:f>ROUND(F38-F37,1)</x:f>
-        <x:v>-443.2</x:v>
-      </x:c>
-      <x:c r="H38" s="24" t="n">
-        <x:f>IFERROR(F38/F37-1,"")</x:f>
-        <x:v>-0.062325973843341265</x:v>
-      </x:c>
-      <x:c r="I38" s="26" t="n">
-        <x:f>ROUND(D38-E38,1)</x:f>
-        <x:v>532.4</x:v>
-      </x:c>
-      <x:c r="J38" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K38" s="22" t="n">
+      <x:c r="C59" s="23" t="n">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="D59" s="23" t="n">
+        <x:v>2794</x:v>
+      </x:c>
+      <x:c r="E59" s="23" t="n">
+        <x:v>2677.6</x:v>
+      </x:c>
+      <x:c r="F59" s="23" t="n">
+        <x:v>2704.6</x:v>
+      </x:c>
+      <x:c r="G59" s="23" t="n">
+        <x:f>ROUND(F59-F58,1)</x:f>
+        <x:v>-59.4</x:v>
+      </x:c>
+      <x:c r="H59" s="24" t="n">
+        <x:f>IFERROR(F59/F58-1,"")</x:f>
+        <x:v>-0.0214905933429812</x:v>
+      </x:c>
+      <x:c r="I59" s="26" t="n">
+        <x:f>ROUND(D59-E59,1)</x:f>
+        <x:v>116.4</x:v>
+      </x:c>
+      <x:c r="J59" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K59" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="22" t="n">
+    <x:row r="60">
+      <x:c r="A60" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B39" s="22" t="str">
+      <x:c r="B60" s="22" t="str">
         <x:v>10月19日-10月23日</x:v>
       </x:c>
-      <x:c r="C39" s="23" t="n">
-        <x:v>6670.2</x:v>
-      </x:c>
-      <x:c r="D39" s="23" t="n">
-        <x:v>6864</x:v>
-      </x:c>
-      <x:c r="E39" s="23" t="n">
-        <x:v>6340</x:v>
-      </x:c>
-      <x:c r="F39" s="23" t="n">
-        <x:v>6742</x:v>
-      </x:c>
-      <x:c r="G39" s="23" t="n">
-        <x:f>ROUND(F39-F38,1)</x:f>
-        <x:v>74.2</x:v>
-      </x:c>
-      <x:c r="H39" s="24" t="n">
-        <x:f>IFERROR(F39/F38-1,"")</x:f>
-        <x:v>0.011128108221602373</x:v>
-      </x:c>
-      <x:c r="I39" s="26" t="n">
-        <x:f>ROUND(D39-E39,1)</x:f>
-        <x:v>524</x:v>
-      </x:c>
-      <x:c r="J39" s="22" t="str">
-        <x:v>IC2612</x:v>
-      </x:c>
-      <x:c r="K39" s="22" t="n">
+      <x:c r="C60" s="23" t="n">
+        <x:v>2690</x:v>
+      </x:c>
+      <x:c r="D60" s="23" t="n">
+        <x:v>2754.6</x:v>
+      </x:c>
+      <x:c r="E60" s="23" t="n">
+        <x:v>2638</x:v>
+      </x:c>
+      <x:c r="F60" s="23" t="n">
+        <x:v>2719</x:v>
+      </x:c>
+      <x:c r="G60" s="23" t="n">
+        <x:f>ROUND(F60-F59,1)</x:f>
+        <x:v>14.4</x:v>
+      </x:c>
+      <x:c r="H60" s="24" t="n">
+        <x:f>IFERROR(F60/F59-1,"")</x:f>
+        <x:v>0.0053242623678178</x:v>
+      </x:c>
+      <x:c r="I60" s="26" t="n">
+        <x:f>ROUND(D60-E60,1)</x:f>
+        <x:v>116.6</x:v>
+      </x:c>
+      <x:c r="J60" s="22" t="str">
+        <x:v>IH2612</x:v>
+      </x:c>
+      <x:c r="K60" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="31" t="str">
+    <x:row r="61">
+      <x:c r="A61" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B40" s="30" t="n">
+      <x:c r="B61" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="30"/>
-      <x:c r="H40" s="30"/>
-      <x:c r="I40" s="32" t="n">
-        <x:f>ROUND(SUM(I37:I39),1)</x:f>
-        <x:v>1479.4</x:v>
-      </x:c>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="30"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="31" t="str">
+      <x:c r="C61" s="30"/>
+      <x:c r="D61" s="30"/>
+      <x:c r="E61" s="30"/>
+      <x:c r="F61" s="30"/>
+      <x:c r="G61" s="30"/>
+      <x:c r="H61" s="30"/>
+      <x:c r="I61" s="32" t="n">
+        <x:f>ROUND(SUM(I58:I60),1)</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="J61" s="30"/>
+      <x:c r="K61" s="30"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="30"/>
-      <x:c r="H41" s="30"/>
-      <x:c r="I41" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I37:I39),0),1)</x:f>
-        <x:v>493.1</x:v>
-      </x:c>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="30"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="17" t="str">
-        <x:v>IF主力</x:v>
-      </x:c>
-      <x:c r="B43" s="17"/>
-      <x:c r="C43" s="17"/>
-      <x:c r="D43" s="17"/>
-      <x:c r="E43" s="17"/>
-      <x:c r="F43" s="17"/>
-      <x:c r="G43" s="17"/>
-      <x:c r="H43" s="17"/>
-      <x:c r="I43" s="17"/>
-      <x:c r="J43" s="17"/>
-      <x:c r="K43" s="17"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="20" t="str">
+      <x:c r="B62" s="30"/>
+      <x:c r="C62" s="30"/>
+      <x:c r="D62" s="30"/>
+      <x:c r="E62" s="30"/>
+      <x:c r="F62" s="30"/>
+      <x:c r="G62" s="30"/>
+      <x:c r="H62" s="30"/>
+      <x:c r="I62" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I58:I60),0),1)</x:f>
+        <x:v>98.8</x:v>
+      </x:c>
+      <x:c r="J62" s="30"/>
+      <x:c r="K62" s="30"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="17" t="str">
+        <x:v>碳酸锂2610</x:v>
+      </x:c>
+      <x:c r="B64" s="17"/>
+      <x:c r="C64" s="17"/>
+      <x:c r="D64" s="17"/>
+      <x:c r="E64" s="17"/>
+      <x:c r="F64" s="17"/>
+      <x:c r="G64" s="17"/>
+      <x:c r="H64" s="17"/>
+      <x:c r="I64" s="17"/>
+      <x:c r="J64" s="17"/>
+      <x:c r="K64" s="17"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="20" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B44" s="20" t="str">
+      <x:c r="B65" s="20" t="str">
         <x:v>周期</x:v>
       </x:c>
-      <x:c r="C44" s="20" t="str">
+      <x:c r="C65" s="20" t="str">
         <x:v>开盘</x:v>
       </x:c>
-      <x:c r="D44" s="20" t="str">
+      <x:c r="D65" s="20" t="str">
         <x:v>高点</x:v>
       </x:c>
-      <x:c r="E44" s="20" t="str">
+      <x:c r="E65" s="20" t="str">
         <x:v>低点</x:v>
       </x:c>
-      <x:c r="F44" s="20" t="str">
+      <x:c r="F65" s="20" t="str">
         <x:v>收盘</x:v>
       </x:c>
-      <x:c r="G44" s="20" t="str">
+      <x:c r="G65" s="20" t="str">
         <x:v>涨跌点数</x:v>
       </x:c>
-      <x:c r="H44" s="20" t="str">
+      <x:c r="H65" s="20" t="str">
         <x:v>涨幅</x:v>
       </x:c>
-      <x:c r="I44" s="20" t="str">
+      <x:c r="I65" s="20" t="str">
         <x:v>振幅</x:v>
       </x:c>
-      <x:c r="J44" s="20" t="str">
+      <x:c r="J65" s="20" t="str">
         <x:v>标的</x:v>
       </x:c>
-      <x:c r="K44" s="20" t="str">
+      <x:c r="K65" s="20" t="str">
         <x:v>交易日</x:v>
       </x:c>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="22" t="n">
+    <x:row r="66">
+      <x:c r="A66" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B45" s="22" t="str">
+      <x:c r="B66" s="22" t="str">
         <x:v>10月8日-10月9日</x:v>
       </x:c>
-      <x:c r="C45" s="23" t="n">
-        <x:v>4300.8</x:v>
-      </x:c>
-      <x:c r="D45" s="23" t="n">
-        <x:v>4331.6</x:v>
-      </x:c>
-      <x:c r="E45" s="23" t="n">
-        <x:v>4180.4</x:v>
-      </x:c>
-      <x:c r="F45" s="23" t="n">
-        <x:v>4244.8</x:v>
-      </x:c>
-      <x:c r="G45" s="23"/>
-      <x:c r="H45" s="24"/>
-      <x:c r="I45" s="26" t="n">
-        <x:f>ROUND(D45-E45,1)</x:f>
-        <x:v>151.2</x:v>
-      </x:c>
-      <x:c r="J45" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K45" s="22" t="n">
+      <x:c r="C66" s="23" t="n">
+        <x:v>120020</x:v>
+      </x:c>
+      <x:c r="D66" s="23" t="n">
+        <x:v>126800</x:v>
+      </x:c>
+      <x:c r="E66" s="23" t="n">
+        <x:v>119000</x:v>
+      </x:c>
+      <x:c r="F66" s="23" t="n">
+        <x:v>121000</x:v>
+      </x:c>
+      <x:c r="G66" s="23"/>
+      <x:c r="H66" s="24"/>
+      <x:c r="I66" s="26" t="n">
+        <x:f>ROUND(D66-E66,1)</x:f>
+        <x:v>7800</x:v>
+      </x:c>
+      <x:c r="J66" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K66" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="22" t="n">
+    <x:row r="67">
+      <x:c r="A67" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B46" s="22" t="str">
+      <x:c r="B67" s="22" t="str">
         <x:v>10月12日-10月16日</x:v>
       </x:c>
-      <x:c r="C46" s="23" t="n">
-        <x:v>4240.4</x:v>
-      </x:c>
-      <x:c r="D46" s="23" t="n">
-        <x:v>4273.6</x:v>
-      </x:c>
-      <x:c r="E46" s="23" t="n">
-        <x:v>4045.2</x:v>
-      </x:c>
-      <x:c r="F46" s="23" t="n">
-        <x:v>4088.8</x:v>
-      </x:c>
-      <x:c r="G46" s="28" t="n">
-        <x:f>ROUND(F46-F45,1)</x:f>
-        <x:v>-156</x:v>
-      </x:c>
-      <x:c r="H46" s="24" t="n">
-        <x:f>IFERROR(F46/F45-1,"")</x:f>
-        <x:v>-0.03675084809649454</x:v>
-      </x:c>
-      <x:c r="I46" s="26" t="n">
-        <x:f>ROUND(D46-E46,1)</x:f>
-        <x:v>228.4</x:v>
-      </x:c>
-      <x:c r="J46" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K46" s="22" t="n">
+      <x:c r="C67" s="23" t="n">
+        <x:v>125960</x:v>
+      </x:c>
+      <x:c r="D67" s="23" t="n">
+        <x:v>125960</x:v>
+      </x:c>
+      <x:c r="E67" s="23" t="n">
+        <x:v>99500</x:v>
+      </x:c>
+      <x:c r="F67" s="23" t="n">
+        <x:v>99500</x:v>
+      </x:c>
+      <x:c r="G67" s="28" t="n">
+        <x:f>ROUND(F67-F66,1)</x:f>
+        <x:v>-21500</x:v>
+      </x:c>
+      <x:c r="H67" s="24" t="n">
+        <x:f>IFERROR(F67/F66-1,"")</x:f>
+        <x:v>-0.1776859504132231</x:v>
+      </x:c>
+      <x:c r="I67" s="26" t="n">
+        <x:f>ROUND(D67-E67,1)</x:f>
+        <x:v>26460</x:v>
+      </x:c>
+      <x:c r="J67" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K67" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="22" t="n">
+    <x:row r="68">
+      <x:c r="A68" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>10月19日-10月23日</x:v>
-      </x:c>
-      <x:c r="C47" s="23" t="n">
-        <x:v>4086.4</x:v>
-      </x:c>
-      <x:c r="D47" s="23" t="n">
-        <x:v>4140.2</x:v>
-      </x:c>
-      <x:c r="E47" s="23" t="n">
-        <x:v>3897.6</x:v>
-      </x:c>
-      <x:c r="F47" s="23" t="n">
-        <x:v>4055</x:v>
-      </x:c>
-      <x:c r="G47" s="23" t="n">
-        <x:f>ROUND(F47-F46,1)</x:f>
-        <x:v>-33.8</x:v>
-      </x:c>
-      <x:c r="H47" s="24" t="n">
-        <x:f>IFERROR(F47/F46-1,"")</x:f>
-        <x:v>-0.00826648405400121</x:v>
-      </x:c>
-      <x:c r="I47" s="26" t="n">
-        <x:f>ROUND(D47-E47,1)</x:f>
-        <x:v>242.6</x:v>
-      </x:c>
-      <x:c r="J47" s="22" t="str">
-        <x:v>IF2612</x:v>
-      </x:c>
-      <x:c r="K47" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="31" t="str">
+      <x:c r="B68" s="22" t="str">
+        <x:v>10月19日-10月21日</x:v>
+      </x:c>
+      <x:c r="C68" s="23" t="n">
+        <x:v>99600</x:v>
+      </x:c>
+      <x:c r="D68" s="23" t="n">
+        <x:v>103420</x:v>
+      </x:c>
+      <x:c r="E68" s="23" t="n">
+        <x:v>98000</x:v>
+      </x:c>
+      <x:c r="F68" s="23" t="n">
+        <x:v>98540</x:v>
+      </x:c>
+      <x:c r="G68" s="28" t="n">
+        <x:f>ROUND(F68-F67,1)</x:f>
+        <x:v>-960</x:v>
+      </x:c>
+      <x:c r="H68" s="24" t="n">
+        <x:f>IFERROR(F68/F67-1,"")</x:f>
+        <x:v>-0.00964824120603014</x:v>
+      </x:c>
+      <x:c r="I68" s="23" t="n">
+        <x:f>ROUND(D68-E68,1)</x:f>
+        <x:v>5420</x:v>
+      </x:c>
+      <x:c r="J68" s="22" t="str">
+        <x:v>LC2610</x:v>
+      </x:c>
+      <x:c r="K68" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="31" t="str">
         <x:v>合计</x:v>
       </x:c>
-      <x:c r="B48" s="30" t="n">
+      <x:c r="B69" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C48" s="30"/>
-      <x:c r="D48" s="30"/>
-      <x:c r="E48" s="30"/>
-      <x:c r="F48" s="30"/>
-      <x:c r="G48" s="30"/>
-      <x:c r="H48" s="30"/>
-      <x:c r="I48" s="32" t="n">
-        <x:f>ROUND(SUM(I45:I47),1)</x:f>
-        <x:v>622.2</x:v>
-      </x:c>
-      <x:c r="J48" s="30"/>
-      <x:c r="K48" s="30"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="31" t="str">
+      <x:c r="C69" s="30"/>
+      <x:c r="D69" s="30"/>
+      <x:c r="E69" s="30"/>
+      <x:c r="F69" s="30"/>
+      <x:c r="G69" s="30"/>
+      <x:c r="H69" s="30"/>
+      <x:c r="I69" s="32" t="n">
+        <x:f>ROUND(SUM(I66:I68),1)</x:f>
+        <x:v>39680</x:v>
+      </x:c>
+      <x:c r="J69" s="30"/>
+      <x:c r="K69" s="30"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="31" t="str">
         <x:v>均值</x:v>
       </x:c>
-      <x:c r="B49" s="30"/>
-      <x:c r="C49" s="30"/>
-      <x:c r="D49" s="30"/>
-      <x:c r="E49" s="30"/>
-      <x:c r="F49" s="30"/>
-      <x:c r="G49" s="30"/>
-      <x:c r="H49" s="30"/>
-      <x:c r="I49" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I45:I47),0),1)</x:f>
-        <x:v>207.4</x:v>
-      </x:c>
-      <x:c r="J49" s="30"/>
-      <x:c r="K49" s="30"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="17" t="str">
-        <x:v>IH主力</x:v>
-      </x:c>
-      <x:c r="B51" s="17"/>
-      <x:c r="C51" s="17"/>
-      <x:c r="D51" s="17"/>
-      <x:c r="E51" s="17"/>
-      <x:c r="F51" s="17"/>
-      <x:c r="G51" s="17"/>
-      <x:c r="H51" s="17"/>
-      <x:c r="I51" s="17"/>
-      <x:c r="J51" s="17"/>
-      <x:c r="K51" s="17"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B52" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C52" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D52" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E52" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F52" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G52" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H52" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I52" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J52" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K52" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B53" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C53" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="D53" s="23" t="n">
-        <x:v>2798.4</x:v>
-      </x:c>
-      <x:c r="E53" s="23" t="n">
-        <x:v>2735</x:v>
-      </x:c>
-      <x:c r="F53" s="23" t="n">
-        <x:v>2764</x:v>
-      </x:c>
-      <x:c r="G53" s="23"/>
-      <x:c r="H53" s="24"/>
-      <x:c r="I53" s="26" t="n">
-        <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>63.4</x:v>
-      </x:c>
-      <x:c r="J53" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K53" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B54" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
-      </x:c>
-      <x:c r="C54" s="23" t="n">
-        <x:v>2762</x:v>
-      </x:c>
-      <x:c r="D54" s="23" t="n">
-        <x:v>2794</x:v>
-      </x:c>
-      <x:c r="E54" s="23" t="n">
-        <x:v>2677.6</x:v>
-      </x:c>
-      <x:c r="F54" s="23" t="n">
-        <x:v>2704.6</x:v>
-      </x:c>
-      <x:c r="G54" s="23" t="n">
-        <x:f>ROUND(F54-F53,1)</x:f>
-        <x:v>-59.4</x:v>
-      </x:c>
-      <x:c r="H54" s="24" t="n">
-        <x:f>IFERROR(F54/F53-1,"")</x:f>
-        <x:v>-0.0214905933429812</x:v>
-      </x:c>
-      <x:c r="I54" s="26" t="n">
-        <x:f>ROUND(D54-E54,1)</x:f>
-        <x:v>116.4</x:v>
-      </x:c>
-      <x:c r="J54" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K54" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>10月19日-10月23日</x:v>
-      </x:c>
-      <x:c r="C55" s="23" t="n">
-        <x:v>2690</x:v>
-      </x:c>
-      <x:c r="D55" s="23" t="n">
-        <x:v>2754.6</x:v>
-      </x:c>
-      <x:c r="E55" s="23" t="n">
-        <x:v>2638</x:v>
-      </x:c>
-      <x:c r="F55" s="23" t="n">
-        <x:v>2719</x:v>
-      </x:c>
-      <x:c r="G55" s="23" t="n">
-        <x:f>ROUND(F55-F54,1)</x:f>
-        <x:v>14.4</x:v>
-      </x:c>
-      <x:c r="H55" s="24" t="n">
-        <x:f>IFERROR(F55/F54-1,"")</x:f>
-        <x:v>0.0053242623678178</x:v>
-      </x:c>
-      <x:c r="I55" s="26" t="n">
-        <x:f>ROUND(D55-E55,1)</x:f>
-        <x:v>116.6</x:v>
-      </x:c>
-      <x:c r="J55" s="22" t="str">
-        <x:v>IH2612</x:v>
-      </x:c>
-      <x:c r="K55" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B56" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C56" s="30"/>
-      <x:c r="D56" s="30"/>
-      <x:c r="E56" s="30"/>
-      <x:c r="F56" s="30"/>
-      <x:c r="G56" s="30"/>
-      <x:c r="H56" s="30"/>
-      <x:c r="I56" s="32" t="n">
-        <x:f>ROUND(SUM(I53:I55),1)</x:f>
-        <x:v>296.4</x:v>
-      </x:c>
-      <x:c r="J56" s="30"/>
-      <x:c r="K56" s="30"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B57" s="30"/>
-      <x:c r="C57" s="30"/>
-      <x:c r="D57" s="30"/>
-      <x:c r="E57" s="30"/>
-      <x:c r="F57" s="30"/>
-      <x:c r="G57" s="30"/>
-      <x:c r="H57" s="30"/>
-      <x:c r="I57" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I53:I55),0),1)</x:f>
-        <x:v>98.8</x:v>
-      </x:c>
-      <x:c r="J57" s="30"/>
-      <x:c r="K57" s="30"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="17" t="str">
-        <x:v>碳酸锂2610</x:v>
-      </x:c>
-      <x:c r="B59" s="17"/>
-      <x:c r="C59" s="17"/>
-      <x:c r="D59" s="17"/>
-      <x:c r="E59" s="17"/>
-      <x:c r="F59" s="17"/>
-      <x:c r="G59" s="17"/>
-      <x:c r="H59" s="17"/>
-      <x:c r="I59" s="17"/>
-      <x:c r="J59" s="17"/>
-      <x:c r="K59" s="17"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="20" t="str">
-        <x:v>序号</x:v>
-      </x:c>
-      <x:c r="B60" s="20" t="str">
-        <x:v>周期</x:v>
-      </x:c>
-      <x:c r="C60" s="20" t="str">
-        <x:v>开盘</x:v>
-      </x:c>
-      <x:c r="D60" s="20" t="str">
-        <x:v>高点</x:v>
-      </x:c>
-      <x:c r="E60" s="20" t="str">
-        <x:v>低点</x:v>
-      </x:c>
-      <x:c r="F60" s="20" t="str">
-        <x:v>收盘</x:v>
-      </x:c>
-      <x:c r="G60" s="20" t="str">
-        <x:v>涨跌点数</x:v>
-      </x:c>
-      <x:c r="H60" s="20" t="str">
-        <x:v>涨幅</x:v>
-      </x:c>
-      <x:c r="I60" s="20" t="str">
-        <x:v>振幅</x:v>
-      </x:c>
-      <x:c r="J60" s="20" t="str">
-        <x:v>标的</x:v>
-      </x:c>
-      <x:c r="K60" s="20" t="str">
-        <x:v>交易日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="22" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B61" s="22" t="str">
-        <x:v>10月8日-10月9日</x:v>
-      </x:c>
-      <x:c r="C61" s="23" t="n">
-        <x:v>120020</x:v>
-      </x:c>
-      <x:c r="D61" s="23" t="n">
-        <x:v>126800</x:v>
-      </x:c>
-      <x:c r="E61" s="23" t="n">
-        <x:v>119000</x:v>
-      </x:c>
-      <x:c r="F61" s="23" t="n">
-        <x:v>121000</x:v>
-      </x:c>
-      <x:c r="G61" s="23"/>
-      <x:c r="H61" s="24"/>
-      <x:c r="I61" s="26" t="n">
-        <x:f>ROUND(D61-E61,1)</x:f>
-        <x:v>7800</x:v>
-      </x:c>
-      <x:c r="J61" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K61" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="22" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B62" s="22" t="str">
-        <x:v>10月12日-10月16日</x:v>
-      </x:c>
-      <x:c r="C62" s="23" t="n">
-        <x:v>125960</x:v>
-      </x:c>
-      <x:c r="D62" s="23" t="n">
-        <x:v>125960</x:v>
-      </x:c>
-      <x:c r="E62" s="23" t="n">
-        <x:v>99500</x:v>
-      </x:c>
-      <x:c r="F62" s="23" t="n">
-        <x:v>99500</x:v>
-      </x:c>
-      <x:c r="G62" s="28" t="n">
-        <x:f>ROUND(F62-F61,1)</x:f>
-        <x:v>-21500</x:v>
-      </x:c>
-      <x:c r="H62" s="24" t="n">
-        <x:f>IFERROR(F62/F61-1,"")</x:f>
-        <x:v>-0.1776859504132231</x:v>
-      </x:c>
-      <x:c r="I62" s="26" t="n">
-        <x:f>ROUND(D62-E62,1)</x:f>
-        <x:v>26460</x:v>
-      </x:c>
-      <x:c r="J62" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K62" s="22" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B63" s="22" t="str">
-        <x:v>10月19日-10月21日</x:v>
-      </x:c>
-      <x:c r="C63" s="23" t="n">
-        <x:v>99600</x:v>
-      </x:c>
-      <x:c r="D63" s="23" t="n">
-        <x:v>103420</x:v>
-      </x:c>
-      <x:c r="E63" s="23" t="n">
-        <x:v>98000</x:v>
-      </x:c>
-      <x:c r="F63" s="23" t="n">
-        <x:v>98540</x:v>
-      </x:c>
-      <x:c r="G63" s="28" t="n">
-        <x:f>ROUND(F63-F62,1)</x:f>
-        <x:v>-960</x:v>
-      </x:c>
-      <x:c r="H63" s="24" t="n">
-        <x:f>IFERROR(F63/F62-1,"")</x:f>
-        <x:v>-0.00964824120603014</x:v>
-      </x:c>
-      <x:c r="I63" s="23" t="n">
-        <x:f>ROUND(D63-E63,1)</x:f>
-        <x:v>5420</x:v>
-      </x:c>
-      <x:c r="J63" s="22" t="str">
-        <x:v>LC2610</x:v>
-      </x:c>
-      <x:c r="K63" s="22" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B64" s="30" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C64" s="30"/>
-      <x:c r="D64" s="30"/>
-      <x:c r="E64" s="30"/>
-      <x:c r="F64" s="30"/>
-      <x:c r="G64" s="30"/>
-      <x:c r="H64" s="30"/>
-      <x:c r="I64" s="32" t="n">
-        <x:f>ROUND(SUM(I61:I63),1)</x:f>
-        <x:v>39680</x:v>
-      </x:c>
-      <x:c r="J64" s="30"/>
-      <x:c r="K64" s="30"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B65" s="30"/>
-      <x:c r="C65" s="30"/>
-      <x:c r="D65" s="30"/>
-      <x:c r="E65" s="30"/>
-      <x:c r="F65" s="30"/>
-      <x:c r="G65" s="30"/>
-      <x:c r="H65" s="30"/>
-      <x:c r="I65" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(I61:I63),0),1)</x:f>
+      <x:c r="B70" s="30"/>
+      <x:c r="C70" s="30"/>
+      <x:c r="D70" s="30"/>
+      <x:c r="E70" s="30"/>
+      <x:c r="F70" s="30"/>
+      <x:c r="G70" s="30"/>
+      <x:c r="H70" s="30"/>
+      <x:c r="I70" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(I66:I68),0),1)</x:f>
         <x:v>13226.7</x:v>
       </x:c>
-      <x:c r="J65" s="30"/>
-      <x:c r="K65" s="30"/>
+      <x:c r="J70" s="30"/>
+      <x:c r="K70" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A3:K3"/>
-    <x:mergeCell ref="A11:K11"/>
-    <x:mergeCell ref="A19:K19"/>
-    <x:mergeCell ref="A27:K27"/>
-    <x:mergeCell ref="A35:K35"/>
-    <x:mergeCell ref="A43:K43"/>
-    <x:mergeCell ref="A51:K51"/>
-    <x:mergeCell ref="A59:K59"/>
+    <x:mergeCell ref="A12:K12"/>
+    <x:mergeCell ref="A21:K21"/>
+    <x:mergeCell ref="A30:K30"/>
+    <x:mergeCell ref="A38:K38"/>
+    <x:mergeCell ref="A47:K47"/>
+    <x:mergeCell ref="A56:K56"/>
+    <x:mergeCell ref="A64:K64"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3439,31 +3629,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>2570.7999999999997</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>6684.93</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>6704.68</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>6589.13</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>6630.78</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-103.8</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.015408601911040876</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>115.6</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -3471,11 +3679,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>214.2</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2686.3999999999996</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>206.6</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3974,31 +4200,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>2384.6</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>6756.46</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>6787.32</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>6674.4</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>6712.73</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-101.7</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.0149256578677045</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>112.9</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -4006,11 +4250,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>198.7</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2497.5</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>192.1</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4509,31 +4771,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>737</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>3671</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>3699.01</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>3664.82</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>3697.52</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>0.0019076109340789849</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>34.2</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -4541,11 +4821,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>61.4</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>771.2</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>59.3</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5579,31 +5877,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>2630.6</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>6700</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>6711.4</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>6573.6</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>6637</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-105</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.015574013645802465</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>137.8</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -5611,11 +5927,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>219.2</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>2768.4</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6114,31 +6448,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B18" s="30" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C18" s="30"/>
-      <x:c r="D18" s="30"/>
-      <x:c r="E18" s="30"/>
-      <x:c r="F18" s="30"/>
-      <x:c r="G18" s="30"/>
-      <x:c r="H18" s="30"/>
-      <x:c r="I18" s="30"/>
-      <x:c r="J18" s="32" t="n">
-        <x:f>SUM(J4:J15)</x:f>
-        <x:v>1070.6000000000001</x:v>
-      </x:c>
-      <x:c r="K18" s="30"/>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>10月26日</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="n">
+        <x:v>4034</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="n">
+        <x:v>4049.8</x:v>
+      </x:c>
+      <x:c r="F16" s="23" t="n">
+        <x:v>3996.4</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="n">
+        <x:v>4049</x:v>
+      </x:c>
+      <x:c r="H16" s="23" t="n">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="n">
+        <x:v>-0.0014796547472256671</x:v>
+      </x:c>
+      <x:c r="J16" s="23" t="n">
+        <x:f>ROUND(E16-F16,1)</x:f>
+        <x:v>53.4</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B19" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="C19" s="30"/>
       <x:c r="D19" s="30"/>
       <x:c r="E19" s="30"/>
@@ -6146,11 +6498,29 @@
       <x:c r="G19" s="30"/>
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="30"/>
-      <x:c r="J19" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J15),0),1)</x:f>
-        <x:v>89.2</x:v>
+      <x:c r="J19" s="32" t="n">
+        <x:f>SUM(J4:J16)</x:f>
+        <x:v>1124.0000000000002</x:v>
       </x:c>
       <x:c r="K19" s="30"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="30"/>
+      <x:c r="J20" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
+        <x:v>86.5</x:v>
+      </x:c>
+      <x:c r="K20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-27
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Rf84368c529bb4b39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Re61cdfe2734f44e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R54ecd4dcc73047d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R52ee679d281f4b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf25f5d267cb94f46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rac3871daa08d48dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R4fa1cdde7fa14a5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rcfb5e916cd574136"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R47623ef079d74707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R5756bae3d5b44fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R1a0655f6961c4fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R68be562840604713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R6fe868b208d14e2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rbb5463243b1842c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R5c57aad3bd934a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R74282c0a1a5b468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R982cb0163607439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rd105b92454e3455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rdd481a9f4b414a6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Rd2570a5e72304bd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6704.68</x:v>
+        <x:v>6717.99</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6589.13</x:v>
+        <x:v>6427.17</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>115.6</x:v>
+        <x:v>290.8</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2686.4</x:v>
+        <x:v>2977.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>206.6</x:v>
+        <x:v>212.7</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6787.32</x:v>
+        <x:v>6784.25</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6674.4</x:v>
+        <x:v>6511.37</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>112.9</x:v>
+        <x:v>272.9</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2497.5</x:v>
+        <x:v>2770.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>192.1</x:v>
+        <x:v>197.9</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3699.01</x:v>
+        <x:v>3708.2</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3664.82</x:v>
+        <x:v>3648.3</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>34.2</x:v>
+        <x:v>59.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>771.2</x:v>
+        <x:v>831.1</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>59.3</x:v>
+        <x:v>59.4</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -607,25 +607,25 @@
         <x:v>IM主力</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n">
-        <x:v>6630</x:v>
+        <x:v>6670.8</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
-        <x:v>6494</x:v>
+        <x:v>6333.2</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>136</x:v>
+        <x:v>337.6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G7" s="10" t="n">
-        <x:v>2868</x:v>
+        <x:v>3205.6</x:v>
       </x:c>
       <x:c r="H7" s="10" t="n">
-        <x:v>220.6</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="I7" s="10" t="n">
         <x:v>190</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6711.4</x:v>
+        <x:v>6732.2</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6573.6</x:v>
+        <x:v>6405.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>137.8</x:v>
+        <x:v>326.6</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>2768.4</x:v>
+        <x:v>3095</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>213</x:v>
+        <x:v>221.1</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4049.8</x:v>
+        <x:v>4066.6</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>3996.4</x:v>
+        <x:v>3989.8</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>53.4</x:v>
+        <x:v>76.8</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1124</x:v>
+        <x:v>1200.8</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>86.5</x:v>
+        <x:v>85.8</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-26</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1529,37 +1529,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>6684.93</x:v>
       </x:c>
       <x:c r="D8" s="23" t="n">
-        <x:v>6704.68</x:v>
+        <x:v>6717.99</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>6589.13</x:v>
+        <x:v>6427.17</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>6630.78</x:v>
-      </x:c>
-      <x:c r="G8" s="23" t="n">
+        <x:v>6427.17</x:v>
+      </x:c>
+      <x:c r="G8" s="28" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-103.8</x:v>
+        <x:v>-307.4</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.015408601911040876</x:v>
-      </x:c>
-      <x:c r="I8" s="23" t="n">
+        <x:v>-0.04564224781165782</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>115.6</x:v>
+        <x:v>290.8</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1577,7 +1577,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1654.2</x:v>
+        <x:v>1829.4</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1595,7 +1595,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>413.6</x:v>
+        <x:v>457.4</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -1763,7 +1763,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>6756.46</x:v>
@@ -1772,28 +1772,28 @@
         <x:v>6787.32</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>6674.4</x:v>
+        <x:v>6511.37</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>6712.73</x:v>
-      </x:c>
-      <x:c r="G17" s="23" t="n">
+        <x:v>6511.42</x:v>
+      </x:c>
+      <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-101.7</x:v>
+        <x:v>-303</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.0149256578677045</x:v>
-      </x:c>
-      <x:c r="I17" s="23" t="n">
+        <x:v>-0.04446733700788319</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>112.9</x:v>
+        <x:v>275.9</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1811,7 +1811,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1543.9</x:v>
+        <x:v>1706.9</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -1829,7 +1829,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>386</x:v>
+        <x:v>426.7</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -1997,37 +1997,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3671</x:v>
       </x:c>
       <x:c r="D26" s="23" t="n">
-        <x:v>3699.01</x:v>
+        <x:v>3708.2</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3664.82</x:v>
+        <x:v>3648.3</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3697.52</x:v>
+        <x:v>3648.3</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>7</x:v>
+        <x:v>-42.2</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>0.0019076109340789849</x:v>
-      </x:c>
-      <x:c r="I26" s="23" t="n">
+        <x:v>-0.01142940755674049</x:v>
+      </x:c>
+      <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>34.2</x:v>
+        <x:v>59.9</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2045,7 +2045,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>467.1</x:v>
+        <x:v>492.8</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2063,7 +2063,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>116.8</x:v>
+        <x:v>123.2</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2231,37 +2231,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C35" s="23" t="n">
         <x:v>6618</x:v>
       </x:c>
       <x:c r="D35" s="23" t="n">
-        <x:v>6630</x:v>
+        <x:v>6670.8</x:v>
       </x:c>
       <x:c r="E35" s="23" t="n">
-        <x:v>6494</x:v>
+        <x:v>6333.2</x:v>
       </x:c>
       <x:c r="F35" s="23" t="n">
-        <x:v>6555.8</x:v>
-      </x:c>
-      <x:c r="G35" s="23" t="n">
+        <x:v>6339.2</x:v>
+      </x:c>
+      <x:c r="G35" s="28" t="n">
         <x:f>ROUND(F35-F34,1)</x:f>
-        <x:v>-104.2</x:v>
+        <x:v>-320.8</x:v>
       </x:c>
       <x:c r="H35" s="24" t="n">
         <x:f>IFERROR(F35/F34-1,"")</x:f>
-        <x:v>-0.015645645645645634</x:v>
-      </x:c>
-      <x:c r="I35" s="23" t="n">
+        <x:v>-0.04816816816816816</x:v>
+      </x:c>
+      <x:c r="I35" s="26" t="n">
         <x:f>ROUND(D35-E35,1)</x:f>
-        <x:v>136</x:v>
+        <x:v>337.6</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
         <x:v>IM2612</x:v>
       </x:c>
       <x:c r="K35" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2279,7 +2279,7 @@
       <x:c r="H36" s="30"/>
       <x:c r="I36" s="32" t="n">
         <x:f>ROUND(SUM(I32:I35),1)</x:f>
-        <x:v>1667.2</x:v>
+        <x:v>1868.8</x:v>
       </x:c>
       <x:c r="J36" s="30"/>
       <x:c r="K36" s="30"/>
@@ -2297,7 +2297,7 @@
       <x:c r="H37" s="30"/>
       <x:c r="I37" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I32:I35),0),1)</x:f>
-        <x:v>416.8</x:v>
+        <x:v>467.2</x:v>
       </x:c>
       <x:c r="J37" s="30"/>
       <x:c r="K37" s="30"/>
@@ -2465,37 +2465,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>6700</x:v>
       </x:c>
       <x:c r="D44" s="23" t="n">
-        <x:v>6711.4</x:v>
+        <x:v>6732.2</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
-        <x:v>6573.6</x:v>
+        <x:v>6405.6</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>6637</x:v>
-      </x:c>
-      <x:c r="G44" s="23" t="n">
+        <x:v>6407.6</x:v>
+      </x:c>
+      <x:c r="G44" s="28" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-105</x:v>
+        <x:v>-334.4</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.015574013645802465</x:v>
-      </x:c>
-      <x:c r="I44" s="23" t="n">
+        <x:v>-0.049599525363393626</x:v>
+      </x:c>
+      <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>137.8</x:v>
+        <x:v>326.6</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2513,7 +2513,7 @@
       <x:c r="H45" s="30"/>
       <x:c r="I45" s="32" t="n">
         <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1617.2</x:v>
+        <x:v>1806</x:v>
       </x:c>
       <x:c r="J45" s="30"/>
       <x:c r="K45" s="30"/>
@@ -2531,7 +2531,7 @@
       <x:c r="H46" s="30"/>
       <x:c r="I46" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>404.3</x:v>
+        <x:v>451.5</x:v>
       </x:c>
       <x:c r="J46" s="30"/>
       <x:c r="K46" s="30"/>
@@ -2699,37 +2699,37 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>10月26日</x:v>
+        <x:v>10月26日-10月27日</x:v>
       </x:c>
       <x:c r="C53" s="23" t="n">
         <x:v>4034</x:v>
       </x:c>
       <x:c r="D53" s="23" t="n">
-        <x:v>4049.8</x:v>
+        <x:v>4066.6</x:v>
       </x:c>
       <x:c r="E53" s="23" t="n">
-        <x:v>3996.4</x:v>
+        <x:v>3989.8</x:v>
       </x:c>
       <x:c r="F53" s="23" t="n">
-        <x:v>4049</x:v>
+        <x:v>3991.2</x:v>
       </x:c>
       <x:c r="G53" s="23" t="n">
         <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>-6</x:v>
+        <x:v>-63.8</x:v>
       </x:c>
       <x:c r="H53" s="24" t="n">
         <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>-0.0014796547472256671</x:v>
+        <x:v>-0.015733662145499427</x:v>
       </x:c>
       <x:c r="I53" s="23" t="n">
         <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>53.4</x:v>
+        <x:v>76.8</x:v>
       </x:c>
       <x:c r="J53" s="22" t="str">
         <x:v>IF2612</x:v>
       </x:c>
       <x:c r="K53" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2747,7 +2747,7 @@
       <x:c r="H54" s="30"/>
       <x:c r="I54" s="32" t="n">
         <x:f>ROUND(SUM(I50:I53),1)</x:f>
-        <x:v>675.6</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="J54" s="30"/>
       <x:c r="K54" s="30"/>
@@ -2765,7 +2765,7 @@
       <x:c r="H55" s="30"/>
       <x:c r="I55" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I50:I53),0),1)</x:f>
-        <x:v>168.9</x:v>
+        <x:v>174.8</x:v>
       </x:c>
       <x:c r="J55" s="30"/>
       <x:c r="K55" s="30"/>
@@ -3741,31 +3741,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2686.3999999999996</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>6664.61</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>6717.99</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>6427.17</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>6427.17</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>-203.6</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.030706794675739446</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>290.8</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -3773,11 +3791,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>206.6</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2977.2</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>212.7</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4312,31 +4348,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2497.5</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>6745.72</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>6784.25</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>6511.37</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>6511.42</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>-201.3</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.029989289007601894</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>272.9</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -4344,11 +4398,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>192.1</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>2770.4</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>197.9</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4883,31 +4955,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>771.2</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>3698.44</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>3708.2</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>3648.3</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>3648.3</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>-49.2</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.01331162508924899</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>59.9</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -4915,11 +5005,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>59.3</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>831.1</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>59.4</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5454,31 +5562,49 @@
         <x:v>IM2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2868.0000000000005</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>6622.4</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>6670.8</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>6333.2</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>6339.2</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>-216.6</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.0330394459867599</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>337.6</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>IM2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -5486,11 +5612,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>220.6</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3205.6000000000004</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6025,31 +6169,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>2768.4</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>6700</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>6732.2</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>6405.6</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>6407.6</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="n">
+        <x:v>-229.4</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.03456380894982669</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>326.6</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -6057,11 +6219,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>213</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>3095</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>221.1</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6596,31 +6776,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B19" s="30" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="30"/>
-      <x:c r="D19" s="30"/>
-      <x:c r="E19" s="30"/>
-      <x:c r="F19" s="30"/>
-      <x:c r="G19" s="30"/>
-      <x:c r="H19" s="30"/>
-      <x:c r="I19" s="30"/>
-      <x:c r="J19" s="32" t="n">
-        <x:f>SUM(J4:J16)</x:f>
-        <x:v>1124.0000000000002</x:v>
-      </x:c>
-      <x:c r="K19" s="30"/>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>10月27日</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:v>4059.6</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="n">
+        <x:v>4066.6</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="n">
+        <x:v>3989.8</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="n">
+        <x:v>3991.2</x:v>
+      </x:c>
+      <x:c r="H17" s="23" t="n">
+        <x:v>-57.8</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="n">
+        <x:v>-0.014275129661644903</x:v>
+      </x:c>
+      <x:c r="J17" s="23" t="n">
+        <x:f>ROUND(E17-F17,1)</x:f>
+        <x:v>76.8</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B20" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="C20" s="30"/>
       <x:c r="D20" s="30"/>
       <x:c r="E20" s="30"/>
@@ -6628,11 +6826,29 @@
       <x:c r="G20" s="30"/>
       <x:c r="H20" s="30"/>
       <x:c r="I20" s="30"/>
-      <x:c r="J20" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J16),0),1)</x:f>
-        <x:v>86.5</x:v>
+      <x:c r="J20" s="32" t="n">
+        <x:f>SUM(J4:J17)</x:f>
+        <x:v>1200.8000000000002</x:v>
       </x:c>
       <x:c r="K20" s="30"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="30"/>
+      <x:c r="E21" s="30"/>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="30"/>
+      <x:c r="J21" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
+        <x:v>85.8</x:v>
+      </x:c>
+      <x:c r="K21" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-28
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R222e76c3a43947c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R83396736878943ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R5bda2cc2985b4b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R23a3efc57e804185"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R38bc15203e9d4ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R9fd2f6e157a24849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rc0656cbc880442c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R7bf36d414cea4355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf389d15dac36421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R5ee3883454064011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R44f28365e829494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R31e777f014384505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rfcb4cda6661b4315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R198f0368c7e545b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R588d3b994f2e4f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R2d8f4c28688e48ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R398fdd6a7b804f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R9be525c631444102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rff10f00ffab248d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R4259167678f14b6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-27</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6717.99</x:v>
+        <x:v>6634.76</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6427.17</x:v>
+        <x:v>6444.21</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>290.8</x:v>
+        <x:v>190.6</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>2977.2</x:v>
+        <x:v>3167.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>212.7</x:v>
+        <x:v>211.2</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-27</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6784.25</x:v>
+        <x:v>6694.67</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6511.37</x:v>
+        <x:v>6534.65</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>272.9</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2770.4</x:v>
+        <x:v>2930.4</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>197.9</x:v>
+        <x:v>195.4</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-27</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3708.2</x:v>
+        <x:v>3684.49</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3648.3</x:v>
+        <x:v>3652.37</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>59.9</x:v>
+        <x:v>32.1</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>831.1</x:v>
+        <x:v>863.2</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>59.4</x:v>
+        <x:v>57.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-27</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6732.2</x:v>
+        <x:v>6639.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6405.6</x:v>
+        <x:v>6460.2</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>326.6</x:v>
+        <x:v>179.6</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3095</x:v>
+        <x:v>3274.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>221.1</x:v>
+        <x:v>218.3</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-27</x:v>
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1529,7 +1529,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>10月26日-10月27日</x:v>
+        <x:v>10月26日-10月28日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>6684.93</x:v>
@@ -1541,15 +1541,15 @@
         <x:v>6427.17</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>6427.17</x:v>
+        <x:v>6578.1</x:v>
       </x:c>
       <x:c r="G8" s="28" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-307.4</x:v>
+        <x:v>-156.4</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.04564224781165782</x:v>
+        <x:v>-0.02323095084304072</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
@@ -1559,7 +1559,7 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1763,7 +1763,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>10月26日-10月27日</x:v>
+        <x:v>10月26日-10月28日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>6756.46</x:v>
@@ -1775,15 +1775,15 @@
         <x:v>6511.37</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>6511.42</x:v>
+        <x:v>6640.89</x:v>
       </x:c>
       <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-303</x:v>
+        <x:v>-173.5</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.04446733700788319</x:v>
+        <x:v>-0.025467976825681804</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
@@ -1793,7 +1793,7 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1997,7 +1997,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>10月26日-10月27日</x:v>
+        <x:v>10月26日-10月28日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3671</x:v>
@@ -2009,15 +2009,15 @@
         <x:v>3648.3</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3648.3</x:v>
+        <x:v>3681.47</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-42.2</x:v>
+        <x:v>-9</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.01142940755674049</x:v>
+        <x:v>-0.0024414168346665877</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
@@ -2027,7 +2027,7 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2465,7 +2465,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>10月26日-10月27日</x:v>
+        <x:v>10月26日-10月28日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>6700</x:v>
@@ -2477,15 +2477,15 @@
         <x:v>6405.6</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>6407.6</x:v>
+        <x:v>6564</x:v>
       </x:c>
       <x:c r="G44" s="28" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-334.4</x:v>
+        <x:v>-178</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.049599525363393626</x:v>
+        <x:v>-0.026401661228122264</x:v>
       </x:c>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
@@ -2495,7 +2495,7 @@
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3777,31 +3777,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>2977.2</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>10月28日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>6487.84</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>6634.76</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>6444.21</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>6578.1</x:v>
+      </x:c>
+      <x:c r="H18" s="28" t="n">
+        <x:v>150.9</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.02348311932001179</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>190.6</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -3809,11 +3827,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>212.7</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>3167.7999999999997</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>211.2</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4384,31 +4420,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>2770.4</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>10月28日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>6572.8</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>6694.67</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>6534.65</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>6640.89</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="n">
+        <x:v>129.5</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.019883527709777526</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -4416,11 +4470,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>197.9</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>2930.4</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>195.4</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4991,31 +5063,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>831.1</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>10月28日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>3676.92</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>3684.49</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>3652.37</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>3681.47</x:v>
+      </x:c>
+      <x:c r="H18" s="23" t="n">
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.009091905819148538</x:v>
+      </x:c>
+      <x:c r="J18" s="23" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>32.1</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -5023,11 +5113,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>59.4</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>863.2</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>57.5</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6205,31 +6313,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B20" s="30" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C20" s="30"/>
-      <x:c r="D20" s="30"/>
-      <x:c r="E20" s="30"/>
-      <x:c r="F20" s="30"/>
-      <x:c r="G20" s="30"/>
-      <x:c r="H20" s="30"/>
-      <x:c r="I20" s="30"/>
-      <x:c r="J20" s="32" t="n">
-        <x:f>SUM(J4:J17)</x:f>
-        <x:v>3095</x:v>
-      </x:c>
-      <x:c r="K20" s="30"/>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>10月28日</x:v>
+      </x:c>
+      <x:c r="D18" s="23" t="n">
+        <x:v>6498</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="n">
+        <x:v>6639.8</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="n">
+        <x:v>6460.2</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="n">
+        <x:v>6564</x:v>
+      </x:c>
+      <x:c r="H18" s="28" t="n">
+        <x:v>156.4</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="n">
+        <x:v>0.024408514888569766</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:f>ROUND(E18-F18,1)</x:f>
+        <x:v>179.6</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B21" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="C21" s="30"/>
       <x:c r="D21" s="30"/>
       <x:c r="E21" s="30"/>
@@ -6237,11 +6363,29 @@
       <x:c r="G21" s="30"/>
       <x:c r="H21" s="30"/>
       <x:c r="I21" s="30"/>
-      <x:c r="J21" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J17),0),1)</x:f>
-        <x:v>221.1</x:v>
+      <x:c r="J21" s="32" t="n">
+        <x:f>SUM(J4:J18)</x:f>
+        <x:v>3274.6</x:v>
       </x:c>
       <x:c r="K21" s="30"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="30"/>
+      <x:c r="E22" s="30"/>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="30"/>
+      <x:c r="J22" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
+        <x:v>218.3</x:v>
+      </x:c>
+      <x:c r="K22" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-29
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="Re8248f8243bd43af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R88d7c7138c8f49ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R82ab6425341d4573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R3ae8c5f9ad894a1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R1a3223102ff44c40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="Rf4b563cc7b014783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Rff4d106b9c3e4036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R2949158d057246a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R45df513965fa401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R1e8761ede58a4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R8e64f9b807da4486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R4956363f5bf9492f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Raa32ca7cd04b4a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R5495932a87c04376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rcdcf02723ddc400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R0baaf87c0491466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ref195854249945fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="Rb1160f72410f4741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R42f68d07d7c14af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R39f6d7e0b5644554"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6634.76</x:v>
+        <x:v>6538.05</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6444.21</x:v>
+        <x:v>6378.01</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>190.6</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3167.8</x:v>
+        <x:v>3327.8</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>211.2</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6694.67</x:v>
+        <x:v>6604.65</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6534.65</x:v>
+        <x:v>6450.54</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>160</x:v>
+        <x:v>154.1</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>2930.4</x:v>
+        <x:v>3084.5</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>195.4</x:v>
+        <x:v>192.8</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3684.49</x:v>
+        <x:v>3678.46</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3652.37</x:v>
+        <x:v>3645.26</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>32.1</x:v>
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>863.2</x:v>
+        <x:v>896.4</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>57.5</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6639.8</x:v>
+        <x:v>6533</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6460.2</x:v>
+        <x:v>6358.8</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>179.6</x:v>
+        <x:v>174.2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3274.6</x:v>
+        <x:v>3448.8</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>218.3</x:v>
+        <x:v>215.6</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1529,7 +1529,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>10月26日-10月28日</x:v>
+        <x:v>10月26日-10月29日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>6684.93</x:v>
@@ -1538,28 +1538,28 @@
         <x:v>6717.99</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>6427.17</x:v>
+        <x:v>6378.01</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>6578.1</x:v>
+        <x:v>6378.78</x:v>
       </x:c>
       <x:c r="G8" s="28" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-156.4</x:v>
+        <x:v>-355.8</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.02323095084304072</x:v>
+        <x:v>-0.05282758313473068</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>290.8</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1577,7 +1577,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1829.4</x:v>
+        <x:v>1878.6</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1595,7 +1595,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>457.4</x:v>
+        <x:v>469.7</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -1763,7 +1763,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>10月26日-10月28日</x:v>
+        <x:v>10月26日-10月29日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>6756.46</x:v>
@@ -1772,28 +1772,28 @@
         <x:v>6787.32</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>6511.37</x:v>
+        <x:v>6450.54</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>6640.89</x:v>
+        <x:v>6453.72</x:v>
       </x:c>
       <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-173.5</x:v>
+        <x:v>-360.7</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.025467976825681804</x:v>
+        <x:v>-0.052934650536214156</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>275.9</x:v>
+        <x:v>336.8</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1811,7 +1811,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1706.9</x:v>
+        <x:v>1767.8</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -1829,7 +1829,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>426.7</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -1997,7 +1997,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>10月26日-10月28日</x:v>
+        <x:v>10月26日-10月29日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3671</x:v>
@@ -2006,28 +2006,28 @@
         <x:v>3708.2</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3648.3</x:v>
+        <x:v>3645.26</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3681.47</x:v>
+        <x:v>3651.43</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-9</x:v>
+        <x:v>-39.1</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.0024414168346665877</x:v>
+        <x:v>-0.010581279399969667</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>59.9</x:v>
+        <x:v>62.9</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2045,7 +2045,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>492.8</x:v>
+        <x:v>495.8</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2063,7 +2063,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>123.2</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2465,7 +2465,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>10月26日-10月28日</x:v>
+        <x:v>10月26日-10月29日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>6700</x:v>
@@ -2474,28 +2474,28 @@
         <x:v>6732.2</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
-        <x:v>6405.6</x:v>
+        <x:v>6358.8</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>6564</x:v>
+        <x:v>6374.6</x:v>
       </x:c>
       <x:c r="G44" s="28" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-178</x:v>
+        <x:v>-367.4</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.026401661228122264</x:v>
+        <x:v>-0.05449421536636012</x:v>
       </x:c>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>326.6</x:v>
+        <x:v>373.4</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2513,7 +2513,7 @@
       <x:c r="H45" s="30"/>
       <x:c r="I45" s="32" t="n">
         <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1806</x:v>
+        <x:v>1852.8</x:v>
       </x:c>
       <x:c r="J45" s="30"/>
       <x:c r="K45" s="30"/>
@@ -2531,7 +2531,7 @@
       <x:c r="H46" s="30"/>
       <x:c r="I46" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>451.5</x:v>
+        <x:v>463.2</x:v>
       </x:c>
       <x:c r="J46" s="30"/>
       <x:c r="K46" s="30"/>
@@ -3813,31 +3813,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>3167.7999999999997</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>10月29日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>6538.05</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>6538.05</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>6378.01</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>6378.78</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="n">
+        <x:v>-199.3</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.030300542709901124</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -3845,11 +3863,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>211.2</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>3327.7999999999997</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4456,31 +4492,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>2930.4</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>10月29日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>6604.65</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>6604.65</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>6450.54</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>6453.72</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="n">
+        <x:v>-187.2</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.028184475273645537</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>154.1</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -4488,11 +4542,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>195.4</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>3084.5</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>192.8</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5099,31 +5171,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>863.2</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>10月29日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>3676.77</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>3678.46</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>3645.26</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>3651.43</x:v>
+      </x:c>
+      <x:c r="H19" s="23" t="n">
+        <x:v>-30</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.008159783999326375</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>33.2</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -5131,11 +5221,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>57.5</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>896.4000000000001</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6385,31 +6493,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B21" s="30" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C21" s="30"/>
-      <x:c r="D21" s="30"/>
-      <x:c r="E21" s="30"/>
-      <x:c r="F21" s="30"/>
-      <x:c r="G21" s="30"/>
-      <x:c r="H21" s="30"/>
-      <x:c r="I21" s="30"/>
-      <x:c r="J21" s="32" t="n">
-        <x:f>SUM(J4:J18)</x:f>
-        <x:v>3274.6</x:v>
-      </x:c>
-      <x:c r="K21" s="30"/>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>10月29日</x:v>
+      </x:c>
+      <x:c r="D19" s="23" t="n">
+        <x:v>6532.8</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="n">
+        <x:v>6533</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="n">
+        <x:v>6358.8</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="n">
+        <x:v>6374.6</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="n">
+        <x:v>-189.4</x:v>
+      </x:c>
+      <x:c r="I19" s="24" t="n">
+        <x:v>-0.028854357099329597</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:f>ROUND(E19-F19,1)</x:f>
+        <x:v>174.2</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B22" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="C22" s="30"/>
       <x:c r="D22" s="30"/>
       <x:c r="E22" s="30"/>
@@ -6417,11 +6543,29 @@
       <x:c r="G22" s="30"/>
       <x:c r="H22" s="30"/>
       <x:c r="I22" s="30"/>
-      <x:c r="J22" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J18),0),1)</x:f>
-        <x:v>218.3</x:v>
+      <x:c r="J22" s="32" t="n">
+        <x:f>SUM(J4:J19)</x:f>
+        <x:v>3448.7999999999997</x:v>
       </x:c>
       <x:c r="K22" s="30"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="30"/>
+      <x:c r="E23" s="30"/>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="30"/>
+      <x:c r="J23" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
+        <x:v>215.6</x:v>
+      </x:c>
+      <x:c r="K23" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update amplitude website 2026-10-30
</commit_message>
<xml_diff>
--- a/每日振幅统计.xlsx
+++ b/每日振幅统计.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R4d956480d8ec4733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="R03b2df38777840a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="R816611fa332c4940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="R64aa92b73dd04df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="Rf6750b13b2b8469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R6d8765e031c1424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="Ra49c289202a049dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R878cf571fa854638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="R9f8578c52e7246db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="Ra030e6814e9f497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R6834f71009204e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周振幅统计" sheetId="2" r:id="Rbb9922ace82045e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="3" r:id="Rf5b9d785544b4b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="4" r:id="Rdbdb1c5d96ba4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="5" r:id="R78f14a59bdd24910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="6" r:id="R479b397834d542ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="7" r:id="R47c0d5543ef44199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="8" r:id="R1395b0f3dd7f4db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="9" r:id="Rf4f9d07d3f2d4970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="碳酸锂2610" sheetId="10" r:id="R232877d2cdfd448e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,25 +520,25 @@
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C4" s="10" t="n">
-        <x:v>6538.05</x:v>
+        <x:v>6428.58</x:v>
       </x:c>
       <x:c r="D4" s="10" t="n">
-        <x:v>6378.01</x:v>
+        <x:v>6161.23</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>160</x:v>
+        <x:v>267.4</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G4" s="10" t="n">
-        <x:v>3327.8</x:v>
+        <x:v>3595.2</x:v>
       </x:c>
       <x:c r="H4" s="10" t="n">
-        <x:v>208</x:v>
+        <x:v>211.5</x:v>
       </x:c>
       <x:c r="I4" s="10" t="n">
         <x:v>180</x:v>
@@ -549,25 +549,25 @@
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C5" s="10" t="n">
-        <x:v>6604.65</x:v>
+        <x:v>6483.01</x:v>
       </x:c>
       <x:c r="D5" s="10" t="n">
-        <x:v>6450.54</x:v>
+        <x:v>6266.19</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>154.1</x:v>
+        <x:v>216.8</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G5" s="10" t="n">
-        <x:v>3084.5</x:v>
+        <x:v>3301.3</x:v>
       </x:c>
       <x:c r="H5" s="10" t="n">
-        <x:v>192.8</x:v>
+        <x:v>194.2</x:v>
       </x:c>
       <x:c r="I5" s="10" t="n">
         <x:v>160</x:v>
@@ -578,25 +578,25 @@
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C6" s="10" t="n">
-        <x:v>3678.46</x:v>
+        <x:v>3660.21</x:v>
       </x:c>
       <x:c r="D6" s="10" t="n">
-        <x:v>3645.26</x:v>
+        <x:v>3595.26</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>33.2</x:v>
+        <x:v>64.9</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G6" s="10" t="n">
-        <x:v>896.4</x:v>
+        <x:v>961.3</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
-        <x:v>56</x:v>
+        <x:v>56.5</x:v>
       </x:c>
       <x:c r="I6" s="10" t="n">
         <x:v>50</x:v>
@@ -636,25 +636,25 @@
         <x:v>IC主力</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n">
-        <x:v>6533</x:v>
+        <x:v>6416.8</x:v>
       </x:c>
       <x:c r="D8" s="10" t="n">
-        <x:v>6358.8</x:v>
+        <x:v>6186</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
-        <x:v>174.2</x:v>
+        <x:v>230.8</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G8" s="10" t="n">
-        <x:v>3448.8</x:v>
+        <x:v>3679.6</x:v>
       </x:c>
       <x:c r="H8" s="10" t="n">
-        <x:v>215.6</x:v>
+        <x:v>216.4</x:v>
       </x:c>
       <x:c r="I8" s="10" t="n">
         <x:v>150</x:v>
@@ -665,25 +665,25 @@
         <x:v>IF主力</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C9" s="10" t="n">
-        <x:v>4021.8</x:v>
+        <x:v>4000.8</x:v>
       </x:c>
       <x:c r="D9" s="10" t="n">
-        <x:v>3970.4</x:v>
+        <x:v>3914.2</x:v>
       </x:c>
       <x:c r="E9" s="12" t="n">
-        <x:v>51.4</x:v>
+        <x:v>86.6</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>1292.8</x:v>
+        <x:v>1379.4</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>80.8</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
         <x:v>90</x:v>
@@ -755,7 +755,7 @@
         <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>2026-10-29</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
         <x:v>数据源</x:v>
@@ -1529,7 +1529,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>10月26日-10月29日</x:v>
+        <x:v>10月26日-10月30日</x:v>
       </x:c>
       <x:c r="C8" s="23" t="n">
         <x:v>6684.93</x:v>
@@ -1538,28 +1538,28 @@
         <x:v>6717.99</x:v>
       </x:c>
       <x:c r="E8" s="23" t="n">
-        <x:v>6378.01</x:v>
+        <x:v>6161.23</x:v>
       </x:c>
       <x:c r="F8" s="23" t="n">
-        <x:v>6378.78</x:v>
+        <x:v>6161.23</x:v>
       </x:c>
       <x:c r="G8" s="28" t="n">
         <x:f>ROUND(F8-F7,1)</x:f>
-        <x:v>-355.8</x:v>
+        <x:v>-573.3</x:v>
       </x:c>
       <x:c r="H8" s="24" t="n">
         <x:f>IFERROR(F8/F7-1,"")</x:f>
-        <x:v>-0.05282758313473068</x:v>
+        <x:v>-0.08513115204430888</x:v>
       </x:c>
       <x:c r="I8" s="26" t="n">
         <x:f>ROUND(D8-E8,1)</x:f>
-        <x:v>340</x:v>
+        <x:v>556.8</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
         <x:v>中证1000</x:v>
       </x:c>
       <x:c r="K8" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1577,7 +1577,7 @@
       <x:c r="H9" s="30"/>
       <x:c r="I9" s="32" t="n">
         <x:f>ROUND(SUM(I5:I8),1)</x:f>
-        <x:v>1878.6</x:v>
+        <x:v>2095.4</x:v>
       </x:c>
       <x:c r="J9" s="30"/>
       <x:c r="K9" s="30"/>
@@ -1595,7 +1595,7 @@
       <x:c r="H10" s="30"/>
       <x:c r="I10" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I5:I8),0),1)</x:f>
-        <x:v>469.7</x:v>
+        <x:v>523.8</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30"/>
@@ -1763,7 +1763,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>10月26日-10月29日</x:v>
+        <x:v>10月26日-10月30日</x:v>
       </x:c>
       <x:c r="C17" s="23" t="n">
         <x:v>6756.46</x:v>
@@ -1772,28 +1772,28 @@
         <x:v>6787.32</x:v>
       </x:c>
       <x:c r="E17" s="23" t="n">
-        <x:v>6450.54</x:v>
+        <x:v>6266.19</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n">
-        <x:v>6453.72</x:v>
+        <x:v>6266.19</x:v>
       </x:c>
       <x:c r="G17" s="28" t="n">
         <x:f>ROUND(F17-F16,1)</x:f>
-        <x:v>-360.7</x:v>
+        <x:v>-548.2</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
         <x:f>IFERROR(F17/F16-1,"")</x:f>
-        <x:v>-0.052934650536214156</x:v>
+        <x:v>-0.08045415323929772</x:v>
       </x:c>
       <x:c r="I17" s="26" t="n">
         <x:f>ROUND(D17-E17,1)</x:f>
-        <x:v>336.8</x:v>
+        <x:v>521.1</x:v>
       </x:c>
       <x:c r="J17" s="22" t="str">
         <x:v>中证500</x:v>
       </x:c>
       <x:c r="K17" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1811,7 +1811,7 @@
       <x:c r="H18" s="30"/>
       <x:c r="I18" s="32" t="n">
         <x:f>ROUND(SUM(I14:I17),1)</x:f>
-        <x:v>1767.8</x:v>
+        <x:v>1952.1</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30"/>
@@ -1829,7 +1829,7 @@
       <x:c r="H19" s="30"/>
       <x:c r="I19" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I14:I17),0),1)</x:f>
-        <x:v>442</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30"/>
@@ -1997,7 +1997,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>10月26日-10月29日</x:v>
+        <x:v>10月26日-10月30日</x:v>
       </x:c>
       <x:c r="C26" s="23" t="n">
         <x:v>3671</x:v>
@@ -2006,28 +2006,28 @@
         <x:v>3708.2</x:v>
       </x:c>
       <x:c r="E26" s="23" t="n">
-        <x:v>3645.26</x:v>
+        <x:v>3595.26</x:v>
       </x:c>
       <x:c r="F26" s="23" t="n">
-        <x:v>3651.43</x:v>
+        <x:v>3599.02</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
         <x:f>ROUND(F26-F25,1)</x:f>
-        <x:v>-39.1</x:v>
+        <x:v>-91.5</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
         <x:f>IFERROR(F26/F25-1,"")</x:f>
-        <x:v>-0.010581279399969667</x:v>
+        <x:v>-0.024782684095293828</x:v>
       </x:c>
       <x:c r="I26" s="26" t="n">
         <x:f>ROUND(D26-E26,1)</x:f>
-        <x:v>62.9</x:v>
+        <x:v>112.9</x:v>
       </x:c>
       <x:c r="J26" s="22" t="str">
         <x:v>上证指数</x:v>
       </x:c>
       <x:c r="K26" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2045,7 +2045,7 @@
       <x:c r="H27" s="30"/>
       <x:c r="I27" s="32" t="n">
         <x:f>ROUND(SUM(I23:I26),1)</x:f>
-        <x:v>495.8</x:v>
+        <x:v>545.8</x:v>
       </x:c>
       <x:c r="J27" s="30"/>
       <x:c r="K27" s="30"/>
@@ -2063,7 +2063,7 @@
       <x:c r="H28" s="30"/>
       <x:c r="I28" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I23:I26),0),1)</x:f>
-        <x:v>124</x:v>
+        <x:v>136.5</x:v>
       </x:c>
       <x:c r="J28" s="30"/>
       <x:c r="K28" s="30"/>
@@ -2465,7 +2465,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>10月26日-10月29日</x:v>
+        <x:v>10月26日-10月30日</x:v>
       </x:c>
       <x:c r="C44" s="23" t="n">
         <x:v>6700</x:v>
@@ -2474,28 +2474,28 @@
         <x:v>6732.2</x:v>
       </x:c>
       <x:c r="E44" s="23" t="n">
-        <x:v>6358.8</x:v>
+        <x:v>6186</x:v>
       </x:c>
       <x:c r="F44" s="23" t="n">
-        <x:v>6374.6</x:v>
+        <x:v>6187.2</x:v>
       </x:c>
       <x:c r="G44" s="28" t="n">
         <x:f>ROUND(F44-F43,1)</x:f>
-        <x:v>-367.4</x:v>
+        <x:v>-554.8</x:v>
       </x:c>
       <x:c r="H44" s="24" t="n">
         <x:f>IFERROR(F44/F43-1,"")</x:f>
-        <x:v>-0.05449421536636012</x:v>
+        <x:v>-0.08229012162563043</x:v>
       </x:c>
       <x:c r="I44" s="26" t="n">
         <x:f>ROUND(D44-E44,1)</x:f>
-        <x:v>373.4</x:v>
+        <x:v>546.2</x:v>
       </x:c>
       <x:c r="J44" s="22" t="str">
         <x:v>IC2612</x:v>
       </x:c>
       <x:c r="K44" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2513,7 +2513,7 @@
       <x:c r="H45" s="30"/>
       <x:c r="I45" s="32" t="n">
         <x:f>ROUND(SUM(I41:I44),1)</x:f>
-        <x:v>1852.8</x:v>
+        <x:v>2025.6</x:v>
       </x:c>
       <x:c r="J45" s="30"/>
       <x:c r="K45" s="30"/>
@@ -2531,7 +2531,7 @@
       <x:c r="H46" s="30"/>
       <x:c r="I46" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I41:I44),0),1)</x:f>
-        <x:v>463.2</x:v>
+        <x:v>506.4</x:v>
       </x:c>
       <x:c r="J46" s="30"/>
       <x:c r="K46" s="30"/>
@@ -2699,7 +2699,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>10月26日-10月29日</x:v>
+        <x:v>10月26日-10月30日</x:v>
       </x:c>
       <x:c r="C53" s="23" t="n">
         <x:v>4034</x:v>
@@ -2708,28 +2708,28 @@
         <x:v>4066.6</x:v>
       </x:c>
       <x:c r="E53" s="23" t="n">
-        <x:v>3970.4</x:v>
+        <x:v>3914.2</x:v>
       </x:c>
       <x:c r="F53" s="23" t="n">
-        <x:v>3980.4</x:v>
+        <x:v>3928</x:v>
       </x:c>
       <x:c r="G53" s="23" t="n">
         <x:f>ROUND(F53-F52,1)</x:f>
-        <x:v>-74.6</x:v>
+        <x:v>-127</x:v>
       </x:c>
       <x:c r="H53" s="24" t="n">
         <x:f>IFERROR(F53/F52-1,"")</x:f>
-        <x:v>-0.018397040690505517</x:v>
+        <x:v>-0.03131935881627623</x:v>
       </x:c>
       <x:c r="I53" s="26" t="n">
         <x:f>ROUND(D53-E53,1)</x:f>
-        <x:v>96.2</x:v>
+        <x:v>152.4</x:v>
       </x:c>
       <x:c r="J53" s="22" t="str">
         <x:v>IF2612</x:v>
       </x:c>
       <x:c r="K53" s="22" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2747,7 +2747,7 @@
       <x:c r="H54" s="30"/>
       <x:c r="I54" s="32" t="n">
         <x:f>ROUND(SUM(I50:I53),1)</x:f>
-        <x:v>718.4</x:v>
+        <x:v>774.6</x:v>
       </x:c>
       <x:c r="J54" s="30"/>
       <x:c r="K54" s="30"/>
@@ -2765,7 +2765,7 @@
       <x:c r="H55" s="30"/>
       <x:c r="I55" s="34" t="n">
         <x:f>ROUND(IFERROR(AVERAGE(I50:I53),0),1)</x:f>
-        <x:v>179.6</x:v>
+        <x:v>193.7</x:v>
       </x:c>
       <x:c r="J55" s="30"/>
       <x:c r="K55" s="30"/>
@@ -3849,31 +3849,49 @@
         <x:v>中证1000</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>3327.7999999999997</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>10月30日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>6243.98</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>6428.58</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>6161.23</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>6161.23</x:v>
+      </x:c>
+      <x:c r="H20" s="28" t="n">
+        <x:v>-217.6</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.034105267778478</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>267.4</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证1000</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -3881,11 +3899,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>208</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>3595.2</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>211.5</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4528,31 +4564,49 @@
         <x:v>中证500</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>3084.5</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>10月30日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>6318.16</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>6483.01</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>6266.19</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>6266.19</x:v>
+      </x:c>
+      <x:c r="H20" s="28" t="n">
+        <x:v>-187.5</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.029057659768319755</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>216.8</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>中证500</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -4560,11 +4614,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>192.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>3301.3</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>194.2</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5207,31 +5279,49 @@
         <x:v>上证指数</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>896.4000000000001</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>10月30日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3605.65</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>3660.21</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3595.26</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>3599.02</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-52.4</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.01435328076945197</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>64.9</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>上证指数</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -5239,11 +5329,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>56</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>961.3000000000001</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>56.5</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6565,31 +6673,49 @@
         <x:v>IC2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>3448.7999999999997</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>10月30日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>6247.8</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>6416.8</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>6186</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>6187.2</x:v>
+      </x:c>
+      <x:c r="H20" s="28" t="n">
+        <x:v>-187.4</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.02939792300693389</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>230.8</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>IC2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -6597,11 +6723,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>215.6</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>3679.6</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>216.4</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7244,31 +7388,49 @@
         <x:v>IF2612</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="31" t="str">
-        <x:v>合计</x:v>
-      </x:c>
-      <x:c r="B22" s="30" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C22" s="30"/>
-      <x:c r="D22" s="30"/>
-      <x:c r="E22" s="30"/>
-      <x:c r="F22" s="30"/>
-      <x:c r="G22" s="30"/>
-      <x:c r="H22" s="30"/>
-      <x:c r="I22" s="30"/>
-      <x:c r="J22" s="32" t="n">
-        <x:f>SUM(J4:J19)</x:f>
-        <x:v>1292.8000000000002</x:v>
-      </x:c>
-      <x:c r="K22" s="30"/>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>10月30日</x:v>
+      </x:c>
+      <x:c r="D20" s="23" t="n">
+        <x:v>3936.4</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="n">
+        <x:v>4000.8</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="n">
+        <x:v>3914.2</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="n">
+        <x:v>3928</x:v>
+      </x:c>
+      <x:c r="H20" s="23" t="n">
+        <x:v>-52.4</x:v>
+      </x:c>
+      <x:c r="I20" s="24" t="n">
+        <x:v>-0.013164506079791027</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:f>ROUND(E20-F20,1)</x:f>
+        <x:v>86.6</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="str">
+        <x:v>IF2612</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="31" t="str">
-        <x:v>均值</x:v>
-      </x:c>
-      <x:c r="B23" s="30"/>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="C23" s="30"/>
       <x:c r="D23" s="30"/>
       <x:c r="E23" s="30"/>
@@ -7276,11 +7438,29 @@
       <x:c r="G23" s="30"/>
       <x:c r="H23" s="30"/>
       <x:c r="I23" s="30"/>
-      <x:c r="J23" s="34" t="n">
-        <x:f>ROUND(IFERROR(AVERAGE(J4:J19),0),1)</x:f>
-        <x:v>80.8</x:v>
+      <x:c r="J23" s="32" t="n">
+        <x:f>SUM(J4:J20)</x:f>
+        <x:v>1379.4</x:v>
       </x:c>
       <x:c r="K23" s="30"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="31" t="str">
+        <x:v>均值</x:v>
+      </x:c>
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="30"/>
+      <x:c r="E24" s="30"/>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="30"/>
+      <x:c r="J24" s="34" t="n">
+        <x:f>ROUND(IFERROR(AVERAGE(J4:J20),0),1)</x:f>
+        <x:v>81.1</x:v>
+      </x:c>
+      <x:c r="K24" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>